<commit_message>
Atualiza programacao-hoje.xlsx (14/09/2026 15:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3283CE51-E0C7-4434-BEAA-A881EE318FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74FE1944-98F9-4560-90E2-63DB9D1AC4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FAVINCO EMBALAGENS 1197" sheetId="150" r:id="rId1"/>
@@ -33138,6 +33138,9 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC1CA626-F30A-4671-8B85-D3FC298D272A}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -33342,1121 +33345,1121 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="116">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="161">
         <v>1</v>
       </c>
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="116" t="s">
+      <c r="C3" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E3" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="116">
+      <c r="E3" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="161">
         <v>262497</v>
       </c>
-      <c r="G3" s="116" t="s">
+      <c r="G3" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H3" s="116">
+      <c r="H3" s="161">
         <v>225</v>
       </c>
-      <c r="I3" s="117">
+      <c r="I3" s="163">
         <v>1.548</v>
       </c>
-      <c r="J3" s="117">
+      <c r="J3" s="163">
         <v>1.62</v>
       </c>
-      <c r="K3" s="116" t="s">
+      <c r="K3" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="113">
+      <c r="L3" s="163">
         <v>564.24599999999998</v>
       </c>
-      <c r="M3" s="115">
+      <c r="M3" s="164">
         <v>364.5</v>
       </c>
-      <c r="N3" s="112">
+      <c r="N3" s="165">
         <v>0.1013</v>
       </c>
-      <c r="O3" s="114">
+      <c r="O3" s="166">
         <v>6.08</v>
       </c>
-      <c r="P3" s="111">
+      <c r="P3" s="161">
         <v>334.6</v>
       </c>
-      <c r="Q3" s="111">
+      <c r="Q3" s="161">
         <v>1</v>
       </c>
-      <c r="R3" s="111">
+      <c r="R3" s="161">
         <v>1600</v>
       </c>
-      <c r="S3" s="113">
+      <c r="S3" s="163">
         <v>1.548</v>
       </c>
-      <c r="T3" s="111">
+      <c r="T3" s="161">
         <v>52</v>
       </c>
-      <c r="U3" s="112">
+      <c r="U3" s="165">
         <v>3.2500000000000001E-2</v>
       </c>
-      <c r="V3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="111" t="s">
+      <c r="V3" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="111" t="s">
+      <c r="X3" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="161" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="111" t="s">
+      <c r="AB3" s="161" t="s">
         <v>553</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="116">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="161">
         <v>2</v>
       </c>
-      <c r="B4" s="118" t="s">
+      <c r="B4" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="116" t="s">
+      <c r="C4" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="116" t="s">
+      <c r="D4" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E4" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="116">
+      <c r="E4" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="161">
         <v>262501</v>
       </c>
-      <c r="G4" s="116" t="s">
+      <c r="G4" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H4" s="116">
+      <c r="H4" s="161">
         <v>510</v>
       </c>
-      <c r="I4" s="117">
+      <c r="I4" s="163">
         <v>0.76600000000000001</v>
       </c>
-      <c r="J4" s="117">
+      <c r="J4" s="163">
         <v>1.43</v>
       </c>
-      <c r="K4" s="116" t="s">
+      <c r="K4" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="113">
+      <c r="L4" s="163">
         <v>558.64400000000001</v>
       </c>
-      <c r="M4" s="115">
+      <c r="M4" s="164">
         <v>364.6</v>
       </c>
-      <c r="N4" s="112">
+      <c r="N4" s="165">
         <v>5.0599999999999999E-2</v>
       </c>
-      <c r="O4" s="114">
+      <c r="O4" s="166">
         <v>3.04</v>
       </c>
-      <c r="P4" s="111">
+      <c r="P4" s="161">
         <v>331.3</v>
       </c>
-      <c r="Q4" s="111">
+      <c r="Q4" s="161">
         <v>2</v>
       </c>
-      <c r="R4" s="111">
+      <c r="R4" s="161">
         <v>1600</v>
       </c>
-      <c r="S4" s="113">
+      <c r="S4" s="163">
         <v>1.532</v>
       </c>
-      <c r="T4" s="111">
+      <c r="T4" s="161">
         <v>68</v>
       </c>
-      <c r="U4" s="112">
+      <c r="U4" s="165">
         <v>4.2500000000000003E-2</v>
       </c>
-      <c r="V4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="111" t="s">
+      <c r="V4" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="111" t="s">
+      <c r="X4" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="161" t="s">
         <v>30</v>
       </c>
-      <c r="AB4" s="111" t="s">
+      <c r="AB4" s="161" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="116">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="161">
         <v>3</v>
       </c>
-      <c r="B5" s="118" t="s">
+      <c r="B5" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="116" t="s">
+      <c r="C5" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="116" t="s">
+      <c r="D5" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E5" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="116">
+      <c r="E5" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="161">
         <v>262495</v>
       </c>
-      <c r="G5" s="116" t="s">
+      <c r="G5" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H5" s="116">
+      <c r="H5" s="161">
         <v>395</v>
       </c>
-      <c r="I5" s="117">
+      <c r="I5" s="163">
         <v>0.69</v>
       </c>
-      <c r="J5" s="117">
+      <c r="J5" s="163">
         <v>2.0699999999999998</v>
       </c>
-      <c r="K5" s="116" t="s">
+      <c r="K5" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="113">
+      <c r="L5" s="163">
         <v>564.178</v>
       </c>
-      <c r="M5" s="115">
+      <c r="M5" s="164">
         <v>408.8</v>
       </c>
-      <c r="N5" s="112">
+      <c r="N5" s="165">
         <v>5.6800000000000003E-2</v>
       </c>
-      <c r="O5" s="114">
+      <c r="O5" s="166">
         <v>3.41</v>
       </c>
-      <c r="P5" s="111">
+      <c r="P5" s="161">
         <v>334.6</v>
       </c>
-      <c r="Q5" s="111">
+      <c r="Q5" s="161">
         <v>2</v>
       </c>
-      <c r="R5" s="111">
+      <c r="R5" s="161">
         <v>1400</v>
       </c>
-      <c r="S5" s="113">
+      <c r="S5" s="163">
         <v>1.38</v>
       </c>
-      <c r="T5" s="111">
+      <c r="T5" s="161">
         <v>20</v>
       </c>
-      <c r="U5" s="112">
+      <c r="U5" s="165">
         <v>1.43E-2</v>
       </c>
-      <c r="V5" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="111" t="s">
+      <c r="V5" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="111" t="s">
+      <c r="X5" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="161" t="s">
         <v>30</v>
       </c>
-      <c r="AB5" s="111" t="s">
+      <c r="AB5" s="161" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="116">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="161">
         <v>4</v>
       </c>
-      <c r="B6" s="118" t="s">
+      <c r="B6" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="116" t="s">
+      <c r="C6" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="116" t="s">
+      <c r="D6" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E6" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="116">
+      <c r="E6" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="161">
         <v>262496</v>
       </c>
-      <c r="G6" s="116" t="s">
+      <c r="G6" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H6" s="116">
+      <c r="H6" s="161">
         <v>610</v>
       </c>
-      <c r="I6" s="117">
+      <c r="I6" s="163">
         <v>1.29</v>
       </c>
-      <c r="J6" s="117">
+      <c r="J6" s="163">
         <v>1.59</v>
       </c>
-      <c r="K6" s="116" t="s">
+      <c r="K6" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="113">
+      <c r="L6" s="163">
         <v>1251.171</v>
       </c>
-      <c r="M6" s="115">
+      <c r="M6" s="164">
         <v>969.9</v>
       </c>
-      <c r="N6" s="112">
+      <c r="N6" s="165">
         <v>0.26939999999999997</v>
       </c>
-      <c r="O6" s="114">
+      <c r="O6" s="166">
         <v>16.170000000000002</v>
       </c>
-      <c r="P6" s="111">
+      <c r="P6" s="161">
         <v>741.9</v>
       </c>
-      <c r="Q6" s="111">
+      <c r="Q6" s="161">
         <v>1</v>
       </c>
-      <c r="R6" s="111">
+      <c r="R6" s="161">
         <v>1350</v>
       </c>
-      <c r="S6" s="113">
+      <c r="S6" s="163">
         <v>1.29</v>
       </c>
-      <c r="T6" s="111">
+      <c r="T6" s="161">
         <v>60</v>
       </c>
-      <c r="U6" s="112">
+      <c r="U6" s="165">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="V6" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="111" t="s">
+      <c r="V6" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="111" t="s">
+      <c r="X6" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="161" t="s">
         <v>32</v>
       </c>
-      <c r="AB6" s="111" t="s">
+      <c r="AB6" s="161" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="116">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="161">
         <v>5</v>
       </c>
-      <c r="B7" s="118" t="s">
+      <c r="B7" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="116" t="s">
+      <c r="C7" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="116" t="s">
+      <c r="D7" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E7" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="116">
+      <c r="E7" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="161">
         <v>262494</v>
       </c>
-      <c r="G7" s="116" t="s">
+      <c r="G7" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H7" s="116">
+      <c r="H7" s="161">
         <v>700</v>
       </c>
-      <c r="I7" s="117">
+      <c r="I7" s="163">
         <v>1.0740000000000001</v>
       </c>
-      <c r="J7" s="117">
+      <c r="J7" s="163">
         <v>1.27</v>
       </c>
-      <c r="K7" s="116" t="s">
+      <c r="K7" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="113">
+      <c r="L7" s="163">
         <v>954.78599999999994</v>
       </c>
-      <c r="M7" s="115">
+      <c r="M7" s="164">
         <v>889</v>
       </c>
-      <c r="N7" s="112">
+      <c r="N7" s="165">
         <v>0.24690000000000001</v>
       </c>
-      <c r="O7" s="114">
+      <c r="O7" s="166">
         <v>14.82</v>
       </c>
-      <c r="P7" s="111">
+      <c r="P7" s="161">
         <v>566.20000000000005</v>
       </c>
-      <c r="Q7" s="111">
+      <c r="Q7" s="161">
         <v>1</v>
       </c>
-      <c r="R7" s="111">
+      <c r="R7" s="161">
         <v>1100</v>
       </c>
-      <c r="S7" s="113">
+      <c r="S7" s="163">
         <v>1.0740000000000001</v>
       </c>
-      <c r="T7" s="111">
+      <c r="T7" s="161">
         <v>26</v>
       </c>
-      <c r="U7" s="112">
+      <c r="U7" s="165">
         <v>2.3599999999999999E-2</v>
       </c>
-      <c r="V7" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="111" t="s">
+      <c r="V7" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="111" t="s">
+      <c r="X7" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="161" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="111" t="s">
+      <c r="AB7" s="161" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="116">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="161">
         <v>6</v>
       </c>
-      <c r="B8" s="118" t="s">
+      <c r="B8" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C8" s="116" t="s">
+      <c r="C8" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="116" t="s">
+      <c r="D8" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E8" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="116">
+      <c r="E8" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="161">
         <v>262502</v>
       </c>
-      <c r="G8" s="116" t="s">
+      <c r="G8" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H8" s="116">
+      <c r="H8" s="161">
         <v>550</v>
       </c>
-      <c r="I8" s="117">
+      <c r="I8" s="163">
         <v>0.95599999999999996</v>
       </c>
-      <c r="J8" s="117">
+      <c r="J8" s="163">
         <v>1.23</v>
       </c>
-      <c r="K8" s="116" t="s">
+      <c r="K8" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="113">
+      <c r="L8" s="163">
         <v>646.73400000000004</v>
       </c>
-      <c r="M8" s="115">
+      <c r="M8" s="164">
         <v>676.5</v>
       </c>
-      <c r="N8" s="112">
+      <c r="N8" s="165">
         <v>0.18790000000000001</v>
       </c>
-      <c r="O8" s="114">
+      <c r="O8" s="166">
         <v>11.28</v>
       </c>
-      <c r="P8" s="111">
+      <c r="P8" s="161">
         <v>383.5</v>
       </c>
-      <c r="Q8" s="111">
+      <c r="Q8" s="161">
         <v>1</v>
       </c>
-      <c r="R8" s="111">
+      <c r="R8" s="161">
         <v>1000</v>
       </c>
-      <c r="S8" s="113">
+      <c r="S8" s="163">
         <v>0.95599999999999996</v>
       </c>
-      <c r="T8" s="111">
+      <c r="T8" s="161">
         <v>44</v>
       </c>
-      <c r="U8" s="112">
+      <c r="U8" s="165">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="V8" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="111" t="s">
+      <c r="V8" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X8" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z8" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA8" s="111" t="s">
+      <c r="X8" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8" s="161" t="s">
         <v>30</v>
       </c>
-      <c r="AB8" s="111" t="s">
+      <c r="AB8" s="161" t="s">
         <v>549</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A9" s="116">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="161">
         <v>7</v>
       </c>
-      <c r="B9" s="118" t="s">
+      <c r="B9" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="116" t="s">
+      <c r="D9" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E9" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="116">
+      <c r="E9" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="161">
         <v>262503</v>
       </c>
-      <c r="G9" s="116" t="s">
+      <c r="G9" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H9" s="116">
+      <c r="H9" s="161">
         <v>550</v>
       </c>
-      <c r="I9" s="117">
+      <c r="I9" s="163">
         <v>0.97099999999999997</v>
       </c>
-      <c r="J9" s="117">
+      <c r="J9" s="163">
         <v>1.26</v>
       </c>
-      <c r="K9" s="116" t="s">
+      <c r="K9" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="113">
+      <c r="L9" s="163">
         <v>672.90300000000002</v>
       </c>
-      <c r="M9" s="115">
+      <c r="M9" s="164">
         <v>693</v>
       </c>
-      <c r="N9" s="112">
+      <c r="N9" s="165">
         <v>0.1925</v>
       </c>
-      <c r="O9" s="114">
+      <c r="O9" s="166">
         <v>11.55</v>
       </c>
-      <c r="P9" s="111">
+      <c r="P9" s="161">
         <v>399</v>
       </c>
-      <c r="Q9" s="111">
+      <c r="Q9" s="161">
         <v>1</v>
       </c>
-      <c r="R9" s="111">
+      <c r="R9" s="161">
         <v>1000</v>
       </c>
-      <c r="S9" s="113">
+      <c r="S9" s="163">
         <v>0.97099999999999997</v>
       </c>
-      <c r="T9" s="111">
+      <c r="T9" s="161">
         <v>29</v>
       </c>
-      <c r="U9" s="112">
+      <c r="U9" s="165">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="V9" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="111" t="s">
+      <c r="V9" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X9" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z9" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA9" s="111" t="s">
+      <c r="X9" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z9" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA9" s="161" t="s">
         <v>30</v>
       </c>
-      <c r="AB9" s="111" t="s">
+      <c r="AB9" s="161" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A10" s="116">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="161">
         <v>8</v>
       </c>
-      <c r="B10" s="118" t="s">
+      <c r="B10" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="116" t="s">
+      <c r="C10" s="161" t="s">
         <v>296</v>
       </c>
-      <c r="D10" s="116" t="s">
+      <c r="D10" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E10" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="116">
+      <c r="E10" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="161">
         <v>262504</v>
       </c>
-      <c r="G10" s="116" t="s">
+      <c r="G10" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H10" s="116">
+      <c r="H10" s="161">
         <v>375</v>
       </c>
-      <c r="I10" s="117">
+      <c r="I10" s="163">
         <v>1.44</v>
       </c>
-      <c r="J10" s="117">
+      <c r="J10" s="163">
         <v>1.538</v>
       </c>
-      <c r="K10" s="116" t="s">
+      <c r="K10" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L10" s="113">
+      <c r="L10" s="163">
         <v>830.52</v>
       </c>
-      <c r="M10" s="115">
+      <c r="M10" s="164">
         <v>576.79999999999995</v>
       </c>
-      <c r="N10" s="112">
+      <c r="N10" s="165">
         <v>0.16020000000000001</v>
       </c>
-      <c r="O10" s="114">
+      <c r="O10" s="166">
         <v>9.61</v>
       </c>
-      <c r="P10" s="111">
+      <c r="P10" s="161">
         <v>318.10000000000002</v>
       </c>
-      <c r="Q10" s="111">
+      <c r="Q10" s="161">
         <v>1</v>
       </c>
-      <c r="R10" s="111">
+      <c r="R10" s="161">
         <v>1500</v>
       </c>
-      <c r="S10" s="113">
+      <c r="S10" s="163">
         <v>1.44</v>
       </c>
-      <c r="T10" s="111">
+      <c r="T10" s="161">
         <v>60</v>
       </c>
-      <c r="U10" s="112">
+      <c r="U10" s="165">
         <v>0.04</v>
       </c>
-      <c r="V10" s="111" t="s">
+      <c r="V10" s="161" t="s">
         <v>42</v>
       </c>
-      <c r="W10" s="111" t="s">
+      <c r="W10" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X10" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="111" t="s">
+      <c r="X10" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="161" t="s">
         <v>39</v>
       </c>
-      <c r="AB10" s="111" t="s">
+      <c r="AB10" s="161" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" s="116">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="161">
         <v>9</v>
       </c>
-      <c r="B11" s="118" t="s">
+      <c r="B11" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C11" s="116" t="s">
+      <c r="C11" s="161" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="116" t="s">
+      <c r="D11" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E11" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="116">
+      <c r="E11" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="161">
         <v>262505</v>
       </c>
-      <c r="G11" s="116" t="s">
+      <c r="G11" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H11" s="116">
+      <c r="H11" s="161">
         <v>1750</v>
       </c>
-      <c r="I11" s="117">
+      <c r="I11" s="163">
         <v>0.74</v>
       </c>
-      <c r="J11" s="117">
+      <c r="J11" s="163">
         <v>0.75</v>
       </c>
-      <c r="K11" s="116" t="s">
+      <c r="K11" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="113">
+      <c r="L11" s="163">
         <v>971.25</v>
       </c>
-      <c r="M11" s="115">
+      <c r="M11" s="164">
         <v>656.3</v>
       </c>
-      <c r="N11" s="112">
+      <c r="N11" s="165">
         <v>9.11E-2</v>
       </c>
-      <c r="O11" s="114">
+      <c r="O11" s="166">
         <v>5.47</v>
       </c>
-      <c r="P11" s="111">
+      <c r="P11" s="161">
         <v>335.1</v>
       </c>
-      <c r="Q11" s="111">
+      <c r="Q11" s="161">
         <v>2</v>
       </c>
-      <c r="R11" s="111">
+      <c r="R11" s="161">
         <v>1500</v>
       </c>
-      <c r="S11" s="113">
+      <c r="S11" s="163">
         <v>1.48</v>
       </c>
-      <c r="T11" s="111">
+      <c r="T11" s="161">
         <v>20</v>
       </c>
-      <c r="U11" s="112">
+      <c r="U11" s="165">
         <v>1.3299999999999999E-2</v>
       </c>
-      <c r="V11" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="111" t="s">
+      <c r="V11" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="161" t="s">
         <v>30</v>
       </c>
-      <c r="AB11" s="111" t="s">
+      <c r="AB11" s="161" t="s">
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" s="116">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="161">
         <v>10</v>
       </c>
-      <c r="B12" s="118" t="s">
+      <c r="B12" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="116" t="s">
+      <c r="C12" s="161" t="s">
         <v>296</v>
       </c>
-      <c r="D12" s="116" t="s">
+      <c r="D12" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E12" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="116">
+      <c r="E12" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="161">
         <v>262499</v>
       </c>
-      <c r="G12" s="116" t="s">
+      <c r="G12" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H12" s="116">
+      <c r="H12" s="161">
         <v>3200</v>
       </c>
-      <c r="I12" s="117">
+      <c r="I12" s="163">
         <v>0.46100000000000002</v>
       </c>
-      <c r="J12" s="117">
+      <c r="J12" s="163">
         <v>1.32</v>
       </c>
-      <c r="K12" s="116" t="s">
+      <c r="K12" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L12" s="113">
+      <c r="L12" s="163">
         <v>1947.2639999999999</v>
       </c>
-      <c r="M12" s="115">
+      <c r="M12" s="164">
         <v>1408</v>
       </c>
-      <c r="N12" s="112">
+      <c r="N12" s="165">
         <v>0.13039999999999999</v>
       </c>
-      <c r="O12" s="114">
+      <c r="O12" s="166">
         <v>7.82</v>
       </c>
-      <c r="P12" s="111">
+      <c r="P12" s="161">
         <v>745.8</v>
       </c>
-      <c r="Q12" s="111">
+      <c r="Q12" s="161">
         <v>3</v>
       </c>
-      <c r="R12" s="111">
+      <c r="R12" s="161">
         <v>1450</v>
       </c>
-      <c r="S12" s="113">
+      <c r="S12" s="163">
         <v>1.383</v>
       </c>
-      <c r="T12" s="111">
+      <c r="T12" s="161">
         <v>67</v>
       </c>
-      <c r="U12" s="112">
+      <c r="U12" s="165">
         <v>4.6199999999999998E-2</v>
       </c>
-      <c r="V12" s="111" t="s">
+      <c r="V12" s="161" t="s">
         <v>42</v>
       </c>
-      <c r="W12" s="111" t="s">
+      <c r="W12" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X12" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="111" t="s">
+      <c r="X12" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="161" t="s">
         <v>32</v>
       </c>
-      <c r="AB12" s="111" t="s">
+      <c r="AB12" s="161" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" s="116">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="161">
         <v>11</v>
       </c>
-      <c r="B13" s="118" t="s">
+      <c r="B13" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C13" s="116" t="s">
+      <c r="C13" s="161" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="116" t="s">
+      <c r="D13" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E13" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="116">
+      <c r="E13" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="161">
         <v>262498</v>
       </c>
-      <c r="G13" s="116" t="s">
+      <c r="G13" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H13" s="116">
+      <c r="H13" s="161">
         <v>3550</v>
       </c>
-      <c r="I13" s="117">
+      <c r="I13" s="163">
         <v>0.3</v>
       </c>
-      <c r="J13" s="117">
+      <c r="J13" s="163">
         <v>0.9</v>
       </c>
-      <c r="K13" s="116" t="s">
+      <c r="K13" s="161" t="s">
         <v>34</v>
       </c>
-      <c r="L13" s="113">
+      <c r="L13" s="163">
         <v>958.5</v>
       </c>
-      <c r="M13" s="115">
+      <c r="M13" s="164">
         <v>1065</v>
       </c>
-      <c r="N13" s="112">
+      <c r="N13" s="165">
         <v>9.8599999999999993E-2</v>
       </c>
-      <c r="O13" s="114">
+      <c r="O13" s="166">
         <v>5.92</v>
       </c>
-      <c r="P13" s="111">
+      <c r="P13" s="161">
         <v>330.7</v>
       </c>
-      <c r="Q13" s="111">
+      <c r="Q13" s="161">
         <v>3</v>
       </c>
-      <c r="R13" s="111">
+      <c r="R13" s="161">
         <v>950</v>
       </c>
-      <c r="S13" s="113">
+      <c r="S13" s="163">
         <v>0.9</v>
       </c>
-      <c r="T13" s="111">
+      <c r="T13" s="161">
         <v>50</v>
       </c>
-      <c r="U13" s="112">
+      <c r="U13" s="165">
         <v>5.2600000000000001E-2</v>
       </c>
-      <c r="V13" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W13" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="X13" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y13" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="111" t="s">
+      <c r="V13" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="161" t="s">
         <v>33</v>
       </c>
-      <c r="AB13" s="111" t="s">
+      <c r="AB13" s="161" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A14" s="116">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="161">
         <v>12</v>
       </c>
-      <c r="B14" s="118" t="s">
+      <c r="B14" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="C14" s="116" t="s">
+      <c r="C14" s="161" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="116" t="s">
+      <c r="D14" s="161" t="s">
         <v>543</v>
       </c>
-      <c r="E14" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="116">
+      <c r="E14" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="161">
         <v>262500</v>
       </c>
-      <c r="G14" s="116" t="s">
+      <c r="G14" s="161" t="s">
         <v>542</v>
       </c>
-      <c r="H14" s="116">
+      <c r="H14" s="161">
         <v>6000</v>
       </c>
-      <c r="I14" s="117">
+      <c r="I14" s="163">
         <v>0.374</v>
       </c>
-      <c r="J14" s="117">
+      <c r="J14" s="163">
         <v>0.44</v>
       </c>
-      <c r="K14" s="116" t="s">
+      <c r="K14" s="161" t="s">
         <v>541</v>
       </c>
-      <c r="L14" s="113">
+      <c r="L14" s="163">
         <v>987.36</v>
       </c>
-      <c r="M14" s="115">
+      <c r="M14" s="164">
         <v>1320</v>
       </c>
-      <c r="N14" s="112">
+      <c r="N14" s="165">
         <v>0.18329999999999999</v>
       </c>
-      <c r="O14" s="114">
+      <c r="O14" s="166">
         <v>11</v>
       </c>
-      <c r="P14" s="111">
+      <c r="P14" s="161">
         <v>340.6</v>
       </c>
-      <c r="Q14" s="111">
+      <c r="Q14" s="161">
         <v>2</v>
       </c>
-      <c r="R14" s="111">
+      <c r="R14" s="161">
         <v>800</v>
       </c>
-      <c r="S14" s="113">
+      <c r="S14" s="163">
         <v>0.748</v>
       </c>
-      <c r="T14" s="111">
+      <c r="T14" s="161">
         <v>52</v>
       </c>
-      <c r="U14" s="112">
+      <c r="U14" s="165">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="V14" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W14" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="X14" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y14" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z14" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA14" s="111" t="s">
+      <c r="V14" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="161" t="s">
         <v>33</v>
       </c>
-      <c r="AB14" s="111" t="s">
+      <c r="AB14" s="161" t="s">
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="G15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="H15" s="110">
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="168">
         <v>18415</v>
       </c>
-      <c r="I15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="J15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="K15" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="L15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="M15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="N15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="O15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="P15" s="109">
+      <c r="I15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="J15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="M15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="O15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="P15" s="168">
         <v>5161.3999999999996</v>
       </c>
-      <c r="Q15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="R15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="S15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="T15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="U15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="V15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="W15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="X15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB15" s="109" t="s">
+      <c r="Q15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="R15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="S15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="T15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="U15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="V15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="W15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="X15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB15" s="168" t="s">
         <v>27</v>
       </c>
     </row>
@@ -34465,7 +34468,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="94" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (14/09/2026 16:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74FE1944-98F9-4560-90E2-63DB9D1AC4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45F1420-DE6A-44A6-A928-8DE15E351028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FAVINCO EMBALAGENS 1197" sheetId="150" r:id="rId1"/>
@@ -2887,7 +2887,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3120,21 +3120,24 @@
     <col min="3" max="3" width="7.77734375" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.6640625" style="108" customWidth="1"/>
-    <col min="6" max="6" width="8.77734375" style="108" customWidth="1"/>
+    <col min="6" max="6" width="8.44140625" style="108" customWidth="1"/>
     <col min="7" max="7" width="4.44140625" style="108" customWidth="1"/>
-    <col min="8" max="8" width="6" style="108" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" style="108" customWidth="1"/>
-    <col min="10" max="10" width="6.77734375" style="108" customWidth="1"/>
-    <col min="11" max="11" width="22.77734375" style="108" customWidth="1"/>
+    <col min="8" max="8" width="5.6640625" style="108" customWidth="1"/>
+    <col min="9" max="9" width="6.109375" style="108" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="108" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="108" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="8.77734375" style="108" customWidth="1"/>
-    <col min="18" max="18" width="13.77734375" style="108" customWidth="1"/>
-    <col min="19" max="19" width="11.77734375" style="108" customWidth="1"/>
+    <col min="16" max="16" width="7.109375" style="108" customWidth="1"/>
+    <col min="17" max="17" width="3.88671875" style="108" customWidth="1"/>
+    <col min="18" max="18" width="6.5546875" style="108" customWidth="1"/>
+    <col min="19" max="19" width="6.77734375" style="108" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="22" max="26" width="11.77734375" style="108" customWidth="1"/>
+    <col min="22" max="23" width="8.109375" style="108" customWidth="1"/>
+    <col min="24" max="24" width="8.6640625" style="108" customWidth="1"/>
+    <col min="25" max="26" width="11.77734375" style="108" customWidth="1"/>
     <col min="27" max="27" width="10.77734375" style="108" customWidth="1"/>
     <col min="28" max="28" width="16.77734375" style="108" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="108"/>
@@ -3226,7 +3229,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -3312,491 +3315,501 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="116">
+    <row r="3" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="161">
         <v>1</v>
       </c>
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="162" t="s">
         <v>480</v>
       </c>
-      <c r="C3" s="116" t="s">
+      <c r="C3" s="161" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="161" t="s">
         <v>602</v>
       </c>
-      <c r="E3" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="116">
+      <c r="E3" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="161">
         <v>262575</v>
       </c>
-      <c r="G3" s="116" t="s">
+      <c r="G3" s="161" t="s">
         <v>668</v>
       </c>
-      <c r="H3" s="116">
+      <c r="H3" s="161">
         <v>600</v>
       </c>
-      <c r="I3" s="117">
+      <c r="I3" s="163">
         <v>0.54300000000000004</v>
       </c>
-      <c r="J3" s="117">
+      <c r="J3" s="163">
         <v>0.95</v>
       </c>
-      <c r="K3" s="116" t="s">
+      <c r="K3" s="161" t="s">
         <v>667</v>
       </c>
-      <c r="L3" s="113">
+      <c r="L3" s="163">
         <v>309.51</v>
       </c>
-      <c r="M3" s="115">
+      <c r="M3" s="164">
         <v>285</v>
       </c>
-      <c r="N3" s="112">
+      <c r="N3" s="165">
         <v>3.9600000000000003E-2</v>
       </c>
-      <c r="O3" s="114">
+      <c r="O3" s="166">
         <v>2.38</v>
       </c>
-      <c r="P3" s="111">
+      <c r="P3" s="161">
         <v>193.8</v>
       </c>
-      <c r="Q3" s="111">
+      <c r="Q3" s="161">
         <v>2</v>
       </c>
-      <c r="R3" s="111">
+      <c r="R3" s="161">
         <v>1150</v>
       </c>
-      <c r="S3" s="113">
+      <c r="S3" s="163">
         <v>1.0860000000000001</v>
       </c>
-      <c r="T3" s="111">
+      <c r="T3" s="161">
         <v>64</v>
       </c>
-      <c r="U3" s="112">
+      <c r="U3" s="165">
         <v>5.57E-2</v>
       </c>
-      <c r="V3" s="111" t="s">
+      <c r="V3" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="W3" s="111" t="s">
+      <c r="W3" s="161" t="s">
         <v>40</v>
       </c>
-      <c r="X3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="111" t="s">
+      <c r="X3" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="AA3" s="111" t="s">
+      <c r="AA3" s="161" t="s">
         <v>39</v>
       </c>
-      <c r="AB3" s="111" t="s">
+      <c r="AB3" s="161" t="s">
         <v>666</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="116"/>
-      <c r="B4" s="118" t="s">
+    <row r="4" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="161">
+        <v>5</v>
+      </c>
+      <c r="B4" s="162" t="s">
         <v>480</v>
       </c>
-      <c r="C4" s="116" t="s">
-        <v>670</v>
+      <c r="C4" s="161" t="s">
+        <v>62</v>
       </c>
       <c r="D4" s="200">
         <v>46279</v>
       </c>
-      <c r="E4" s="116"/>
-      <c r="F4" s="116">
-        <v>262576</v>
-      </c>
-      <c r="G4" s="116">
+      <c r="E4" s="161"/>
+      <c r="F4" s="161">
+        <v>262579</v>
+      </c>
+      <c r="G4" s="161">
         <v>69</v>
       </c>
-      <c r="H4" s="116">
-        <v>500</v>
-      </c>
-      <c r="I4" s="117">
-        <v>0.45</v>
-      </c>
-      <c r="J4" s="117">
-        <v>1.59</v>
-      </c>
-      <c r="K4" s="116" t="s">
-        <v>671</v>
-      </c>
-      <c r="L4" s="113">
-        <v>357.75</v>
-      </c>
-      <c r="M4" s="115">
-        <v>397.5</v>
-      </c>
-      <c r="N4" s="112">
-        <v>5.5199999999999999E-2</v>
-      </c>
-      <c r="O4" s="114">
-        <v>3.31</v>
-      </c>
-      <c r="P4" s="111">
-        <v>138.80000000000001</v>
-      </c>
-      <c r="Q4" s="111">
+      <c r="H4" s="161">
+        <v>300</v>
+      </c>
+      <c r="I4" s="163">
+        <v>1.113</v>
+      </c>
+      <c r="J4" s="163">
+        <v>2.41</v>
+      </c>
+      <c r="K4" s="161" t="s">
+        <v>676</v>
+      </c>
+      <c r="L4" s="163">
+        <v>804.69899999999996</v>
+      </c>
+      <c r="M4" s="164">
+        <v>723</v>
+      </c>
+      <c r="N4" s="165">
+        <v>0.20080000000000001</v>
+      </c>
+      <c r="O4" s="166">
+        <v>12.05</v>
+      </c>
+      <c r="P4" s="161">
+        <v>503.7</v>
+      </c>
+      <c r="Q4" s="161">
+        <v>1</v>
+      </c>
+      <c r="R4" s="161">
+        <v>1150</v>
+      </c>
+      <c r="S4" s="163">
+        <v>1.113</v>
+      </c>
+      <c r="T4" s="161">
+        <v>37</v>
+      </c>
+      <c r="U4" s="165">
+        <v>3.2199999999999999E-2</v>
+      </c>
+      <c r="V4" s="161" t="s">
+        <v>29</v>
+      </c>
+      <c r="W4" s="161" t="s">
+        <v>40</v>
+      </c>
+      <c r="X4" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="161" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA4" s="161">
         <v>2</v>
       </c>
-      <c r="R4" s="111">
-        <v>1150</v>
-      </c>
-      <c r="S4" s="113">
-        <v>0.9</v>
-      </c>
-      <c r="T4" s="111">
-        <v>250</v>
-      </c>
-      <c r="U4" s="112">
-        <v>0.21740000000000001</v>
-      </c>
-      <c r="V4" s="111" t="s">
-        <v>40</v>
-      </c>
-      <c r="W4" s="111" t="s">
-        <v>29</v>
-      </c>
-      <c r="X4" s="111" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y4" s="111"/>
-      <c r="Z4" s="111"/>
-      <c r="AA4" s="111">
-        <v>1</v>
-      </c>
-      <c r="AB4" s="111" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="116"/>
-      <c r="B5" s="118" t="s">
+      <c r="AB4" s="161" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="161">
+        <v>2</v>
+      </c>
+      <c r="B5" s="162" t="s">
         <v>480</v>
       </c>
-      <c r="C5" s="116" t="s">
+      <c r="C5" s="161" t="s">
         <v>670</v>
       </c>
       <c r="D5" s="200">
         <v>46279</v>
       </c>
-      <c r="E5" s="116"/>
-      <c r="F5" s="116">
-        <v>262578</v>
-      </c>
-      <c r="G5" s="116">
+      <c r="E5" s="161"/>
+      <c r="F5" s="161">
+        <v>262576</v>
+      </c>
+      <c r="G5" s="161">
         <v>69</v>
       </c>
-      <c r="H5" s="116">
-        <v>600</v>
-      </c>
-      <c r="I5" s="117">
-        <v>0.54600000000000004</v>
-      </c>
-      <c r="J5" s="117">
-        <v>1.41</v>
-      </c>
-      <c r="K5" s="116" t="s">
-        <v>674</v>
-      </c>
-      <c r="L5" s="113">
-        <v>461.916</v>
-      </c>
-      <c r="M5" s="115">
-        <v>423</v>
-      </c>
-      <c r="N5" s="112">
-        <v>5.8700000000000002E-2</v>
-      </c>
-      <c r="O5" s="114">
-        <v>3.52</v>
-      </c>
-      <c r="P5" s="111">
-        <v>179.2</v>
-      </c>
-      <c r="Q5" s="111">
+      <c r="H5" s="161">
+        <v>500</v>
+      </c>
+      <c r="I5" s="163">
+        <v>0.45</v>
+      </c>
+      <c r="J5" s="163">
+        <v>1.59</v>
+      </c>
+      <c r="K5" s="161" t="s">
+        <v>671</v>
+      </c>
+      <c r="L5" s="163">
+        <v>357.75</v>
+      </c>
+      <c r="M5" s="164">
+        <v>397.5</v>
+      </c>
+      <c r="N5" s="165">
+        <v>5.5199999999999999E-2</v>
+      </c>
+      <c r="O5" s="166">
+        <v>3.31</v>
+      </c>
+      <c r="P5" s="161">
+        <v>138.80000000000001</v>
+      </c>
+      <c r="Q5" s="161">
         <v>2</v>
       </c>
-      <c r="R5" s="111">
+      <c r="R5" s="161">
         <v>1150</v>
       </c>
-      <c r="S5" s="113">
-        <v>1.0920000000000001</v>
-      </c>
-      <c r="T5" s="111">
-        <v>58</v>
-      </c>
-      <c r="U5" s="112">
-        <v>5.04E-2</v>
-      </c>
-      <c r="V5" s="111" t="s">
+      <c r="S5" s="163">
+        <v>0.9</v>
+      </c>
+      <c r="T5" s="161">
+        <v>250</v>
+      </c>
+      <c r="U5" s="165">
+        <v>0.21740000000000001</v>
+      </c>
+      <c r="V5" s="161" t="s">
         <v>40</v>
       </c>
-      <c r="W5" s="111" t="s">
+      <c r="W5" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="111" t="s">
+      <c r="X5" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="Y5" s="111"/>
-      <c r="Z5" s="111"/>
-      <c r="AA5" s="111">
+      <c r="Y5" s="161"/>
+      <c r="Z5" s="161"/>
+      <c r="AA5" s="161">
         <v>1</v>
       </c>
-      <c r="AB5" s="111" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="116"/>
-      <c r="B6" s="118" t="s">
+      <c r="AB5" s="161" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="161">
+        <v>3</v>
+      </c>
+      <c r="B6" s="162" t="s">
         <v>480</v>
       </c>
-      <c r="C6" s="116" t="s">
+      <c r="C6" s="161" t="s">
         <v>670</v>
       </c>
       <c r="D6" s="200">
         <v>46279</v>
       </c>
-      <c r="E6" s="116"/>
-      <c r="F6" s="116">
-        <v>262577</v>
-      </c>
-      <c r="G6" s="116">
+      <c r="E6" s="161"/>
+      <c r="F6" s="161">
+        <v>262578</v>
+      </c>
+      <c r="G6" s="161">
         <v>69</v>
       </c>
-      <c r="H6" s="116">
-        <v>1000</v>
-      </c>
-      <c r="I6" s="117">
-        <v>0.52500000000000002</v>
-      </c>
-      <c r="J6" s="117">
-        <v>1.29</v>
-      </c>
-      <c r="K6" s="116" t="s">
-        <v>672</v>
-      </c>
-      <c r="L6" s="113">
-        <v>677.25</v>
-      </c>
-      <c r="M6" s="115">
-        <v>645</v>
-      </c>
-      <c r="N6" s="112">
-        <v>8.9599999999999999E-2</v>
-      </c>
-      <c r="O6" s="114">
-        <v>5.38</v>
-      </c>
-      <c r="P6" s="111">
-        <v>262.8</v>
-      </c>
-      <c r="Q6" s="111">
+      <c r="H6" s="161">
+        <v>600</v>
+      </c>
+      <c r="I6" s="163">
+        <v>0.54600000000000004</v>
+      </c>
+      <c r="J6" s="163">
+        <v>1.41</v>
+      </c>
+      <c r="K6" s="161" t="s">
+        <v>674</v>
+      </c>
+      <c r="L6" s="163">
+        <v>461.916</v>
+      </c>
+      <c r="M6" s="164">
+        <v>423</v>
+      </c>
+      <c r="N6" s="165">
+        <v>5.8700000000000002E-2</v>
+      </c>
+      <c r="O6" s="166">
+        <v>3.52</v>
+      </c>
+      <c r="P6" s="161">
+        <v>179.2</v>
+      </c>
+      <c r="Q6" s="161">
         <v>2</v>
       </c>
-      <c r="R6" s="111">
-        <v>1100</v>
-      </c>
-      <c r="S6" s="113">
-        <v>1.05</v>
-      </c>
-      <c r="T6" s="111">
-        <v>50</v>
-      </c>
-      <c r="U6" s="112">
-        <v>4.5499999999999999E-2</v>
-      </c>
-      <c r="V6" s="111" t="s">
+      <c r="R6" s="161">
+        <v>1150</v>
+      </c>
+      <c r="S6" s="163">
+        <v>1.0920000000000001</v>
+      </c>
+      <c r="T6" s="161">
+        <v>58</v>
+      </c>
+      <c r="U6" s="165">
+        <v>5.04E-2</v>
+      </c>
+      <c r="V6" s="161" t="s">
         <v>40</v>
       </c>
-      <c r="W6" s="111" t="s">
+      <c r="W6" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="111" t="s">
+      <c r="X6" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="Y6" s="111"/>
-      <c r="Z6" s="111"/>
-      <c r="AA6" s="111">
-        <v>2</v>
-      </c>
-      <c r="AB6" s="111" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="116"/>
-      <c r="B7" s="118" t="s">
+      <c r="Y6" s="161"/>
+      <c r="Z6" s="161"/>
+      <c r="AA6" s="161">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="161" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="161">
+        <v>4</v>
+      </c>
+      <c r="B7" s="162" t="s">
         <v>480</v>
       </c>
-      <c r="C7" s="116" t="s">
-        <v>62</v>
+      <c r="C7" s="161" t="s">
+        <v>670</v>
       </c>
       <c r="D7" s="200">
         <v>46279</v>
       </c>
-      <c r="E7" s="116"/>
-      <c r="F7" s="116">
-        <v>262579</v>
-      </c>
-      <c r="G7" s="116">
+      <c r="E7" s="161"/>
+      <c r="F7" s="161">
+        <v>262577</v>
+      </c>
+      <c r="G7" s="161">
         <v>69</v>
       </c>
-      <c r="H7" s="116">
-        <v>300</v>
-      </c>
-      <c r="I7" s="117">
-        <v>1.113</v>
-      </c>
-      <c r="J7" s="117">
-        <v>2.41</v>
-      </c>
-      <c r="K7" s="116" t="s">
-        <v>676</v>
-      </c>
-      <c r="L7" s="113">
-        <v>804.69899999999996</v>
-      </c>
-      <c r="M7" s="115">
-        <v>723</v>
-      </c>
-      <c r="N7" s="112">
-        <v>0.20080000000000001</v>
-      </c>
-      <c r="O7" s="114">
-        <v>12.05</v>
-      </c>
-      <c r="P7" s="111">
-        <v>503.7</v>
-      </c>
-      <c r="Q7" s="111">
-        <v>1</v>
-      </c>
-      <c r="R7" s="111">
-        <v>1150</v>
-      </c>
-      <c r="S7" s="113">
-        <v>1.113</v>
-      </c>
-      <c r="T7" s="111">
-        <v>37</v>
-      </c>
-      <c r="U7" s="112">
-        <v>3.2199999999999999E-2</v>
-      </c>
-      <c r="V7" s="111" t="s">
+      <c r="H7" s="161">
+        <v>1000</v>
+      </c>
+      <c r="I7" s="163">
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="J7" s="163">
+        <v>1.29</v>
+      </c>
+      <c r="K7" s="161" t="s">
+        <v>672</v>
+      </c>
+      <c r="L7" s="163">
+        <v>677.25</v>
+      </c>
+      <c r="M7" s="164">
+        <v>645</v>
+      </c>
+      <c r="N7" s="165">
+        <v>8.9599999999999999E-2</v>
+      </c>
+      <c r="O7" s="166">
+        <v>5.38</v>
+      </c>
+      <c r="P7" s="161">
+        <v>262.8</v>
+      </c>
+      <c r="Q7" s="161">
+        <v>2</v>
+      </c>
+      <c r="R7" s="161">
+        <v>1100</v>
+      </c>
+      <c r="S7" s="163">
+        <v>1.05</v>
+      </c>
+      <c r="T7" s="161">
+        <v>50</v>
+      </c>
+      <c r="U7" s="165">
+        <v>4.5499999999999999E-2</v>
+      </c>
+      <c r="V7" s="161" t="s">
+        <v>40</v>
+      </c>
+      <c r="W7" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="W7" s="111" t="s">
-        <v>40</v>
-      </c>
-      <c r="X7" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="111" t="s">
+      <c r="X7" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="AA7" s="111">
+      <c r="Y7" s="161"/>
+      <c r="Z7" s="161"/>
+      <c r="AA7" s="161">
         <v>2</v>
       </c>
-      <c r="AB7" s="111" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="110">
-        <v>600</v>
-      </c>
-      <c r="I8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="N8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="O8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="109">
-        <v>193.8</v>
-      </c>
-      <c r="Q8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="R8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="T8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="V8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="W8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="X8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB8" s="109" t="s">
+      <c r="AB7" s="161" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="168">
+        <f>SUM(H3:H7)</f>
+        <v>3000</v>
+      </c>
+      <c r="I8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="168">
+        <f>SUM(P3:P7)</f>
+        <v>1278.3</v>
+      </c>
+      <c r="Q8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="168" t="s">
         <v>27</v>
       </c>
     </row>
@@ -31996,7 +32009,8 @@
         <v>27</v>
       </c>
       <c r="H6" s="157">
-        <v>550</v>
+        <f>SUM(H3:H5)</f>
+        <v>3550</v>
       </c>
       <c r="I6" s="157" t="s">
         <v>27</v>
@@ -32020,7 +32034,8 @@
         <v>27</v>
       </c>
       <c r="P6" s="157">
-        <v>116</v>
+        <f>SUM(P3:P5)</f>
+        <v>405.9</v>
       </c>
       <c r="Q6" s="157" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (15/09/2026 10:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51D4E5CA-76F0-4112-9CC5-C2FAB367F7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6A4196-E620-41F3-AED5-10AFD3F573EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3471,433 +3471,433 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28">
-      <c r="A3" s="34">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="5" t="s">
         <v>680</v>
       </c>
-      <c r="E3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="34">
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
         <v>262601</v>
       </c>
-      <c r="G3" s="34" t="s">
+      <c r="G3" s="5" t="s">
         <v>704</v>
       </c>
-      <c r="H3" s="34">
+      <c r="H3" s="5">
         <v>1000</v>
       </c>
-      <c r="I3" s="35">
+      <c r="I3" s="7">
         <v>0.71199999999999997</v>
       </c>
-      <c r="J3" s="35">
+      <c r="J3" s="7">
         <v>2.19</v>
       </c>
-      <c r="K3" s="34" t="s">
+      <c r="K3" s="5" t="s">
         <v>709</v>
       </c>
-      <c r="L3" s="31">
+      <c r="L3" s="7">
         <v>1559.28</v>
       </c>
-      <c r="M3" s="33">
+      <c r="M3" s="9">
         <v>1095</v>
       </c>
-      <c r="N3" s="30">
+      <c r="N3" s="6">
         <v>0.15210000000000001</v>
       </c>
-      <c r="O3" s="32">
+      <c r="O3" s="8">
         <v>9.1300000000000008</v>
       </c>
-      <c r="P3" s="29">
+      <c r="P3" s="5">
         <v>838.9</v>
       </c>
-      <c r="Q3" s="29">
+      <c r="Q3" s="5">
         <v>2</v>
       </c>
-      <c r="R3" s="29">
+      <c r="R3" s="5">
         <v>1450</v>
       </c>
-      <c r="S3" s="31">
+      <c r="S3" s="7">
         <v>1.4239999999999999</v>
       </c>
-      <c r="T3" s="29">
+      <c r="T3" s="5">
         <v>26</v>
       </c>
-      <c r="U3" s="30">
+      <c r="U3" s="6">
         <v>1.7899999999999999E-2</v>
       </c>
-      <c r="V3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="29" t="s">
+      <c r="V3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="29" t="s">
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="AB3" s="29" t="s">
+      <c r="AB3" s="5" t="s">
         <v>708</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
-      <c r="A4" s="34">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="5" t="s">
         <v>680</v>
       </c>
-      <c r="E4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="34">
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
         <v>262600</v>
       </c>
-      <c r="G4" s="34" t="s">
+      <c r="G4" s="5" t="s">
         <v>704</v>
       </c>
-      <c r="H4" s="34">
+      <c r="H4" s="5">
         <v>900</v>
       </c>
-      <c r="I4" s="35">
+      <c r="I4" s="7">
         <v>0.64200000000000002</v>
       </c>
-      <c r="J4" s="35">
+      <c r="J4" s="7">
         <v>2.0779999999999998</v>
       </c>
-      <c r="K4" s="34" t="s">
+      <c r="K4" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="L4" s="31">
+      <c r="L4" s="7">
         <v>1200.6679999999999</v>
       </c>
-      <c r="M4" s="33">
+      <c r="M4" s="9">
         <v>935.1</v>
       </c>
-      <c r="N4" s="30">
+      <c r="N4" s="6">
         <v>0.12989999999999999</v>
       </c>
-      <c r="O4" s="32">
+      <c r="O4" s="8">
         <v>7.79</v>
       </c>
-      <c r="P4" s="29">
+      <c r="P4" s="5">
         <v>646</v>
       </c>
-      <c r="Q4" s="29">
+      <c r="Q4" s="5">
         <v>2</v>
       </c>
-      <c r="R4" s="29">
+      <c r="R4" s="5">
         <v>1350</v>
       </c>
-      <c r="S4" s="31">
+      <c r="S4" s="7">
         <v>1.284</v>
       </c>
-      <c r="T4" s="29">
+      <c r="T4" s="5">
         <v>66</v>
       </c>
-      <c r="U4" s="30">
+      <c r="U4" s="6">
         <v>4.8899999999999999E-2</v>
       </c>
-      <c r="V4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="29" t="s">
+      <c r="V4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="29" t="s">
+      <c r="X4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="AB4" s="29" t="s">
+      <c r="AB4" s="5" t="s">
         <v>707</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
-      <c r="A5" s="34">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="5" t="s">
         <v>680</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="34">
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
         <v>262599</v>
       </c>
-      <c r="G5" s="34" t="s">
+      <c r="G5" s="5" t="s">
         <v>704</v>
       </c>
-      <c r="H5" s="34">
+      <c r="H5" s="5">
         <v>450</v>
       </c>
-      <c r="I5" s="35">
+      <c r="I5" s="7">
         <v>0.622</v>
       </c>
-      <c r="J5" s="35">
+      <c r="J5" s="7">
         <v>2.2000000000000002</v>
       </c>
-      <c r="K5" s="34" t="s">
+      <c r="K5" s="5" t="s">
         <v>706</v>
       </c>
-      <c r="L5" s="31">
+      <c r="L5" s="7">
         <v>615.78</v>
       </c>
-      <c r="M5" s="33">
+      <c r="M5" s="9">
         <v>495</v>
       </c>
-      <c r="N5" s="30">
+      <c r="N5" s="6">
         <v>6.88E-2</v>
       </c>
-      <c r="O5" s="32">
+      <c r="O5" s="8">
         <v>4.13</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="5">
         <v>331.3</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="5">
         <v>2</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="5">
         <v>1300</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="7">
         <v>1.244</v>
       </c>
-      <c r="T5" s="29">
+      <c r="T5" s="5">
         <v>56</v>
       </c>
-      <c r="U5" s="30">
+      <c r="U5" s="6">
         <v>4.3099999999999999E-2</v>
       </c>
-      <c r="V5" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="29" t="s">
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="29" t="s">
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AB5" s="29" t="s">
+      <c r="AB5" s="5" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="6" spans="1:28">
-      <c r="A6" s="34">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="5">
         <v>4</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="5" t="s">
         <v>680</v>
       </c>
-      <c r="E6" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="34">
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
         <v>262598</v>
       </c>
-      <c r="G6" s="34" t="s">
+      <c r="G6" s="5" t="s">
         <v>704</v>
       </c>
-      <c r="H6" s="34">
+      <c r="H6" s="5">
         <v>550</v>
       </c>
-      <c r="I6" s="35">
+      <c r="I6" s="7">
         <v>0.96199999999999997</v>
       </c>
-      <c r="J6" s="35">
+      <c r="J6" s="7">
         <v>2.1190000000000002</v>
       </c>
-      <c r="K6" s="34" t="s">
+      <c r="K6" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L6" s="31">
+      <c r="L6" s="7">
         <v>1121.163</v>
       </c>
-      <c r="M6" s="33">
+      <c r="M6" s="9">
         <v>1165.5</v>
       </c>
-      <c r="N6" s="30">
+      <c r="N6" s="6">
         <v>0.32369999999999999</v>
       </c>
-      <c r="O6" s="32">
+      <c r="O6" s="8">
         <v>19.420000000000002</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="5">
         <v>603.20000000000005</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="5">
         <v>1</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="5">
         <v>1000</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="7">
         <v>0.96199999999999997</v>
       </c>
-      <c r="T6" s="29">
+      <c r="T6" s="5">
         <v>38</v>
       </c>
-      <c r="U6" s="30">
+      <c r="U6" s="6">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="V6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="29" t="s">
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="29" t="s">
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AB6" s="29" t="s">
+      <c r="AB6" s="5" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="7" spans="1:28">
-      <c r="A7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="28">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="11">
         <v>2900</v>
       </c>
-      <c r="I7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="27">
+      <c r="I7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P7" s="11">
         <v>2419.3000000000002</v>
       </c>
-      <c r="Q7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB7" s="27" t="s">
+      <c r="Q7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB7" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (15/09/2026 14:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F3C1CD4-46EC-4BD2-A68C-77BCDB3D04CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1688667D-7199-447B-B9B4-AFA4325846F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>
@@ -36271,7 +36271,7 @@
         <v>624</v>
       </c>
       <c r="H13" s="161">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="I13" s="163">
         <v>0.432</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (15/09/2026 14:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1688667D-7199-447B-B9B4-AFA4325846F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE7989C1-838F-4DFE-A69D-179E27CD3EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6668" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6685" uniqueCount="728">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2241,6 +2241,18 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - IPE EMBALAGENS LTDA - PCBOX EMBALAGENS LTDA  —  OF: 001203</t>
+  </si>
+  <si>
+    <t>W55R15</t>
+  </si>
+  <si>
+    <t>1156x1820</t>
+  </si>
+  <si>
+    <t>150x345x150</t>
+  </si>
+  <si>
+    <t>665x1546</t>
   </si>
 </sst>
 </file>
@@ -2466,7 +2478,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="216">
+  <cellXfs count="228">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3038,6 +3050,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3081,6 +3096,37 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5610,88 +5656,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="202" t="s">
+      <c r="A1" s="203" t="s">
         <v>554</v>
       </c>
-      <c r="B1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="202" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="202" t="s">
+      <c r="B1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="203" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5781,89 +5827,89 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="203">
+    <row r="3" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="204">
         <v>1</v>
       </c>
-      <c r="B3" s="204" t="s">
+      <c r="B3" s="205" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="203" t="s">
+      <c r="C3" s="204" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="203" t="s">
+      <c r="D3" s="204" t="s">
         <v>543</v>
       </c>
-      <c r="E3" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="203">
+      <c r="E3" s="204" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="204">
         <v>262497</v>
       </c>
-      <c r="G3" s="203" t="s">
+      <c r="G3" s="204" t="s">
         <v>542</v>
       </c>
-      <c r="H3" s="203">
+      <c r="H3" s="204">
         <v>225</v>
       </c>
-      <c r="I3" s="205">
+      <c r="I3" s="206">
         <v>1.548</v>
       </c>
-      <c r="J3" s="205">
+      <c r="J3" s="206">
         <v>1.62</v>
       </c>
-      <c r="K3" s="203" t="s">
+      <c r="K3" s="204" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="205">
+      <c r="L3" s="206">
         <v>564.24599999999998</v>
       </c>
-      <c r="M3" s="206">
+      <c r="M3" s="207">
         <v>364.5</v>
       </c>
-      <c r="N3" s="207">
+      <c r="N3" s="208">
         <v>0.1013</v>
       </c>
-      <c r="O3" s="208">
+      <c r="O3" s="209">
         <v>6.08</v>
       </c>
-      <c r="P3" s="203">
+      <c r="P3" s="204">
         <v>334.6</v>
       </c>
-      <c r="Q3" s="203">
+      <c r="Q3" s="204">
         <v>1</v>
       </c>
-      <c r="R3" s="203">
+      <c r="R3" s="204">
         <v>1600</v>
       </c>
-      <c r="S3" s="205">
+      <c r="S3" s="206">
         <v>1.548</v>
       </c>
-      <c r="T3" s="203">
+      <c r="T3" s="204">
         <v>52</v>
       </c>
-      <c r="U3" s="207">
+      <c r="U3" s="208">
         <v>3.2500000000000001E-2</v>
       </c>
-      <c r="V3" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="203" t="s">
+      <c r="V3" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="204" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="203" t="s">
+      <c r="X3" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="204" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="203" t="s">
+      <c r="AB3" s="204" t="s">
         <v>553</v>
       </c>
     </row>
@@ -5953,261 +5999,261 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="203">
+    <row r="5" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="204">
         <v>3</v>
       </c>
-      <c r="B5" s="204" t="s">
+      <c r="B5" s="205" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="203" t="s">
+      <c r="C5" s="204" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="203" t="s">
+      <c r="D5" s="204" t="s">
         <v>543</v>
       </c>
-      <c r="E5" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="203">
+      <c r="E5" s="204" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="204">
         <v>262495</v>
       </c>
-      <c r="G5" s="203" t="s">
+      <c r="G5" s="204" t="s">
         <v>542</v>
       </c>
-      <c r="H5" s="203">
+      <c r="H5" s="204">
         <v>395</v>
       </c>
-      <c r="I5" s="205">
+      <c r="I5" s="206">
         <v>0.69</v>
       </c>
-      <c r="J5" s="205">
+      <c r="J5" s="206">
         <v>2.0699999999999998</v>
       </c>
-      <c r="K5" s="203" t="s">
+      <c r="K5" s="204" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="205">
+      <c r="L5" s="206">
         <v>564.178</v>
       </c>
-      <c r="M5" s="206">
+      <c r="M5" s="207">
         <v>408.8</v>
       </c>
-      <c r="N5" s="207">
+      <c r="N5" s="208">
         <v>5.6800000000000003E-2</v>
       </c>
-      <c r="O5" s="208">
+      <c r="O5" s="209">
         <v>3.41</v>
       </c>
-      <c r="P5" s="203">
+      <c r="P5" s="204">
         <v>334.6</v>
       </c>
-      <c r="Q5" s="203">
+      <c r="Q5" s="204">
         <v>2</v>
       </c>
-      <c r="R5" s="203">
+      <c r="R5" s="204">
         <v>1400</v>
       </c>
-      <c r="S5" s="205">
+      <c r="S5" s="206">
         <v>1.38</v>
       </c>
-      <c r="T5" s="203">
+      <c r="T5" s="204">
         <v>20</v>
       </c>
-      <c r="U5" s="207">
+      <c r="U5" s="208">
         <v>1.43E-2</v>
       </c>
-      <c r="V5" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="203" t="s">
+      <c r="V5" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="204" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="203" t="s">
+      <c r="X5" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="204" t="s">
         <v>30</v>
       </c>
-      <c r="AB5" s="203" t="s">
+      <c r="AB5" s="204" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="203">
+    <row r="6" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="204">
         <v>4</v>
       </c>
-      <c r="B6" s="204" t="s">
+      <c r="B6" s="205" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="203" t="s">
+      <c r="C6" s="204" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="203" t="s">
+      <c r="D6" s="204" t="s">
         <v>543</v>
       </c>
-      <c r="E6" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="203">
+      <c r="E6" s="204" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="204">
         <v>262496</v>
       </c>
-      <c r="G6" s="203" t="s">
+      <c r="G6" s="204" t="s">
         <v>542</v>
       </c>
-      <c r="H6" s="203">
+      <c r="H6" s="204">
         <v>610</v>
       </c>
-      <c r="I6" s="205">
+      <c r="I6" s="206">
         <v>1.29</v>
       </c>
-      <c r="J6" s="205">
+      <c r="J6" s="206">
         <v>1.59</v>
       </c>
-      <c r="K6" s="203" t="s">
+      <c r="K6" s="204" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="205">
+      <c r="L6" s="206">
         <v>1251.171</v>
       </c>
-      <c r="M6" s="206">
+      <c r="M6" s="207">
         <v>969.9</v>
       </c>
-      <c r="N6" s="207">
+      <c r="N6" s="208">
         <v>0.26939999999999997</v>
       </c>
-      <c r="O6" s="208">
+      <c r="O6" s="209">
         <v>16.170000000000002</v>
       </c>
-      <c r="P6" s="203">
+      <c r="P6" s="204">
         <v>741.9</v>
       </c>
-      <c r="Q6" s="203">
+      <c r="Q6" s="204">
         <v>1</v>
       </c>
-      <c r="R6" s="203">
+      <c r="R6" s="204">
         <v>1350</v>
       </c>
-      <c r="S6" s="205">
+      <c r="S6" s="206">
         <v>1.29</v>
       </c>
-      <c r="T6" s="203">
+      <c r="T6" s="204">
         <v>60</v>
       </c>
-      <c r="U6" s="207">
+      <c r="U6" s="208">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="V6" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="203" t="s">
+      <c r="V6" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="204" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="203" t="s">
+      <c r="X6" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="204" t="s">
         <v>32</v>
       </c>
-      <c r="AB6" s="203" t="s">
+      <c r="AB6" s="204" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="203">
+    <row r="7" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="204">
         <v>5</v>
       </c>
-      <c r="B7" s="204" t="s">
+      <c r="B7" s="205" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="203" t="s">
+      <c r="C7" s="204" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="203" t="s">
+      <c r="D7" s="204" t="s">
         <v>543</v>
       </c>
-      <c r="E7" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="203">
+      <c r="E7" s="204" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="204">
         <v>262494</v>
       </c>
-      <c r="G7" s="203" t="s">
+      <c r="G7" s="204" t="s">
         <v>542</v>
       </c>
-      <c r="H7" s="203">
+      <c r="H7" s="204">
         <v>700</v>
       </c>
-      <c r="I7" s="205">
+      <c r="I7" s="206">
         <v>1.0740000000000001</v>
       </c>
-      <c r="J7" s="205">
+      <c r="J7" s="206">
         <v>1.27</v>
       </c>
-      <c r="K7" s="203" t="s">
+      <c r="K7" s="204" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="205">
+      <c r="L7" s="206">
         <v>954.78599999999994</v>
       </c>
-      <c r="M7" s="206">
+      <c r="M7" s="207">
         <v>889</v>
       </c>
-      <c r="N7" s="207">
+      <c r="N7" s="208">
         <v>0.24690000000000001</v>
       </c>
-      <c r="O7" s="208">
+      <c r="O7" s="209">
         <v>14.82</v>
       </c>
-      <c r="P7" s="203">
+      <c r="P7" s="204">
         <v>566.20000000000005</v>
       </c>
-      <c r="Q7" s="203">
+      <c r="Q7" s="204">
         <v>1</v>
       </c>
-      <c r="R7" s="203">
+      <c r="R7" s="204">
         <v>1100</v>
       </c>
-      <c r="S7" s="205">
+      <c r="S7" s="206">
         <v>1.0740000000000001</v>
       </c>
-      <c r="T7" s="203">
+      <c r="T7" s="204">
         <v>26</v>
       </c>
-      <c r="U7" s="207">
+      <c r="U7" s="208">
         <v>2.3599999999999999E-2</v>
       </c>
-      <c r="V7" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="203" t="s">
+      <c r="V7" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="204" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="203" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="203" t="s">
+      <c r="X7" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="204" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="204" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="203" t="s">
+      <c r="AB7" s="204" t="s">
         <v>550</v>
       </c>
     </row>
@@ -10749,7 +10795,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4063489B-9360-4477-96A2-DD5FB6D3203C}">
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
@@ -11210,90 +11256,88 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="133">
+    <row r="6" spans="1:28" s="227" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="225">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="226" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="219" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>489</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="5">
-        <v>262467</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>488</v>
-      </c>
-      <c r="H6" s="5">
-        <v>800</v>
-      </c>
-      <c r="I6" s="7">
-        <v>0.56799999999999995</v>
-      </c>
-      <c r="J6" s="7">
-        <v>1.508</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="L6" s="7">
-        <v>685.23500000000001</v>
-      </c>
-      <c r="M6" s="9">
-        <v>603.20000000000005</v>
-      </c>
-      <c r="N6" s="6">
-        <v>8.3799999999999999E-2</v>
-      </c>
-      <c r="O6" s="8">
-        <v>5.03</v>
-      </c>
-      <c r="P6" s="5">
-        <v>406.3</v>
-      </c>
-      <c r="Q6" s="5">
+      <c r="D6" s="220">
+        <v>46279</v>
+      </c>
+      <c r="E6" s="219"/>
+      <c r="F6" s="219">
+        <v>262610</v>
+      </c>
+      <c r="G6" s="219">
+        <v>8235</v>
+      </c>
+      <c r="H6" s="219">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="221">
+        <v>0.64500000000000002</v>
+      </c>
+      <c r="J6" s="221">
+        <v>1.526</v>
+      </c>
+      <c r="K6" s="219" t="s">
+        <v>726</v>
+      </c>
+      <c r="L6" s="221">
+        <v>984.27</v>
+      </c>
+      <c r="M6" s="222">
+        <v>763</v>
+      </c>
+      <c r="N6" s="223">
+        <v>0.106</v>
+      </c>
+      <c r="O6" s="224">
+        <v>6.36</v>
+      </c>
+      <c r="P6" s="219">
+        <v>529.5</v>
+      </c>
+      <c r="Q6" s="219">
         <v>2</v>
       </c>
-      <c r="R6" s="5">
-        <v>1200</v>
-      </c>
-      <c r="S6" s="7">
-        <v>1.1359999999999999</v>
-      </c>
-      <c r="T6" s="5">
-        <v>64</v>
-      </c>
-      <c r="U6" s="6">
-        <v>5.33E-2</v>
-      </c>
-      <c r="V6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="5" t="s">
+      <c r="R6" s="219">
+        <v>1350</v>
+      </c>
+      <c r="S6" s="221">
+        <v>1.29</v>
+      </c>
+      <c r="T6" s="219">
+        <v>60</v>
+      </c>
+      <c r="U6" s="223">
+        <v>4.4400000000000002E-2</v>
+      </c>
+      <c r="V6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="219" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB6" s="5" t="s">
-        <v>494</v>
+      <c r="X6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="219">
+        <v>6</v>
+      </c>
+      <c r="AB6" s="219" t="s">
+        <v>727</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11313,52 +11357,52 @@
         <v>27</v>
       </c>
       <c r="F7" s="5">
-        <v>262468</v>
+        <v>262467</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>488</v>
       </c>
       <c r="H7" s="5">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="I7" s="7">
-        <v>0.46400000000000002</v>
+        <v>0.56799999999999995</v>
       </c>
       <c r="J7" s="7">
-        <v>1.208</v>
+        <v>1.508</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="L7" s="7">
-        <v>560.51199999999994</v>
+        <v>685.23500000000001</v>
       </c>
       <c r="M7" s="9">
-        <v>604</v>
+        <v>603.20000000000005</v>
       </c>
       <c r="N7" s="6">
-        <v>8.3900000000000002E-2</v>
+        <v>8.3799999999999999E-2</v>
       </c>
       <c r="O7" s="8">
         <v>5.03</v>
       </c>
       <c r="P7" s="5">
-        <v>332.4</v>
+        <v>406.3</v>
       </c>
       <c r="Q7" s="5">
         <v>2</v>
       </c>
       <c r="R7" s="5">
-        <v>950</v>
+        <v>1200</v>
       </c>
       <c r="S7" s="7">
-        <v>0.92800000000000005</v>
+        <v>1.1359999999999999</v>
       </c>
       <c r="T7" s="5">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="U7" s="6">
-        <v>2.3199999999999998E-2</v>
+        <v>5.33E-2</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>28</v>
@@ -11379,7 +11423,7 @@
         <v>30</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11390,7 +11434,7 @@
         <v>63</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>489</v>
@@ -11399,159 +11443,159 @@
         <v>27</v>
       </c>
       <c r="F8" s="5">
-        <v>262465</v>
+        <v>262468</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>488</v>
       </c>
       <c r="H8" s="5">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="I8" s="7">
-        <v>0.78200000000000003</v>
+        <v>0.46400000000000002</v>
       </c>
       <c r="J8" s="7">
-        <v>1.5680000000000001</v>
+        <v>1.208</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="L8" s="7">
-        <v>1103.558</v>
+        <v>560.51199999999994</v>
       </c>
       <c r="M8" s="9">
-        <v>705.6</v>
+        <v>604</v>
       </c>
       <c r="N8" s="6">
-        <v>9.8000000000000004E-2</v>
+        <v>8.3900000000000002E-2</v>
       </c>
       <c r="O8" s="8">
-        <v>5.88</v>
+        <v>5.03</v>
       </c>
       <c r="P8" s="5">
-        <v>380.7</v>
+        <v>332.4</v>
       </c>
       <c r="Q8" s="5">
         <v>2</v>
       </c>
       <c r="R8" s="5">
-        <v>1600</v>
+        <v>950</v>
       </c>
       <c r="S8" s="7">
-        <v>1.5640000000000001</v>
+        <v>0.92800000000000005</v>
       </c>
       <c r="T8" s="5">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="U8" s="6">
-        <v>2.2499999999999999E-2</v>
+        <v>2.3199999999999998E-2</v>
       </c>
       <c r="V8" s="5" t="s">
         <v>28</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X8" s="5" t="s">
         <v>28</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z8" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA8" s="5" t="s">
         <v>30</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="133">
         <v>7</v>
       </c>
-      <c r="B9" s="134" t="s">
+      <c r="B9" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="133" t="s">
+      <c r="C9" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="133" t="s">
-        <v>534</v>
-      </c>
-      <c r="E9" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="133">
-        <v>262510</v>
-      </c>
-      <c r="G9" s="133" t="s">
-        <v>557</v>
-      </c>
-      <c r="H9" s="133">
-        <v>1100</v>
-      </c>
-      <c r="I9" s="135">
-        <v>0.77200000000000002</v>
-      </c>
-      <c r="J9" s="135">
-        <v>1.7589999999999999</v>
-      </c>
-      <c r="K9" s="133" t="s">
-        <v>556</v>
-      </c>
-      <c r="L9" s="135">
-        <v>1493.7429999999999</v>
-      </c>
-      <c r="M9" s="136">
-        <v>967.4</v>
-      </c>
-      <c r="N9" s="137">
-        <v>0.13439999999999999</v>
-      </c>
-      <c r="O9" s="138">
-        <v>8.06</v>
-      </c>
-      <c r="P9" s="133">
-        <v>515.29999999999995</v>
-      </c>
-      <c r="Q9" s="133">
+      <c r="D9" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5">
+        <v>262465</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="H9" s="5">
+        <v>900</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0.78200000000000003</v>
+      </c>
+      <c r="J9" s="7">
+        <v>1.5680000000000001</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="L9" s="7">
+        <v>1103.558</v>
+      </c>
+      <c r="M9" s="9">
+        <v>705.6</v>
+      </c>
+      <c r="N9" s="6">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="O9" s="8">
+        <v>5.88</v>
+      </c>
+      <c r="P9" s="5">
+        <v>380.7</v>
+      </c>
+      <c r="Q9" s="5">
         <v>2</v>
       </c>
-      <c r="R9" s="133">
+      <c r="R9" s="5">
         <v>1600</v>
       </c>
-      <c r="S9" s="135">
-        <v>1.544</v>
-      </c>
-      <c r="T9" s="133">
-        <v>56</v>
-      </c>
-      <c r="U9" s="137">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="V9" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="133" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB9" s="133" t="s">
-        <v>562</v>
+      <c r="S9" s="7">
+        <v>1.5640000000000001</v>
+      </c>
+      <c r="T9" s="5">
+        <v>36</v>
+      </c>
+      <c r="U9" s="6">
+        <v>2.2499999999999999E-2</v>
+      </c>
+      <c r="V9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB9" s="5" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11571,73 +11615,73 @@
         <v>27</v>
       </c>
       <c r="F10" s="133">
-        <v>262509</v>
+        <v>262510</v>
       </c>
       <c r="G10" s="133" t="s">
         <v>557</v>
       </c>
       <c r="H10" s="133">
-        <v>650</v>
+        <v>1100</v>
       </c>
       <c r="I10" s="135">
-        <v>1.0680000000000001</v>
+        <v>0.77200000000000002</v>
       </c>
       <c r="J10" s="135">
-        <v>1.375</v>
+        <v>1.7589999999999999</v>
       </c>
       <c r="K10" s="133" t="s">
-        <v>120</v>
+        <v>556</v>
       </c>
       <c r="L10" s="135">
-        <v>954.52499999999998</v>
+        <v>1493.7429999999999</v>
       </c>
       <c r="M10" s="136">
-        <v>893.8</v>
+        <v>967.4</v>
       </c>
       <c r="N10" s="137">
-        <v>0.24829999999999999</v>
+        <v>0.13439999999999999</v>
       </c>
       <c r="O10" s="138">
-        <v>14.9</v>
+        <v>8.06</v>
       </c>
       <c r="P10" s="133">
-        <v>329.3</v>
+        <v>515.29999999999995</v>
       </c>
       <c r="Q10" s="133">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="133">
-        <v>1100</v>
+        <v>1600</v>
       </c>
       <c r="S10" s="135">
-        <v>1.0680000000000001</v>
+        <v>1.544</v>
       </c>
       <c r="T10" s="133">
+        <v>56</v>
+      </c>
+      <c r="U10" s="137">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="V10" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="133" t="s">
         <v>32</v>
       </c>
-      <c r="U10" s="137">
-        <v>2.9100000000000001E-2</v>
-      </c>
-      <c r="V10" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="133" t="s">
-        <v>30</v>
-      </c>
       <c r="AB10" s="133" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11648,7 +11692,7 @@
         <v>63</v>
       </c>
       <c r="C11" s="133" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D11" s="133" t="s">
         <v>534</v>
@@ -11657,52 +11701,52 @@
         <v>27</v>
       </c>
       <c r="F11" s="133">
-        <v>262508</v>
+        <v>262509</v>
       </c>
       <c r="G11" s="133" t="s">
         <v>557</v>
       </c>
       <c r="H11" s="133">
-        <v>1650</v>
+        <v>650</v>
       </c>
       <c r="I11" s="135">
-        <v>0.47199999999999998</v>
+        <v>1.0680000000000001</v>
       </c>
       <c r="J11" s="135">
-        <v>1.2589999999999999</v>
+        <v>1.375</v>
       </c>
       <c r="K11" s="133" t="s">
-        <v>564</v>
+        <v>120</v>
       </c>
       <c r="L11" s="135">
-        <v>980.50900000000001</v>
+        <v>954.52499999999998</v>
       </c>
       <c r="M11" s="136">
-        <v>1038.7</v>
+        <v>893.8</v>
       </c>
       <c r="N11" s="137">
-        <v>0.14430000000000001</v>
+        <v>0.24829999999999999</v>
       </c>
       <c r="O11" s="138">
-        <v>8.66</v>
+        <v>14.9</v>
       </c>
       <c r="P11" s="133">
-        <v>338.3</v>
+        <v>329.3</v>
       </c>
       <c r="Q11" s="133">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R11" s="133">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="S11" s="135">
-        <v>0.94399999999999995</v>
+        <v>1.0680000000000001</v>
       </c>
       <c r="T11" s="133">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="U11" s="137">
-        <v>5.6000000000000001E-2</v>
+        <v>2.9100000000000001E-2</v>
       </c>
       <c r="V11" s="133" t="s">
         <v>28</v>
@@ -11723,180 +11767,266 @@
         <v>30</v>
       </c>
       <c r="AB11" s="133" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="133">
         <v>10</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="134" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="133" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="133" t="s">
+        <v>534</v>
+      </c>
+      <c r="E12" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="133">
+        <v>262508</v>
+      </c>
+      <c r="G12" s="133" t="s">
+        <v>557</v>
+      </c>
+      <c r="H12" s="133">
+        <v>1650</v>
+      </c>
+      <c r="I12" s="135">
+        <v>0.47199999999999998</v>
+      </c>
+      <c r="J12" s="135">
+        <v>1.2589999999999999</v>
+      </c>
+      <c r="K12" s="133" t="s">
+        <v>564</v>
+      </c>
+      <c r="L12" s="135">
+        <v>980.50900000000001</v>
+      </c>
+      <c r="M12" s="136">
+        <v>1038.7</v>
+      </c>
+      <c r="N12" s="137">
+        <v>0.14430000000000001</v>
+      </c>
+      <c r="O12" s="138">
+        <v>8.66</v>
+      </c>
+      <c r="P12" s="133">
+        <v>338.3</v>
+      </c>
+      <c r="Q12" s="133">
+        <v>2</v>
+      </c>
+      <c r="R12" s="133">
+        <v>1000</v>
+      </c>
+      <c r="S12" s="135">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="T12" s="133">
+        <v>56</v>
+      </c>
+      <c r="U12" s="137">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="V12" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="133" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB12" s="133" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="133">
+        <v>11</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="5">
+      <c r="E13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="5">
         <v>262466</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>488</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H13" s="5">
         <v>2000</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I13" s="7">
         <v>0.90900000000000003</v>
       </c>
-      <c r="J12" s="7">
+      <c r="J13" s="7">
         <v>0.65900000000000003</v>
       </c>
-      <c r="K12" s="5" t="s">
+      <c r="K13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L13" s="7">
         <v>1198.0619999999999</v>
       </c>
-      <c r="M12" s="9">
+      <c r="M13" s="9">
         <v>1318</v>
       </c>
-      <c r="N12" s="6">
+      <c r="N13" s="6">
         <v>0.36609999999999998</v>
       </c>
-      <c r="O12" s="8">
+      <c r="O13" s="8">
         <v>21.97</v>
       </c>
-      <c r="P12" s="5">
+      <c r="P13" s="5">
         <v>413.3</v>
       </c>
-      <c r="Q12" s="5">
+      <c r="Q13" s="5">
         <v>1</v>
       </c>
-      <c r="R12" s="5">
+      <c r="R13" s="5">
         <v>950</v>
       </c>
-      <c r="S12" s="7">
+      <c r="S13" s="7">
         <v>0.90900000000000003</v>
       </c>
-      <c r="T12" s="5">
+      <c r="T13" s="5">
         <v>41</v>
       </c>
-      <c r="U12" s="6">
+      <c r="U13" s="6">
         <v>4.3200000000000002E-2</v>
       </c>
-      <c r="V12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="5" t="s">
+      <c r="V13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB12" s="5" t="s">
+      <c r="AB13" s="5" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="11">
-        <f>SUM(H3:H12)</f>
-        <v>10300</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P13" s="11">
-        <f>SUM(P3:P12)</f>
-        <v>4288</v>
-      </c>
-      <c r="Q13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB13" s="11" t="s">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="11">
+        <f>SUM(H3:H13)</f>
+        <v>11300</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P14" s="11">
+        <f>SUM(P3:P13)</f>
+        <v>4817.5000000000009</v>
+      </c>
+      <c r="Q14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB14" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -23921,261 +24051,261 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="209" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="210">
+    <row r="4" spans="1:28" s="210" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="211">
         <v>2</v>
       </c>
-      <c r="B4" s="215" t="s">
+      <c r="B4" s="216" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="210" t="s">
+      <c r="C4" s="211" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="210" t="s">
+      <c r="D4" s="211" t="s">
         <v>680</v>
       </c>
-      <c r="E4" s="210" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="210">
+      <c r="E4" s="211" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="211">
         <v>262597</v>
       </c>
-      <c r="G4" s="210" t="s">
+      <c r="G4" s="211" t="s">
         <v>700</v>
       </c>
-      <c r="H4" s="210">
+      <c r="H4" s="211">
         <v>600</v>
       </c>
-      <c r="I4" s="212">
+      <c r="I4" s="213">
         <v>1.236</v>
       </c>
-      <c r="J4" s="212">
+      <c r="J4" s="213">
         <v>2.5910000000000002</v>
       </c>
-      <c r="K4" s="210" t="s">
+      <c r="K4" s="211" t="s">
         <v>522</v>
       </c>
-      <c r="L4" s="212">
+      <c r="L4" s="213">
         <v>1921.4860000000001</v>
       </c>
-      <c r="M4" s="214">
+      <c r="M4" s="215">
         <v>1554.6</v>
       </c>
-      <c r="N4" s="211">
+      <c r="N4" s="212">
         <v>0.43180000000000002</v>
       </c>
-      <c r="O4" s="213">
+      <c r="O4" s="214">
         <v>25.91</v>
       </c>
-      <c r="P4" s="210">
+      <c r="P4" s="211">
         <v>1214.4000000000001</v>
       </c>
-      <c r="Q4" s="210">
+      <c r="Q4" s="211">
         <v>1</v>
       </c>
-      <c r="R4" s="210">
+      <c r="R4" s="211">
         <v>1300</v>
       </c>
-      <c r="S4" s="212">
+      <c r="S4" s="213">
         <v>1.236</v>
       </c>
-      <c r="T4" s="210">
+      <c r="T4" s="211">
         <v>64</v>
       </c>
-      <c r="U4" s="211">
+      <c r="U4" s="212">
         <v>4.9200000000000001E-2</v>
       </c>
-      <c r="V4" s="210" t="s">
+      <c r="V4" s="211" t="s">
         <v>29</v>
       </c>
-      <c r="W4" s="210" t="s">
+      <c r="W4" s="211" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="210" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="210" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="210" t="s">
+      <c r="X4" s="211" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="211" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="211" t="s">
         <v>29</v>
       </c>
-      <c r="AA4" s="210" t="s">
+      <c r="AA4" s="211" t="s">
         <v>32</v>
       </c>
-      <c r="AB4" s="210" t="s">
+      <c r="AB4" s="211" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="209" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="210">
+    <row r="5" spans="1:28" s="210" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="211">
         <v>3</v>
       </c>
-      <c r="B5" s="215" t="s">
+      <c r="B5" s="216" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="210" t="s">
+      <c r="C5" s="211" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="210" t="s">
+      <c r="D5" s="211" t="s">
         <v>680</v>
       </c>
-      <c r="E5" s="210" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="210">
+      <c r="E5" s="211" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="211">
         <v>262596</v>
       </c>
-      <c r="G5" s="210" t="s">
+      <c r="G5" s="211" t="s">
         <v>700</v>
       </c>
-      <c r="H5" s="210">
+      <c r="H5" s="211">
         <v>2000</v>
       </c>
-      <c r="I5" s="212">
+      <c r="I5" s="213">
         <v>1.196</v>
       </c>
-      <c r="J5" s="212">
+      <c r="J5" s="213">
         <v>1.6910000000000001</v>
       </c>
-      <c r="K5" s="210" t="s">
+      <c r="K5" s="211" t="s">
         <v>519</v>
       </c>
-      <c r="L5" s="212">
+      <c r="L5" s="213">
         <v>4044.8719999999998</v>
       </c>
-      <c r="M5" s="214">
+      <c r="M5" s="215">
         <v>3382</v>
       </c>
-      <c r="N5" s="211">
+      <c r="N5" s="212">
         <v>0.93940000000000001</v>
       </c>
-      <c r="O5" s="213">
+      <c r="O5" s="214">
         <v>56.37</v>
       </c>
-      <c r="P5" s="210">
+      <c r="P5" s="211">
         <v>2556.4</v>
       </c>
-      <c r="Q5" s="210">
+      <c r="Q5" s="211">
         <v>1</v>
       </c>
-      <c r="R5" s="210">
+      <c r="R5" s="211">
         <v>1250</v>
       </c>
-      <c r="S5" s="212">
+      <c r="S5" s="213">
         <v>1.196</v>
       </c>
-      <c r="T5" s="210">
+      <c r="T5" s="211">
         <v>54</v>
       </c>
-      <c r="U5" s="211">
+      <c r="U5" s="212">
         <v>4.3200000000000002E-2</v>
       </c>
-      <c r="V5" s="210" t="s">
+      <c r="V5" s="211" t="s">
         <v>29</v>
       </c>
-      <c r="W5" s="210" t="s">
+      <c r="W5" s="211" t="s">
         <v>40</v>
       </c>
-      <c r="X5" s="210" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="210" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="210" t="s">
+      <c r="X5" s="211" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="211" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="211" t="s">
         <v>29</v>
       </c>
-      <c r="AA5" s="210" t="s">
+      <c r="AA5" s="211" t="s">
         <v>72</v>
       </c>
-      <c r="AB5" s="210" t="s">
+      <c r="AB5" s="211" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="209" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="210">
+    <row r="6" spans="1:28" s="210" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="211">
         <v>4</v>
       </c>
-      <c r="B6" s="215" t="s">
+      <c r="B6" s="216" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="210" t="s">
+      <c r="C6" s="211" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="210" t="s">
+      <c r="D6" s="211" t="s">
         <v>680</v>
       </c>
-      <c r="E6" s="210" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="210">
+      <c r="E6" s="211" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="211">
         <v>262595</v>
       </c>
-      <c r="G6" s="210" t="s">
+      <c r="G6" s="211" t="s">
         <v>700</v>
       </c>
-      <c r="H6" s="210">
+      <c r="H6" s="211">
         <v>1400</v>
       </c>
-      <c r="I6" s="212">
+      <c r="I6" s="213">
         <v>1.2050000000000001</v>
       </c>
-      <c r="J6" s="212">
+      <c r="J6" s="213">
         <v>2.5910000000000002</v>
       </c>
-      <c r="K6" s="210" t="s">
+      <c r="K6" s="211" t="s">
         <v>53</v>
       </c>
-      <c r="L6" s="212">
+      <c r="L6" s="213">
         <v>4371.0169999999998</v>
       </c>
-      <c r="M6" s="214">
+      <c r="M6" s="215">
         <v>3627.4</v>
       </c>
-      <c r="N6" s="211">
+      <c r="N6" s="212">
         <v>1.0076000000000001</v>
       </c>
-      <c r="O6" s="213">
+      <c r="O6" s="214">
         <v>60.46</v>
       </c>
-      <c r="P6" s="210">
+      <c r="P6" s="211">
         <v>2482.6999999999998</v>
       </c>
-      <c r="Q6" s="210">
+      <c r="Q6" s="211">
         <v>1</v>
       </c>
-      <c r="R6" s="210">
+      <c r="R6" s="211">
         <v>1250</v>
       </c>
-      <c r="S6" s="212">
+      <c r="S6" s="213">
         <v>1.2050000000000001</v>
       </c>
-      <c r="T6" s="210">
+      <c r="T6" s="211">
         <v>45</v>
       </c>
-      <c r="U6" s="211">
+      <c r="U6" s="212">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="V6" s="210" t="s">
+      <c r="V6" s="211" t="s">
         <v>35</v>
       </c>
-      <c r="W6" s="210" t="s">
+      <c r="W6" s="211" t="s">
         <v>40</v>
       </c>
-      <c r="X6" s="210" t="s">
+      <c r="X6" s="211" t="s">
         <v>35</v>
       </c>
-      <c r="Y6" s="210" t="s">
+      <c r="Y6" s="211" t="s">
         <v>35</v>
       </c>
-      <c r="Z6" s="210" t="s">
+      <c r="Z6" s="211" t="s">
         <v>35</v>
       </c>
-      <c r="AA6" s="210" t="s">
+      <c r="AA6" s="211" t="s">
         <v>55</v>
       </c>
-      <c r="AB6" s="210" t="s">
+      <c r="AB6" s="211" t="s">
         <v>54</v>
       </c>
     </row>
@@ -35184,11 +35314,11 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0213073B-7DC6-44F4-9A79-2376A05B9E79}">
-  <dimension ref="A1:AB27"/>
+  <dimension ref="A1:AB29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="108" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.5546875" style="108" customWidth="1"/>
@@ -35392,7 +35522,7 @@
       <c r="A3" s="161">
         <v>1</v>
       </c>
-      <c r="B3" s="162" t="s">
+      <c r="B3" s="217" t="s">
         <v>626</v>
       </c>
       <c r="C3" s="161" t="s">
@@ -37030,82 +37160,76 @@
         <v>626</v>
       </c>
       <c r="C22" s="161" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="161" t="s">
-        <v>625</v>
-      </c>
-      <c r="E22" s="161" t="s">
-        <v>27</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="D22" s="191">
+        <v>46280</v>
+      </c>
+      <c r="E22" s="161"/>
       <c r="F22" s="161">
-        <v>262554</v>
+        <v>262609</v>
       </c>
       <c r="G22" s="161" t="s">
-        <v>624</v>
+        <v>724</v>
       </c>
       <c r="H22" s="161">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="I22" s="163">
-        <v>0.40400000000000003</v>
+        <v>0.28399999999999997</v>
       </c>
       <c r="J22" s="163">
-        <v>0.84</v>
-      </c>
-      <c r="K22" s="161" t="s">
-        <v>630</v>
+        <v>1.8</v>
+      </c>
+      <c r="K22" s="201" t="s">
+        <v>44</v>
       </c>
       <c r="L22" s="163">
-        <v>509.04</v>
+        <v>511.2</v>
       </c>
       <c r="M22" s="164">
-        <v>630</v>
+        <v>600</v>
       </c>
       <c r="N22" s="165">
-        <v>8.7499999999999994E-2</v>
+        <v>5.5599999999999997E-2</v>
       </c>
       <c r="O22" s="166">
-        <v>5.25</v>
+        <v>3.33</v>
       </c>
       <c r="P22" s="161">
-        <v>175.6</v>
+        <v>176.4</v>
       </c>
       <c r="Q22" s="161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R22" s="161">
-        <v>850</v>
+        <v>900</v>
       </c>
       <c r="S22" s="163">
-        <v>0.80800000000000005</v>
+        <v>0.85199999999999998</v>
       </c>
       <c r="T22" s="161">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="U22" s="165">
-        <v>4.9399999999999999E-2</v>
+        <v>5.33E-2</v>
       </c>
       <c r="V22" s="161" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W22" s="161" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X22" s="161" t="s">
         <v>28</v>
       </c>
-      <c r="Y22" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z22" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA22" s="161" t="s">
-        <v>39</v>
+      <c r="Y22" s="161"/>
+      <c r="Z22" s="161"/>
+      <c r="AA22" s="161">
+        <v>1</v>
       </c>
       <c r="AB22" s="161" t="s">
-        <v>629</v>
+        <v>725</v>
       </c>
     </row>
     <row r="23" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
@@ -37116,7 +37240,7 @@
         <v>626</v>
       </c>
       <c r="C23" s="161" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D23" s="161" t="s">
         <v>625</v>
@@ -37125,37 +37249,37 @@
         <v>27</v>
       </c>
       <c r="F23" s="161">
-        <v>262551</v>
+        <v>262554</v>
       </c>
       <c r="G23" s="161" t="s">
         <v>624</v>
       </c>
       <c r="H23" s="161">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="I23" s="163">
         <v>0.40400000000000003</v>
       </c>
       <c r="J23" s="163">
-        <v>1.39</v>
+        <v>0.84</v>
       </c>
       <c r="K23" s="161" t="s">
-        <v>279</v>
+        <v>630</v>
       </c>
       <c r="L23" s="163">
-        <v>280.77999999999997</v>
+        <v>509.04</v>
       </c>
       <c r="M23" s="164">
-        <v>347.5</v>
+        <v>630</v>
       </c>
       <c r="N23" s="165">
-        <v>4.8300000000000003E-2</v>
+        <v>8.7499999999999994E-2</v>
       </c>
       <c r="O23" s="166">
-        <v>2.9</v>
+        <v>5.25</v>
       </c>
       <c r="P23" s="161">
-        <v>103.3</v>
+        <v>175.6</v>
       </c>
       <c r="Q23" s="161">
         <v>2</v>
@@ -37173,10 +37297,10 @@
         <v>4.9399999999999999E-2</v>
       </c>
       <c r="V23" s="161" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W23" s="161" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X23" s="161" t="s">
         <v>28</v>
@@ -37191,7 +37315,7 @@
         <v>39</v>
       </c>
       <c r="AB23" s="161" t="s">
-        <v>278</v>
+        <v>629</v>
       </c>
     </row>
     <row r="24" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
@@ -37202,7 +37326,7 @@
         <v>626</v>
       </c>
       <c r="C24" s="161" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D24" s="161" t="s">
         <v>625</v>
@@ -37211,13 +37335,13 @@
         <v>27</v>
       </c>
       <c r="F24" s="161">
-        <v>262552</v>
+        <v>262551</v>
       </c>
       <c r="G24" s="161" t="s">
         <v>624</v>
       </c>
       <c r="H24" s="161">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="I24" s="163">
         <v>0.40400000000000003</v>
@@ -37229,19 +37353,19 @@
         <v>279</v>
       </c>
       <c r="L24" s="163">
-        <v>1684.68</v>
+        <v>280.77999999999997</v>
       </c>
       <c r="M24" s="164">
-        <v>2085</v>
+        <v>347.5</v>
       </c>
       <c r="N24" s="165">
-        <v>0.28960000000000002</v>
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="O24" s="166">
-        <v>17.38</v>
+        <v>2.9</v>
       </c>
       <c r="P24" s="161">
-        <v>581.20000000000005</v>
+        <v>103.3</v>
       </c>
       <c r="Q24" s="161">
         <v>2</v>
@@ -37259,10 +37383,10 @@
         <v>4.9399999999999999E-2</v>
       </c>
       <c r="V24" s="161" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W24" s="161" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X24" s="161" t="s">
         <v>28</v>
@@ -37274,7 +37398,7 @@
         <v>27</v>
       </c>
       <c r="AA24" s="161" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="AB24" s="161" t="s">
         <v>278</v>
@@ -37297,52 +37421,52 @@
         <v>27</v>
       </c>
       <c r="F25" s="161">
-        <v>262553</v>
+        <v>262552</v>
       </c>
       <c r="G25" s="161" t="s">
         <v>624</v>
       </c>
       <c r="H25" s="161">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="I25" s="163">
-        <v>0.34399999999999997</v>
+        <v>0.40400000000000003</v>
       </c>
       <c r="J25" s="163">
-        <v>1.26</v>
+        <v>1.39</v>
       </c>
       <c r="K25" s="161" t="s">
-        <v>628</v>
+        <v>279</v>
       </c>
       <c r="L25" s="163">
-        <v>866.88</v>
+        <v>1684.68</v>
       </c>
       <c r="M25" s="164">
-        <v>1260</v>
+        <v>2085</v>
       </c>
       <c r="N25" s="165">
-        <v>0.17499999999999999</v>
+        <v>0.28960000000000002</v>
       </c>
       <c r="O25" s="166">
-        <v>10.5</v>
+        <v>17.38</v>
       </c>
       <c r="P25" s="161">
-        <v>299.10000000000002</v>
+        <v>581.20000000000005</v>
       </c>
       <c r="Q25" s="161">
         <v>2</v>
       </c>
       <c r="R25" s="161">
-        <v>750</v>
+        <v>850</v>
       </c>
       <c r="S25" s="163">
-        <v>0.68799999999999994</v>
+        <v>0.80800000000000005</v>
       </c>
       <c r="T25" s="161">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="U25" s="165">
-        <v>8.2699999999999996E-2</v>
+        <v>4.9399999999999999E-2</v>
       </c>
       <c r="V25" s="161" t="s">
         <v>28</v>
@@ -37360,10 +37484,10 @@
         <v>27</v>
       </c>
       <c r="AA25" s="161" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AB25" s="161" t="s">
-        <v>627</v>
+        <v>278</v>
       </c>
     </row>
     <row r="26" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
@@ -37383,160 +37507,249 @@
         <v>27</v>
       </c>
       <c r="F26" s="161">
-        <v>262557</v>
+        <v>262553</v>
       </c>
       <c r="G26" s="161" t="s">
         <v>624</v>
       </c>
       <c r="H26" s="161">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="I26" s="163">
-        <v>0.30399999999999999</v>
+        <v>0.34399999999999997</v>
       </c>
       <c r="J26" s="163">
-        <v>0.84</v>
+        <v>1.26</v>
       </c>
       <c r="K26" s="161" t="s">
-        <v>319</v>
+        <v>628</v>
       </c>
       <c r="L26" s="163">
-        <v>383.04</v>
+        <v>866.88</v>
       </c>
       <c r="M26" s="164">
-        <v>630</v>
+        <v>1260</v>
       </c>
       <c r="N26" s="165">
-        <v>8.7499999999999994E-2</v>
+        <v>0.17499999999999999</v>
       </c>
       <c r="O26" s="166">
-        <v>5.25</v>
+        <v>10.5</v>
       </c>
       <c r="P26" s="161">
-        <v>132.1</v>
+        <v>299.10000000000002</v>
       </c>
       <c r="Q26" s="161">
         <v>2</v>
       </c>
       <c r="R26" s="161">
+        <v>750</v>
+      </c>
+      <c r="S26" s="163">
+        <v>0.68799999999999994</v>
+      </c>
+      <c r="T26" s="161">
+        <v>62</v>
+      </c>
+      <c r="U26" s="165">
+        <v>8.2699999999999996E-2</v>
+      </c>
+      <c r="V26" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W26" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X26" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y26" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z26" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA26" s="161" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB26" s="161" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="161">
+        <v>25</v>
+      </c>
+      <c r="B27" s="162" t="s">
+        <v>626</v>
+      </c>
+      <c r="C27" s="161" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" s="161" t="s">
+        <v>625</v>
+      </c>
+      <c r="E27" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="161">
+        <v>262557</v>
+      </c>
+      <c r="G27" s="161" t="s">
+        <v>624</v>
+      </c>
+      <c r="H27" s="161">
+        <v>1500</v>
+      </c>
+      <c r="I27" s="163">
+        <v>0.30399999999999999</v>
+      </c>
+      <c r="J27" s="163">
+        <v>0.84</v>
+      </c>
+      <c r="K27" s="161" t="s">
+        <v>319</v>
+      </c>
+      <c r="L27" s="163">
+        <v>383.04</v>
+      </c>
+      <c r="M27" s="164">
+        <v>630</v>
+      </c>
+      <c r="N27" s="165">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="O27" s="166">
+        <v>5.25</v>
+      </c>
+      <c r="P27" s="161">
+        <v>132.1</v>
+      </c>
+      <c r="Q27" s="161">
+        <v>2</v>
+      </c>
+      <c r="R27" s="161">
         <v>650</v>
       </c>
-      <c r="S26" s="163">
+      <c r="S27" s="163">
         <v>0.60799999999999998</v>
       </c>
-      <c r="T26" s="161">
+      <c r="T27" s="161">
         <v>42</v>
       </c>
-      <c r="U26" s="165">
+      <c r="U27" s="165">
         <v>6.4600000000000005E-2</v>
       </c>
-      <c r="V26" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W26" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X26" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y26" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z26" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA26" s="161" t="s">
+      <c r="V27" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W27" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X27" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y27" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z27" s="161" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA27" s="161" t="s">
         <v>39</v>
       </c>
-      <c r="AB26" s="161" t="s">
+      <c r="AB27" s="161" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="C27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="D27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="E27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="F27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="G27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="H27" s="168">
+    <row r="28" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="G28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" s="168">
         <v>25800</v>
       </c>
-      <c r="I27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="J27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="K27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="L27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="M27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="N27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="O27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="P27" s="168">
+      <c r="I28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="K28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="L28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="M28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="N28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="O28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="P28" s="168">
         <v>5957.9</v>
       </c>
-      <c r="Q27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="R27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="S27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="T27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="U27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="V27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="W27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="X27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA27" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB27" s="168" t="s">
-        <v>27</v>
-      </c>
+      <c r="Q28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="R28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="S28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="T28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="U28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="V28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="W28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="X28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA28" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB28" s="168" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B29" s="218"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (15/09/2026 15:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7746A5D-8BB2-46D9-9A55-8AABDF275D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1BD8DF-3335-49C9-B9C2-72AFCA772BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
     <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId15"/>
     <sheet name="RM Embalagens 1179 P" sheetId="136" r:id="rId16"/>
     <sheet name="Tolecaixas 1181 P" sheetId="138" r:id="rId17"/>
-    <sheet name="ABAPEL 1178" sheetId="135" r:id="rId18"/>
+    <sheet name="ABAPEL 1178 P" sheetId="135" r:id="rId18"/>
     <sheet name="FAVINCO EMBALAGENS 1177 P" sheetId="134" r:id="rId19"/>
     <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId20"/>
     <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId21"/>
@@ -2490,7 +2490,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="228">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3114,34 +3114,31 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="18" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="18" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -10847,88 +10844,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1">
-      <c r="A1" s="195" t="s">
+      <c r="A1" s="194" t="s">
         <v>496</v>
       </c>
-      <c r="B1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="195" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="195" t="s">
+      <c r="B1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="194" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="194" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11274,175 +11271,177 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="227" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A6" s="220"/>
-      <c r="B6" s="219" t="s">
+    <row r="6" spans="1:28" s="226" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="219">
+        <v>4</v>
+      </c>
+      <c r="B6" s="220" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="220" t="s">
+      <c r="C6" s="219" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="222">
+      <c r="D6" s="221">
         <v>46274</v>
       </c>
-      <c r="E6" s="220"/>
-      <c r="F6" s="220">
+      <c r="E6" s="219"/>
+      <c r="F6" s="219">
         <v>262613</v>
       </c>
-      <c r="G6" s="220">
+      <c r="G6" s="219">
         <v>8223</v>
       </c>
-      <c r="H6" s="220">
+      <c r="H6" s="219">
         <v>700</v>
       </c>
-      <c r="I6" s="223">
+      <c r="I6" s="222">
         <v>0.64200000000000002</v>
       </c>
-      <c r="J6" s="223">
+      <c r="J6" s="222">
         <v>2.0790000000000002</v>
       </c>
-      <c r="K6" s="220" t="s">
+      <c r="K6" s="219" t="s">
         <v>129</v>
       </c>
-      <c r="L6" s="223">
+      <c r="L6" s="222">
         <v>934.303</v>
       </c>
-      <c r="M6" s="224">
+      <c r="M6" s="223">
         <v>727.7</v>
       </c>
-      <c r="N6" s="225">
+      <c r="N6" s="224">
         <v>0.1011</v>
       </c>
-      <c r="O6" s="226">
+      <c r="O6" s="225">
         <v>6.06</v>
       </c>
-      <c r="P6" s="220">
+      <c r="P6" s="219">
         <v>502.7</v>
       </c>
-      <c r="Q6" s="220">
+      <c r="Q6" s="219">
         <v>2</v>
       </c>
-      <c r="R6" s="220">
+      <c r="R6" s="219">
         <v>1350</v>
       </c>
-      <c r="S6" s="223">
+      <c r="S6" s="222">
         <v>1.284</v>
       </c>
-      <c r="T6" s="220">
+      <c r="T6" s="219">
         <v>66</v>
       </c>
-      <c r="U6" s="225">
+      <c r="U6" s="224">
         <v>4.8899999999999999E-2</v>
       </c>
-      <c r="V6" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="220" t="s">
+      <c r="V6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="219" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="220">
+      <c r="X6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="219">
         <v>4</v>
       </c>
-      <c r="AB6" s="220" t="s">
+      <c r="AB6" s="219" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="227" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A7" s="220">
-        <v>4</v>
-      </c>
-      <c r="B7" s="221" t="s">
+    <row r="7" spans="1:28" s="226" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="219">
+        <v>5</v>
+      </c>
+      <c r="B7" s="220" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="220" t="s">
+      <c r="C7" s="219" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="222">
+      <c r="D7" s="221">
         <v>46279</v>
       </c>
-      <c r="E7" s="220"/>
-      <c r="F7" s="220">
+      <c r="E7" s="219"/>
+      <c r="F7" s="219">
         <v>262610</v>
       </c>
-      <c r="G7" s="220">
+      <c r="G7" s="219">
         <v>8235</v>
       </c>
-      <c r="H7" s="220">
+      <c r="H7" s="219">
         <v>1000</v>
       </c>
-      <c r="I7" s="223">
+      <c r="I7" s="222">
         <v>0.64500000000000002</v>
       </c>
-      <c r="J7" s="223">
+      <c r="J7" s="222">
         <v>1.526</v>
       </c>
-      <c r="K7" s="220" t="s">
+      <c r="K7" s="219" t="s">
         <v>726</v>
       </c>
-      <c r="L7" s="223">
+      <c r="L7" s="222">
         <v>984.27</v>
       </c>
-      <c r="M7" s="224">
+      <c r="M7" s="223">
         <v>763</v>
       </c>
-      <c r="N7" s="225">
+      <c r="N7" s="224">
         <v>0.106</v>
       </c>
-      <c r="O7" s="226">
+      <c r="O7" s="225">
         <v>6.36</v>
       </c>
-      <c r="P7" s="220">
+      <c r="P7" s="219">
         <v>529.5</v>
       </c>
-      <c r="Q7" s="220">
+      <c r="Q7" s="219">
         <v>2</v>
       </c>
-      <c r="R7" s="220">
+      <c r="R7" s="219">
         <v>1350</v>
       </c>
-      <c r="S7" s="223">
+      <c r="S7" s="222">
         <v>1.29</v>
       </c>
-      <c r="T7" s="220">
+      <c r="T7" s="219">
         <v>60</v>
       </c>
-      <c r="U7" s="225">
+      <c r="U7" s="224">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="V7" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="220" t="s">
+      <c r="V7" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="219" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="220" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="220">
+      <c r="X7" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="219" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="219">
         <v>6</v>
       </c>
-      <c r="AB7" s="220" t="s">
+      <c r="AB7" s="219" t="s">
         <v>727</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="133">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>63</v>
@@ -11527,90 +11526,92 @@
       </c>
     </row>
     <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A9" s="220"/>
-      <c r="B9" s="98" t="s">
+      <c r="A9" s="219">
+        <v>7</v>
+      </c>
+      <c r="B9" s="186" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="97" t="s">
+      <c r="C9" s="185" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="228">
+      <c r="D9" s="227">
         <v>46274</v>
       </c>
-      <c r="E9" s="97"/>
-      <c r="F9" s="97">
+      <c r="E9" s="185"/>
+      <c r="F9" s="185">
         <v>262612</v>
       </c>
-      <c r="G9" s="97">
+      <c r="G9" s="185">
         <v>8223</v>
       </c>
-      <c r="H9" s="97">
+      <c r="H9" s="185">
         <v>835</v>
       </c>
-      <c r="I9" s="99">
+      <c r="I9" s="187">
         <v>1.018</v>
       </c>
-      <c r="J9" s="99">
+      <c r="J9" s="187">
         <v>0.64500000000000002</v>
       </c>
-      <c r="K9" s="97" t="s">
+      <c r="K9" s="185" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="99">
+      <c r="L9" s="187">
         <v>548.26900000000001</v>
       </c>
-      <c r="M9" s="100">
+      <c r="M9" s="188">
         <v>538.6</v>
       </c>
-      <c r="N9" s="101">
+      <c r="N9" s="189">
         <v>0.14960000000000001</v>
       </c>
-      <c r="O9" s="102">
+      <c r="O9" s="190">
         <v>8.98</v>
       </c>
-      <c r="P9" s="97">
+      <c r="P9" s="185">
         <v>295</v>
       </c>
-      <c r="Q9" s="97">
+      <c r="Q9" s="185">
         <v>1</v>
       </c>
-      <c r="R9" s="97">
+      <c r="R9" s="185">
         <v>1050</v>
       </c>
-      <c r="S9" s="99">
+      <c r="S9" s="187">
         <v>1.018</v>
       </c>
-      <c r="T9" s="97">
+      <c r="T9" s="185">
         <v>32</v>
       </c>
-      <c r="U9" s="101">
+      <c r="U9" s="189">
         <v>3.0499999999999999E-2</v>
       </c>
-      <c r="V9" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="97" t="s">
+      <c r="V9" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="185" t="s">
         <v>29</v>
       </c>
-      <c r="X9" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z9" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA9" s="97">
+      <c r="X9" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z9" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA9" s="185">
         <v>2</v>
       </c>
-      <c r="AB9" s="97" t="s">
+      <c r="AB9" s="185" t="s">
         <v>728</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="133">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>63</v>
@@ -11695,90 +11696,92 @@
       </c>
     </row>
     <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A11" s="220"/>
-      <c r="B11" s="98" t="s">
+      <c r="A11" s="219">
+        <v>9</v>
+      </c>
+      <c r="B11" s="186" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="97" t="s">
+      <c r="C11" s="185" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="228">
+      <c r="D11" s="227">
         <v>46274</v>
       </c>
-      <c r="E11" s="97"/>
-      <c r="F11" s="97">
+      <c r="E11" s="185"/>
+      <c r="F11" s="185">
         <v>262614</v>
       </c>
-      <c r="G11" s="97">
+      <c r="G11" s="185">
         <v>8223</v>
       </c>
-      <c r="H11" s="97">
+      <c r="H11" s="185">
         <v>3300</v>
       </c>
-      <c r="I11" s="99">
+      <c r="I11" s="187">
         <v>0.39700000000000002</v>
       </c>
-      <c r="J11" s="99">
+      <c r="J11" s="187">
         <v>1.04</v>
       </c>
-      <c r="K11" s="97" t="s">
+      <c r="K11" s="185" t="s">
         <v>730</v>
       </c>
-      <c r="L11" s="99">
+      <c r="L11" s="187">
         <v>1362.5039999999999</v>
       </c>
-      <c r="M11" s="100">
+      <c r="M11" s="188">
         <v>1716</v>
       </c>
-      <c r="N11" s="101">
+      <c r="N11" s="189">
         <v>0.23830000000000001</v>
       </c>
-      <c r="O11" s="102">
+      <c r="O11" s="190">
         <v>14.3</v>
       </c>
-      <c r="P11" s="97">
+      <c r="P11" s="185">
         <v>733</v>
       </c>
-      <c r="Q11" s="97">
+      <c r="Q11" s="185">
         <v>2</v>
       </c>
-      <c r="R11" s="97">
+      <c r="R11" s="185">
         <v>850</v>
       </c>
-      <c r="S11" s="99">
+      <c r="S11" s="187">
         <v>0.79400000000000004</v>
       </c>
-      <c r="T11" s="97">
+      <c r="T11" s="185">
         <v>56</v>
       </c>
-      <c r="U11" s="101">
+      <c r="U11" s="189">
         <v>6.59E-2</v>
       </c>
-      <c r="V11" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="97" t="s">
+      <c r="V11" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="185" t="s">
         <v>29</v>
       </c>
-      <c r="X11" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z11" s="97" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA11" s="97">
+      <c r="X11" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z11" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA11" s="185">
         <v>5</v>
       </c>
-      <c r="AB11" s="97" t="s">
+      <c r="AB11" s="185" t="s">
         <v>731</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="133">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>63</v>
@@ -11864,7 +11867,7 @@
     </row>
     <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="133">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B13" s="134" t="s">
         <v>63</v>
@@ -11950,7 +11953,7 @@
     </row>
     <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="133">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B14" s="134" t="s">
         <v>63</v>
@@ -12036,7 +12039,7 @@
     </row>
     <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="133">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B15" s="134" t="s">
         <v>63</v>
@@ -12122,7 +12125,7 @@
     </row>
     <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="133">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>63</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (15/09/2026 16:05)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1BD8DF-3335-49C9-B9C2-72AFCA772BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B1B6E1C-8B16-4D57-8425-FDE4588754AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (15/09/2026 16:45)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B1B6E1C-8B16-4D57-8425-FDE4588754AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4A1AFD-EC1E-4B21-B956-A4EAAB8713E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="HARMONY EMBALAGENS 1199" sheetId="151" r:id="rId4"/>
     <sheet name="FAVINCO EMBALAGENS 1197" sheetId="150" r:id="rId5"/>
     <sheet name="ABAPEL 1196" sheetId="149" r:id="rId6"/>
-    <sheet name="CARPELL LTDA 1195" sheetId="147" r:id="rId7"/>
+    <sheet name="CARPELL LTDA 1195 P" sheetId="147" r:id="rId7"/>
     <sheet name="Renovapel 1192 P" sheetId="146" r:id="rId8"/>
     <sheet name="DR EMBALAGENS 1189  P" sheetId="144" r:id="rId9"/>
     <sheet name="FAVINCO EMBALAGENS 1188 R" sheetId="143" r:id="rId10"/>
@@ -2419,7 +2419,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2456,6 +2456,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3062,9 +3068,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3110,9 +3113,6 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3139,6 +3139,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5668,88 +5674,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="202" t="s">
         <v>554</v>
       </c>
-      <c r="B1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="203" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="203" t="s">
+      <c r="B1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="202" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="202" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5839,89 +5845,89 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A3" s="204">
+    <row r="3" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A3" s="203">
         <v>1</v>
       </c>
-      <c r="B3" s="205" t="s">
+      <c r="B3" s="204" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="204" t="s">
+      <c r="C3" s="203" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="204" t="s">
+      <c r="D3" s="203" t="s">
         <v>543</v>
       </c>
-      <c r="E3" s="204" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="204">
+      <c r="E3" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="203">
         <v>262497</v>
       </c>
-      <c r="G3" s="204" t="s">
+      <c r="G3" s="203" t="s">
         <v>542</v>
       </c>
-      <c r="H3" s="204">
+      <c r="H3" s="203">
         <v>225</v>
       </c>
-      <c r="I3" s="206">
+      <c r="I3" s="205">
         <v>1.548</v>
       </c>
-      <c r="J3" s="206">
+      <c r="J3" s="205">
         <v>1.62</v>
       </c>
-      <c r="K3" s="204" t="s">
+      <c r="K3" s="203" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="206">
+      <c r="L3" s="205">
         <v>564.24599999999998</v>
       </c>
-      <c r="M3" s="207">
+      <c r="M3" s="206">
         <v>364.5</v>
       </c>
-      <c r="N3" s="208">
+      <c r="N3" s="207">
         <v>0.1013</v>
       </c>
-      <c r="O3" s="209">
+      <c r="O3" s="208">
         <v>6.08</v>
       </c>
-      <c r="P3" s="204">
+      <c r="P3" s="203">
         <v>334.6</v>
       </c>
-      <c r="Q3" s="204">
+      <c r="Q3" s="203">
         <v>1</v>
       </c>
-      <c r="R3" s="204">
+      <c r="R3" s="203">
         <v>1600</v>
       </c>
-      <c r="S3" s="206">
+      <c r="S3" s="205">
         <v>1.548</v>
       </c>
-      <c r="T3" s="204">
+      <c r="T3" s="203">
         <v>52</v>
       </c>
-      <c r="U3" s="208">
+      <c r="U3" s="207">
         <v>3.2500000000000001E-2</v>
       </c>
-      <c r="V3" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="204" t="s">
+      <c r="V3" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="203" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="204" t="s">
+      <c r="X3" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="203" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="204" t="s">
+      <c r="AB3" s="203" t="s">
         <v>553</v>
       </c>
     </row>
@@ -6011,261 +6017,261 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A5" s="204">
+    <row r="5" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="203">
         <v>3</v>
       </c>
-      <c r="B5" s="205" t="s">
+      <c r="B5" s="204" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="204" t="s">
+      <c r="C5" s="203" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="204" t="s">
+      <c r="D5" s="203" t="s">
         <v>543</v>
       </c>
-      <c r="E5" s="204" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="204">
+      <c r="E5" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="203">
         <v>262495</v>
       </c>
-      <c r="G5" s="204" t="s">
+      <c r="G5" s="203" t="s">
         <v>542</v>
       </c>
-      <c r="H5" s="204">
+      <c r="H5" s="203">
         <v>395</v>
       </c>
-      <c r="I5" s="206">
+      <c r="I5" s="205">
         <v>0.69</v>
       </c>
-      <c r="J5" s="206">
+      <c r="J5" s="205">
         <v>2.0699999999999998</v>
       </c>
-      <c r="K5" s="204" t="s">
+      <c r="K5" s="203" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="206">
+      <c r="L5" s="205">
         <v>564.178</v>
       </c>
-      <c r="M5" s="207">
+      <c r="M5" s="206">
         <v>408.8</v>
       </c>
-      <c r="N5" s="208">
+      <c r="N5" s="207">
         <v>5.6800000000000003E-2</v>
       </c>
-      <c r="O5" s="209">
+      <c r="O5" s="208">
         <v>3.41</v>
       </c>
-      <c r="P5" s="204">
+      <c r="P5" s="203">
         <v>334.6</v>
       </c>
-      <c r="Q5" s="204">
+      <c r="Q5" s="203">
         <v>2</v>
       </c>
-      <c r="R5" s="204">
+      <c r="R5" s="203">
         <v>1400</v>
       </c>
-      <c r="S5" s="206">
+      <c r="S5" s="205">
         <v>1.38</v>
       </c>
-      <c r="T5" s="204">
+      <c r="T5" s="203">
         <v>20</v>
       </c>
-      <c r="U5" s="208">
+      <c r="U5" s="207">
         <v>1.43E-2</v>
       </c>
-      <c r="V5" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="204" t="s">
+      <c r="V5" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="203" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="204" t="s">
+      <c r="X5" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="203" t="s">
         <v>30</v>
       </c>
-      <c r="AB5" s="204" t="s">
+      <c r="AB5" s="203" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A6" s="204">
+    <row r="6" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="203">
         <v>4</v>
       </c>
-      <c r="B6" s="205" t="s">
+      <c r="B6" s="204" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="204" t="s">
+      <c r="C6" s="203" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="204" t="s">
+      <c r="D6" s="203" t="s">
         <v>543</v>
       </c>
-      <c r="E6" s="204" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="204">
+      <c r="E6" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="203">
         <v>262496</v>
       </c>
-      <c r="G6" s="204" t="s">
+      <c r="G6" s="203" t="s">
         <v>542</v>
       </c>
-      <c r="H6" s="204">
+      <c r="H6" s="203">
         <v>610</v>
       </c>
-      <c r="I6" s="206">
+      <c r="I6" s="205">
         <v>1.29</v>
       </c>
-      <c r="J6" s="206">
+      <c r="J6" s="205">
         <v>1.59</v>
       </c>
-      <c r="K6" s="204" t="s">
+      <c r="K6" s="203" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="206">
+      <c r="L6" s="205">
         <v>1251.171</v>
       </c>
-      <c r="M6" s="207">
+      <c r="M6" s="206">
         <v>969.9</v>
       </c>
-      <c r="N6" s="208">
+      <c r="N6" s="207">
         <v>0.26939999999999997</v>
       </c>
-      <c r="O6" s="209">
+      <c r="O6" s="208">
         <v>16.170000000000002</v>
       </c>
-      <c r="P6" s="204">
+      <c r="P6" s="203">
         <v>741.9</v>
       </c>
-      <c r="Q6" s="204">
+      <c r="Q6" s="203">
         <v>1</v>
       </c>
-      <c r="R6" s="204">
+      <c r="R6" s="203">
         <v>1350</v>
       </c>
-      <c r="S6" s="206">
+      <c r="S6" s="205">
         <v>1.29</v>
       </c>
-      <c r="T6" s="204">
+      <c r="T6" s="203">
         <v>60</v>
       </c>
-      <c r="U6" s="208">
+      <c r="U6" s="207">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="V6" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="204" t="s">
+      <c r="V6" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="203" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="204" t="s">
+      <c r="X6" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="203" t="s">
         <v>32</v>
       </c>
-      <c r="AB6" s="204" t="s">
+      <c r="AB6" s="203" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="202" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A7" s="204">
+    <row r="7" spans="1:28" s="201" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="203">
         <v>5</v>
       </c>
-      <c r="B7" s="205" t="s">
+      <c r="B7" s="204" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="204" t="s">
+      <c r="C7" s="203" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="204" t="s">
+      <c r="D7" s="203" t="s">
         <v>543</v>
       </c>
-      <c r="E7" s="204" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="204">
+      <c r="E7" s="203" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="203">
         <v>262494</v>
       </c>
-      <c r="G7" s="204" t="s">
+      <c r="G7" s="203" t="s">
         <v>542</v>
       </c>
-      <c r="H7" s="204">
+      <c r="H7" s="203">
         <v>700</v>
       </c>
-      <c r="I7" s="206">
+      <c r="I7" s="205">
         <v>1.0740000000000001</v>
       </c>
-      <c r="J7" s="206">
+      <c r="J7" s="205">
         <v>1.27</v>
       </c>
-      <c r="K7" s="204" t="s">
+      <c r="K7" s="203" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="206">
+      <c r="L7" s="205">
         <v>954.78599999999994</v>
       </c>
-      <c r="M7" s="207">
+      <c r="M7" s="206">
         <v>889</v>
       </c>
-      <c r="N7" s="208">
+      <c r="N7" s="207">
         <v>0.24690000000000001</v>
       </c>
-      <c r="O7" s="209">
+      <c r="O7" s="208">
         <v>14.82</v>
       </c>
-      <c r="P7" s="204">
+      <c r="P7" s="203">
         <v>566.20000000000005</v>
       </c>
-      <c r="Q7" s="204">
+      <c r="Q7" s="203">
         <v>1</v>
       </c>
-      <c r="R7" s="204">
+      <c r="R7" s="203">
         <v>1100</v>
       </c>
-      <c r="S7" s="206">
+      <c r="S7" s="205">
         <v>1.0740000000000001</v>
       </c>
-      <c r="T7" s="204">
+      <c r="T7" s="203">
         <v>26</v>
       </c>
-      <c r="U7" s="208">
+      <c r="U7" s="207">
         <v>2.3599999999999999E-2</v>
       </c>
-      <c r="V7" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="204" t="s">
+      <c r="V7" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="203" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="204" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="204" t="s">
+      <c r="X7" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="203" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="203" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="204" t="s">
+      <c r="AB7" s="203" t="s">
         <v>550</v>
       </c>
     </row>
@@ -11271,171 +11277,171 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="226" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A6" s="219">
+    <row r="6" spans="1:28" s="224" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="217">
         <v>4</v>
       </c>
-      <c r="B6" s="220" t="s">
+      <c r="B6" s="218" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="219" t="s">
+      <c r="C6" s="217" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="221">
+      <c r="D6" s="219">
         <v>46274</v>
       </c>
-      <c r="E6" s="219"/>
-      <c r="F6" s="219">
+      <c r="E6" s="217"/>
+      <c r="F6" s="217">
         <v>262613</v>
       </c>
-      <c r="G6" s="219">
+      <c r="G6" s="217">
         <v>8223</v>
       </c>
-      <c r="H6" s="219">
+      <c r="H6" s="217">
         <v>700</v>
       </c>
-      <c r="I6" s="222">
+      <c r="I6" s="220">
         <v>0.64200000000000002</v>
       </c>
-      <c r="J6" s="222">
+      <c r="J6" s="220">
         <v>2.0790000000000002</v>
       </c>
-      <c r="K6" s="219" t="s">
+      <c r="K6" s="217" t="s">
         <v>129</v>
       </c>
-      <c r="L6" s="222">
+      <c r="L6" s="220">
         <v>934.303</v>
       </c>
-      <c r="M6" s="223">
+      <c r="M6" s="221">
         <v>727.7</v>
       </c>
-      <c r="N6" s="224">
+      <c r="N6" s="222">
         <v>0.1011</v>
       </c>
-      <c r="O6" s="225">
+      <c r="O6" s="223">
         <v>6.06</v>
       </c>
-      <c r="P6" s="219">
+      <c r="P6" s="217">
         <v>502.7</v>
       </c>
-      <c r="Q6" s="219">
+      <c r="Q6" s="217">
         <v>2</v>
       </c>
-      <c r="R6" s="219">
+      <c r="R6" s="217">
         <v>1350</v>
       </c>
-      <c r="S6" s="222">
+      <c r="S6" s="220">
         <v>1.284</v>
       </c>
-      <c r="T6" s="219">
+      <c r="T6" s="217">
         <v>66</v>
       </c>
-      <c r="U6" s="224">
+      <c r="U6" s="222">
         <v>4.8899999999999999E-2</v>
       </c>
-      <c r="V6" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="219" t="s">
+      <c r="V6" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="217" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="219">
+      <c r="X6" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="217">
         <v>4</v>
       </c>
-      <c r="AB6" s="219" t="s">
+      <c r="AB6" s="217" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="226" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A7" s="219">
+    <row r="7" spans="1:28" s="224" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="217">
         <v>5</v>
       </c>
-      <c r="B7" s="220" t="s">
+      <c r="B7" s="218" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="219" t="s">
+      <c r="C7" s="217" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="221">
+      <c r="D7" s="219">
         <v>46279</v>
       </c>
-      <c r="E7" s="219"/>
-      <c r="F7" s="219">
+      <c r="E7" s="217"/>
+      <c r="F7" s="217">
         <v>262610</v>
       </c>
-      <c r="G7" s="219">
+      <c r="G7" s="217">
         <v>8235</v>
       </c>
-      <c r="H7" s="219">
+      <c r="H7" s="217">
         <v>1000</v>
       </c>
-      <c r="I7" s="222">
+      <c r="I7" s="220">
         <v>0.64500000000000002</v>
       </c>
-      <c r="J7" s="222">
+      <c r="J7" s="220">
         <v>1.526</v>
       </c>
-      <c r="K7" s="219" t="s">
+      <c r="K7" s="217" t="s">
         <v>726</v>
       </c>
-      <c r="L7" s="222">
+      <c r="L7" s="220">
         <v>984.27</v>
       </c>
-      <c r="M7" s="223">
+      <c r="M7" s="221">
         <v>763</v>
       </c>
-      <c r="N7" s="224">
+      <c r="N7" s="222">
         <v>0.106</v>
       </c>
-      <c r="O7" s="225">
+      <c r="O7" s="223">
         <v>6.36</v>
       </c>
-      <c r="P7" s="219">
+      <c r="P7" s="217">
         <v>529.5</v>
       </c>
-      <c r="Q7" s="219">
+      <c r="Q7" s="217">
         <v>2</v>
       </c>
-      <c r="R7" s="219">
+      <c r="R7" s="217">
         <v>1350</v>
       </c>
-      <c r="S7" s="222">
+      <c r="S7" s="220">
         <v>1.29</v>
       </c>
-      <c r="T7" s="219">
+      <c r="T7" s="217">
         <v>60</v>
       </c>
-      <c r="U7" s="224">
+      <c r="U7" s="222">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="V7" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="219" t="s">
+      <c r="V7" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="217" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="219" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="219">
+      <c r="X7" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="217" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="217">
         <v>6</v>
       </c>
-      <c r="AB7" s="219" t="s">
+      <c r="AB7" s="217" t="s">
         <v>727</v>
       </c>
     </row>
@@ -11526,7 +11532,7 @@
       </c>
     </row>
     <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A9" s="219">
+      <c r="A9" s="217">
         <v>7</v>
       </c>
       <c r="B9" s="186" t="s">
@@ -11535,7 +11541,7 @@
       <c r="C9" s="185" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="227">
+      <c r="D9" s="225">
         <v>46274</v>
       </c>
       <c r="E9" s="185"/>
@@ -11696,7 +11702,7 @@
       </c>
     </row>
     <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A11" s="219">
+      <c r="A11" s="217">
         <v>9</v>
       </c>
       <c r="B11" s="186" t="s">
@@ -11705,7 +11711,7 @@
       <c r="C11" s="185" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="227">
+      <c r="D11" s="225">
         <v>46274</v>
       </c>
       <c r="E11" s="185"/>
@@ -24319,261 +24325,261 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="210" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A4" s="211">
+    <row r="4" spans="1:28" s="209" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A4" s="210">
         <v>2</v>
       </c>
-      <c r="B4" s="216" t="s">
+      <c r="B4" s="215" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="211" t="s">
+      <c r="C4" s="210" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="211" t="s">
+      <c r="D4" s="210" t="s">
         <v>680</v>
       </c>
-      <c r="E4" s="211" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="211">
+      <c r="E4" s="210" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="210">
         <v>262597</v>
       </c>
-      <c r="G4" s="211" t="s">
+      <c r="G4" s="210" t="s">
         <v>700</v>
       </c>
-      <c r="H4" s="211">
+      <c r="H4" s="210">
         <v>600</v>
       </c>
-      <c r="I4" s="213">
+      <c r="I4" s="212">
         <v>1.236</v>
       </c>
-      <c r="J4" s="213">
+      <c r="J4" s="212">
         <v>2.5910000000000002</v>
       </c>
-      <c r="K4" s="211" t="s">
+      <c r="K4" s="210" t="s">
         <v>522</v>
       </c>
-      <c r="L4" s="213">
+      <c r="L4" s="212">
         <v>1921.4860000000001</v>
       </c>
-      <c r="M4" s="215">
+      <c r="M4" s="214">
         <v>1554.6</v>
       </c>
-      <c r="N4" s="212">
+      <c r="N4" s="211">
         <v>0.43180000000000002</v>
       </c>
-      <c r="O4" s="214">
+      <c r="O4" s="213">
         <v>25.91</v>
       </c>
-      <c r="P4" s="211">
+      <c r="P4" s="210">
         <v>1214.4000000000001</v>
       </c>
-      <c r="Q4" s="211">
+      <c r="Q4" s="210">
         <v>1</v>
       </c>
-      <c r="R4" s="211">
+      <c r="R4" s="210">
         <v>1300</v>
       </c>
-      <c r="S4" s="213">
+      <c r="S4" s="212">
         <v>1.236</v>
       </c>
-      <c r="T4" s="211">
+      <c r="T4" s="210">
         <v>64</v>
       </c>
-      <c r="U4" s="212">
+      <c r="U4" s="211">
         <v>4.9200000000000001E-2</v>
       </c>
-      <c r="V4" s="211" t="s">
+      <c r="V4" s="210" t="s">
         <v>29</v>
       </c>
-      <c r="W4" s="211" t="s">
+      <c r="W4" s="210" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="211" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="211" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="211" t="s">
+      <c r="X4" s="210" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="210" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="210" t="s">
         <v>29</v>
       </c>
-      <c r="AA4" s="211" t="s">
+      <c r="AA4" s="210" t="s">
         <v>32</v>
       </c>
-      <c r="AB4" s="211" t="s">
+      <c r="AB4" s="210" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="210" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A5" s="211">
+    <row r="5" spans="1:28" s="209" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="210">
         <v>3</v>
       </c>
-      <c r="B5" s="216" t="s">
+      <c r="B5" s="215" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="211" t="s">
+      <c r="C5" s="210" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="211" t="s">
+      <c r="D5" s="210" t="s">
         <v>680</v>
       </c>
-      <c r="E5" s="211" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="211">
+      <c r="E5" s="210" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="210">
         <v>262596</v>
       </c>
-      <c r="G5" s="211" t="s">
+      <c r="G5" s="210" t="s">
         <v>700</v>
       </c>
-      <c r="H5" s="211">
+      <c r="H5" s="210">
         <v>2000</v>
       </c>
-      <c r="I5" s="213">
+      <c r="I5" s="212">
         <v>1.196</v>
       </c>
-      <c r="J5" s="213">
+      <c r="J5" s="212">
         <v>1.6910000000000001</v>
       </c>
-      <c r="K5" s="211" t="s">
+      <c r="K5" s="210" t="s">
         <v>519</v>
       </c>
-      <c r="L5" s="213">
+      <c r="L5" s="212">
         <v>4044.8719999999998</v>
       </c>
-      <c r="M5" s="215">
+      <c r="M5" s="214">
         <v>3382</v>
       </c>
-      <c r="N5" s="212">
+      <c r="N5" s="211">
         <v>0.93940000000000001</v>
       </c>
-      <c r="O5" s="214">
+      <c r="O5" s="213">
         <v>56.37</v>
       </c>
-      <c r="P5" s="211">
+      <c r="P5" s="210">
         <v>2556.4</v>
       </c>
-      <c r="Q5" s="211">
+      <c r="Q5" s="210">
         <v>1</v>
       </c>
-      <c r="R5" s="211">
+      <c r="R5" s="210">
         <v>1250</v>
       </c>
-      <c r="S5" s="213">
+      <c r="S5" s="212">
         <v>1.196</v>
       </c>
-      <c r="T5" s="211">
+      <c r="T5" s="210">
         <v>54</v>
       </c>
-      <c r="U5" s="212">
+      <c r="U5" s="211">
         <v>4.3200000000000002E-2</v>
       </c>
-      <c r="V5" s="211" t="s">
+      <c r="V5" s="210" t="s">
         <v>29</v>
       </c>
-      <c r="W5" s="211" t="s">
+      <c r="W5" s="210" t="s">
         <v>40</v>
       </c>
-      <c r="X5" s="211" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="211" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="211" t="s">
+      <c r="X5" s="210" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="210" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="210" t="s">
         <v>29</v>
       </c>
-      <c r="AA5" s="211" t="s">
+      <c r="AA5" s="210" t="s">
         <v>72</v>
       </c>
-      <c r="AB5" s="211" t="s">
+      <c r="AB5" s="210" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="210" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A6" s="211">
+    <row r="6" spans="1:28" s="209" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="210">
         <v>4</v>
       </c>
-      <c r="B6" s="216" t="s">
+      <c r="B6" s="215" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="211" t="s">
+      <c r="C6" s="210" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="211" t="s">
+      <c r="D6" s="210" t="s">
         <v>680</v>
       </c>
-      <c r="E6" s="211" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="211">
+      <c r="E6" s="210" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="210">
         <v>262595</v>
       </c>
-      <c r="G6" s="211" t="s">
+      <c r="G6" s="210" t="s">
         <v>700</v>
       </c>
-      <c r="H6" s="211">
+      <c r="H6" s="210">
         <v>1400</v>
       </c>
-      <c r="I6" s="213">
+      <c r="I6" s="212">
         <v>1.2050000000000001</v>
       </c>
-      <c r="J6" s="213">
+      <c r="J6" s="212">
         <v>2.5910000000000002</v>
       </c>
-      <c r="K6" s="211" t="s">
+      <c r="K6" s="210" t="s">
         <v>53</v>
       </c>
-      <c r="L6" s="213">
+      <c r="L6" s="212">
         <v>4371.0169999999998</v>
       </c>
-      <c r="M6" s="215">
+      <c r="M6" s="214">
         <v>3627.4</v>
       </c>
-      <c r="N6" s="212">
+      <c r="N6" s="211">
         <v>1.0076000000000001</v>
       </c>
-      <c r="O6" s="214">
+      <c r="O6" s="213">
         <v>60.46</v>
       </c>
-      <c r="P6" s="211">
+      <c r="P6" s="210">
         <v>2482.6999999999998</v>
       </c>
-      <c r="Q6" s="211">
+      <c r="Q6" s="210">
         <v>1</v>
       </c>
-      <c r="R6" s="211">
+      <c r="R6" s="210">
         <v>1250</v>
       </c>
-      <c r="S6" s="213">
+      <c r="S6" s="212">
         <v>1.2050000000000001</v>
       </c>
-      <c r="T6" s="211">
+      <c r="T6" s="210">
         <v>45</v>
       </c>
-      <c r="U6" s="212">
+      <c r="U6" s="211">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="V6" s="211" t="s">
+      <c r="V6" s="210" t="s">
         <v>35</v>
       </c>
-      <c r="W6" s="211" t="s">
+      <c r="W6" s="210" t="s">
         <v>40</v>
       </c>
-      <c r="X6" s="211" t="s">
+      <c r="X6" s="210" t="s">
         <v>35</v>
       </c>
-      <c r="Y6" s="211" t="s">
+      <c r="Y6" s="210" t="s">
         <v>35</v>
       </c>
-      <c r="Z6" s="211" t="s">
+      <c r="Z6" s="210" t="s">
         <v>35</v>
       </c>
-      <c r="AA6" s="211" t="s">
+      <c r="AA6" s="210" t="s">
         <v>55</v>
       </c>
-      <c r="AB6" s="211" t="s">
+      <c r="AB6" s="210" t="s">
         <v>54</v>
       </c>
     </row>
@@ -35582,11 +35588,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0213073B-7DC6-44F4-9A79-2376A05B9E79}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB29"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="108" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.5546875" style="108" customWidth="1"/>
@@ -35609,94 +35618,94 @@
     <col min="23" max="23" width="7.88671875" style="108" customWidth="1"/>
     <col min="24" max="24" width="8.6640625" style="108" customWidth="1"/>
     <col min="25" max="26" width="7" style="108" customWidth="1"/>
-    <col min="27" max="27" width="4.21875" style="108" customWidth="1"/>
-    <col min="28" max="28" width="11.5546875" style="108" customWidth="1"/>
+    <col min="27" max="27" width="9.33203125" style="108" customWidth="1"/>
+    <col min="28" max="28" width="19.88671875" style="108" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1">
-      <c r="A1" s="192" t="s">
+      <c r="A1" s="193" t="s">
         <v>652</v>
       </c>
-      <c r="B1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="192" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="192" t="s">
+      <c r="B1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="193" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="193" t="s">
         <v>27</v>
       </c>
     </row>
@@ -35786,2244 +35795,2245 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1">
-      <c r="A3" s="161">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A3" s="150">
         <v>1</v>
       </c>
-      <c r="B3" s="217" t="s">
+      <c r="B3" s="226" t="s">
         <v>626</v>
       </c>
-      <c r="C3" s="161" t="s">
+      <c r="C3" s="150" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="161" t="s">
+      <c r="D3" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E3" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="161">
+      <c r="E3" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="150">
         <v>262546</v>
       </c>
-      <c r="G3" s="161" t="s">
+      <c r="G3" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H3" s="161">
+      <c r="H3" s="150">
         <v>300</v>
       </c>
-      <c r="I3" s="163">
+      <c r="I3" s="152">
         <v>0.71</v>
       </c>
-      <c r="J3" s="163">
+      <c r="J3" s="152">
         <v>1.26</v>
       </c>
-      <c r="K3" s="161" t="s">
+      <c r="K3" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="163">
+      <c r="L3" s="152">
         <v>268.38</v>
       </c>
-      <c r="M3" s="164">
+      <c r="M3" s="153">
         <v>189</v>
       </c>
-      <c r="N3" s="165">
+      <c r="N3" s="154">
         <v>2.6200000000000001E-2</v>
       </c>
-      <c r="O3" s="166">
+      <c r="O3" s="155">
         <v>1.57</v>
       </c>
-      <c r="P3" s="161">
+      <c r="P3" s="150">
         <v>162.6</v>
       </c>
-      <c r="Q3" s="161">
+      <c r="Q3" s="150">
         <v>2</v>
       </c>
-      <c r="R3" s="161">
+      <c r="R3" s="150">
         <v>1450</v>
       </c>
-      <c r="S3" s="163">
+      <c r="S3" s="152">
         <v>1.42</v>
       </c>
-      <c r="T3" s="161">
+      <c r="T3" s="150">
         <v>30</v>
       </c>
-      <c r="U3" s="165">
+      <c r="U3" s="154">
         <v>2.07E-2</v>
       </c>
-      <c r="V3" s="161" t="s">
+      <c r="V3" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="W3" s="161" t="s">
+      <c r="W3" s="150" t="s">
         <v>40</v>
       </c>
-      <c r="X3" s="161" t="s">
+      <c r="X3" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="Y3" s="161" t="s">
+      <c r="Y3" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="Z3" s="161" t="s">
+      <c r="Z3" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="AA3" s="161" t="s">
+      <c r="AA3" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="161" t="s">
+      <c r="AB3" s="150" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1">
-      <c r="A4" s="161">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A4" s="150">
         <v>2</v>
       </c>
-      <c r="B4" s="162" t="s">
+      <c r="B4" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C4" s="161" t="s">
+      <c r="C4" s="150" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="161" t="s">
+      <c r="D4" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E4" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="161">
+      <c r="E4" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="150">
         <v>262547</v>
       </c>
-      <c r="G4" s="161" t="s">
+      <c r="G4" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H4" s="161">
+      <c r="H4" s="150">
         <v>300</v>
       </c>
-      <c r="I4" s="163">
+      <c r="I4" s="152">
         <v>0.71</v>
       </c>
-      <c r="J4" s="163">
+      <c r="J4" s="152">
         <v>1.46</v>
       </c>
-      <c r="K4" s="161" t="s">
+      <c r="K4" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="163">
+      <c r="L4" s="152">
         <v>310.98</v>
       </c>
-      <c r="M4" s="164">
+      <c r="M4" s="153">
         <v>219</v>
       </c>
-      <c r="N4" s="165">
+      <c r="N4" s="154">
         <v>3.04E-2</v>
       </c>
-      <c r="O4" s="166">
+      <c r="O4" s="155">
         <v>1.82</v>
       </c>
-      <c r="P4" s="161">
+      <c r="P4" s="150">
         <v>188.5</v>
       </c>
-      <c r="Q4" s="161">
+      <c r="Q4" s="150">
         <v>2</v>
       </c>
-      <c r="R4" s="161">
+      <c r="R4" s="150">
         <v>1450</v>
       </c>
-      <c r="S4" s="163">
+      <c r="S4" s="152">
         <v>1.42</v>
       </c>
-      <c r="T4" s="161">
+      <c r="T4" s="150">
         <v>30</v>
       </c>
-      <c r="U4" s="165">
+      <c r="U4" s="154">
         <v>2.07E-2</v>
       </c>
-      <c r="V4" s="161" t="s">
+      <c r="V4" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="W4" s="161" t="s">
+      <c r="W4" s="150" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="161" t="s">
+      <c r="X4" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="Y4" s="161" t="s">
+      <c r="Y4" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="Z4" s="161" t="s">
+      <c r="Z4" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="AA4" s="161" t="s">
+      <c r="AA4" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB4" s="161" t="s">
+      <c r="AB4" s="150" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1">
-      <c r="A5" s="161">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="150">
         <v>3</v>
       </c>
-      <c r="B5" s="162" t="s">
+      <c r="B5" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C5" s="161" t="s">
+      <c r="C5" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="161" t="s">
+      <c r="D5" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E5" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="161">
+      <c r="E5" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="150">
         <v>262560</v>
       </c>
-      <c r="G5" s="161" t="s">
+      <c r="G5" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H5" s="161">
+      <c r="H5" s="150">
         <v>500</v>
       </c>
-      <c r="I5" s="163">
+      <c r="I5" s="152">
         <v>0.49399999999999999</v>
       </c>
-      <c r="J5" s="163">
+      <c r="J5" s="152">
         <v>1.56</v>
       </c>
-      <c r="K5" s="161" t="s">
+      <c r="K5" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="163">
+      <c r="L5" s="152">
         <v>385.32</v>
       </c>
-      <c r="M5" s="164">
+      <c r="M5" s="153">
         <v>260</v>
       </c>
-      <c r="N5" s="165">
+      <c r="N5" s="154">
         <v>2.41E-2</v>
       </c>
-      <c r="O5" s="166">
+      <c r="O5" s="155">
         <v>1.44</v>
       </c>
-      <c r="P5" s="161">
+      <c r="P5" s="150">
         <v>132.9</v>
       </c>
-      <c r="Q5" s="161">
+      <c r="Q5" s="150">
         <v>3</v>
       </c>
-      <c r="R5" s="161">
+      <c r="R5" s="150">
         <v>1550</v>
       </c>
-      <c r="S5" s="163">
+      <c r="S5" s="152">
         <v>1.482</v>
       </c>
-      <c r="T5" s="161">
+      <c r="T5" s="150">
         <v>68</v>
       </c>
-      <c r="U5" s="165">
+      <c r="U5" s="154">
         <v>4.3900000000000002E-2</v>
       </c>
-      <c r="V5" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="161" t="s">
+      <c r="V5" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB5" s="161" t="s">
+      <c r="AB5" s="150" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1">
-      <c r="A6" s="161">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="150">
         <v>4</v>
       </c>
-      <c r="B6" s="162" t="s">
+      <c r="B6" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C6" s="161" t="s">
+      <c r="C6" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="161" t="s">
+      <c r="D6" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E6" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="161">
+      <c r="E6" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="150">
         <v>262542</v>
       </c>
-      <c r="G6" s="161" t="s">
+      <c r="G6" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H6" s="161">
+      <c r="H6" s="150">
         <v>1000</v>
       </c>
-      <c r="I6" s="163">
+      <c r="I6" s="152">
         <v>0.70899999999999996</v>
       </c>
-      <c r="J6" s="163">
+      <c r="J6" s="152">
         <v>1.28</v>
       </c>
-      <c r="K6" s="161" t="s">
+      <c r="K6" s="150" t="s">
         <v>647</v>
       </c>
-      <c r="L6" s="163">
+      <c r="L6" s="152">
         <v>907.52</v>
       </c>
-      <c r="M6" s="164">
+      <c r="M6" s="153">
         <v>640</v>
       </c>
-      <c r="N6" s="165">
+      <c r="N6" s="154">
         <v>8.8900000000000007E-2</v>
       </c>
-      <c r="O6" s="166">
+      <c r="O6" s="155">
         <v>5.33</v>
       </c>
-      <c r="P6" s="161">
+      <c r="P6" s="150">
         <v>313.10000000000002</v>
       </c>
-      <c r="Q6" s="161">
+      <c r="Q6" s="150">
         <v>2</v>
       </c>
-      <c r="R6" s="161">
+      <c r="R6" s="150">
         <v>1450</v>
       </c>
-      <c r="S6" s="163">
+      <c r="S6" s="152">
         <v>1.4179999999999999</v>
       </c>
-      <c r="T6" s="161">
+      <c r="T6" s="150">
         <v>32</v>
       </c>
-      <c r="U6" s="165">
+      <c r="U6" s="154">
         <v>2.2100000000000002E-2</v>
       </c>
-      <c r="V6" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="161" t="s">
+      <c r="V6" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="150" t="s">
         <v>30</v>
       </c>
-      <c r="AB6" s="161" t="s">
+      <c r="AB6" s="150" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1">
-      <c r="A7" s="161">
+    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="150">
         <v>5</v>
       </c>
-      <c r="B7" s="162" t="s">
+      <c r="B7" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C7" s="161" t="s">
+      <c r="C7" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="161" t="s">
+      <c r="D7" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E7" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="161">
+      <c r="E7" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="150">
         <v>262543</v>
       </c>
-      <c r="G7" s="161" t="s">
+      <c r="G7" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H7" s="161">
+      <c r="H7" s="150">
         <v>1000</v>
       </c>
-      <c r="I7" s="163">
+      <c r="I7" s="152">
         <v>0.70899999999999996</v>
       </c>
-      <c r="J7" s="163">
+      <c r="J7" s="152">
         <v>1.9</v>
       </c>
-      <c r="K7" s="161" t="s">
+      <c r="K7" s="150" t="s">
         <v>647</v>
       </c>
-      <c r="L7" s="163">
+      <c r="L7" s="152">
         <v>1347.1</v>
       </c>
-      <c r="M7" s="164">
+      <c r="M7" s="153">
         <v>950</v>
       </c>
-      <c r="N7" s="165">
+      <c r="N7" s="154">
         <v>0.13189999999999999</v>
       </c>
-      <c r="O7" s="166">
+      <c r="O7" s="155">
         <v>7.92</v>
       </c>
-      <c r="P7" s="161">
+      <c r="P7" s="150">
         <v>464.7</v>
       </c>
-      <c r="Q7" s="161">
+      <c r="Q7" s="150">
         <v>2</v>
       </c>
-      <c r="R7" s="161">
+      <c r="R7" s="150">
         <v>1450</v>
       </c>
-      <c r="S7" s="163">
+      <c r="S7" s="152">
         <v>1.4179999999999999</v>
       </c>
-      <c r="T7" s="161">
+      <c r="T7" s="150">
         <v>32</v>
       </c>
-      <c r="U7" s="165">
+      <c r="U7" s="154">
         <v>2.2100000000000002E-2</v>
       </c>
-      <c r="V7" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="161" t="s">
+      <c r="V7" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="150" t="s">
         <v>30</v>
       </c>
-      <c r="AB7" s="161" t="s">
+      <c r="AB7" s="150" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1">
-      <c r="A8" s="161">
+    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A8" s="150">
         <v>6</v>
       </c>
-      <c r="B8" s="162" t="s">
+      <c r="B8" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C8" s="161" t="s">
+      <c r="C8" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="161" t="s">
+      <c r="D8" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E8" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="161">
+      <c r="E8" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="150">
         <v>262550</v>
       </c>
-      <c r="G8" s="161" t="s">
+      <c r="G8" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H8" s="161">
+      <c r="H8" s="150">
         <v>1000</v>
       </c>
-      <c r="I8" s="163">
+      <c r="I8" s="152">
         <v>0.71</v>
       </c>
-      <c r="J8" s="163">
+      <c r="J8" s="152">
         <v>1.36</v>
       </c>
-      <c r="K8" s="161" t="s">
+      <c r="K8" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="163">
+      <c r="L8" s="152">
         <v>965.6</v>
       </c>
-      <c r="M8" s="164">
+      <c r="M8" s="153">
         <v>680</v>
       </c>
-      <c r="N8" s="165">
+      <c r="N8" s="154">
         <v>9.4399999999999998E-2</v>
       </c>
-      <c r="O8" s="166">
+      <c r="O8" s="155">
         <v>5.67</v>
       </c>
-      <c r="P8" s="161">
+      <c r="P8" s="150">
         <v>333.1</v>
       </c>
-      <c r="Q8" s="161">
+      <c r="Q8" s="150">
         <v>2</v>
       </c>
-      <c r="R8" s="161">
+      <c r="R8" s="150">
         <v>1450</v>
       </c>
-      <c r="S8" s="163">
+      <c r="S8" s="152">
         <v>1.42</v>
       </c>
-      <c r="T8" s="161">
+      <c r="T8" s="150">
         <v>30</v>
       </c>
-      <c r="U8" s="165">
+      <c r="U8" s="154">
         <v>2.07E-2</v>
       </c>
-      <c r="V8" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="161" t="s">
+      <c r="V8" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="150" t="s">
         <v>30</v>
       </c>
-      <c r="AB8" s="161" t="s">
+      <c r="AB8" s="150" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1">
-      <c r="A9" s="161">
+    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A9" s="150">
         <v>7</v>
       </c>
-      <c r="B9" s="162" t="s">
+      <c r="B9" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C9" s="161" t="s">
+      <c r="C9" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="161" t="s">
+      <c r="D9" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E9" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="161">
+      <c r="E9" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="150">
         <v>262555</v>
       </c>
-      <c r="G9" s="161" t="s">
+      <c r="G9" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H9" s="161">
+      <c r="H9" s="150">
         <v>2000</v>
       </c>
-      <c r="I9" s="163">
+      <c r="I9" s="152">
         <v>0.45</v>
       </c>
-      <c r="J9" s="163">
+      <c r="J9" s="152">
         <v>0.75</v>
       </c>
-      <c r="K9" s="161" t="s">
+      <c r="K9" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="163">
+      <c r="L9" s="152">
         <v>675</v>
       </c>
-      <c r="M9" s="164">
+      <c r="M9" s="153">
         <v>500</v>
       </c>
-      <c r="N9" s="165">
+      <c r="N9" s="154">
         <v>4.6300000000000001E-2</v>
       </c>
-      <c r="O9" s="166">
+      <c r="O9" s="155">
         <v>2.78</v>
       </c>
-      <c r="P9" s="161">
+      <c r="P9" s="150">
         <v>232.9</v>
       </c>
-      <c r="Q9" s="161">
+      <c r="Q9" s="150">
         <v>3</v>
       </c>
-      <c r="R9" s="161">
+      <c r="R9" s="150">
         <v>1400</v>
       </c>
-      <c r="S9" s="163">
+      <c r="S9" s="152">
         <v>1.35</v>
       </c>
-      <c r="T9" s="161">
+      <c r="T9" s="150">
         <v>50</v>
       </c>
-      <c r="U9" s="165">
+      <c r="U9" s="154">
         <v>3.5700000000000003E-2</v>
       </c>
-      <c r="V9" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="161" t="s">
+      <c r="V9" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB9" s="161" t="s">
+      <c r="AB9" s="150" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1">
-      <c r="A10" s="161">
+    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A10" s="150">
         <v>8</v>
       </c>
-      <c r="B10" s="162" t="s">
+      <c r="B10" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C10" s="161" t="s">
+      <c r="C10" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="161" t="s">
+      <c r="D10" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E10" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="161">
+      <c r="E10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="150">
         <v>262556</v>
       </c>
-      <c r="G10" s="161" t="s">
+      <c r="G10" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H10" s="161">
+      <c r="H10" s="150">
         <v>1500</v>
       </c>
-      <c r="I10" s="163">
+      <c r="I10" s="152">
         <v>0.45</v>
       </c>
-      <c r="J10" s="163">
+      <c r="J10" s="152">
         <v>0.65</v>
       </c>
-      <c r="K10" s="161" t="s">
+      <c r="K10" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L10" s="163">
+      <c r="L10" s="152">
         <v>438.75</v>
       </c>
-      <c r="M10" s="164">
+      <c r="M10" s="153">
         <v>325</v>
       </c>
-      <c r="N10" s="165">
+      <c r="N10" s="154">
         <v>3.0099999999999998E-2</v>
       </c>
-      <c r="O10" s="166">
+      <c r="O10" s="155">
         <v>1.81</v>
       </c>
-      <c r="P10" s="161">
+      <c r="P10" s="150">
         <v>151.4</v>
       </c>
-      <c r="Q10" s="161">
+      <c r="Q10" s="150">
         <v>3</v>
       </c>
-      <c r="R10" s="161">
+      <c r="R10" s="150">
         <v>1400</v>
       </c>
-      <c r="S10" s="163">
+      <c r="S10" s="152">
         <v>1.35</v>
       </c>
-      <c r="T10" s="161">
+      <c r="T10" s="150">
         <v>50</v>
       </c>
-      <c r="U10" s="165">
+      <c r="U10" s="154">
         <v>3.5700000000000003E-2</v>
       </c>
-      <c r="V10" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="161" t="s">
+      <c r="V10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB10" s="161" t="s">
+      <c r="AB10" s="150" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1">
-      <c r="A11" s="161">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A11" s="150">
         <v>9</v>
       </c>
-      <c r="B11" s="162" t="s">
+      <c r="B11" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C11" s="161" t="s">
+      <c r="C11" s="150" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="161" t="s">
+      <c r="D11" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E11" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="161">
+      <c r="E11" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="150">
         <v>262565</v>
       </c>
-      <c r="G11" s="161" t="s">
+      <c r="G11" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H11" s="161">
+      <c r="H11" s="150">
         <v>500</v>
       </c>
-      <c r="I11" s="163">
+      <c r="I11" s="152">
         <v>0.46</v>
       </c>
-      <c r="J11" s="163">
+      <c r="J11" s="152">
         <v>0.9</v>
       </c>
-      <c r="K11" s="161" t="s">
+      <c r="K11" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="163">
+      <c r="L11" s="152">
         <v>207</v>
       </c>
-      <c r="M11" s="164">
+      <c r="M11" s="153">
         <v>150</v>
       </c>
-      <c r="N11" s="165">
+      <c r="N11" s="154">
         <v>1.3899999999999999E-2</v>
       </c>
-      <c r="O11" s="166">
+      <c r="O11" s="155">
         <v>0.83</v>
       </c>
-      <c r="P11" s="161">
+      <c r="P11" s="150">
         <v>78.2</v>
       </c>
-      <c r="Q11" s="161">
+      <c r="Q11" s="150">
         <v>3</v>
       </c>
-      <c r="R11" s="161">
+      <c r="R11" s="150">
         <v>1400</v>
       </c>
-      <c r="S11" s="163">
+      <c r="S11" s="152">
         <v>1.38</v>
       </c>
-      <c r="T11" s="161">
+      <c r="T11" s="150">
         <v>20</v>
       </c>
-      <c r="U11" s="165">
+      <c r="U11" s="154">
         <v>1.43E-2</v>
       </c>
-      <c r="V11" s="161" t="s">
+      <c r="V11" s="150" t="s">
         <v>38</v>
       </c>
-      <c r="W11" s="161" t="s">
+      <c r="W11" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="X11" s="161" t="s">
+      <c r="X11" s="150" t="s">
         <v>35</v>
       </c>
-      <c r="Y11" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="161" t="s">
+      <c r="Y11" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB11" s="161" t="s">
+      <c r="AB11" s="150" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1">
-      <c r="A12" s="161">
+    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A12" s="150">
         <v>10</v>
       </c>
-      <c r="B12" s="162" t="s">
+      <c r="B12" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C12" s="161" t="s">
+      <c r="C12" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="161" t="s">
+      <c r="D12" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E12" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="161">
+      <c r="E12" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="150">
         <v>262563</v>
       </c>
-      <c r="G12" s="161" t="s">
+      <c r="G12" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H12" s="161">
+      <c r="H12" s="150">
         <v>500</v>
       </c>
-      <c r="I12" s="163">
+      <c r="I12" s="152">
         <v>0.66</v>
       </c>
-      <c r="J12" s="163">
+      <c r="J12" s="152">
         <v>1.2</v>
       </c>
-      <c r="K12" s="161" t="s">
+      <c r="K12" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L12" s="163">
+      <c r="L12" s="152">
         <v>396</v>
       </c>
-      <c r="M12" s="164">
+      <c r="M12" s="153">
         <v>300</v>
       </c>
-      <c r="N12" s="165">
+      <c r="N12" s="154">
         <v>4.1700000000000001E-2</v>
       </c>
-      <c r="O12" s="166">
+      <c r="O12" s="155">
         <v>2.5</v>
       </c>
-      <c r="P12" s="161">
+      <c r="P12" s="150">
         <v>136.6</v>
       </c>
-      <c r="Q12" s="161">
+      <c r="Q12" s="150">
         <v>2</v>
       </c>
-      <c r="R12" s="161">
+      <c r="R12" s="150">
         <v>1350</v>
       </c>
-      <c r="S12" s="163">
+      <c r="S12" s="152">
         <v>1.32</v>
       </c>
-      <c r="T12" s="161">
+      <c r="T12" s="150">
         <v>30</v>
       </c>
-      <c r="U12" s="165">
+      <c r="U12" s="154">
         <v>2.2200000000000001E-2</v>
       </c>
-      <c r="V12" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X12" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="161" t="s">
+      <c r="V12" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB12" s="161" t="s">
+      <c r="AB12" s="150" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1">
-      <c r="A13" s="161">
+    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A13" s="150">
         <v>11</v>
       </c>
-      <c r="B13" s="162" t="s">
+      <c r="B13" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C13" s="161" t="s">
+      <c r="C13" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="161" t="s">
+      <c r="D13" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E13" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="161">
+      <c r="E13" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="150">
         <v>262564</v>
       </c>
-      <c r="G13" s="161" t="s">
+      <c r="G13" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H13" s="161">
+      <c r="H13" s="150">
         <v>1000</v>
       </c>
-      <c r="I13" s="163">
+      <c r="I13" s="152">
         <v>0.432</v>
       </c>
-      <c r="J13" s="163">
+      <c r="J13" s="152">
         <v>1.44</v>
       </c>
-      <c r="K13" s="161" t="s">
+      <c r="K13" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L13" s="163">
+      <c r="L13" s="152">
         <v>311.04000000000002</v>
       </c>
-      <c r="M13" s="164">
+      <c r="M13" s="153">
         <v>240</v>
       </c>
-      <c r="N13" s="165">
+      <c r="N13" s="154">
         <v>2.2200000000000001E-2</v>
       </c>
-      <c r="O13" s="166">
+      <c r="O13" s="155">
         <v>1.33</v>
       </c>
-      <c r="P13" s="161">
+      <c r="P13" s="150">
         <v>107.3</v>
       </c>
-      <c r="Q13" s="161">
+      <c r="Q13" s="150">
         <v>3</v>
       </c>
-      <c r="R13" s="161">
+      <c r="R13" s="150">
         <v>1350</v>
       </c>
-      <c r="S13" s="163">
+      <c r="S13" s="152">
         <v>1.296</v>
       </c>
-      <c r="T13" s="161">
+      <c r="T13" s="150">
         <v>54</v>
       </c>
-      <c r="U13" s="165">
+      <c r="U13" s="154">
         <v>0.04</v>
       </c>
-      <c r="V13" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W13" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X13" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y13" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="161" t="s">
+      <c r="V13" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB13" s="161" t="s">
+      <c r="AB13" s="150" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1">
-      <c r="A14" s="161">
+    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A14" s="150">
         <v>12</v>
       </c>
-      <c r="B14" s="162" t="s">
+      <c r="B14" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C14" s="161" t="s">
+      <c r="C14" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="161" t="s">
+      <c r="D14" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E14" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="161">
+      <c r="E14" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="150">
         <v>262544</v>
       </c>
-      <c r="G14" s="161" t="s">
+      <c r="G14" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H14" s="161">
+      <c r="H14" s="150">
         <v>500</v>
       </c>
-      <c r="I14" s="163">
+      <c r="I14" s="152">
         <v>0.6</v>
       </c>
-      <c r="J14" s="163">
+      <c r="J14" s="152">
         <v>1.1399999999999999</v>
       </c>
-      <c r="K14" s="161" t="s">
+      <c r="K14" s="150" t="s">
         <v>640</v>
       </c>
-      <c r="L14" s="163">
+      <c r="L14" s="152">
         <v>342</v>
       </c>
-      <c r="M14" s="164">
+      <c r="M14" s="153">
         <v>285</v>
       </c>
-      <c r="N14" s="165">
+      <c r="N14" s="154">
         <v>3.9600000000000003E-2</v>
       </c>
-      <c r="O14" s="166">
+      <c r="O14" s="155">
         <v>2.38</v>
       </c>
-      <c r="P14" s="161">
+      <c r="P14" s="150">
         <v>118</v>
       </c>
-      <c r="Q14" s="161">
+      <c r="Q14" s="150">
         <v>2</v>
       </c>
-      <c r="R14" s="161">
+      <c r="R14" s="150">
         <v>1250</v>
       </c>
-      <c r="S14" s="163">
+      <c r="S14" s="152">
         <v>1.2</v>
       </c>
-      <c r="T14" s="161">
+      <c r="T14" s="150">
         <v>50</v>
       </c>
-      <c r="U14" s="165">
+      <c r="U14" s="154">
         <v>0.04</v>
       </c>
-      <c r="V14" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W14" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X14" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y14" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z14" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA14" s="161" t="s">
+      <c r="V14" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB14" s="161" t="s">
+      <c r="AB14" s="150" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1">
-      <c r="A15" s="161">
+    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A15" s="150">
         <v>13</v>
       </c>
-      <c r="B15" s="162" t="s">
+      <c r="B15" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C15" s="161" t="s">
+      <c r="C15" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="161" t="s">
+      <c r="D15" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E15" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="161">
+      <c r="E15" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="150">
         <v>262561</v>
       </c>
-      <c r="G15" s="161" t="s">
+      <c r="G15" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H15" s="161">
+      <c r="H15" s="150">
         <v>500</v>
       </c>
-      <c r="I15" s="163">
+      <c r="I15" s="152">
         <v>0.61499999999999999</v>
       </c>
-      <c r="J15" s="163">
+      <c r="J15" s="152">
         <v>0.9</v>
       </c>
-      <c r="K15" s="161" t="s">
+      <c r="K15" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L15" s="163">
+      <c r="L15" s="152">
         <v>276.75</v>
       </c>
-      <c r="M15" s="164">
+      <c r="M15" s="153">
         <v>225</v>
       </c>
-      <c r="N15" s="165">
+      <c r="N15" s="154">
         <v>3.1300000000000001E-2</v>
       </c>
-      <c r="O15" s="166">
+      <c r="O15" s="155">
         <v>1.88</v>
       </c>
-      <c r="P15" s="161">
+      <c r="P15" s="150">
         <v>95.5</v>
       </c>
-      <c r="Q15" s="161">
+      <c r="Q15" s="150">
         <v>2</v>
       </c>
-      <c r="R15" s="161">
+      <c r="R15" s="150">
         <v>1250</v>
       </c>
-      <c r="S15" s="163">
+      <c r="S15" s="152">
         <v>1.23</v>
       </c>
-      <c r="T15" s="161">
+      <c r="T15" s="150">
         <v>20</v>
       </c>
-      <c r="U15" s="165">
+      <c r="U15" s="154">
         <v>1.6E-2</v>
       </c>
-      <c r="V15" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X15" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="161" t="s">
+      <c r="V15" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB15" s="161" t="s">
+      <c r="AB15" s="150" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="167" customFormat="1">
-      <c r="A16" s="161">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A16" s="150">
         <v>14</v>
       </c>
-      <c r="B16" s="162" t="s">
+      <c r="B16" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C16" s="161" t="s">
+      <c r="C16" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="161" t="s">
+      <c r="D16" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E16" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="161">
+      <c r="E16" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="150">
         <v>262559</v>
       </c>
-      <c r="G16" s="161" t="s">
+      <c r="G16" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H16" s="161">
+      <c r="H16" s="150">
         <v>700</v>
       </c>
-      <c r="I16" s="163">
+      <c r="I16" s="152">
         <v>0.57999999999999996</v>
       </c>
-      <c r="J16" s="163">
+      <c r="J16" s="152">
         <v>0.54</v>
       </c>
-      <c r="K16" s="161" t="s">
+      <c r="K16" s="150" t="s">
         <v>638</v>
       </c>
-      <c r="L16" s="163">
+      <c r="L16" s="152">
         <v>219.24</v>
       </c>
-      <c r="M16" s="164">
+      <c r="M16" s="153">
         <v>189</v>
       </c>
-      <c r="N16" s="165">
+      <c r="N16" s="154">
         <v>2.6200000000000001E-2</v>
       </c>
-      <c r="O16" s="166">
+      <c r="O16" s="155">
         <v>1.57</v>
       </c>
-      <c r="P16" s="161">
+      <c r="P16" s="150">
         <v>75.599999999999994</v>
       </c>
-      <c r="Q16" s="161">
+      <c r="Q16" s="150">
         <v>2</v>
       </c>
-      <c r="R16" s="161">
+      <c r="R16" s="150">
         <v>1200</v>
       </c>
-      <c r="S16" s="163">
+      <c r="S16" s="152">
         <v>1.1599999999999999</v>
       </c>
-      <c r="T16" s="161">
+      <c r="T16" s="150">
         <v>40</v>
       </c>
-      <c r="U16" s="165">
+      <c r="U16" s="154">
         <v>3.3300000000000003E-2</v>
       </c>
-      <c r="V16" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W16" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X16" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y16" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z16" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA16" s="161" t="s">
+      <c r="V16" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y16" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z16" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA16" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB16" s="161" t="s">
+      <c r="AB16" s="150" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="167" customFormat="1">
-      <c r="A17" s="161">
+    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A17" s="150">
         <v>15</v>
       </c>
-      <c r="B17" s="162" t="s">
+      <c r="B17" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C17" s="161" t="s">
+      <c r="C17" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="161" t="s">
+      <c r="D17" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E17" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="161">
+      <c r="E17" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="150">
         <v>262558</v>
       </c>
-      <c r="G17" s="161" t="s">
+      <c r="G17" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H17" s="161">
+      <c r="H17" s="150">
         <v>1000</v>
       </c>
-      <c r="I17" s="163">
+      <c r="I17" s="152">
         <v>0.59</v>
       </c>
-      <c r="J17" s="163">
+      <c r="J17" s="152">
         <v>0.5</v>
       </c>
-      <c r="K17" s="161" t="s">
+      <c r="K17" s="150" t="s">
         <v>636</v>
       </c>
-      <c r="L17" s="163">
+      <c r="L17" s="152">
         <v>295</v>
       </c>
-      <c r="M17" s="164">
+      <c r="M17" s="153">
         <v>250</v>
       </c>
-      <c r="N17" s="165">
+      <c r="N17" s="154">
         <v>3.4700000000000002E-2</v>
       </c>
-      <c r="O17" s="166">
+      <c r="O17" s="155">
         <v>2.08</v>
       </c>
-      <c r="P17" s="161">
+      <c r="P17" s="150">
         <v>101.8</v>
       </c>
-      <c r="Q17" s="161">
+      <c r="Q17" s="150">
         <v>2</v>
       </c>
-      <c r="R17" s="161">
+      <c r="R17" s="150">
         <v>1200</v>
       </c>
-      <c r="S17" s="163">
+      <c r="S17" s="152">
         <v>1.18</v>
       </c>
-      <c r="T17" s="161">
+      <c r="T17" s="150">
         <v>20</v>
       </c>
-      <c r="U17" s="165">
+      <c r="U17" s="154">
         <v>1.67E-2</v>
       </c>
-      <c r="V17" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W17" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X17" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y17" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z17" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA17" s="161" t="s">
+      <c r="V17" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W17" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X17" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y17" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB17" s="161" t="s">
+      <c r="AB17" s="150" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="167" customFormat="1">
-      <c r="A18" s="161">
+    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A18" s="150">
         <v>16</v>
       </c>
-      <c r="B18" s="162" t="s">
+      <c r="B18" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C18" s="161" t="s">
+      <c r="C18" s="150" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="161" t="s">
+      <c r="D18" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E18" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="161">
+      <c r="E18" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="150">
         <v>262548</v>
       </c>
-      <c r="G18" s="161" t="s">
+      <c r="G18" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H18" s="161">
+      <c r="H18" s="150">
         <v>1000</v>
       </c>
-      <c r="I18" s="163">
+      <c r="I18" s="152">
         <v>0.55400000000000005</v>
       </c>
-      <c r="J18" s="163">
+      <c r="J18" s="152">
         <v>2.2040000000000002</v>
       </c>
-      <c r="K18" s="161" t="s">
+      <c r="K18" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L18" s="163">
+      <c r="L18" s="152">
         <v>1221.0160000000001</v>
       </c>
-      <c r="M18" s="164">
+      <c r="M18" s="153">
         <v>1102</v>
       </c>
-      <c r="N18" s="165">
+      <c r="N18" s="154">
         <v>0.15310000000000001</v>
       </c>
-      <c r="O18" s="166">
+      <c r="O18" s="155">
         <v>9.18</v>
       </c>
-      <c r="P18" s="161">
+      <c r="P18" s="150">
         <v>449.3</v>
       </c>
-      <c r="Q18" s="161">
+      <c r="Q18" s="150">
         <v>2</v>
       </c>
-      <c r="R18" s="161">
+      <c r="R18" s="150">
         <v>1150</v>
       </c>
-      <c r="S18" s="163">
+      <c r="S18" s="152">
         <v>1.1080000000000001</v>
       </c>
-      <c r="T18" s="161">
+      <c r="T18" s="150">
         <v>42</v>
       </c>
-      <c r="U18" s="165">
+      <c r="U18" s="154">
         <v>3.6499999999999998E-2</v>
       </c>
-      <c r="V18" s="161" t="s">
+      <c r="V18" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="W18" s="161" t="s">
+      <c r="W18" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="X18" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y18" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z18" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA18" s="161" t="s">
+      <c r="X18" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y18" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="150" t="s">
         <v>30</v>
       </c>
-      <c r="AB18" s="161" t="s">
+      <c r="AB18" s="150" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="167" customFormat="1">
-      <c r="A19" s="161">
+    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A19" s="150">
         <v>17</v>
       </c>
-      <c r="B19" s="162" t="s">
+      <c r="B19" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C19" s="161" t="s">
+      <c r="C19" s="150" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="161" t="s">
+      <c r="D19" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E19" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="161">
+      <c r="E19" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="150">
         <v>262549</v>
       </c>
-      <c r="G19" s="161" t="s">
+      <c r="G19" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H19" s="161">
+      <c r="H19" s="150">
         <v>1500</v>
       </c>
-      <c r="I19" s="163">
+      <c r="I19" s="152">
         <v>0.56399999999999995</v>
       </c>
-      <c r="J19" s="163">
+      <c r="J19" s="152">
         <v>2.16</v>
       </c>
-      <c r="K19" s="161" t="s">
+      <c r="K19" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L19" s="163">
+      <c r="L19" s="152">
         <v>1827.36</v>
       </c>
-      <c r="M19" s="164">
+      <c r="M19" s="153">
         <v>1620</v>
       </c>
-      <c r="N19" s="165">
+      <c r="N19" s="154">
         <v>0.22500000000000001</v>
       </c>
-      <c r="O19" s="166">
+      <c r="O19" s="155">
         <v>13.5</v>
       </c>
-      <c r="P19" s="161">
+      <c r="P19" s="150">
         <v>672.5</v>
       </c>
-      <c r="Q19" s="161">
+      <c r="Q19" s="150">
         <v>2</v>
       </c>
-      <c r="R19" s="161">
+      <c r="R19" s="150">
         <v>1150</v>
       </c>
-      <c r="S19" s="163">
+      <c r="S19" s="152">
         <v>1.1279999999999999</v>
       </c>
-      <c r="T19" s="161">
+      <c r="T19" s="150">
         <v>22</v>
       </c>
-      <c r="U19" s="165">
+      <c r="U19" s="154">
         <v>1.9099999999999999E-2</v>
       </c>
-      <c r="V19" s="161" t="s">
+      <c r="V19" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="W19" s="161" t="s">
+      <c r="W19" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="X19" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y19" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z19" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA19" s="161" t="s">
+      <c r="X19" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y19" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB19" s="161" t="s">
+      <c r="AB19" s="150" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="167" customFormat="1">
-      <c r="A20" s="161">
+    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A20" s="150">
         <v>18</v>
       </c>
-      <c r="B20" s="162" t="s">
+      <c r="B20" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C20" s="161" t="s">
+      <c r="C20" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="161" t="s">
+      <c r="D20" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E20" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F20" s="161">
+      <c r="E20" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="150">
         <v>262562</v>
       </c>
-      <c r="G20" s="161" t="s">
+      <c r="G20" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H20" s="161">
+      <c r="H20" s="150">
         <v>1000</v>
       </c>
-      <c r="I20" s="163">
+      <c r="I20" s="152">
         <v>0.33</v>
       </c>
-      <c r="J20" s="163">
+      <c r="J20" s="152">
         <v>0.76</v>
       </c>
-      <c r="K20" s="161" t="s">
+      <c r="K20" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="L20" s="163">
+      <c r="L20" s="152">
         <v>250.8</v>
       </c>
-      <c r="M20" s="164">
+      <c r="M20" s="153">
         <v>253.3</v>
       </c>
-      <c r="N20" s="165">
+      <c r="N20" s="154">
         <v>2.35E-2</v>
       </c>
-      <c r="O20" s="166">
+      <c r="O20" s="155">
         <v>1.41</v>
       </c>
-      <c r="P20" s="161">
+      <c r="P20" s="150">
         <v>86.5</v>
       </c>
-      <c r="Q20" s="161">
+      <c r="Q20" s="150">
         <v>3</v>
       </c>
-      <c r="R20" s="161">
+      <c r="R20" s="150">
         <v>1050</v>
       </c>
-      <c r="S20" s="163">
+      <c r="S20" s="152">
         <v>0.99</v>
       </c>
-      <c r="T20" s="161">
+      <c r="T20" s="150">
         <v>60</v>
       </c>
-      <c r="U20" s="165">
+      <c r="U20" s="154">
         <v>5.7099999999999998E-2</v>
       </c>
-      <c r="V20" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W20" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X20" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y20" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z20" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA20" s="161" t="s">
+      <c r="V20" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W20" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X20" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y20" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z20" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA20" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB20" s="161" t="s">
+      <c r="AB20" s="150" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="21" spans="1:28" s="167" customFormat="1">
-      <c r="A21" s="161">
+    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A21" s="150">
         <v>19</v>
       </c>
-      <c r="B21" s="162" t="s">
+      <c r="B21" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C21" s="161" t="s">
+      <c r="C21" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="161" t="s">
+      <c r="D21" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E21" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F21" s="161">
+      <c r="E21" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="150">
         <v>262545</v>
       </c>
-      <c r="G21" s="161" t="s">
+      <c r="G21" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H21" s="161">
+      <c r="H21" s="150">
         <v>2000</v>
       </c>
-      <c r="I21" s="163">
+      <c r="I21" s="152">
         <v>0.92500000000000004</v>
       </c>
-      <c r="J21" s="163">
+      <c r="J21" s="152">
         <v>1.2</v>
       </c>
-      <c r="K21" s="161" t="s">
+      <c r="K21" s="150" t="s">
         <v>632</v>
       </c>
-      <c r="L21" s="163">
+      <c r="L21" s="152">
         <v>2220</v>
       </c>
-      <c r="M21" s="164">
+      <c r="M21" s="153">
         <v>2400</v>
       </c>
-      <c r="N21" s="165">
+      <c r="N21" s="154">
         <v>0.66669999999999996</v>
       </c>
-      <c r="O21" s="166">
+      <c r="O21" s="155">
         <v>40</v>
       </c>
-      <c r="P21" s="161">
+      <c r="P21" s="150">
         <v>765.9</v>
       </c>
-      <c r="Q21" s="161">
+      <c r="Q21" s="150">
         <v>1</v>
       </c>
-      <c r="R21" s="161">
+      <c r="R21" s="150">
         <v>950</v>
       </c>
-      <c r="S21" s="163">
+      <c r="S21" s="152">
         <v>0.92500000000000004</v>
       </c>
-      <c r="T21" s="161">
+      <c r="T21" s="150">
         <v>25</v>
       </c>
-      <c r="U21" s="165">
+      <c r="U21" s="154">
         <v>2.63E-2</v>
       </c>
-      <c r="V21" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W21" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X21" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y21" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z21" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA21" s="161" t="s">
+      <c r="V21" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W21" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X21" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y21" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z21" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA21" s="150" t="s">
         <v>49</v>
       </c>
-      <c r="AB21" s="161" t="s">
+      <c r="AB21" s="150" t="s">
         <v>631</v>
       </c>
     </row>
-    <row r="22" spans="1:28" s="167" customFormat="1">
-      <c r="A22" s="161">
+    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A22" s="150">
         <v>20</v>
       </c>
-      <c r="B22" s="162" t="s">
+      <c r="B22" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C22" s="161" t="s">
+      <c r="C22" s="150" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="191">
+      <c r="D22" s="177">
         <v>46280</v>
       </c>
-      <c r="E22" s="161"/>
-      <c r="F22" s="161">
+      <c r="E22" s="150"/>
+      <c r="F22" s="150">
         <v>262609</v>
       </c>
-      <c r="G22" s="161" t="s">
+      <c r="G22" s="150" t="s">
         <v>724</v>
       </c>
-      <c r="H22" s="161">
+      <c r="H22" s="150">
         <v>1000</v>
       </c>
-      <c r="I22" s="163">
+      <c r="I22" s="152">
         <v>0.28399999999999997</v>
       </c>
-      <c r="J22" s="163">
+      <c r="J22" s="152">
         <v>1.8</v>
       </c>
-      <c r="K22" s="201" t="s">
+      <c r="K22" s="227" t="s">
         <v>44</v>
       </c>
-      <c r="L22" s="163">
+      <c r="L22" s="152">
         <v>511.2</v>
       </c>
-      <c r="M22" s="164">
+      <c r="M22" s="153">
         <v>600</v>
       </c>
-      <c r="N22" s="165">
+      <c r="N22" s="154">
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="O22" s="166">
+      <c r="O22" s="155">
         <v>3.33</v>
       </c>
-      <c r="P22" s="161">
+      <c r="P22" s="150">
         <v>176.4</v>
       </c>
-      <c r="Q22" s="161">
+      <c r="Q22" s="150">
         <v>3</v>
       </c>
-      <c r="R22" s="161">
+      <c r="R22" s="150">
         <v>900</v>
       </c>
-      <c r="S22" s="163">
+      <c r="S22" s="152">
         <v>0.85199999999999998</v>
       </c>
-      <c r="T22" s="161">
+      <c r="T22" s="150">
         <v>48</v>
       </c>
-      <c r="U22" s="165">
+      <c r="U22" s="154">
         <v>5.33E-2</v>
       </c>
-      <c r="V22" s="161" t="s">
+      <c r="V22" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="W22" s="161" t="s">
+      <c r="W22" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="X22" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y22" s="161"/>
-      <c r="Z22" s="161"/>
-      <c r="AA22" s="161">
+      <c r="X22" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y22" s="150"/>
+      <c r="Z22" s="150"/>
+      <c r="AA22" s="150">
         <v>1</v>
       </c>
-      <c r="AB22" s="161" t="s">
+      <c r="AB22" s="150" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="23" spans="1:28" s="167" customFormat="1">
-      <c r="A23" s="161">
+    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A23" s="150">
         <v>21</v>
       </c>
-      <c r="B23" s="162" t="s">
+      <c r="B23" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C23" s="161" t="s">
+      <c r="C23" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D23" s="161" t="s">
+      <c r="D23" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E23" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F23" s="161">
+      <c r="E23" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23" s="150">
         <v>262554</v>
       </c>
-      <c r="G23" s="161" t="s">
+      <c r="G23" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H23" s="161">
+      <c r="H23" s="150">
         <v>1500</v>
       </c>
-      <c r="I23" s="163">
+      <c r="I23" s="152">
         <v>0.40400000000000003</v>
       </c>
-      <c r="J23" s="163">
+      <c r="J23" s="152">
         <v>0.84</v>
       </c>
-      <c r="K23" s="161" t="s">
+      <c r="K23" s="150" t="s">
         <v>630</v>
       </c>
-      <c r="L23" s="163">
+      <c r="L23" s="152">
         <v>509.04</v>
       </c>
-      <c r="M23" s="164">
+      <c r="M23" s="153">
         <v>630</v>
       </c>
-      <c r="N23" s="165">
+      <c r="N23" s="154">
         <v>8.7499999999999994E-2</v>
       </c>
-      <c r="O23" s="166">
+      <c r="O23" s="155">
         <v>5.25</v>
       </c>
-      <c r="P23" s="161">
+      <c r="P23" s="150">
         <v>175.6</v>
       </c>
-      <c r="Q23" s="161">
+      <c r="Q23" s="150">
         <v>2</v>
       </c>
-      <c r="R23" s="161">
+      <c r="R23" s="150">
         <v>850</v>
       </c>
-      <c r="S23" s="163">
+      <c r="S23" s="152">
         <v>0.80800000000000005</v>
       </c>
-      <c r="T23" s="161">
+      <c r="T23" s="150">
         <v>42</v>
       </c>
-      <c r="U23" s="165">
+      <c r="U23" s="154">
         <v>4.9399999999999999E-2</v>
       </c>
-      <c r="V23" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W23" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X23" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y23" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z23" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA23" s="161" t="s">
+      <c r="V23" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W23" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X23" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y23" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z23" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA23" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB23" s="161" t="s">
+      <c r="AB23" s="150" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="24" spans="1:28" s="167" customFormat="1">
-      <c r="A24" s="161">
+    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A24" s="150">
         <v>22</v>
       </c>
-      <c r="B24" s="162" t="s">
+      <c r="B24" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C24" s="161" t="s">
+      <c r="C24" s="150" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="161" t="s">
+      <c r="D24" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E24" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F24" s="161">
+      <c r="E24" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="150">
         <v>262551</v>
       </c>
-      <c r="G24" s="161" t="s">
+      <c r="G24" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H24" s="161">
+      <c r="H24" s="150">
         <v>500</v>
       </c>
-      <c r="I24" s="163">
+      <c r="I24" s="152">
         <v>0.40400000000000003</v>
       </c>
-      <c r="J24" s="163">
+      <c r="J24" s="152">
         <v>1.39</v>
       </c>
-      <c r="K24" s="161" t="s">
+      <c r="K24" s="150" t="s">
         <v>279</v>
       </c>
-      <c r="L24" s="163">
+      <c r="L24" s="152">
         <v>280.77999999999997</v>
       </c>
-      <c r="M24" s="164">
+      <c r="M24" s="153">
         <v>347.5</v>
       </c>
-      <c r="N24" s="165">
+      <c r="N24" s="154">
         <v>4.8300000000000003E-2</v>
       </c>
-      <c r="O24" s="166">
+      <c r="O24" s="155">
         <v>2.9</v>
       </c>
-      <c r="P24" s="161">
+      <c r="P24" s="150">
         <v>103.3</v>
       </c>
-      <c r="Q24" s="161">
+      <c r="Q24" s="150">
         <v>2</v>
       </c>
-      <c r="R24" s="161">
+      <c r="R24" s="150">
         <v>850</v>
       </c>
-      <c r="S24" s="163">
+      <c r="S24" s="152">
         <v>0.80800000000000005</v>
       </c>
-      <c r="T24" s="161">
+      <c r="T24" s="150">
         <v>42</v>
       </c>
-      <c r="U24" s="165">
+      <c r="U24" s="154">
         <v>4.9399999999999999E-2</v>
       </c>
-      <c r="V24" s="161" t="s">
+      <c r="V24" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="W24" s="161" t="s">
+      <c r="W24" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="X24" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y24" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z24" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA24" s="161" t="s">
+      <c r="X24" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y24" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z24" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA24" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB24" s="161" t="s">
+      <c r="AB24" s="150" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="25" spans="1:28" s="167" customFormat="1">
-      <c r="A25" s="161">
+    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A25" s="150">
         <v>23</v>
       </c>
-      <c r="B25" s="162" t="s">
+      <c r="B25" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C25" s="161" t="s">
+      <c r="C25" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="161" t="s">
+      <c r="D25" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E25" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F25" s="161">
+      <c r="E25" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F25" s="150">
         <v>262552</v>
       </c>
-      <c r="G25" s="161" t="s">
+      <c r="G25" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H25" s="161">
+      <c r="H25" s="150">
         <v>3000</v>
       </c>
-      <c r="I25" s="163">
+      <c r="I25" s="152">
         <v>0.40400000000000003</v>
       </c>
-      <c r="J25" s="163">
+      <c r="J25" s="152">
         <v>1.39</v>
       </c>
-      <c r="K25" s="161" t="s">
+      <c r="K25" s="150" t="s">
         <v>279</v>
       </c>
-      <c r="L25" s="163">
+      <c r="L25" s="152">
         <v>1684.68</v>
       </c>
-      <c r="M25" s="164">
+      <c r="M25" s="153">
         <v>2085</v>
       </c>
-      <c r="N25" s="165">
+      <c r="N25" s="154">
         <v>0.28960000000000002</v>
       </c>
-      <c r="O25" s="166">
+      <c r="O25" s="155">
         <v>17.38</v>
       </c>
-      <c r="P25" s="161">
+      <c r="P25" s="150">
         <v>581.20000000000005</v>
       </c>
-      <c r="Q25" s="161">
+      <c r="Q25" s="150">
         <v>2</v>
       </c>
-      <c r="R25" s="161">
+      <c r="R25" s="150">
         <v>850</v>
       </c>
-      <c r="S25" s="163">
+      <c r="S25" s="152">
         <v>0.80800000000000005</v>
       </c>
-      <c r="T25" s="161">
+      <c r="T25" s="150">
         <v>42</v>
       </c>
-      <c r="U25" s="165">
+      <c r="U25" s="154">
         <v>4.9399999999999999E-2</v>
       </c>
-      <c r="V25" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W25" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X25" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y25" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z25" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA25" s="161" t="s">
+      <c r="V25" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W25" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X25" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y25" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z25" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA25" s="150" t="s">
         <v>32</v>
       </c>
-      <c r="AB25" s="161" t="s">
+      <c r="AB25" s="150" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="26" spans="1:28" s="167" customFormat="1">
-      <c r="A26" s="161">
+    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A26" s="150">
         <v>24</v>
       </c>
-      <c r="B26" s="162" t="s">
+      <c r="B26" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C26" s="161" t="s">
+      <c r="C26" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D26" s="161" t="s">
+      <c r="D26" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E26" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F26" s="161">
+      <c r="E26" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F26" s="150">
         <v>262553</v>
       </c>
-      <c r="G26" s="161" t="s">
+      <c r="G26" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H26" s="161">
+      <c r="H26" s="150">
         <v>2000</v>
       </c>
-      <c r="I26" s="163">
+      <c r="I26" s="152">
         <v>0.34399999999999997</v>
       </c>
-      <c r="J26" s="163">
+      <c r="J26" s="152">
         <v>1.26</v>
       </c>
-      <c r="K26" s="161" t="s">
+      <c r="K26" s="150" t="s">
         <v>628</v>
       </c>
-      <c r="L26" s="163">
+      <c r="L26" s="152">
         <v>866.88</v>
       </c>
-      <c r="M26" s="164">
+      <c r="M26" s="153">
         <v>1260</v>
       </c>
-      <c r="N26" s="165">
+      <c r="N26" s="154">
         <v>0.17499999999999999</v>
       </c>
-      <c r="O26" s="166">
+      <c r="O26" s="155">
         <v>10.5</v>
       </c>
-      <c r="P26" s="161">
+      <c r="P26" s="150">
         <v>299.10000000000002</v>
       </c>
-      <c r="Q26" s="161">
+      <c r="Q26" s="150">
         <v>2</v>
       </c>
-      <c r="R26" s="161">
+      <c r="R26" s="150">
         <v>750</v>
       </c>
-      <c r="S26" s="163">
+      <c r="S26" s="152">
         <v>0.68799999999999994</v>
       </c>
-      <c r="T26" s="161">
+      <c r="T26" s="150">
         <v>62</v>
       </c>
-      <c r="U26" s="165">
+      <c r="U26" s="154">
         <v>8.2699999999999996E-2</v>
       </c>
-      <c r="V26" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W26" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X26" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y26" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z26" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA26" s="161" t="s">
+      <c r="V26" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W26" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X26" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y26" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z26" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA26" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB26" s="161" t="s">
+      <c r="AB26" s="150" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="167" customFormat="1">
-      <c r="A27" s="161">
+    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A27" s="150">
         <v>25</v>
       </c>
-      <c r="B27" s="162" t="s">
+      <c r="B27" s="151" t="s">
         <v>626</v>
       </c>
-      <c r="C27" s="161" t="s">
+      <c r="C27" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="161" t="s">
+      <c r="D27" s="150" t="s">
         <v>625</v>
       </c>
-      <c r="E27" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="F27" s="161">
+      <c r="E27" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="150">
         <v>262557</v>
       </c>
-      <c r="G27" s="161" t="s">
+      <c r="G27" s="150" t="s">
         <v>624</v>
       </c>
-      <c r="H27" s="161">
+      <c r="H27" s="150">
         <v>1500</v>
       </c>
-      <c r="I27" s="163">
+      <c r="I27" s="152">
         <v>0.30399999999999999</v>
       </c>
-      <c r="J27" s="163">
+      <c r="J27" s="152">
         <v>0.84</v>
       </c>
-      <c r="K27" s="161" t="s">
+      <c r="K27" s="150" t="s">
         <v>319</v>
       </c>
-      <c r="L27" s="163">
+      <c r="L27" s="152">
         <v>383.04</v>
       </c>
-      <c r="M27" s="164">
+      <c r="M27" s="153">
         <v>630</v>
       </c>
-      <c r="N27" s="165">
+      <c r="N27" s="154">
         <v>8.7499999999999994E-2</v>
       </c>
-      <c r="O27" s="166">
+      <c r="O27" s="155">
         <v>5.25</v>
       </c>
-      <c r="P27" s="161">
+      <c r="P27" s="150">
         <v>132.1</v>
       </c>
-      <c r="Q27" s="161">
+      <c r="Q27" s="150">
         <v>2</v>
       </c>
-      <c r="R27" s="161">
+      <c r="R27" s="150">
         <v>650</v>
       </c>
-      <c r="S27" s="163">
+      <c r="S27" s="152">
         <v>0.60799999999999998</v>
       </c>
-      <c r="T27" s="161">
+      <c r="T27" s="150">
         <v>42</v>
       </c>
-      <c r="U27" s="165">
+      <c r="U27" s="154">
         <v>6.4600000000000005E-2</v>
       </c>
-      <c r="V27" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="W27" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="X27" s="161" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y27" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z27" s="161" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA27" s="161" t="s">
+      <c r="V27" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W27" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X27" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y27" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z27" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA27" s="150" t="s">
         <v>39</v>
       </c>
-      <c r="AB27" s="161" t="s">
+      <c r="AB27" s="150" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="28" spans="1:28" s="167" customFormat="1">
-      <c r="A28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="C28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="E28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="F28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="G28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="H28" s="168">
+    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="F28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="G28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" s="157">
         <v>25800</v>
       </c>
-      <c r="I28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="J28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="K28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="L28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="M28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="N28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="O28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="P28" s="168">
+      <c r="I28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="K28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="L28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="M28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="N28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="O28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="P28" s="157">
         <v>5957.9</v>
       </c>
-      <c r="Q28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="R28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="S28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="T28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="U28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="V28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="W28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="X28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA28" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB28" s="168" t="s">
+      <c r="Q28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="R28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="S28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="T28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="U28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="V28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="W28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="X28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA28" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB28" s="157" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:28">
-      <c r="B29" s="218"/>
+      <c r="B29" s="216"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.89" right="0.39" top="0.48" bottom="0.26" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="74" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (16/09/2026 10:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88979F9C-1FAA-4AD1-ACBA-4C9533CC7BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9C717A-CB33-4A34-9F0A-91D6A7693055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="23" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (16/09/2026 14:15)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9C717A-CB33-4A34-9F0A-91D6A7693055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F300661C-53F0-4D62-B280-59DE4F0B4DB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="23" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>
@@ -51,7 +51,6 @@
     <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId36"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -70,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6712" uniqueCount="732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6719" uniqueCount="734">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2266,6 +2265,12 @@
   </si>
   <si>
     <t>814x2100</t>
+  </si>
+  <si>
+    <t>162x190x162</t>
+  </si>
+  <si>
+    <t>1048x1362</t>
   </si>
 </sst>
 </file>
@@ -2277,7 +2282,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3372,7 +3377,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22CC649A-4A24-4BCE-A798-0B107F907AA7}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -3404,7 +3409,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>723</v>
       </c>
@@ -3490,7 +3495,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1">
+    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3576,7 +3581,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -3662,7 +3667,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -3748,7 +3753,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -3834,7 +3839,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -3920,7 +3925,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -4020,7 +4025,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.5546875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -4050,7 +4055,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>599</v>
       </c>
@@ -4136,7 +4141,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -4222,7 +4227,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -4308,7 +4313,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -4394,7 +4399,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="150"/>
       <c r="B5" s="151" t="s">
         <v>621</v>
@@ -4472,7 +4477,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="157" t="s">
         <v>27</v>
       </c>
@@ -4560,7 +4565,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:28">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="D8" s="158"/>
       <c r="J8" s="159"/>
       <c r="L8" s="159"/>
@@ -4580,7 +4585,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -4608,7 +4613,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>592</v>
       </c>
@@ -4694,7 +4699,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1">
+    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4780,7 +4785,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -4866,7 +4871,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -4952,7 +4957,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -5038,7 +5043,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -5118,7 +5123,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -5198,7 +5203,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -5284,7 +5289,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -5370,7 +5375,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -5456,7 +5461,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -5542,7 +5547,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -5643,7 +5648,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -5674,7 +5679,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="222" t="s">
         <v>554</v>
       </c>
@@ -5760,7 +5765,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -5846,7 +5851,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="193">
         <v>1</v>
       </c>
@@ -5932,7 +5937,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -6018,7 +6023,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="193">
         <v>3</v>
       </c>
@@ -6104,7 +6109,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="193">
         <v>4</v>
       </c>
@@ -6190,7 +6195,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="193">
         <v>5</v>
       </c>
@@ -6276,7 +6281,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -6362,7 +6367,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -6448,7 +6453,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -6534,7 +6539,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -6620,7 +6625,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -6706,7 +6711,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -6792,7 +6797,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -6878,7 +6883,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="157" t="s">
         <v>27</v>
       </c>
@@ -6979,7 +6984,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -7011,7 +7016,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>539</v>
       </c>
@@ -7097,7 +7102,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -7183,7 +7188,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="126">
         <v>1</v>
       </c>
@@ -7269,7 +7274,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -7355,7 +7360,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="126">
         <v>2</v>
       </c>
@@ -7441,7 +7446,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>3</v>
       </c>
@@ -7527,7 +7532,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -7613,7 +7618,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -7699,7 +7704,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -7785,7 +7790,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="10" spans="1:28">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>27</v>
       </c>
@@ -7883,7 +7888,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
   <dimension ref="A1:AB5"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -7915,7 +7920,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>535</v>
       </c>
@@ -8001,7 +8006,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -8087,7 +8092,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -8173,7 +8178,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -8259,7 +8264,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
         <v>27</v>
       </c>
@@ -8359,7 +8364,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -8391,7 +8396,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="223" t="s">
         <v>523</v>
       </c>
@@ -8477,7 +8482,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="43.2" customHeight="1">
+    <row r="2" spans="1:28" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="107" t="s">
         <v>0</v>
       </c>
@@ -8563,7 +8568,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="90">
         <v>1</v>
       </c>
@@ -8649,7 +8654,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="90">
         <v>2</v>
       </c>
@@ -8735,7 +8740,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="90">
         <v>3</v>
       </c>
@@ -8821,7 +8826,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="90">
         <v>4</v>
       </c>
@@ -8907,7 +8912,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="106" t="s">
         <v>27</v>
       </c>
@@ -9008,7 +9013,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" style="3" hidden="1" customWidth="1"/>
@@ -9040,7 +9045,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>512</v>
       </c>
@@ -9126,7 +9131,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -9212,7 +9217,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" customFormat="1">
+    <row r="3" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="120">
         <v>1</v>
       </c>
@@ -9298,7 +9303,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="4" spans="1:28" customFormat="1">
+    <row r="4" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="120">
         <v>2</v>
       </c>
@@ -9384,7 +9389,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:28" customFormat="1">
+    <row r="5" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="120">
         <v>3</v>
       </c>
@@ -9470,7 +9475,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="6" spans="1:28" customFormat="1">
+    <row r="6" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -9556,7 +9561,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="7" spans="1:28" customFormat="1">
+    <row r="7" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="120">
         <v>5</v>
       </c>
@@ -9642,7 +9647,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="8" spans="1:28" customFormat="1">
+    <row r="8" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="47">
         <v>6</v>
       </c>
@@ -9728,7 +9733,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="9" spans="1:28" customFormat="1">
+    <row r="9" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>7</v>
       </c>
@@ -9814,7 +9819,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="10" spans="1:28" customFormat="1">
+    <row r="10" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="120">
         <v>8</v>
       </c>
@@ -9900,7 +9905,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>9</v>
       </c>
@@ -9986,7 +9991,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="45" customFormat="1">
+    <row r="12" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="46" t="s">
         <v>27</v>
       </c>
@@ -10084,7 +10089,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -10115,7 +10120,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>531</v>
       </c>
@@ -10201,7 +10206,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39" customHeight="1">
+    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -10287,7 +10292,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -10373,7 +10378,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -10459,7 +10464,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -10545,7 +10550,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -10631,7 +10636,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -10717,7 +10722,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="110" t="s">
         <v>27</v>
       </c>
@@ -10818,7 +10823,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -10850,7 +10855,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>496</v>
       </c>
@@ -10936,7 +10941,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -11022,7 +11027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="133">
         <v>1</v>
       </c>
@@ -11108,7 +11113,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="133">
         <v>2</v>
       </c>
@@ -11192,7 +11197,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="133">
         <v>3</v>
       </c>
@@ -11278,7 +11283,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="207">
         <v>4</v>
       </c>
@@ -11362,7 +11367,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="207">
         <v>5</v>
       </c>
@@ -11446,7 +11451,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="133">
         <v>6</v>
       </c>
@@ -11532,7 +11537,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="207">
         <v>7</v>
       </c>
@@ -11616,7 +11621,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="133">
         <v>8</v>
       </c>
@@ -11702,7 +11707,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="207">
         <v>9</v>
       </c>
@@ -11786,7 +11791,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="133">
         <v>10</v>
       </c>
@@ -11872,7 +11877,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="133">
         <v>11</v>
       </c>
@@ -11958,7 +11963,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="133">
         <v>12</v>
       </c>
@@ -12044,7 +12049,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="133">
         <v>13</v>
       </c>
@@ -12130,7 +12135,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="133">
         <v>14</v>
       </c>
@@ -12216,7 +12221,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>27</v>
       </c>
@@ -12319,7 +12324,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -12349,7 +12354,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>486</v>
       </c>
@@ -12435,7 +12440,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -12521,7 +12526,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -12607,7 +12612,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="139">
         <v>2</v>
       </c>
@@ -12693,7 +12698,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="139"/>
       <c r="B5" s="140" t="s">
         <v>480</v>
@@ -12771,7 +12776,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="139"/>
       <c r="B6" s="140" t="s">
         <v>480</v>
@@ -12849,7 +12854,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34">
         <v>3</v>
       </c>
@@ -12935,7 +12940,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="28" t="s">
         <v>27</v>
       </c>
@@ -13035,7 +13040,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5AF4CA-00D7-4A30-8F64-AC13CDBB2809}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13067,7 +13072,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>710</v>
       </c>
@@ -13153,7 +13158,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54" customHeight="1">
+    <row r="2" spans="1:28" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13239,7 +13244,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -13325,7 +13330,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -13411,7 +13416,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -13497,7 +13502,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -13583,7 +13588,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -13683,7 +13688,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13713,7 +13718,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>475</v>
       </c>
@@ -13799,7 +13804,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13885,7 +13890,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="97">
         <v>1</v>
       </c>
@@ -13971,7 +13976,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="97">
         <v>2</v>
       </c>
@@ -14057,7 +14062,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="97">
         <v>3</v>
       </c>
@@ -14143,7 +14148,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="97">
         <v>4</v>
       </c>
@@ -14229,7 +14234,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="97">
         <v>5</v>
       </c>
@@ -14315,7 +14320,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="97">
         <v>6</v>
       </c>
@@ -14401,7 +14406,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="97">
         <v>7</v>
       </c>
@@ -14487,7 +14492,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="97">
         <v>8</v>
       </c>
@@ -14573,7 +14578,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="97">
         <v>9</v>
       </c>
@@ -14659,7 +14664,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="97">
         <v>10</v>
       </c>
@@ -14745,7 +14750,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>27</v>
       </c>
@@ -14846,7 +14851,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -14878,7 +14883,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>454</v>
       </c>
@@ -14964,7 +14969,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="50.4" customHeight="1">
+    <row r="2" spans="1:28" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -15050,7 +15055,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -15136,7 +15141,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -15222,7 +15227,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -15308,7 +15313,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -15394,7 +15399,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -15480,7 +15485,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -15581,7 +15586,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -15613,7 +15618,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="33" customHeight="1">
+    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>440</v>
       </c>
@@ -15699,7 +15704,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -15785,7 +15790,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -15871,7 +15876,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -15957,7 +15962,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -16043,7 +16048,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -16129,7 +16134,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -16215,7 +16220,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -16301,7 +16306,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -16387,7 +16392,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
@@ -16488,7 +16493,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -16519,7 +16524,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>403</v>
       </c>
@@ -16605,7 +16610,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1">
+    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -16691,7 +16696,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -16777,7 +16782,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -16861,7 +16866,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -16947,7 +16952,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -17033,7 +17038,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -17117,7 +17122,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -17201,7 +17206,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
@@ -17302,7 +17307,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" customWidth="1"/>
@@ -17332,7 +17337,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="225" t="s">
         <v>380</v>
       </c>
@@ -17418,7 +17423,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="89" t="s">
         <v>0</v>
       </c>
@@ -17504,7 +17509,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14">
         <v>1</v>
       </c>
@@ -17590,7 +17595,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14">
         <v>2</v>
       </c>
@@ -17676,7 +17681,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14">
         <v>3</v>
       </c>
@@ -17762,7 +17767,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14">
         <v>4</v>
       </c>
@@ -17848,7 +17853,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>5</v>
       </c>
@@ -17934,7 +17939,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>6</v>
       </c>
@@ -18020,7 +18025,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>7</v>
       </c>
@@ -18106,7 +18111,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>8</v>
       </c>
@@ -18192,7 +18197,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>9</v>
       </c>
@@ -18278,7 +18283,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>10</v>
       </c>
@@ -18364,7 +18369,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>11</v>
       </c>
@@ -18450,7 +18455,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
         <v>12</v>
       </c>
@@ -18536,7 +18541,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>13</v>
       </c>
@@ -18622,7 +18627,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
         <v>14</v>
       </c>
@@ -18708,7 +18713,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14">
         <v>15</v>
       </c>
@@ -18794,7 +18799,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14">
         <v>16</v>
       </c>
@@ -18880,7 +18885,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14">
         <v>17</v>
       </c>
@@ -18966,7 +18971,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14">
         <v>18</v>
       </c>
@@ -19052,7 +19057,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="25.05" customHeight="1">
+    <row r="21" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="14">
         <v>19</v>
       </c>
@@ -19138,7 +19143,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.05" customHeight="1">
+    <row r="22" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14">
         <v>20</v>
       </c>
@@ -19224,7 +19229,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.05" customHeight="1">
+    <row r="23" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14">
         <v>21</v>
       </c>
@@ -19310,7 +19315,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.05" customHeight="1">
+    <row r="24" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14">
         <v>22</v>
       </c>
@@ -19396,7 +19401,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.05" customHeight="1">
+    <row r="25" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14">
         <v>23</v>
       </c>
@@ -19482,7 +19487,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.05" customHeight="1">
+    <row r="26" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14">
         <v>24</v>
       </c>
@@ -19568,7 +19573,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="90">
         <v>10</v>
       </c>
@@ -19654,7 +19659,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.05" customHeight="1">
+    <row r="28" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="20" t="s">
         <v>27</v>
       </c>
@@ -19755,7 +19760,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" style="3" customWidth="1"/>
@@ -19787,7 +19792,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>332</v>
       </c>
@@ -19873,7 +19878,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -19959,7 +19964,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -20045,7 +20050,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -20131,7 +20136,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -20217,7 +20222,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -20303,7 +20308,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -20389,7 +20394,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:28">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="F14" s="3" t="s">
         <v>395</v>
       </c>
@@ -20409,7 +20414,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -20440,7 +20445,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>329</v>
       </c>
@@ -20526,7 +20531,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20612,7 +20617,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="81">
         <v>1</v>
       </c>
@@ -20698,7 +20703,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="81">
         <v>2</v>
       </c>
@@ -20784,7 +20789,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37" t="s">
         <v>27</v>
       </c>
@@ -20870,8 +20875,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
-    <row r="8" spans="1:28">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="D8" s="160"/>
     </row>
   </sheetData>
@@ -20889,7 +20894,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
@@ -20919,7 +20924,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>324</v>
       </c>
@@ -21005,7 +21010,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -21091,7 +21096,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -21177,7 +21182,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="34">
         <v>2</v>
       </c>
@@ -21263,7 +21268,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -21349,7 +21354,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34">
         <v>4</v>
       </c>
@@ -21435,7 +21440,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34">
         <v>5</v>
       </c>
@@ -21521,7 +21526,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="34">
         <v>6</v>
       </c>
@@ -21607,7 +21612,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="28" t="s">
         <v>27</v>
       </c>
@@ -21708,7 +21713,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -21739,7 +21744,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>281</v>
       </c>
@@ -21825,7 +21830,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1">
+    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -21911,7 +21916,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -21997,7 +22002,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -22083,7 +22088,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -22169,7 +22174,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -22255,7 +22260,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -22356,7 +22361,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB27"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -22387,7 +22392,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>258</v>
       </c>
@@ -22473,7 +22478,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -22559,7 +22564,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -22645,7 +22650,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -22731,7 +22736,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -22817,7 +22822,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -22903,7 +22908,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -22989,7 +22994,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -23075,7 +23080,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -23161,7 +23166,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -23247,7 +23252,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -23333,7 +23338,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -23419,7 +23424,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -23505,7 +23510,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -23589,7 +23594,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -23675,7 +23680,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -23761,7 +23766,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -23847,7 +23852,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -23933,7 +23938,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>27</v>
       </c>
@@ -24019,7 +24024,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:28">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
       <c r="K27" s="1" t="s">
         <v>259</v>
       </c>
@@ -24036,7 +24041,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15B73F0-D53E-458D-8A18-622E142F07EE}">
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -24068,7 +24073,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>702</v>
       </c>
@@ -24154,7 +24159,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="42.6" customHeight="1">
+    <row r="2" spans="1:28" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -24240,7 +24245,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -24326,7 +24331,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="200">
         <v>2</v>
       </c>
@@ -24412,7 +24417,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="200">
         <v>3</v>
       </c>
@@ -24498,7 +24503,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="200">
         <v>4</v>
       </c>
@@ -24584,7 +24589,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -24670,7 +24675,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -24756,7 +24761,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -24842,7 +24847,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -24928,7 +24933,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -25014,7 +25019,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -25100,7 +25105,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -25186,7 +25191,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -25272,7 +25277,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -25358,7 +25363,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -25444,7 +25449,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -25530,7 +25535,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -25616,7 +25621,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -25702,7 +25707,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>27</v>
       </c>
@@ -25803,7 +25808,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB18"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -25835,7 +25840,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>240</v>
       </c>
@@ -25921,7 +25926,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -26007,7 +26012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -26093,7 +26098,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -26179,7 +26184,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -26263,7 +26268,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -26349,7 +26354,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -26433,7 +26438,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -26513,7 +26518,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -26593,7 +26598,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -26673,7 +26678,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -26753,7 +26758,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -26839,7 +26844,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -26925,7 +26930,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -27011,7 +27016,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -27097,7 +27102,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -27183,7 +27188,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -27269,7 +27274,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>27</v>
       </c>
@@ -27370,7 +27375,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -27400,7 +27405,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>202</v>
       </c>
@@ -27486,7 +27491,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -27572,7 +27577,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21">
         <v>1</v>
       </c>
@@ -27658,7 +27663,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="185">
         <v>1</v>
       </c>
@@ -27744,7 +27749,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21">
         <v>2</v>
       </c>
@@ -27830,7 +27835,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21">
         <v>3</v>
       </c>
@@ -27916,7 +27921,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -28002,7 +28007,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -28103,7 +28108,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -28133,7 +28138,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>192</v>
       </c>
@@ -28219,7 +28224,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -28305,7 +28310,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -28391,7 +28396,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -28477,7 +28482,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -28563,7 +28568,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -28649,7 +28654,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -28735,7 +28740,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -28821,7 +28826,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -28907,7 +28912,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -28993,7 +28998,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -29079,7 +29084,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -29180,7 +29185,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" style="3" hidden="1" customWidth="1"/>
@@ -29212,7 +29217,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="226" t="s">
         <v>155</v>
       </c>
@@ -29298,7 +29303,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -29384,7 +29389,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="47">
         <v>1</v>
       </c>
@@ -29470,7 +29475,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="47">
         <v>2</v>
       </c>
@@ -29556,7 +29561,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="47">
         <v>3</v>
       </c>
@@ -29642,7 +29647,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -29728,7 +29733,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>1</v>
       </c>
@@ -29814,7 +29819,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21">
         <v>2</v>
       </c>
@@ -29900,7 +29905,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>5</v>
       </c>
@@ -29986,7 +29991,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="47">
         <v>6</v>
       </c>
@@ -30072,7 +30077,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>7</v>
       </c>
@@ -30158,7 +30163,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="47">
         <v>8</v>
       </c>
@@ -30244,7 +30249,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="47">
         <v>9</v>
       </c>
@@ -30330,7 +30335,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="46" t="s">
         <v>27</v>
       </c>
@@ -30431,7 +30436,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="1" hidden="1" customWidth="1"/>
@@ -30463,7 +30468,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>79</v>
       </c>
@@ -30549,7 +30554,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="63.6" customHeight="1">
+    <row r="2" spans="1:28" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -30635,7 +30640,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="53">
         <v>1</v>
       </c>
@@ -30721,7 +30726,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="53">
         <v>2</v>
       </c>
@@ -30807,7 +30812,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="53">
         <v>4</v>
       </c>
@@ -30893,7 +30898,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="53">
         <v>5</v>
       </c>
@@ -30979,7 +30984,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="53">
         <v>6</v>
       </c>
@@ -31065,7 +31070,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="53">
         <v>7</v>
       </c>
@@ -31151,7 +31156,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="53">
         <v>8</v>
       </c>
@@ -31237,7 +31242,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="53">
         <v>9</v>
       </c>
@@ -31323,7 +31328,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="53">
         <v>3</v>
       </c>
@@ -31403,7 +31408,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="53">
         <v>10</v>
       </c>
@@ -31489,7 +31494,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53">
         <v>11</v>
       </c>
@@ -31575,7 +31580,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -31621,7 +31626,7 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -31653,7 +31658,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="21" customHeight="1">
+    <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>134</v>
       </c>
@@ -31739,7 +31744,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="48" customHeight="1">
+    <row r="2" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -31825,7 +31830,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -31911,7 +31916,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>27</v>
       </c>
@@ -32012,7 +32017,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -32044,7 +32049,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="227" t="s">
         <v>109</v>
       </c>
@@ -32130,7 +32135,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -32216,7 +32221,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -32302,7 +32307,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -32388,7 +32393,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -32474,7 +32479,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -32560,7 +32565,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -32646,7 +32651,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -32732,7 +32737,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -32818,7 +32823,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -32904,7 +32909,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -32990,7 +32995,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -33076,7 +33081,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -33162,7 +33167,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
@@ -33260,7 +33265,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C03CE4-617A-4EF9-89C8-ADAA1610BB0C}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -33290,7 +33295,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>681</v>
       </c>
@@ -33376,7 +33381,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="60.6" customHeight="1">
+    <row r="2" spans="1:28" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -33462,7 +33467,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="19.2" customHeight="1">
+    <row r="3" spans="1:28" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -33548,7 +33553,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="110" t="s">
         <v>27</v>
       </c>
@@ -33644,8 +33649,8 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41716D2-EB8A-4484-83AF-D7868E55628C}">
-  <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:AB11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -33675,7 +33680,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>669</v>
       </c>
@@ -33761,7 +33766,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -33847,7 +33852,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1">
+    <row r="3" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -33933,7 +33938,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -34017,7 +34022,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1">
+    <row r="5" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -34097,7 +34102,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1">
+    <row r="6" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -34177,7 +34182,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1">
+    <row r="7" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="161">
         <v>5</v>
       </c>
@@ -34257,7 +34262,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1">
+    <row r="8" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="161">
         <v>6</v>
       </c>
@@ -34337,7 +34342,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1">
+    <row r="9" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="161">
         <v>7</v>
       </c>
@@ -34417,91 +34422,169 @@
         <v>711</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1">
-      <c r="A10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="168">
-        <f>SUM(H3:H8)</f>
-        <v>3600</v>
-      </c>
-      <c r="I10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="K10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="M10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="O10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="P10" s="168">
-        <f>SUM(P3:P8)</f>
-        <v>1408.7</v>
-      </c>
-      <c r="Q10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="R10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="S10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="T10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="U10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="V10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="W10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="X10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB10" s="168" t="s">
+    <row r="10" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="161"/>
+      <c r="B10" s="162" t="s">
+        <v>480</v>
+      </c>
+      <c r="C10" s="161" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="191">
+        <v>46281</v>
+      </c>
+      <c r="E10" s="161"/>
+      <c r="F10" s="161">
+        <v>262615</v>
+      </c>
+      <c r="G10" s="161">
+        <v>71</v>
+      </c>
+      <c r="H10" s="161">
+        <v>2000</v>
+      </c>
+      <c r="I10" s="163">
+        <v>0.51400000000000001</v>
+      </c>
+      <c r="J10" s="163">
+        <v>1.3420000000000001</v>
+      </c>
+      <c r="K10" s="161" t="s">
+        <v>732</v>
+      </c>
+      <c r="L10" s="163">
+        <v>1379.576</v>
+      </c>
+      <c r="M10" s="164">
+        <v>1342</v>
+      </c>
+      <c r="N10" s="165">
+        <v>0.18640000000000001</v>
+      </c>
+      <c r="O10" s="166">
+        <v>11.18</v>
+      </c>
+      <c r="P10" s="161">
+        <v>434.6</v>
+      </c>
+      <c r="Q10" s="161">
+        <v>2</v>
+      </c>
+      <c r="R10" s="161">
+        <v>1050</v>
+      </c>
+      <c r="S10" s="163">
+        <v>1.028</v>
+      </c>
+      <c r="T10" s="161">
+        <v>22</v>
+      </c>
+      <c r="U10" s="165">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="V10" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="161"/>
+      <c r="Z10" s="161"/>
+      <c r="AA10" s="161">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="161" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="168">
+        <f>SUM(H3:H10)</f>
+        <v>6850</v>
+      </c>
+      <c r="I11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="O11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="P11" s="168">
+        <f>SUM(P3:P10)</f>
+        <v>2055.9</v>
+      </c>
+      <c r="Q11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="R11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="S11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="T11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="U11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="V11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="W11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="X11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB11" s="168" t="s">
         <v>27</v>
       </c>
     </row>
@@ -34516,7 +34599,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BFDD7F-F2DE-484D-858D-A0AEE46D68A8}">
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.88671875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -34547,7 +34630,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>665</v>
       </c>
@@ -34633,7 +34716,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1">
+    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -34719,7 +34802,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="184" customFormat="1">
+    <row r="3" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="178">
         <v>1</v>
       </c>
@@ -34805,7 +34888,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="184" customFormat="1">
+    <row r="4" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="178">
         <v>2</v>
       </c>
@@ -34891,7 +34974,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="184" customFormat="1">
+    <row r="5" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="178">
         <v>3</v>
       </c>
@@ -34977,7 +35060,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="184" customFormat="1">
+    <row r="6" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="178">
         <v>4</v>
       </c>
@@ -35063,7 +35146,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="184" customFormat="1">
+    <row r="7" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="178">
         <v>5</v>
       </c>
@@ -35149,7 +35232,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="184" customFormat="1">
+    <row r="8" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="178">
         <v>6</v>
       </c>
@@ -35235,7 +35318,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="184" customFormat="1">
+    <row r="9" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="178">
         <v>7</v>
       </c>
@@ -35321,7 +35404,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="184" customFormat="1">
+    <row r="10" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="178">
         <v>8</v>
       </c>
@@ -35407,7 +35490,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="184" customFormat="1">
+    <row r="11" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="178">
         <v>9</v>
       </c>
@@ -35493,7 +35576,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="168" t="s">
         <v>27</v>
       </c>
@@ -35593,7 +35676,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB29"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -35624,7 +35707,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>652</v>
       </c>
@@ -35710,7 +35793,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -35796,7 +35879,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -35882,7 +35965,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -35968,7 +36051,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="150">
         <v>3</v>
       </c>
@@ -36054,7 +36137,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="150">
         <v>4</v>
       </c>
@@ -36140,7 +36223,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="150">
         <v>5</v>
       </c>
@@ -36226,7 +36309,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -36312,7 +36395,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -36398,7 +36481,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -36484,7 +36567,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -36570,7 +36653,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -36656,7 +36739,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -36742,7 +36825,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -36828,7 +36911,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="150">
         <v>13</v>
       </c>
@@ -36914,7 +36997,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="150">
         <v>14</v>
       </c>
@@ -37000,7 +37083,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="150">
         <v>15</v>
       </c>
@@ -37086,7 +37169,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="150">
         <v>16</v>
       </c>
@@ -37172,7 +37255,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="150">
         <v>17</v>
       </c>
@@ -37258,7 +37341,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="150">
         <v>18</v>
       </c>
@@ -37344,7 +37427,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="150">
         <v>19</v>
       </c>
@@ -37430,7 +37513,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="150">
         <v>20</v>
       </c>
@@ -37510,7 +37593,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="150">
         <v>21</v>
       </c>
@@ -37596,7 +37679,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="150">
         <v>22</v>
       </c>
@@ -37682,7 +37765,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="150">
         <v>23</v>
       </c>
@@ -37768,7 +37851,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="150">
         <v>24</v>
       </c>
@@ -37854,7 +37937,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="150">
         <v>25</v>
       </c>
@@ -37940,7 +38023,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="157" t="s">
         <v>27</v>
       </c>
@@ -38026,7 +38109,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:28">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B29" s="206"/>
     </row>
   </sheetData>
@@ -38044,7 +38127,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -38075,7 +38158,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>618</v>
       </c>
@@ -38161,7 +38244,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -38247,7 +38330,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -38333,7 +38416,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -38419,7 +38502,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -38505,7 +38588,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -38591,7 +38674,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="168" t="s">
         <v>27</v>
       </c>
@@ -38692,7 +38775,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.21875" style="108" customWidth="1"/>
     <col min="2" max="2" width="15.109375" style="108" customWidth="1"/>
@@ -38724,7 +38807,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>606</v>
       </c>
@@ -38810,7 +38893,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -38896,7 +38979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="170">
         <v>1</v>
       </c>
@@ -38982,7 +39065,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="170">
         <v>2</v>
       </c>
@@ -39068,7 +39151,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="170">
         <v>3</v>
       </c>
@@ -39154,7 +39237,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="170">
         <v>4</v>
       </c>
@@ -39240,7 +39323,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="170">
         <v>5</v>
       </c>
@@ -39326,7 +39409,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="170">
         <v>6</v>
       </c>
@@ -39412,7 +39495,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="170">
         <v>7</v>
       </c>
@@ -39498,7 +39581,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="170">
         <v>8</v>
       </c>
@@ -39584,7 +39667,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="157" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (16/09/2026 14:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F300661C-53F0-4D62-B280-59DE4F0B4DB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8A1473-61F9-405D-9D01-CB392F2E9357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34441,7 +34441,7 @@
         <v>71</v>
       </c>
       <c r="H10" s="161">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="I10" s="163">
         <v>0.51400000000000001</v>
@@ -34524,7 +34524,7 @@
       </c>
       <c r="H11" s="168">
         <f>SUM(H3:H10)</f>
-        <v>6850</v>
+        <v>7850</v>
       </c>
       <c r="I11" s="168" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (16/09/2026 17:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8A1473-61F9-405D-9D01-CB392F2E9357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E65A2A-9079-4122-9E11-E41FA40E2C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6719" uniqueCount="734">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6747" uniqueCount="740">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2271,6 +2271,24 @@
   </si>
   <si>
     <t>1048x1362</t>
+  </si>
+  <si>
+    <t>1070x1780</t>
+  </si>
+  <si>
+    <t>995x1620</t>
+  </si>
+  <si>
+    <t>87x105x87</t>
+  </si>
+  <si>
+    <t>1136x2024</t>
+  </si>
+  <si>
+    <t>90x185x90</t>
+  </si>
+  <si>
+    <t>1115x2100</t>
   </si>
 </sst>
 </file>
@@ -33649,7 +33667,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41716D2-EB8A-4484-83AF-D7868E55628C}">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
@@ -34353,56 +34371,56 @@
         <v>36</v>
       </c>
       <c r="D9" s="191">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E9" s="161"/>
       <c r="F9" s="161">
-        <v>262602</v>
+        <v>262616</v>
       </c>
       <c r="G9" s="161">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H9" s="161">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="I9" s="163">
-        <v>0.54</v>
+        <v>0.35</v>
       </c>
       <c r="J9" s="163">
-        <v>1</v>
+        <v>0.88</v>
       </c>
       <c r="K9" s="161" t="s">
         <v>34</v>
       </c>
       <c r="L9" s="163">
-        <v>675</v>
+        <v>308</v>
       </c>
       <c r="M9" s="164">
-        <v>625</v>
+        <v>293.3</v>
       </c>
       <c r="N9" s="165">
-        <v>8.6800000000000002E-2</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="O9" s="166">
-        <v>5.21</v>
+        <v>1.63</v>
       </c>
       <c r="P9" s="161">
-        <v>212.6</v>
+        <v>97</v>
       </c>
       <c r="Q9" s="161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="161">
         <v>1100</v>
       </c>
       <c r="S9" s="163">
-        <v>1.08</v>
+        <v>1.05</v>
       </c>
       <c r="T9" s="161">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="U9" s="165">
-        <v>1.8200000000000001E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V9" s="161" t="s">
         <v>28</v>
@@ -34419,11 +34437,13 @@
         <v>1</v>
       </c>
       <c r="AB9" s="161" t="s">
-        <v>711</v>
+        <v>734</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="161"/>
+      <c r="A10" s="161">
+        <v>8</v>
+      </c>
       <c r="B10" s="162" t="s">
         <v>480</v>
       </c>
@@ -34431,56 +34451,56 @@
         <v>36</v>
       </c>
       <c r="D10" s="191">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="E10" s="161"/>
       <c r="F10" s="161">
-        <v>262615</v>
+        <v>262602</v>
       </c>
       <c r="G10" s="161">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H10" s="161">
-        <v>3000</v>
+        <v>1250</v>
       </c>
       <c r="I10" s="163">
-        <v>0.51400000000000001</v>
+        <v>0.54</v>
       </c>
       <c r="J10" s="163">
-        <v>1.3420000000000001</v>
+        <v>1</v>
       </c>
       <c r="K10" s="161" t="s">
-        <v>732</v>
+        <v>34</v>
       </c>
       <c r="L10" s="163">
-        <v>1379.576</v>
+        <v>675</v>
       </c>
       <c r="M10" s="164">
-        <v>1342</v>
+        <v>625</v>
       </c>
       <c r="N10" s="165">
-        <v>0.18640000000000001</v>
+        <v>8.6800000000000002E-2</v>
       </c>
       <c r="O10" s="166">
-        <v>11.18</v>
+        <v>5.21</v>
       </c>
       <c r="P10" s="161">
-        <v>434.6</v>
+        <v>212.6</v>
       </c>
       <c r="Q10" s="161">
         <v>2</v>
       </c>
       <c r="R10" s="161">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S10" s="163">
-        <v>1.028</v>
+        <v>1.08</v>
       </c>
       <c r="T10" s="161">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="U10" s="165">
-        <v>2.1000000000000001E-2</v>
+        <v>1.8200000000000001E-2</v>
       </c>
       <c r="V10" s="161" t="s">
         <v>28</v>
@@ -34494,97 +34514,417 @@
       <c r="Y10" s="161"/>
       <c r="Z10" s="161"/>
       <c r="AA10" s="161">
+        <v>1</v>
+      </c>
+      <c r="AB10" s="161" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="161">
+        <v>9</v>
+      </c>
+      <c r="B11" s="162" t="s">
+        <v>480</v>
+      </c>
+      <c r="C11" s="161" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="191">
+        <v>46281</v>
+      </c>
+      <c r="E11" s="161"/>
+      <c r="F11" s="161">
+        <v>262615</v>
+      </c>
+      <c r="G11" s="161">
+        <v>71</v>
+      </c>
+      <c r="H11" s="161">
+        <v>3000</v>
+      </c>
+      <c r="I11" s="163">
+        <v>0.51400000000000001</v>
+      </c>
+      <c r="J11" s="163">
+        <v>1.3420000000000001</v>
+      </c>
+      <c r="K11" s="161" t="s">
+        <v>732</v>
+      </c>
+      <c r="L11" s="163">
+        <v>1379.576</v>
+      </c>
+      <c r="M11" s="164">
+        <v>1342</v>
+      </c>
+      <c r="N11" s="165">
+        <v>0.18640000000000001</v>
+      </c>
+      <c r="O11" s="166">
+        <v>11.18</v>
+      </c>
+      <c r="P11" s="161">
+        <v>434.6</v>
+      </c>
+      <c r="Q11" s="161">
+        <v>2</v>
+      </c>
+      <c r="R11" s="161">
+        <v>1050</v>
+      </c>
+      <c r="S11" s="163">
+        <v>1.028</v>
+      </c>
+      <c r="T11" s="161">
+        <v>22</v>
+      </c>
+      <c r="U11" s="165">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="V11" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="161"/>
+      <c r="Z11" s="161"/>
+      <c r="AA11" s="161">
         <v>3</v>
       </c>
-      <c r="AB10" s="161" t="s">
+      <c r="AB11" s="161" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="168">
-        <f>SUM(H3:H10)</f>
-        <v>7850</v>
-      </c>
-      <c r="I11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="K11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="L11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="M11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="N11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="O11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="P11" s="168">
-        <f>SUM(P3:P10)</f>
-        <v>2055.9</v>
-      </c>
-      <c r="Q11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="R11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="S11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="T11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="U11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="V11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="W11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="X11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB11" s="168" t="s">
+    <row r="12" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="161">
+        <v>10</v>
+      </c>
+      <c r="B12" s="162" t="s">
+        <v>480</v>
+      </c>
+      <c r="C12" s="161" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="191">
+        <v>46281</v>
+      </c>
+      <c r="E12" s="161"/>
+      <c r="F12" s="161">
+        <v>262617</v>
+      </c>
+      <c r="G12" s="161">
+        <v>72</v>
+      </c>
+      <c r="H12" s="161">
+        <v>3200</v>
+      </c>
+      <c r="I12" s="163">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="J12" s="163">
+        <v>0.8</v>
+      </c>
+      <c r="K12" s="161" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="163">
+        <v>832</v>
+      </c>
+      <c r="M12" s="164">
+        <v>853.3</v>
+      </c>
+      <c r="N12" s="165">
+        <v>7.9000000000000001E-2</v>
+      </c>
+      <c r="O12" s="166">
+        <v>4.74</v>
+      </c>
+      <c r="P12" s="161">
+        <v>262.10000000000002</v>
+      </c>
+      <c r="Q12" s="161">
+        <v>3</v>
+      </c>
+      <c r="R12" s="161">
+        <v>1000</v>
+      </c>
+      <c r="S12" s="163">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="T12" s="161">
+        <v>25</v>
+      </c>
+      <c r="U12" s="165">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="V12" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="161"/>
+      <c r="Z12" s="161"/>
+      <c r="AA12" s="161">
+        <v>2</v>
+      </c>
+      <c r="AB12" s="161" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="161">
+        <v>11</v>
+      </c>
+      <c r="B13" s="162" t="s">
+        <v>480</v>
+      </c>
+      <c r="C13" s="161" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="191">
+        <v>46281</v>
+      </c>
+      <c r="E13" s="161"/>
+      <c r="F13" s="161">
+        <v>262618</v>
+      </c>
+      <c r="G13" s="161">
+        <v>73</v>
+      </c>
+      <c r="H13" s="161">
+        <v>2000</v>
+      </c>
+      <c r="I13" s="163">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="J13" s="163">
+        <v>1.002</v>
+      </c>
+      <c r="K13" s="161" t="s">
+        <v>736</v>
+      </c>
+      <c r="L13" s="163">
+        <v>559.11599999999999</v>
+      </c>
+      <c r="M13" s="164">
+        <v>1002</v>
+      </c>
+      <c r="N13" s="165">
+        <v>0.13919999999999999</v>
+      </c>
+      <c r="O13" s="166">
+        <v>8.35</v>
+      </c>
+      <c r="P13" s="161">
+        <v>176.1</v>
+      </c>
+      <c r="Q13" s="161">
+        <v>2</v>
+      </c>
+      <c r="R13" s="161">
+        <v>600</v>
+      </c>
+      <c r="S13" s="163">
+        <v>0.55800000000000005</v>
+      </c>
+      <c r="T13" s="161">
+        <v>42</v>
+      </c>
+      <c r="U13" s="165">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V13" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="161"/>
+      <c r="Z13" s="161"/>
+      <c r="AA13" s="161">
+        <v>1</v>
+      </c>
+      <c r="AB13" s="161" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="161">
+        <v>12</v>
+      </c>
+      <c r="B14" s="162" t="s">
+        <v>480</v>
+      </c>
+      <c r="C14" s="161" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="191">
+        <v>46281</v>
+      </c>
+      <c r="E14" s="161"/>
+      <c r="F14" s="161">
+        <v>262619</v>
+      </c>
+      <c r="G14" s="161">
+        <v>73</v>
+      </c>
+      <c r="H14" s="161">
+        <v>6000</v>
+      </c>
+      <c r="I14" s="163">
+        <v>0.36499999999999999</v>
+      </c>
+      <c r="J14" s="163">
+        <v>1.04</v>
+      </c>
+      <c r="K14" s="161" t="s">
+        <v>738</v>
+      </c>
+      <c r="L14" s="163">
+        <v>2277.6</v>
+      </c>
+      <c r="M14" s="164">
+        <v>3120</v>
+      </c>
+      <c r="N14" s="165">
+        <v>0.43330000000000002</v>
+      </c>
+      <c r="O14" s="166">
+        <v>26</v>
+      </c>
+      <c r="P14" s="161">
+        <v>717.4</v>
+      </c>
+      <c r="Q14" s="161">
+        <v>2</v>
+      </c>
+      <c r="R14" s="161">
+        <v>750</v>
+      </c>
+      <c r="S14" s="163">
+        <v>0.73</v>
+      </c>
+      <c r="T14" s="161">
+        <v>20</v>
+      </c>
+      <c r="U14" s="165">
+        <v>2.6700000000000002E-2</v>
+      </c>
+      <c r="V14" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="161"/>
+      <c r="Z14" s="161"/>
+      <c r="AA14" s="161">
+        <v>3</v>
+      </c>
+      <c r="AB14" s="161" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="168">
+        <f>SUM(H3:H14)</f>
+        <v>20050</v>
+      </c>
+      <c r="I15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="J15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="M15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="O15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="P15" s="168">
+        <f>SUM(P3:P14)</f>
+        <v>3308.5</v>
+      </c>
+      <c r="Q15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="R15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="S15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="T15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="U15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="V15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="W15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="X15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB15" s="168" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (16/09/2026 18:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E65A2A-9079-4122-9E11-E41FA40E2C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E638CB-AD61-4674-ADB3-327FE3F42127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (17/09/2026 08:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E638CB-AD61-4674-ADB3-327FE3F42127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94FEA94-1A43-4B4C-9741-2B559B51AE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="IPE - PC BOX 1203" sheetId="154" r:id="rId1"/>
+    <sheet name="IPE - PC BOX 1203P" sheetId="154" r:id="rId1"/>
     <sheet name="ABAPEL 1201" sheetId="153" r:id="rId2"/>
     <sheet name="HARMONY EMBALAGENS 1200" sheetId="152" r:id="rId3"/>
     <sheet name="HARMONY EMBALAGENS 1199" sheetId="151" r:id="rId4"/>
@@ -2300,7 +2300,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3394,8 +3394,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22CC649A-4A24-4BCE-A798-0B107F907AA7}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -3427,93 +3430,93 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="218" t="s">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
+      <c r="A1" s="221" t="s">
         <v>723</v>
       </c>
-      <c r="B1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="218" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="221" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="51" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3599,7 +3602,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -3685,7 +3688,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -3771,7 +3774,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -3857,93 +3860,93 @@
         <v>717</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="185">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="186" t="s">
         <v>448</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="185" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="185" t="s">
         <v>716</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="5">
+      <c r="E6" s="185" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="185">
         <v>262604</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="185" t="s">
         <v>715</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="185">
         <v>3000</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="187">
         <v>0.45600000000000002</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="187">
         <v>1.5609999999999999</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="185" t="s">
         <v>714</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="187">
         <v>2135.4479999999999</v>
       </c>
-      <c r="M6" s="9">
+      <c r="M6" s="188">
         <v>2341.5</v>
       </c>
-      <c r="N6" s="6">
+      <c r="N6" s="189">
         <v>0.32519999999999999</v>
       </c>
-      <c r="O6" s="8">
+      <c r="O6" s="190">
         <v>19.510000000000002</v>
       </c>
-      <c r="P6" s="5">
+      <c r="P6" s="185">
         <v>672.7</v>
       </c>
-      <c r="Q6" s="5">
+      <c r="Q6" s="185">
         <v>2</v>
       </c>
-      <c r="R6" s="5">
+      <c r="R6" s="185">
         <v>950</v>
       </c>
-      <c r="S6" s="7">
+      <c r="S6" s="187">
         <v>0.91200000000000003</v>
       </c>
-      <c r="T6" s="5">
+      <c r="T6" s="185">
         <v>38</v>
       </c>
-      <c r="U6" s="6">
+      <c r="U6" s="189">
         <v>0.04</v>
       </c>
-      <c r="V6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="5" t="s">
+      <c r="V6" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="185" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="185" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="185" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="185" t="s">
         <v>32</v>
       </c>
-      <c r="AB6" s="5" t="s">
+      <c r="AB6" s="185" t="s">
         <v>713</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -4033,7 +4036,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.28000000000000003" right="0.2" top="1.74" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4043,7 +4047,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.5546875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -4073,7 +4077,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="220" t="s">
         <v>599</v>
       </c>
@@ -4159,7 +4163,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -4245,7 +4249,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -4331,7 +4335,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -4417,7 +4421,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="150"/>
       <c r="B5" s="151" t="s">
         <v>621</v>
@@ -4495,7 +4499,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="157" t="s">
         <v>27</v>
       </c>
@@ -4583,7 +4587,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28">
       <c r="D8" s="158"/>
       <c r="J8" s="159"/>
       <c r="L8" s="159"/>
@@ -4603,7 +4607,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -4631,7 +4635,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>592</v>
       </c>
@@ -4717,7 +4721,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4803,7 +4807,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -4889,7 +4893,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -4975,7 +4979,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -5061,7 +5065,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -5141,7 +5145,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -5221,7 +5225,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -5307,7 +5311,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -5393,7 +5397,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -5479,7 +5483,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -5565,7 +5569,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -5666,7 +5670,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -5697,7 +5701,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="222" t="s">
         <v>554</v>
       </c>
@@ -5783,7 +5787,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -5869,7 +5873,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="193">
         <v>1</v>
       </c>
@@ -5955,7 +5959,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -6041,7 +6045,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="193">
         <v>3</v>
       </c>
@@ -6127,7 +6131,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="193">
         <v>4</v>
       </c>
@@ -6213,7 +6217,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="193">
         <v>5</v>
       </c>
@@ -6299,7 +6303,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -6385,7 +6389,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -6471,7 +6475,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -6557,7 +6561,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -6643,7 +6647,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -6729,7 +6733,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -6815,7 +6819,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -6901,7 +6905,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="157" t="s">
         <v>27</v>
       </c>
@@ -7002,7 +7006,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -7034,7 +7038,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>539</v>
       </c>
@@ -7120,7 +7124,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -7206,7 +7210,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="126">
         <v>1</v>
       </c>
@@ -7292,7 +7296,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -7378,7 +7382,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="126">
         <v>2</v>
       </c>
@@ -7464,7 +7468,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>3</v>
       </c>
@@ -7550,7 +7554,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -7636,7 +7640,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -7722,7 +7726,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -7808,7 +7812,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28">
       <c r="A10" s="28" t="s">
         <v>27</v>
       </c>
@@ -7906,7 +7910,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
   <dimension ref="A1:AB5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -7938,7 +7942,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="218" t="s">
         <v>535</v>
       </c>
@@ -8024,7 +8028,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -8110,7 +8114,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -8196,7 +8200,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -8282,7 +8286,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28">
       <c r="A5" s="28" t="s">
         <v>27</v>
       </c>
@@ -8382,7 +8386,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -8414,7 +8418,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="223" t="s">
         <v>523</v>
       </c>
@@ -8500,7 +8504,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="43.2" customHeight="1">
       <c r="A2" s="107" t="s">
         <v>0</v>
       </c>
@@ -8586,7 +8590,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="90">
         <v>1</v>
       </c>
@@ -8672,7 +8676,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="90">
         <v>2</v>
       </c>
@@ -8758,7 +8762,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="90">
         <v>3</v>
       </c>
@@ -8844,7 +8848,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="90">
         <v>4</v>
       </c>
@@ -8930,7 +8934,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="106" t="s">
         <v>27</v>
       </c>
@@ -9031,7 +9035,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" style="3" hidden="1" customWidth="1"/>
@@ -9063,7 +9067,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="224" t="s">
         <v>512</v>
       </c>
@@ -9149,7 +9153,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -9235,7 +9239,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" customFormat="1">
       <c r="A3" s="120">
         <v>1</v>
       </c>
@@ -9321,7 +9325,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="4" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" customFormat="1">
       <c r="A4" s="120">
         <v>2</v>
       </c>
@@ -9407,7 +9411,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" customFormat="1">
       <c r="A5" s="120">
         <v>3</v>
       </c>
@@ -9493,7 +9497,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="6" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" customFormat="1">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -9579,7 +9583,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="7" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" customFormat="1">
       <c r="A7" s="120">
         <v>5</v>
       </c>
@@ -9665,7 +9669,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="8" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" customFormat="1">
       <c r="A8" s="47">
         <v>6</v>
       </c>
@@ -9751,7 +9755,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="9" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" customFormat="1">
       <c r="A9" s="47">
         <v>7</v>
       </c>
@@ -9837,7 +9841,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="10" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" customFormat="1">
       <c r="A10" s="120">
         <v>8</v>
       </c>
@@ -9923,7 +9927,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="45" customFormat="1">
       <c r="A11" s="47">
         <v>9</v>
       </c>
@@ -10009,7 +10013,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="45" customFormat="1">
       <c r="A12" s="46" t="s">
         <v>27</v>
       </c>
@@ -10107,7 +10111,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -10138,7 +10142,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="220" t="s">
         <v>531</v>
       </c>
@@ -10224,7 +10228,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="39" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -10310,7 +10314,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -10396,7 +10400,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -10482,7 +10486,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -10568,7 +10572,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -10654,7 +10658,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -10740,7 +10744,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1">
       <c r="A8" s="110" t="s">
         <v>27</v>
       </c>
@@ -10841,7 +10845,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -10873,7 +10877,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>496</v>
       </c>
@@ -10959,7 +10963,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -11045,7 +11049,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="133">
         <v>1</v>
       </c>
@@ -11131,7 +11135,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="133">
         <v>2</v>
       </c>
@@ -11215,7 +11219,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="133">
         <v>3</v>
       </c>
@@ -11301,7 +11305,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="207">
         <v>4</v>
       </c>
@@ -11385,7 +11389,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="207">
         <v>5</v>
       </c>
@@ -11469,7 +11473,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="133">
         <v>6</v>
       </c>
@@ -11555,7 +11559,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="207">
         <v>7</v>
       </c>
@@ -11639,7 +11643,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="133">
         <v>8</v>
       </c>
@@ -11725,7 +11729,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="207">
         <v>9</v>
       </c>
@@ -11809,7 +11813,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="133">
         <v>10</v>
       </c>
@@ -11895,7 +11899,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="133">
         <v>11</v>
       </c>
@@ -11981,7 +11985,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="133">
         <v>12</v>
       </c>
@@ -12067,7 +12071,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="133">
         <v>13</v>
       </c>
@@ -12153,7 +12157,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="133">
         <v>14</v>
       </c>
@@ -12239,7 +12243,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A17" s="11" t="s">
         <v>27</v>
       </c>
@@ -12342,7 +12346,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -12372,7 +12376,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>486</v>
       </c>
@@ -12458,7 +12462,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -12544,7 +12548,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -12630,7 +12634,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="139">
         <v>2</v>
       </c>
@@ -12716,7 +12720,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="139"/>
       <c r="B5" s="140" t="s">
         <v>480</v>
@@ -12794,7 +12798,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="139"/>
       <c r="B6" s="140" t="s">
         <v>480</v>
@@ -12872,7 +12876,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="34">
         <v>3</v>
       </c>
@@ -12958,7 +12962,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1">
       <c r="A8" s="28" t="s">
         <v>27</v>
       </c>
@@ -13058,7 +13062,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5AF4CA-00D7-4A30-8F64-AC13CDBB2809}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13090,7 +13094,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="218" t="s">
         <v>710</v>
       </c>
@@ -13176,7 +13180,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="54" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13262,7 +13266,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -13348,7 +13352,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -13434,7 +13438,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -13520,7 +13524,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -13606,7 +13610,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -13706,7 +13710,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13736,7 +13740,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>475</v>
       </c>
@@ -13822,7 +13826,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13908,7 +13912,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="97">
         <v>1</v>
       </c>
@@ -13994,7 +13998,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="97">
         <v>2</v>
       </c>
@@ -14080,7 +14084,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="97">
         <v>3</v>
       </c>
@@ -14166,7 +14170,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="97">
         <v>4</v>
       </c>
@@ -14252,7 +14256,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="97">
         <v>5</v>
       </c>
@@ -14338,7 +14342,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="97">
         <v>6</v>
       </c>
@@ -14424,7 +14428,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="97">
         <v>7</v>
       </c>
@@ -14510,7 +14514,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="97">
         <v>8</v>
       </c>
@@ -14596,7 +14600,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="97">
         <v>9</v>
       </c>
@@ -14682,7 +14686,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="97">
         <v>10</v>
       </c>
@@ -14768,7 +14772,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="11" t="s">
         <v>27</v>
       </c>
@@ -14869,7 +14873,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -14901,7 +14905,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>454</v>
       </c>
@@ -14987,7 +14991,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="50.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -15073,7 +15077,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -15159,7 +15163,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -15245,7 +15249,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -15331,7 +15335,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -15417,7 +15421,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -15503,7 +15507,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -15604,7 +15608,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -15636,7 +15640,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="33" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>440</v>
       </c>
@@ -15722,7 +15726,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -15808,7 +15812,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -15894,7 +15898,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -15980,7 +15984,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -16066,7 +16070,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -16152,7 +16156,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -16238,7 +16242,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -16324,7 +16328,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -16410,7 +16414,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
@@ -16511,7 +16515,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -16542,7 +16546,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>403</v>
       </c>
@@ -16628,7 +16632,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -16714,7 +16718,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -16800,7 +16804,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -16884,7 +16888,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -16970,7 +16974,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -17056,7 +17060,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -17140,7 +17144,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -17224,7 +17228,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
@@ -17325,7 +17329,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" customWidth="1"/>
@@ -17355,7 +17359,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="225" t="s">
         <v>380</v>
       </c>
@@ -17441,7 +17445,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1">
       <c r="A2" s="89" t="s">
         <v>0</v>
       </c>
@@ -17527,7 +17531,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="14">
         <v>1</v>
       </c>
@@ -17613,7 +17617,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="14">
         <v>2</v>
       </c>
@@ -17699,7 +17703,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="14">
         <v>3</v>
       </c>
@@ -17785,7 +17789,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="14">
         <v>4</v>
       </c>
@@ -17871,7 +17875,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="14">
         <v>5</v>
       </c>
@@ -17957,7 +17961,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1">
       <c r="A8" s="14">
         <v>6</v>
       </c>
@@ -18043,7 +18047,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1">
       <c r="A9" s="14">
         <v>7</v>
       </c>
@@ -18129,7 +18133,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1">
       <c r="A10" s="14">
         <v>8</v>
       </c>
@@ -18215,7 +18219,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1">
       <c r="A11" s="14">
         <v>9</v>
       </c>
@@ -18301,7 +18305,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1">
       <c r="A12" s="14">
         <v>10</v>
       </c>
@@ -18387,7 +18391,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1">
       <c r="A13" s="14">
         <v>11</v>
       </c>
@@ -18473,7 +18477,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" ht="25.05" customHeight="1">
       <c r="A14" s="14">
         <v>12</v>
       </c>
@@ -18559,7 +18563,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" ht="25.05" customHeight="1">
       <c r="A15" s="14">
         <v>13</v>
       </c>
@@ -18645,7 +18649,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" ht="25.05" customHeight="1">
       <c r="A16" s="14">
         <v>14</v>
       </c>
@@ -18731,7 +18735,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" ht="25.05" customHeight="1">
       <c r="A17" s="14">
         <v>15</v>
       </c>
@@ -18817,7 +18821,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" ht="25.05" customHeight="1">
       <c r="A18" s="14">
         <v>16</v>
       </c>
@@ -18903,7 +18907,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" ht="25.05" customHeight="1">
       <c r="A19" s="14">
         <v>17</v>
       </c>
@@ -18989,7 +18993,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:28" ht="25.05" customHeight="1">
       <c r="A20" s="14">
         <v>18</v>
       </c>
@@ -19075,7 +19079,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:28" ht="25.05" customHeight="1">
       <c r="A21" s="14">
         <v>19</v>
       </c>
@@ -19161,7 +19165,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:28" ht="25.05" customHeight="1">
       <c r="A22" s="14">
         <v>20</v>
       </c>
@@ -19247,7 +19251,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:28" ht="25.05" customHeight="1">
       <c r="A23" s="14">
         <v>21</v>
       </c>
@@ -19333,7 +19337,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:28" ht="25.05" customHeight="1">
       <c r="A24" s="14">
         <v>22</v>
       </c>
@@ -19419,7 +19423,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:28" ht="25.05" customHeight="1">
       <c r="A25" s="14">
         <v>23</v>
       </c>
@@ -19505,7 +19509,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:28" ht="25.05" customHeight="1">
       <c r="A26" s="14">
         <v>24</v>
       </c>
@@ -19591,7 +19595,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A27" s="90">
         <v>10</v>
       </c>
@@ -19677,7 +19681,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:28" ht="25.05" customHeight="1">
       <c r="A28" s="20" t="s">
         <v>27</v>
       </c>
@@ -19778,7 +19782,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" style="3" customWidth="1"/>
@@ -19810,7 +19814,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="224" t="s">
         <v>332</v>
       </c>
@@ -19896,7 +19900,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -19982,7 +19986,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -20068,7 +20072,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -20154,7 +20158,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -20240,7 +20244,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -20326,7 +20330,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -20412,7 +20416,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28">
       <c r="F14" s="3" t="s">
         <v>395</v>
       </c>
@@ -20432,7 +20436,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -20463,7 +20467,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>329</v>
       </c>
@@ -20549,7 +20553,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20635,7 +20639,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="81">
         <v>1</v>
       </c>
@@ -20721,7 +20725,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="81">
         <v>2</v>
       </c>
@@ -20807,7 +20811,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="37" t="s">
         <v>27</v>
       </c>
@@ -20893,8 +20897,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
+    <row r="8" spans="1:28">
       <c r="D8" s="160"/>
     </row>
   </sheetData>
@@ -20912,7 +20916,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
@@ -20942,7 +20946,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>324</v>
       </c>
@@ -21028,7 +21032,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -21114,7 +21118,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -21200,7 +21204,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="34">
         <v>2</v>
       </c>
@@ -21286,7 +21290,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -21372,7 +21376,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="34">
         <v>4</v>
       </c>
@@ -21458,7 +21462,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="34">
         <v>5</v>
       </c>
@@ -21544,7 +21548,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1">
       <c r="A8" s="34">
         <v>6</v>
       </c>
@@ -21630,7 +21634,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1">
       <c r="A9" s="28" t="s">
         <v>27</v>
       </c>
@@ -21731,7 +21735,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -21762,7 +21766,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="224" t="s">
         <v>281</v>
       </c>
@@ -21848,7 +21852,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="51" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -21934,7 +21938,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -22020,7 +22024,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -22106,7 +22110,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -22192,7 +22196,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -22278,7 +22282,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -22379,7 +22383,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -22410,7 +22414,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>258</v>
       </c>
@@ -22496,7 +22500,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -22582,7 +22586,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -22668,7 +22672,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -22754,7 +22758,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -22840,7 +22844,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -22926,7 +22930,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -23012,7 +23016,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -23098,7 +23102,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -23184,7 +23188,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -23270,7 +23274,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -23356,7 +23360,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -23442,7 +23446,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -23528,7 +23532,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -23612,7 +23616,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -23698,7 +23702,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -23784,7 +23788,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -23870,7 +23874,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -23956,7 +23960,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A19" s="11" t="s">
         <v>27</v>
       </c>
@@ -24042,7 +24046,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:28">
       <c r="K27" s="1" t="s">
         <v>259</v>
       </c>
@@ -24059,7 +24063,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15B73F0-D53E-458D-8A18-622E142F07EE}">
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -24091,7 +24095,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="218" t="s">
         <v>702</v>
       </c>
@@ -24177,7 +24181,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="42.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -24263,7 +24267,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -24349,7 +24353,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="200">
         <v>2</v>
       </c>
@@ -24435,7 +24439,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="200">
         <v>3</v>
       </c>
@@ -24521,7 +24525,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="200">
         <v>4</v>
       </c>
@@ -24607,7 +24611,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -24693,7 +24697,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -24779,7 +24783,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -24865,7 +24869,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -24951,7 +24955,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -25037,7 +25041,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -25123,7 +25127,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -25209,7 +25213,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -25295,7 +25299,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -25381,7 +25385,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -25467,7 +25471,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -25553,7 +25557,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -25639,7 +25643,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -25725,7 +25729,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A20" s="11" t="s">
         <v>27</v>
       </c>
@@ -25826,7 +25830,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -25858,7 +25862,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>240</v>
       </c>
@@ -25944,7 +25948,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -26030,7 +26034,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -26116,7 +26120,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -26202,7 +26206,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -26286,7 +26290,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -26372,7 +26376,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -26456,7 +26460,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -26536,7 +26540,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -26616,7 +26620,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -26696,7 +26700,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -26776,7 +26780,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -26862,7 +26866,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -26948,7 +26952,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -27034,7 +27038,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -27120,7 +27124,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -27206,7 +27210,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -27292,7 +27296,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A18" s="11" t="s">
         <v>27</v>
       </c>
@@ -27393,7 +27397,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -27423,7 +27427,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>202</v>
       </c>
@@ -27509,7 +27513,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -27595,7 +27599,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="21">
         <v>1</v>
       </c>
@@ -27681,7 +27685,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="185">
         <v>1</v>
       </c>
@@ -27767,7 +27771,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="21">
         <v>2</v>
       </c>
@@ -27853,7 +27857,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="21">
         <v>3</v>
       </c>
@@ -27939,7 +27943,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -28025,7 +28029,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -28126,7 +28130,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -28156,7 +28160,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>192</v>
       </c>
@@ -28242,7 +28246,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -28328,7 +28332,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -28414,7 +28418,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -28500,7 +28504,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -28586,7 +28590,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -28672,7 +28676,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -28758,7 +28762,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -28844,7 +28848,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -28930,7 +28934,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -29016,7 +29020,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -29102,7 +29106,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -29203,7 +29207,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" style="3" hidden="1" customWidth="1"/>
@@ -29235,7 +29239,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1">
       <c r="A1" s="226" t="s">
         <v>155</v>
       </c>
@@ -29321,7 +29325,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -29407,7 +29411,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A3" s="47">
         <v>1</v>
       </c>
@@ -29493,7 +29497,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A4" s="47">
         <v>2</v>
       </c>
@@ -29579,7 +29583,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A5" s="47">
         <v>3</v>
       </c>
@@ -29665,7 +29669,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -29751,7 +29755,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="21">
         <v>1</v>
       </c>
@@ -29837,7 +29841,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="21">
         <v>2</v>
       </c>
@@ -29923,7 +29927,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A9" s="47">
         <v>5</v>
       </c>
@@ -30009,7 +30013,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A10" s="47">
         <v>6</v>
       </c>
@@ -30095,7 +30099,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A11" s="47">
         <v>7</v>
       </c>
@@ -30181,7 +30185,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A12" s="47">
         <v>8</v>
       </c>
@@ -30267,7 +30271,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A13" s="47">
         <v>9</v>
       </c>
@@ -30353,7 +30357,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A14" s="46" t="s">
         <v>27</v>
       </c>
@@ -30454,7 +30458,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="1" hidden="1" customWidth="1"/>
@@ -30486,7 +30490,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>79</v>
       </c>
@@ -30572,7 +30576,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="63.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -30658,7 +30662,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="53">
         <v>1</v>
       </c>
@@ -30744,7 +30748,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="53">
         <v>2</v>
       </c>
@@ -30830,7 +30834,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="53">
         <v>4</v>
       </c>
@@ -30916,7 +30920,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="53">
         <v>5</v>
       </c>
@@ -31002,7 +31006,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="53">
         <v>6</v>
       </c>
@@ -31088,7 +31092,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="53">
         <v>7</v>
       </c>
@@ -31174,7 +31178,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="53">
         <v>8</v>
       </c>
@@ -31260,7 +31264,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="53">
         <v>9</v>
       </c>
@@ -31346,7 +31350,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="53">
         <v>3</v>
       </c>
@@ -31426,7 +31430,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="53">
         <v>10</v>
       </c>
@@ -31512,7 +31516,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="53">
         <v>11</v>
       </c>
@@ -31598,7 +31602,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -31644,7 +31648,7 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -31676,7 +31680,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="21" customHeight="1">
       <c r="A1" s="221" t="s">
         <v>134</v>
       </c>
@@ -31762,7 +31766,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="48" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -31848,7 +31852,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -31934,7 +31938,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>27</v>
       </c>
@@ -32035,7 +32039,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -32067,7 +32071,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1">
       <c r="A1" s="227" t="s">
         <v>109</v>
       </c>
@@ -32153,7 +32157,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -32239,7 +32243,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -32325,7 +32329,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -32411,7 +32415,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -32497,7 +32501,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -32583,7 +32587,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -32669,7 +32673,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -32755,7 +32759,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -32841,7 +32845,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -32927,7 +32931,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -33013,7 +33017,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -33099,7 +33103,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -33185,7 +33189,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
@@ -33283,7 +33287,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C03CE4-617A-4EF9-89C8-ADAA1610BB0C}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -33313,7 +33317,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="219" t="s">
         <v>681</v>
       </c>
@@ -33399,7 +33403,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="60.6" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -33485,7 +33489,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="19.2" customHeight="1">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -33571,7 +33575,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28">
       <c r="A4" s="110" t="s">
         <v>27</v>
       </c>
@@ -33668,7 +33672,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41716D2-EB8A-4484-83AF-D7868E55628C}">
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -33698,7 +33702,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="219" t="s">
         <v>669</v>
       </c>
@@ -33784,7 +33788,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -33870,7 +33874,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="167" customFormat="1">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -33956,7 +33960,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="167" customFormat="1">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -34040,7 +34044,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="167" customFormat="1">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -34120,7 +34124,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="167" customFormat="1">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -34200,7 +34204,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="167" customFormat="1">
       <c r="A7" s="161">
         <v>5</v>
       </c>
@@ -34280,7 +34284,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="167" customFormat="1">
       <c r="A8" s="161">
         <v>6</v>
       </c>
@@ -34360,7 +34364,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="167" customFormat="1">
       <c r="A9" s="161">
         <v>7</v>
       </c>
@@ -34440,7 +34444,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="167" customFormat="1">
       <c r="A10" s="161">
         <v>8</v>
       </c>
@@ -34520,7 +34524,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="167" customFormat="1">
       <c r="A11" s="161">
         <v>9</v>
       </c>
@@ -34600,7 +34604,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="167" customFormat="1">
       <c r="A12" s="161">
         <v>10</v>
       </c>
@@ -34680,7 +34684,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="167" customFormat="1">
       <c r="A13" s="161">
         <v>11</v>
       </c>
@@ -34760,7 +34764,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="167" customFormat="1">
       <c r="A14" s="161">
         <v>12</v>
       </c>
@@ -34840,7 +34844,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="167" customFormat="1">
       <c r="A15" s="168" t="s">
         <v>27</v>
       </c>
@@ -34939,7 +34943,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BFDD7F-F2DE-484D-858D-A0AEE46D68A8}">
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.88671875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -34970,7 +34974,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="219" t="s">
         <v>665</v>
       </c>
@@ -35056,7 +35060,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -35142,7 +35146,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="184" customFormat="1">
       <c r="A3" s="178">
         <v>1</v>
       </c>
@@ -35228,7 +35232,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="184" customFormat="1">
       <c r="A4" s="178">
         <v>2</v>
       </c>
@@ -35314,7 +35318,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="184" customFormat="1">
       <c r="A5" s="178">
         <v>3</v>
       </c>
@@ -35400,7 +35404,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="184" customFormat="1">
       <c r="A6" s="178">
         <v>4</v>
       </c>
@@ -35486,7 +35490,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="184" customFormat="1">
       <c r="A7" s="178">
         <v>5</v>
       </c>
@@ -35572,7 +35576,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="184" customFormat="1">
       <c r="A8" s="178">
         <v>6</v>
       </c>
@@ -35658,7 +35662,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="184" customFormat="1">
       <c r="A9" s="178">
         <v>7</v>
       </c>
@@ -35744,7 +35748,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="184" customFormat="1">
       <c r="A10" s="178">
         <v>8</v>
       </c>
@@ -35830,7 +35834,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="184" customFormat="1">
       <c r="A11" s="178">
         <v>9</v>
       </c>
@@ -35916,7 +35920,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="167" customFormat="1">
       <c r="A12" s="168" t="s">
         <v>27</v>
       </c>
@@ -36016,7 +36020,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -36047,7 +36051,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="220" t="s">
         <v>652</v>
       </c>
@@ -36133,7 +36137,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="57" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -36219,7 +36223,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -36305,7 +36309,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -36391,7 +36395,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="150">
         <v>3</v>
       </c>
@@ -36477,7 +36481,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="150">
         <v>4</v>
       </c>
@@ -36563,7 +36567,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="150">
         <v>5</v>
       </c>
@@ -36649,7 +36653,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -36735,7 +36739,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -36821,7 +36825,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -36907,7 +36911,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -36993,7 +36997,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -37079,7 +37083,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -37165,7 +37169,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -37251,7 +37255,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="150">
         <v>13</v>
       </c>
@@ -37337,7 +37341,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="150">
         <v>14</v>
       </c>
@@ -37423,7 +37427,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A17" s="150">
         <v>15</v>
       </c>
@@ -37509,7 +37513,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A18" s="150">
         <v>16</v>
       </c>
@@ -37595,7 +37599,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A19" s="150">
         <v>17</v>
       </c>
@@ -37681,7 +37685,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A20" s="150">
         <v>18</v>
       </c>
@@ -37767,7 +37771,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A21" s="150">
         <v>19</v>
       </c>
@@ -37853,7 +37857,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A22" s="150">
         <v>20</v>
       </c>
@@ -37933,7 +37937,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A23" s="150">
         <v>21</v>
       </c>
@@ -38019,7 +38023,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A24" s="150">
         <v>22</v>
       </c>
@@ -38105,7 +38109,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A25" s="150">
         <v>23</v>
       </c>
@@ -38191,7 +38195,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A26" s="150">
         <v>24</v>
       </c>
@@ -38277,7 +38281,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A27" s="150">
         <v>25</v>
       </c>
@@ -38363,7 +38367,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A28" s="157" t="s">
         <v>27</v>
       </c>
@@ -38449,7 +38453,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:28">
       <c r="B29" s="206"/>
     </row>
   </sheetData>
@@ -38467,7 +38471,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -38498,7 +38502,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="220" t="s">
         <v>618</v>
       </c>
@@ -38584,7 +38588,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="57" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -38670,7 +38674,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -38756,7 +38760,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -38842,7 +38846,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -38928,7 +38932,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -39014,7 +39018,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="168" t="s">
         <v>27</v>
       </c>
@@ -39115,7 +39119,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.21875" style="108" customWidth="1"/>
     <col min="2" max="2" width="15.109375" style="108" customWidth="1"/>
@@ -39147,7 +39151,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="220" t="s">
         <v>606</v>
       </c>
@@ -39233,7 +39237,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="57" customHeight="1">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -39319,7 +39323,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="170">
         <v>1</v>
       </c>
@@ -39405,7 +39409,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="170">
         <v>2</v>
       </c>
@@ -39491,7 +39495,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="170">
         <v>3</v>
       </c>
@@ -39577,7 +39581,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="170">
         <v>4</v>
       </c>
@@ -39663,7 +39667,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="170">
         <v>5</v>
       </c>
@@ -39749,7 +39753,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="170">
         <v>6</v>
       </c>
@@ -39835,7 +39839,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="170">
         <v>7</v>
       </c>
@@ -39921,7 +39925,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="170">
         <v>8</v>
       </c>
@@ -40007,7 +40011,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="157" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (17/09/2026 14:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CEA6FFE-A7AB-472C-9327-902FC2319522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CC1DCBD-325D-4AEF-BEC7-CE05D419440C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens 1209" sheetId="156" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6959" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6966" uniqueCount="759">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -35884,7 +35884,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41716D2-EB8A-4484-83AF-D7868E55628C}">
-  <dimension ref="A1:AB15"/>
+  <dimension ref="A1:AB16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
@@ -36087,7 +36087,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -36173,7 +36173,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -36257,7 +36257,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -36337,7 +36337,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -36417,7 +36417,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="161">
         <v>5</v>
       </c>
@@ -36497,7 +36497,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="161">
         <v>6</v>
       </c>
@@ -36577,7 +36577,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="161">
         <v>7</v>
       </c>
@@ -36657,7 +36657,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="161">
         <v>8</v>
       </c>
@@ -36737,7 +36737,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="161">
         <v>9</v>
       </c>
@@ -36817,7 +36817,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="161">
         <v>10</v>
       </c>
@@ -36897,7 +36897,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="161">
         <v>11</v>
       </c>
@@ -36977,7 +36977,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="161">
         <v>12</v>
       </c>
@@ -37057,91 +37057,171 @@
         <v>739</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="G15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="H15" s="168">
-        <f>SUM(H3:H14)</f>
-        <v>20050</v>
-      </c>
-      <c r="I15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="J15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="K15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="L15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="M15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="N15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="O15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="P15" s="168">
-        <f>SUM(P3:P14)</f>
-        <v>3308.5</v>
-      </c>
-      <c r="Q15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="R15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="S15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="T15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="U15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="V15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="W15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="X15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB15" s="168" t="s">
+    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="150">
+        <v>3</v>
+      </c>
+      <c r="B15" s="151" t="s">
+        <v>621</v>
+      </c>
+      <c r="C15" s="150" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="177">
+        <v>46275</v>
+      </c>
+      <c r="E15" s="150"/>
+      <c r="F15" s="150">
+        <v>252541</v>
+      </c>
+      <c r="G15" s="150">
+        <v>67</v>
+      </c>
+      <c r="H15" s="150">
+        <v>3000</v>
+      </c>
+      <c r="I15" s="152">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="J15" s="152">
+        <v>1.004</v>
+      </c>
+      <c r="K15" s="150" t="s">
+        <v>736</v>
+      </c>
+      <c r="L15" s="152">
+        <v>840.34799999999996</v>
+      </c>
+      <c r="M15" s="153">
+        <v>1004</v>
+      </c>
+      <c r="N15" s="154">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="O15" s="155">
+        <v>5.58</v>
+      </c>
+      <c r="P15" s="150">
+        <v>289.89999999999998</v>
+      </c>
+      <c r="Q15" s="150">
+        <v>3</v>
+      </c>
+      <c r="R15" s="150">
+        <v>900</v>
+      </c>
+      <c r="S15" s="152">
+        <v>0.83699999999999997</v>
+      </c>
+      <c r="T15" s="150">
+        <v>63</v>
+      </c>
+      <c r="U15" s="154">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V15" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="150"/>
+      <c r="Z15" s="150"/>
+      <c r="AA15" s="150">
+        <v>1</v>
+      </c>
+      <c r="AB15" s="150" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="168">
+        <f>SUM(H3:H15)</f>
+        <v>23050</v>
+      </c>
+      <c r="I16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="J16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="K16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="L16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="M16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="O16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="P16" s="168">
+        <f>SUM(P3:P15)</f>
+        <v>3598.4</v>
+      </c>
+      <c r="Q16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="R16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="S16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="T16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="U16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="V16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="W16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="X16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA16" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB16" s="168" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (17/09/2026 15:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E16C89D-F23A-47F9-AFDA-FA4F17A51108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380802A0-75AA-4B89-B0D4-E4D0E018464C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Z4A EMBALAGENS LTDA 1210" sheetId="157" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7100" uniqueCount="769">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7107" uniqueCount="770">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2378,6 +2378,9 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - Z4A EMBALAGENS LTDA  —  OF: 001210</t>
+  </si>
+  <si>
+    <t>780x1820</t>
   </si>
 </sst>
 </file>
@@ -3490,7 +3493,7 @@
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" style="108" customWidth="1"/>
+    <col min="5" max="5" width="8.77734375" style="108" customWidth="1"/>
     <col min="6" max="6" width="7.109375" style="108" customWidth="1"/>
     <col min="7" max="8" width="6.21875" style="108" customWidth="1"/>
     <col min="9" max="10" width="6" style="108" customWidth="1"/>
@@ -37206,7 +37209,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41716D2-EB8A-4484-83AF-D7868E55628C}">
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
@@ -37594,52 +37597,52 @@
       </c>
       <c r="E5" s="161"/>
       <c r="F5" s="161">
-        <v>262576</v>
+        <v>262577</v>
       </c>
       <c r="G5" s="161">
         <v>69</v>
       </c>
       <c r="H5" s="161">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="I5" s="163">
-        <v>0.45</v>
+        <v>0.52500000000000002</v>
       </c>
       <c r="J5" s="163">
-        <v>1.59</v>
+        <v>1.29</v>
       </c>
       <c r="K5" s="161" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="L5" s="163">
-        <v>357.75</v>
+        <v>677.25</v>
       </c>
       <c r="M5" s="164">
-        <v>397.5</v>
+        <v>645</v>
       </c>
       <c r="N5" s="165">
-        <v>5.5199999999999999E-2</v>
+        <v>8.9599999999999999E-2</v>
       </c>
       <c r="O5" s="166">
-        <v>3.31</v>
+        <v>5.38</v>
       </c>
       <c r="P5" s="161">
-        <v>138.80000000000001</v>
+        <v>262.8</v>
       </c>
       <c r="Q5" s="161">
         <v>2</v>
       </c>
       <c r="R5" s="161">
-        <v>1150</v>
+        <v>1100</v>
       </c>
       <c r="S5" s="163">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="T5" s="161">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="U5" s="165">
-        <v>0.21740000000000001</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V5" s="161" t="s">
         <v>40</v>
@@ -37653,10 +37656,10 @@
       <c r="Y5" s="161"/>
       <c r="Z5" s="161"/>
       <c r="AA5" s="161">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB5" s="161" t="s">
-        <v>666</v>
+        <v>673</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37674,37 +37677,37 @@
       </c>
       <c r="E6" s="161"/>
       <c r="F6" s="161">
-        <v>262578</v>
+        <v>262576</v>
       </c>
       <c r="G6" s="161">
         <v>69</v>
       </c>
       <c r="H6" s="161">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="I6" s="163">
-        <v>0.54600000000000004</v>
+        <v>0.45</v>
       </c>
       <c r="J6" s="163">
-        <v>1.41</v>
+        <v>1.59</v>
       </c>
       <c r="K6" s="161" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="L6" s="163">
-        <v>461.916</v>
+        <v>357.75</v>
       </c>
       <c r="M6" s="164">
-        <v>423</v>
+        <v>397.5</v>
       </c>
       <c r="N6" s="165">
-        <v>5.8700000000000002E-2</v>
+        <v>5.5199999999999999E-2</v>
       </c>
       <c r="O6" s="166">
-        <v>3.52</v>
+        <v>3.31</v>
       </c>
       <c r="P6" s="161">
-        <v>179.2</v>
+        <v>138.80000000000001</v>
       </c>
       <c r="Q6" s="161">
         <v>2</v>
@@ -37713,13 +37716,13 @@
         <v>1150</v>
       </c>
       <c r="S6" s="163">
-        <v>1.0920000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="T6" s="161">
-        <v>58</v>
+        <v>250</v>
       </c>
       <c r="U6" s="165">
-        <v>5.04E-2</v>
+        <v>0.21740000000000001</v>
       </c>
       <c r="V6" s="161" t="s">
         <v>40</v>
@@ -37736,7 +37739,7 @@
         <v>1</v>
       </c>
       <c r="AB6" s="161" t="s">
-        <v>675</v>
+        <v>666</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37747,68 +37750,68 @@
         <v>480</v>
       </c>
       <c r="C7" s="161" t="s">
-        <v>36</v>
+        <v>670</v>
       </c>
       <c r="D7" s="191">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="E7" s="161"/>
       <c r="F7" s="161">
-        <v>262603</v>
+        <v>262578</v>
       </c>
       <c r="G7" s="161">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H7" s="161">
         <v>600</v>
       </c>
       <c r="I7" s="163">
-        <v>0.69</v>
+        <v>0.54600000000000004</v>
       </c>
       <c r="J7" s="163">
-        <v>1</v>
+        <v>1.41</v>
       </c>
       <c r="K7" s="161" t="s">
-        <v>34</v>
+        <v>674</v>
       </c>
       <c r="L7" s="163">
-        <v>414</v>
+        <v>461.916</v>
       </c>
       <c r="M7" s="164">
-        <v>300</v>
+        <v>423</v>
       </c>
       <c r="N7" s="165">
-        <v>4.1700000000000001E-2</v>
+        <v>5.8700000000000002E-2</v>
       </c>
       <c r="O7" s="166">
-        <v>2.5</v>
+        <v>3.52</v>
       </c>
       <c r="P7" s="161">
-        <v>130.4</v>
+        <v>179.2</v>
       </c>
       <c r="Q7" s="161">
         <v>2</v>
       </c>
       <c r="R7" s="161">
-        <v>1400</v>
+        <v>1150</v>
       </c>
       <c r="S7" s="163">
-        <v>1.38</v>
+        <v>1.0920000000000001</v>
       </c>
       <c r="T7" s="161">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="U7" s="165">
-        <v>1.43E-2</v>
+        <v>5.04E-2</v>
       </c>
       <c r="V7" s="161" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="W7" s="161" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X7" s="161" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Y7" s="161"/>
       <c r="Z7" s="161"/>
@@ -37816,7 +37819,7 @@
         <v>1</v>
       </c>
       <c r="AB7" s="161" t="s">
-        <v>712</v>
+        <v>675</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37827,76 +37830,76 @@
         <v>480</v>
       </c>
       <c r="C8" s="161" t="s">
-        <v>670</v>
+        <v>36</v>
       </c>
       <c r="D8" s="191">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="E8" s="161"/>
       <c r="F8" s="161">
-        <v>262577</v>
+        <v>262634</v>
       </c>
       <c r="G8" s="161">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H8" s="161">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="I8" s="163">
-        <v>0.52500000000000002</v>
+        <v>0.76</v>
       </c>
       <c r="J8" s="163">
-        <v>1.29</v>
+        <v>0.9</v>
       </c>
       <c r="K8" s="161" t="s">
-        <v>672</v>
+        <v>34</v>
       </c>
       <c r="L8" s="163">
-        <v>677.25</v>
+        <v>3420</v>
       </c>
       <c r="M8" s="164">
-        <v>645</v>
+        <v>2250</v>
       </c>
       <c r="N8" s="165">
-        <v>8.9599999999999999E-2</v>
+        <v>0.3125</v>
       </c>
       <c r="O8" s="166">
-        <v>5.38</v>
+        <v>18.75</v>
       </c>
       <c r="P8" s="161">
-        <v>262.8</v>
+        <v>1077.3</v>
       </c>
       <c r="Q8" s="161">
         <v>2</v>
       </c>
       <c r="R8" s="161">
-        <v>1100</v>
+        <v>1550</v>
       </c>
       <c r="S8" s="163">
-        <v>1.05</v>
+        <v>1.52</v>
       </c>
       <c r="T8" s="161">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="U8" s="165">
-        <v>4.5499999999999999E-2</v>
+        <v>1.9400000000000001E-2</v>
       </c>
       <c r="V8" s="161" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="W8" s="161" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X8" s="161" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Y8" s="161"/>
       <c r="Z8" s="161"/>
       <c r="AA8" s="161">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AB8" s="161" t="s">
-        <v>673</v>
+        <v>769</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37910,56 +37913,56 @@
         <v>36</v>
       </c>
       <c r="D9" s="191">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="E9" s="161"/>
       <c r="F9" s="161">
-        <v>262616</v>
+        <v>262603</v>
       </c>
       <c r="G9" s="161">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H9" s="161">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="I9" s="163">
-        <v>0.35</v>
+        <v>0.69</v>
       </c>
       <c r="J9" s="163">
-        <v>0.88</v>
+        <v>1</v>
       </c>
       <c r="K9" s="161" t="s">
         <v>34</v>
       </c>
       <c r="L9" s="163">
-        <v>308</v>
+        <v>414</v>
       </c>
       <c r="M9" s="164">
-        <v>293.3</v>
+        <v>300</v>
       </c>
       <c r="N9" s="165">
-        <v>2.7199999999999998E-2</v>
+        <v>4.1700000000000001E-2</v>
       </c>
       <c r="O9" s="166">
-        <v>1.63</v>
+        <v>2.5</v>
       </c>
       <c r="P9" s="161">
-        <v>97</v>
+        <v>130.4</v>
       </c>
       <c r="Q9" s="161">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="161">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="S9" s="163">
-        <v>1.05</v>
+        <v>1.38</v>
       </c>
       <c r="T9" s="161">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="U9" s="165">
-        <v>4.5499999999999999E-2</v>
+        <v>1.43E-2</v>
       </c>
       <c r="V9" s="161" t="s">
         <v>28</v>
@@ -37976,7 +37979,7 @@
         <v>1</v>
       </c>
       <c r="AB9" s="161" t="s">
-        <v>734</v>
+        <v>712</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37990,56 +37993,56 @@
         <v>36</v>
       </c>
       <c r="D10" s="191">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E10" s="161"/>
       <c r="F10" s="161">
-        <v>262602</v>
+        <v>262616</v>
       </c>
       <c r="G10" s="161">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H10" s="161">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="I10" s="163">
-        <v>0.54</v>
+        <v>0.35</v>
       </c>
       <c r="J10" s="163">
-        <v>1</v>
+        <v>0.88</v>
       </c>
       <c r="K10" s="161" t="s">
         <v>34</v>
       </c>
       <c r="L10" s="163">
-        <v>675</v>
+        <v>308</v>
       </c>
       <c r="M10" s="164">
-        <v>625</v>
+        <v>293.3</v>
       </c>
       <c r="N10" s="165">
-        <v>8.6800000000000002E-2</v>
+        <v>2.7199999999999998E-2</v>
       </c>
       <c r="O10" s="166">
-        <v>5.21</v>
+        <v>1.63</v>
       </c>
       <c r="P10" s="161">
-        <v>212.6</v>
+        <v>97</v>
       </c>
       <c r="Q10" s="161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="161">
         <v>1100</v>
       </c>
       <c r="S10" s="163">
-        <v>1.08</v>
+        <v>1.05</v>
       </c>
       <c r="T10" s="161">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="U10" s="165">
-        <v>1.8200000000000001E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V10" s="161" t="s">
         <v>28</v>
@@ -38056,7 +38059,7 @@
         <v>1</v>
       </c>
       <c r="AB10" s="161" t="s">
-        <v>711</v>
+        <v>734</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -38070,56 +38073,56 @@
         <v>36</v>
       </c>
       <c r="D11" s="191">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="E11" s="161"/>
       <c r="F11" s="161">
-        <v>262615</v>
+        <v>262602</v>
       </c>
       <c r="G11" s="161">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H11" s="161">
-        <v>3000</v>
+        <v>1250</v>
       </c>
       <c r="I11" s="163">
-        <v>0.51400000000000001</v>
+        <v>0.54</v>
       </c>
       <c r="J11" s="163">
-        <v>1.3420000000000001</v>
+        <v>1</v>
       </c>
       <c r="K11" s="161" t="s">
-        <v>732</v>
+        <v>34</v>
       </c>
       <c r="L11" s="163">
-        <v>1379.576</v>
+        <v>675</v>
       </c>
       <c r="M11" s="164">
-        <v>1342</v>
+        <v>625</v>
       </c>
       <c r="N11" s="165">
-        <v>0.18640000000000001</v>
+        <v>8.6800000000000002E-2</v>
       </c>
       <c r="O11" s="166">
-        <v>11.18</v>
+        <v>5.21</v>
       </c>
       <c r="P11" s="161">
-        <v>434.6</v>
+        <v>212.6</v>
       </c>
       <c r="Q11" s="161">
         <v>2</v>
       </c>
       <c r="R11" s="161">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S11" s="163">
-        <v>1.028</v>
+        <v>1.08</v>
       </c>
       <c r="T11" s="161">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="U11" s="165">
-        <v>2.1000000000000001E-2</v>
+        <v>1.8200000000000001E-2</v>
       </c>
       <c r="V11" s="161" t="s">
         <v>28</v>
@@ -38133,10 +38136,10 @@
       <c r="Y11" s="161"/>
       <c r="Z11" s="161"/>
       <c r="AA11" s="161">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB11" s="161" t="s">
-        <v>733</v>
+        <v>711</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -38154,52 +38157,52 @@
       </c>
       <c r="E12" s="161"/>
       <c r="F12" s="161">
-        <v>262617</v>
+        <v>262615</v>
       </c>
       <c r="G12" s="161">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H12" s="161">
-        <v>3200</v>
+        <v>3000</v>
       </c>
       <c r="I12" s="163">
-        <v>0.32500000000000001</v>
+        <v>0.51400000000000001</v>
       </c>
       <c r="J12" s="163">
-        <v>0.8</v>
+        <v>1.3420000000000001</v>
       </c>
       <c r="K12" s="161" t="s">
-        <v>34</v>
+        <v>732</v>
       </c>
       <c r="L12" s="163">
-        <v>832</v>
+        <v>1379.576</v>
       </c>
       <c r="M12" s="164">
-        <v>853.3</v>
+        <v>1342</v>
       </c>
       <c r="N12" s="165">
-        <v>7.9000000000000001E-2</v>
+        <v>0.18640000000000001</v>
       </c>
       <c r="O12" s="166">
-        <v>4.74</v>
+        <v>11.18</v>
       </c>
       <c r="P12" s="161">
-        <v>262.10000000000002</v>
+        <v>434.6</v>
       </c>
       <c r="Q12" s="161">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R12" s="161">
-        <v>1000</v>
+        <v>1050</v>
       </c>
       <c r="S12" s="163">
-        <v>0.97499999999999998</v>
+        <v>1.028</v>
       </c>
       <c r="T12" s="161">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="U12" s="165">
-        <v>2.5000000000000001E-2</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="V12" s="161" t="s">
         <v>28</v>
@@ -38213,10 +38216,10 @@
       <c r="Y12" s="161"/>
       <c r="Z12" s="161"/>
       <c r="AA12" s="161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB12" s="161" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -38234,52 +38237,52 @@
       </c>
       <c r="E13" s="161"/>
       <c r="F13" s="161">
-        <v>262618</v>
+        <v>262617</v>
       </c>
       <c r="G13" s="161">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H13" s="161">
-        <v>2000</v>
+        <v>3200</v>
       </c>
       <c r="I13" s="163">
-        <v>0.27900000000000003</v>
+        <v>0.32500000000000001</v>
       </c>
       <c r="J13" s="163">
-        <v>1.002</v>
+        <v>0.8</v>
       </c>
       <c r="K13" s="161" t="s">
-        <v>736</v>
+        <v>34</v>
       </c>
       <c r="L13" s="163">
-        <v>559.11599999999999</v>
+        <v>832</v>
       </c>
       <c r="M13" s="164">
-        <v>1002</v>
+        <v>853.3</v>
       </c>
       <c r="N13" s="165">
-        <v>0.13919999999999999</v>
+        <v>7.9000000000000001E-2</v>
       </c>
       <c r="O13" s="166">
-        <v>8.35</v>
+        <v>4.74</v>
       </c>
       <c r="P13" s="161">
-        <v>176.1</v>
+        <v>262.10000000000002</v>
       </c>
       <c r="Q13" s="161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="161">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="S13" s="163">
-        <v>0.55800000000000005</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="T13" s="161">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="U13" s="165">
-        <v>7.0000000000000007E-2</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="V13" s="161" t="s">
         <v>28</v>
@@ -38293,10 +38296,10 @@
       <c r="Y13" s="161"/>
       <c r="Z13" s="161"/>
       <c r="AA13" s="161">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB13" s="161" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -38314,52 +38317,52 @@
       </c>
       <c r="E14" s="161"/>
       <c r="F14" s="161">
-        <v>262619</v>
+        <v>262618</v>
       </c>
       <c r="G14" s="161">
         <v>73</v>
       </c>
       <c r="H14" s="161">
-        <v>6000</v>
+        <v>2000</v>
       </c>
       <c r="I14" s="163">
-        <v>0.36499999999999999</v>
+        <v>0.27900000000000003</v>
       </c>
       <c r="J14" s="163">
-        <v>1.04</v>
+        <v>1.002</v>
       </c>
       <c r="K14" s="161" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="L14" s="163">
-        <v>2277.6</v>
+        <v>559.11599999999999</v>
       </c>
       <c r="M14" s="164">
-        <v>3120</v>
+        <v>1002</v>
       </c>
       <c r="N14" s="165">
-        <v>0.43330000000000002</v>
+        <v>0.13919999999999999</v>
       </c>
       <c r="O14" s="166">
-        <v>26</v>
+        <v>8.35</v>
       </c>
       <c r="P14" s="161">
-        <v>717.4</v>
+        <v>176.1</v>
       </c>
       <c r="Q14" s="161">
         <v>2</v>
       </c>
       <c r="R14" s="161">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="S14" s="163">
-        <v>0.73</v>
+        <v>0.55800000000000005</v>
       </c>
       <c r="T14" s="161">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="U14" s="165">
-        <v>2.6700000000000002E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="V14" s="161" t="s">
         <v>28</v>
@@ -38373,177 +38376,257 @@
       <c r="Y14" s="161"/>
       <c r="Z14" s="161"/>
       <c r="AA14" s="161">
+        <v>1</v>
+      </c>
+      <c r="AB14" s="161" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="161">
+        <v>13</v>
+      </c>
+      <c r="B15" s="162" t="s">
+        <v>480</v>
+      </c>
+      <c r="C15" s="161" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="191">
+        <v>46281</v>
+      </c>
+      <c r="E15" s="161"/>
+      <c r="F15" s="161">
+        <v>262619</v>
+      </c>
+      <c r="G15" s="161">
+        <v>73</v>
+      </c>
+      <c r="H15" s="161">
+        <v>6000</v>
+      </c>
+      <c r="I15" s="163">
+        <v>0.36499999999999999</v>
+      </c>
+      <c r="J15" s="163">
+        <v>1.04</v>
+      </c>
+      <c r="K15" s="161" t="s">
+        <v>738</v>
+      </c>
+      <c r="L15" s="163">
+        <v>2277.6</v>
+      </c>
+      <c r="M15" s="164">
+        <v>3120</v>
+      </c>
+      <c r="N15" s="165">
+        <v>0.43330000000000002</v>
+      </c>
+      <c r="O15" s="166">
+        <v>26</v>
+      </c>
+      <c r="P15" s="161">
+        <v>717.4</v>
+      </c>
+      <c r="Q15" s="161">
+        <v>2</v>
+      </c>
+      <c r="R15" s="161">
+        <v>750</v>
+      </c>
+      <c r="S15" s="163">
+        <v>0.73</v>
+      </c>
+      <c r="T15" s="161">
+        <v>20</v>
+      </c>
+      <c r="U15" s="165">
+        <v>2.6700000000000002E-2</v>
+      </c>
+      <c r="V15" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="161"/>
+      <c r="Z15" s="161"/>
+      <c r="AA15" s="161">
         <v>3</v>
       </c>
-      <c r="AB14" s="161" t="s">
+      <c r="AB15" s="161" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="150">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="161">
+        <v>14</v>
+      </c>
+      <c r="B16" s="151" t="s">
+        <v>621</v>
+      </c>
+      <c r="C16" s="150" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="177">
+        <v>46275</v>
+      </c>
+      <c r="E16" s="150"/>
+      <c r="F16" s="150">
+        <v>252541</v>
+      </c>
+      <c r="G16" s="150">
+        <v>67</v>
+      </c>
+      <c r="H16" s="150">
+        <v>3000</v>
+      </c>
+      <c r="I16" s="152">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="J16" s="152">
+        <v>1.004</v>
+      </c>
+      <c r="K16" s="150" t="s">
+        <v>736</v>
+      </c>
+      <c r="L16" s="152">
+        <v>840.34799999999996</v>
+      </c>
+      <c r="M16" s="153">
+        <v>1004</v>
+      </c>
+      <c r="N16" s="154">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="O16" s="155">
+        <v>5.58</v>
+      </c>
+      <c r="P16" s="150">
+        <v>289.89999999999998</v>
+      </c>
+      <c r="Q16" s="150">
         <v>3</v>
       </c>
-      <c r="B15" s="151" t="s">
-        <v>621</v>
-      </c>
-      <c r="C15" s="150" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="177">
-        <v>46275</v>
-      </c>
-      <c r="E15" s="150"/>
-      <c r="F15" s="150">
-        <v>252541</v>
-      </c>
-      <c r="G15" s="150">
-        <v>67</v>
-      </c>
-      <c r="H15" s="150">
-        <v>3000</v>
-      </c>
-      <c r="I15" s="152">
-        <v>0.27900000000000003</v>
-      </c>
-      <c r="J15" s="152">
-        <v>1.004</v>
-      </c>
-      <c r="K15" s="150" t="s">
-        <v>736</v>
-      </c>
-      <c r="L15" s="152">
-        <v>840.34799999999996</v>
-      </c>
-      <c r="M15" s="153">
-        <v>1004</v>
-      </c>
-      <c r="N15" s="154">
-        <v>9.2999999999999999E-2</v>
-      </c>
-      <c r="O15" s="155">
-        <v>5.58</v>
-      </c>
-      <c r="P15" s="150">
-        <v>289.89999999999998</v>
-      </c>
-      <c r="Q15" s="150">
-        <v>3</v>
-      </c>
-      <c r="R15" s="150">
+      <c r="R16" s="150">
         <v>900</v>
       </c>
-      <c r="S15" s="152">
+      <c r="S16" s="152">
         <v>0.83699999999999997</v>
       </c>
-      <c r="T15" s="150">
+      <c r="T16" s="150">
         <v>63</v>
       </c>
-      <c r="U15" s="154">
+      <c r="U16" s="154">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="V15" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="X15" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="150"/>
-      <c r="Z15" s="150"/>
-      <c r="AA15" s="150">
+      <c r="V16" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y16" s="150"/>
+      <c r="Z16" s="150"/>
+      <c r="AA16" s="150">
         <v>1</v>
       </c>
-      <c r="AB15" s="150" t="s">
+      <c r="AB16" s="150" t="s">
         <v>622</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="H16" s="168">
-        <f>SUM(H3:H15)</f>
-        <v>23050</v>
-      </c>
-      <c r="I16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="J16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="K16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="L16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="M16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="N16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="O16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="P16" s="168">
-        <f>SUM(P3:P15)</f>
-        <v>3598.4</v>
-      </c>
-      <c r="Q16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="R16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="S16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="T16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="U16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="V16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="W16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="X16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA16" s="168" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB16" s="168" t="s">
+    <row r="17" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" s="168">
+        <f>SUM(H3:H16)</f>
+        <v>28050</v>
+      </c>
+      <c r="I17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="K17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="L17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="M17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="O17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="P17" s="168">
+        <f>SUM(P3:P16)</f>
+        <v>4675.6999999999989</v>
+      </c>
+      <c r="Q17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="R17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="S17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="T17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="U17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="V17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="W17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="X17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="168" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB17" s="168" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (17/09/2026 16:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFE27BE-A7C6-4750-800E-5E7949E31770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A490F77F-253F-422E-9CC5-BD1F775A69AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PCBOX 1212" sheetId="158" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="ABAPEL 1201" sheetId="153" r:id="rId5"/>
     <sheet name="HARMONY EMBALAGENS 1200" sheetId="152" r:id="rId6"/>
     <sheet name="HARMONY EMBALAGENS 1199" sheetId="151" r:id="rId7"/>
-    <sheet name="FAVINCO EMBALAGENS 1197" sheetId="150" r:id="rId8"/>
+    <sheet name="FAVINCO EMBALAGENS 1197 P" sheetId="150" r:id="rId8"/>
     <sheet name="ABAPEL 1196" sheetId="149" r:id="rId9"/>
     <sheet name="CARPELL LTDA 1195 P" sheetId="147" r:id="rId10"/>
     <sheet name="Renovapel 1192 P" sheetId="146" r:id="rId11"/>
@@ -2429,7 +2429,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3524,7 +3524,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00EADB3A-C171-49AE-8471-729057A3A740}">
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -3556,7 +3556,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>781</v>
       </c>
@@ -3642,7 +3642,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="61.2" customHeight="1">
+    <row r="2" spans="1:28" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -3728,7 +3728,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -3900,7 +3900,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -4072,7 +4072,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="110" t="s">
         <v>27</v>
       </c>
@@ -4258,7 +4258,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB29"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -4289,7 +4289,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>652</v>
       </c>
@@ -4375,7 +4375,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -4633,7 +4633,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="150">
         <v>3</v>
       </c>
@@ -4719,7 +4719,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="150">
         <v>4</v>
       </c>
@@ -4805,7 +4805,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="150">
         <v>5</v>
       </c>
@@ -4891,7 +4891,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -4977,7 +4977,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -5063,7 +5063,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -5149,7 +5149,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -5235,7 +5235,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -5321,7 +5321,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -5407,7 +5407,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="150">
         <v>13</v>
       </c>
@@ -5579,7 +5579,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="150">
         <v>14</v>
       </c>
@@ -5665,7 +5665,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="150">
         <v>15</v>
       </c>
@@ -5751,7 +5751,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="150">
         <v>16</v>
       </c>
@@ -5837,7 +5837,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="150">
         <v>17</v>
       </c>
@@ -5923,7 +5923,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="150">
         <v>18</v>
       </c>
@@ -6009,7 +6009,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="150">
         <v>19</v>
       </c>
@@ -6095,7 +6095,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="150">
         <v>20</v>
       </c>
@@ -6175,7 +6175,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="150">
         <v>21</v>
       </c>
@@ -6261,7 +6261,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="150">
         <v>22</v>
       </c>
@@ -6347,7 +6347,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="150">
         <v>23</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="150">
         <v>24</v>
       </c>
@@ -6519,7 +6519,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="150">
         <v>25</v>
       </c>
@@ -6605,7 +6605,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="157" t="s">
         <v>27</v>
       </c>
@@ -6691,7 +6691,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:28">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B29" s="206"/>
     </row>
   </sheetData>
@@ -6709,7 +6709,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -6740,7 +6740,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>618</v>
       </c>
@@ -6826,7 +6826,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -6912,7 +6912,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -6998,7 +6998,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -7084,7 +7084,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -7170,7 +7170,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="168" t="s">
         <v>27</v>
       </c>
@@ -7357,7 +7357,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.21875" style="108" customWidth="1"/>
     <col min="2" max="2" width="15.109375" style="108" customWidth="1"/>
@@ -7389,7 +7389,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>606</v>
       </c>
@@ -7475,7 +7475,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -7561,7 +7561,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="170">
         <v>1</v>
       </c>
@@ -7647,7 +7647,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="170">
         <v>2</v>
       </c>
@@ -7733,7 +7733,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="170">
         <v>3</v>
       </c>
@@ -7819,7 +7819,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="170">
         <v>4</v>
       </c>
@@ -7905,7 +7905,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="170">
         <v>5</v>
       </c>
@@ -7991,7 +7991,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="170">
         <v>6</v>
       </c>
@@ -8077,7 +8077,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="170">
         <v>7</v>
       </c>
@@ -8163,7 +8163,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="170">
         <v>8</v>
       </c>
@@ -8249,7 +8249,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="157" t="s">
         <v>27</v>
       </c>
@@ -8350,7 +8350,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.5546875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -8380,7 +8380,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>599</v>
       </c>
@@ -8466,7 +8466,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -8552,7 +8552,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -8638,7 +8638,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -8724,7 +8724,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="150">
         <v>3</v>
       </c>
@@ -8804,7 +8804,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="157" t="s">
         <v>27</v>
       </c>
@@ -8892,7 +8892,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:28">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="D8" s="158"/>
       <c r="J8" s="159"/>
       <c r="L8" s="159"/>
@@ -8912,7 +8912,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -8940,7 +8940,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>592</v>
       </c>
@@ -9026,7 +9026,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1">
+    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -9112,7 +9112,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -9198,7 +9198,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -9284,7 +9284,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -9370,7 +9370,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -9450,7 +9450,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -9530,7 +9530,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -9616,7 +9616,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -9702,7 +9702,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -9788,7 +9788,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -9874,7 +9874,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -9975,7 +9975,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -10006,7 +10006,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="222" t="s">
         <v>554</v>
       </c>
@@ -10092,7 +10092,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -10178,7 +10178,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="193">
         <v>1</v>
       </c>
@@ -10264,7 +10264,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -10350,7 +10350,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="193">
         <v>3</v>
       </c>
@@ -10436,7 +10436,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="193">
         <v>4</v>
       </c>
@@ -10522,7 +10522,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="193">
         <v>5</v>
       </c>
@@ -10608,7 +10608,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -10694,7 +10694,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -10780,7 +10780,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -10866,7 +10866,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -10952,7 +10952,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -11038,7 +11038,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -11124,7 +11124,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -11210,7 +11210,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="157" t="s">
         <v>27</v>
       </c>
@@ -11311,7 +11311,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -11343,7 +11343,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>539</v>
       </c>
@@ -11429,7 +11429,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -11515,7 +11515,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="126">
         <v>1</v>
       </c>
@@ -11601,7 +11601,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -11687,7 +11687,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="126">
         <v>2</v>
       </c>
@@ -11773,7 +11773,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>3</v>
       </c>
@@ -11859,7 +11859,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -11945,7 +11945,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -12031,7 +12031,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -12117,7 +12117,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="10" spans="1:28">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>27</v>
       </c>
@@ -12215,7 +12215,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
   <dimension ref="A1:AB5"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -12247,7 +12247,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>535</v>
       </c>
@@ -12333,7 +12333,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -12419,7 +12419,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -12505,7 +12505,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -12591,7 +12591,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
         <v>27</v>
       </c>
@@ -12691,7 +12691,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -12723,7 +12723,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="223" t="s">
         <v>523</v>
       </c>
@@ -12809,7 +12809,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="43.2" customHeight="1">
+    <row r="2" spans="1:28" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="107" t="s">
         <v>0</v>
       </c>
@@ -12895,7 +12895,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="90">
         <v>1</v>
       </c>
@@ -12981,7 +12981,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="90">
         <v>2</v>
       </c>
@@ -13067,7 +13067,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="90">
         <v>3</v>
       </c>
@@ -13153,7 +13153,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="90">
         <v>4</v>
       </c>
@@ -13239,7 +13239,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="106" t="s">
         <v>27</v>
       </c>
@@ -13340,7 +13340,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" style="3" hidden="1" customWidth="1"/>
@@ -13372,7 +13372,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>512</v>
       </c>
@@ -13458,7 +13458,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -13544,7 +13544,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" customFormat="1">
+    <row r="3" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="120">
         <v>1</v>
       </c>
@@ -13630,7 +13630,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="4" spans="1:28" customFormat="1">
+    <row r="4" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="120">
         <v>2</v>
       </c>
@@ -13716,7 +13716,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:28" customFormat="1">
+    <row r="5" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="120">
         <v>3</v>
       </c>
@@ -13802,7 +13802,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="6" spans="1:28" customFormat="1">
+    <row r="6" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -13888,7 +13888,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="7" spans="1:28" customFormat="1">
+    <row r="7" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="120">
         <v>5</v>
       </c>
@@ -13974,7 +13974,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="8" spans="1:28" customFormat="1">
+    <row r="8" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="47">
         <v>6</v>
       </c>
@@ -14060,7 +14060,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="9" spans="1:28" customFormat="1">
+    <row r="9" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>7</v>
       </c>
@@ -14146,7 +14146,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="10" spans="1:28" customFormat="1">
+    <row r="10" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="120">
         <v>8</v>
       </c>
@@ -14232,7 +14232,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>9</v>
       </c>
@@ -14318,7 +14318,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="45" customFormat="1">
+    <row r="12" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="46" t="s">
         <v>27</v>
       </c>
@@ -14416,7 +14416,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A45B5AC-557E-4203-8DD1-DFBBC7E9A9E0}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.77734375" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -14446,7 +14446,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>768</v>
       </c>
@@ -14532,7 +14532,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -14618,7 +14618,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -14704,7 +14704,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -14790,7 +14790,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -14876,7 +14876,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="6" spans="1:28">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -14962,7 +14962,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:28">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="110" t="s">
         <v>27</v>
       </c>
@@ -15059,7 +15059,7 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -15090,7 +15090,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>531</v>
       </c>
@@ -15176,7 +15176,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39" customHeight="1">
+    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -15262,7 +15262,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -15348,7 +15348,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -15434,7 +15434,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -15520,7 +15520,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -15606,7 +15606,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -15692,7 +15692,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="110" t="s">
         <v>27</v>
       </c>
@@ -15793,7 +15793,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -15825,7 +15825,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>496</v>
       </c>
@@ -15911,7 +15911,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -15997,7 +15997,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="133">
         <v>1</v>
       </c>
@@ -16083,7 +16083,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="133">
         <v>2</v>
       </c>
@@ -16167,7 +16167,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="133">
         <v>3</v>
       </c>
@@ -16253,7 +16253,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="207">
         <v>4</v>
       </c>
@@ -16337,7 +16337,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="207">
         <v>5</v>
       </c>
@@ -16421,7 +16421,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="133">
         <v>6</v>
       </c>
@@ -16507,7 +16507,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="207">
         <v>7</v>
       </c>
@@ -16591,7 +16591,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="133">
         <v>8</v>
       </c>
@@ -16677,7 +16677,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="207">
         <v>9</v>
       </c>
@@ -16761,7 +16761,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="133">
         <v>10</v>
       </c>
@@ -16847,7 +16847,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="133">
         <v>11</v>
       </c>
@@ -16933,7 +16933,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="133">
         <v>12</v>
       </c>
@@ -17019,7 +17019,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="133">
         <v>13</v>
       </c>
@@ -17105,7 +17105,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="133">
         <v>14</v>
       </c>
@@ -17191,7 +17191,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>27</v>
       </c>
@@ -17294,7 +17294,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -17324,7 +17324,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>486</v>
       </c>
@@ -17410,7 +17410,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -17496,7 +17496,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -17582,7 +17582,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="139">
         <v>2</v>
       </c>
@@ -17668,7 +17668,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="139"/>
       <c r="B5" s="140" t="s">
         <v>480</v>
@@ -17746,7 +17746,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="139"/>
       <c r="B6" s="140" t="s">
         <v>480</v>
@@ -17824,7 +17824,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34">
         <v>3</v>
       </c>
@@ -17910,7 +17910,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="28" t="s">
         <v>27</v>
       </c>
@@ -18013,7 +18013,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -18043,7 +18043,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>475</v>
       </c>
@@ -18129,7 +18129,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -18215,7 +18215,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="97">
         <v>1</v>
       </c>
@@ -18301,7 +18301,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="97">
         <v>2</v>
       </c>
@@ -18387,7 +18387,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="97">
         <v>3</v>
       </c>
@@ -18473,7 +18473,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="97">
         <v>4</v>
       </c>
@@ -18559,7 +18559,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="97">
         <v>5</v>
       </c>
@@ -18645,7 +18645,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="97">
         <v>6</v>
       </c>
@@ -18731,7 +18731,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="97">
         <v>7</v>
       </c>
@@ -18817,7 +18817,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="97">
         <v>8</v>
       </c>
@@ -18903,7 +18903,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="97">
         <v>9</v>
       </c>
@@ -18989,7 +18989,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="97">
         <v>10</v>
       </c>
@@ -19075,7 +19075,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>27</v>
       </c>
@@ -19176,7 +19176,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -19208,7 +19208,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>454</v>
       </c>
@@ -19294,7 +19294,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="50.4" customHeight="1">
+    <row r="2" spans="1:28" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -19380,7 +19380,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -19466,7 +19466,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -19552,7 +19552,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -19638,7 +19638,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -19724,7 +19724,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -19810,7 +19810,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -19911,7 +19911,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -19943,7 +19943,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="33" customHeight="1">
+    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>440</v>
       </c>
@@ -20029,7 +20029,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20115,7 +20115,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -20201,7 +20201,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -20287,7 +20287,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -20373,7 +20373,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -20459,7 +20459,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -20545,7 +20545,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -20631,7 +20631,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -20717,7 +20717,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
@@ -20818,7 +20818,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -20849,7 +20849,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>403</v>
       </c>
@@ -20935,7 +20935,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1">
+    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -21021,7 +21021,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -21107,7 +21107,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -21191,7 +21191,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -21277,7 +21277,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -21363,7 +21363,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -21447,7 +21447,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -21531,7 +21531,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
@@ -21632,7 +21632,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" customWidth="1"/>
@@ -21662,7 +21662,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="225" t="s">
         <v>380</v>
       </c>
@@ -21748,7 +21748,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="89" t="s">
         <v>0</v>
       </c>
@@ -21834,7 +21834,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14">
         <v>1</v>
       </c>
@@ -21920,7 +21920,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14">
         <v>2</v>
       </c>
@@ -22006,7 +22006,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14">
         <v>3</v>
       </c>
@@ -22092,7 +22092,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14">
         <v>4</v>
       </c>
@@ -22178,7 +22178,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>5</v>
       </c>
@@ -22264,7 +22264,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>6</v>
       </c>
@@ -22350,7 +22350,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>7</v>
       </c>
@@ -22436,7 +22436,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>8</v>
       </c>
@@ -22522,7 +22522,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>9</v>
       </c>
@@ -22608,7 +22608,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>10</v>
       </c>
@@ -22694,7 +22694,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>11</v>
       </c>
@@ -22780,7 +22780,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
         <v>12</v>
       </c>
@@ -22866,7 +22866,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>13</v>
       </c>
@@ -22952,7 +22952,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
         <v>14</v>
       </c>
@@ -23038,7 +23038,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14">
         <v>15</v>
       </c>
@@ -23124,7 +23124,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14">
         <v>16</v>
       </c>
@@ -23210,7 +23210,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14">
         <v>17</v>
       </c>
@@ -23296,7 +23296,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14">
         <v>18</v>
       </c>
@@ -23382,7 +23382,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="25.05" customHeight="1">
+    <row r="21" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="14">
         <v>19</v>
       </c>
@@ -23468,7 +23468,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.05" customHeight="1">
+    <row r="22" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14">
         <v>20</v>
       </c>
@@ -23554,7 +23554,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.05" customHeight="1">
+    <row r="23" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14">
         <v>21</v>
       </c>
@@ -23640,7 +23640,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.05" customHeight="1">
+    <row r="24" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14">
         <v>22</v>
       </c>
@@ -23726,7 +23726,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.05" customHeight="1">
+    <row r="25" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14">
         <v>23</v>
       </c>
@@ -23812,7 +23812,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.05" customHeight="1">
+    <row r="26" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14">
         <v>24</v>
       </c>
@@ -23898,7 +23898,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="90">
         <v>10</v>
       </c>
@@ -23984,7 +23984,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.05" customHeight="1">
+    <row r="28" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="20" t="s">
         <v>27</v>
       </c>
@@ -24085,7 +24085,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" style="3" customWidth="1"/>
@@ -24117,7 +24117,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>332</v>
       </c>
@@ -24203,7 +24203,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -24289,7 +24289,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -24375,7 +24375,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -24461,7 +24461,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -24547,7 +24547,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -24719,7 +24719,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:28">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="F14" s="3" t="s">
         <v>395</v>
       </c>
@@ -24739,7 +24739,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -24770,7 +24770,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>329</v>
       </c>
@@ -24856,7 +24856,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -24942,7 +24942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="81">
         <v>1</v>
       </c>
@@ -25028,7 +25028,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="81">
         <v>2</v>
       </c>
@@ -25114,7 +25114,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37" t="s">
         <v>27</v>
       </c>
@@ -25200,8 +25200,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
-    <row r="8" spans="1:28">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="D8" s="160"/>
     </row>
   </sheetData>
@@ -25216,7 +25216,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E182FEA0-9E29-45AE-8927-1BAD28B275F4}">
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -25247,7 +25247,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>758</v>
       </c>
@@ -25333,7 +25333,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -25419,7 +25419,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -25505,7 +25505,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -25591,7 +25591,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -25677,7 +25677,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -25763,7 +25763,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -25849,7 +25849,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="116">
         <v>6</v>
       </c>
@@ -25935,7 +25935,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="116">
         <v>7</v>
       </c>
@@ -26021,7 +26021,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="116">
         <v>8</v>
       </c>
@@ -26107,7 +26107,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="116">
         <v>9</v>
       </c>
@@ -26193,7 +26193,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="116">
         <v>10</v>
       </c>
@@ -26279,7 +26279,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="110" t="s">
         <v>27</v>
       </c>
@@ -26379,7 +26379,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
@@ -26409,7 +26409,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>324</v>
       </c>
@@ -26495,7 +26495,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -26581,7 +26581,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -26667,7 +26667,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="34">
         <v>2</v>
       </c>
@@ -26753,7 +26753,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -26839,7 +26839,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34">
         <v>4</v>
       </c>
@@ -26925,7 +26925,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34">
         <v>5</v>
       </c>
@@ -27011,7 +27011,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="34">
         <v>6</v>
       </c>
@@ -27097,7 +27097,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="28" t="s">
         <v>27</v>
       </c>
@@ -27198,7 +27198,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -27229,7 +27229,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>281</v>
       </c>
@@ -27315,7 +27315,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1">
+    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -27401,7 +27401,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -27487,7 +27487,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -27573,7 +27573,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -27659,7 +27659,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -27745,7 +27745,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -27846,7 +27846,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB27"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -27877,7 +27877,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>258</v>
       </c>
@@ -27963,7 +27963,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -28049,7 +28049,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -28135,7 +28135,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -28221,7 +28221,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -28307,7 +28307,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -28393,7 +28393,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -28479,7 +28479,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -28565,7 +28565,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -28651,7 +28651,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -28737,7 +28737,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -28823,7 +28823,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -28909,7 +28909,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -28995,7 +28995,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -29079,7 +29079,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -29165,7 +29165,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -29251,7 +29251,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -29337,7 +29337,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -29423,7 +29423,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>27</v>
       </c>
@@ -29509,7 +29509,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:28">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
       <c r="K27" s="1" t="s">
         <v>259</v>
       </c>
@@ -29529,7 +29529,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB18"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -29561,7 +29561,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>240</v>
       </c>
@@ -29647,7 +29647,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -29733,7 +29733,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -29819,7 +29819,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -29905,7 +29905,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -29989,7 +29989,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -30075,7 +30075,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -30159,7 +30159,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -30239,7 +30239,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -30319,7 +30319,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -30399,7 +30399,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -30479,7 +30479,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -30565,7 +30565,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -30651,7 +30651,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -30737,7 +30737,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -30823,7 +30823,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -30909,7 +30909,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -30995,7 +30995,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>27</v>
       </c>
@@ -31096,7 +31096,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -31126,7 +31126,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>202</v>
       </c>
@@ -31212,7 +31212,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -31298,7 +31298,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21">
         <v>1</v>
       </c>
@@ -31384,7 +31384,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="185">
         <v>1</v>
       </c>
@@ -31470,7 +31470,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21">
         <v>2</v>
       </c>
@@ -31556,7 +31556,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21">
         <v>3</v>
       </c>
@@ -31642,7 +31642,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -31728,7 +31728,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -31829,7 +31829,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -31859,7 +31859,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>192</v>
       </c>
@@ -31945,7 +31945,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -32031,7 +32031,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -32117,7 +32117,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -32203,7 +32203,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -32289,7 +32289,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -32375,7 +32375,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -32461,7 +32461,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -32547,7 +32547,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -32633,7 +32633,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -32719,7 +32719,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -32805,7 +32805,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -32906,7 +32906,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" style="3" hidden="1" customWidth="1"/>
@@ -32938,7 +32938,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="226" t="s">
         <v>155</v>
       </c>
@@ -33024,7 +33024,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -33110,7 +33110,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="47">
         <v>1</v>
       </c>
@@ -33196,7 +33196,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="47">
         <v>2</v>
       </c>
@@ -33282,7 +33282,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="47">
         <v>3</v>
       </c>
@@ -33368,7 +33368,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -33454,7 +33454,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>1</v>
       </c>
@@ -33540,7 +33540,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21">
         <v>2</v>
       </c>
@@ -33626,7 +33626,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>5</v>
       </c>
@@ -33712,7 +33712,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="47">
         <v>6</v>
       </c>
@@ -33798,7 +33798,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>7</v>
       </c>
@@ -33884,7 +33884,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="47">
         <v>8</v>
       </c>
@@ -33970,7 +33970,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="47">
         <v>9</v>
       </c>
@@ -34056,7 +34056,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="46" t="s">
         <v>27</v>
       </c>
@@ -34157,7 +34157,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="1" hidden="1" customWidth="1"/>
@@ -34189,7 +34189,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>79</v>
       </c>
@@ -34275,7 +34275,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="63.6" customHeight="1">
+    <row r="2" spans="1:28" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -34361,7 +34361,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="53">
         <v>1</v>
       </c>
@@ -34447,7 +34447,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="53">
         <v>2</v>
       </c>
@@ -34533,7 +34533,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="53">
         <v>4</v>
       </c>
@@ -34619,7 +34619,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="53">
         <v>5</v>
       </c>
@@ -34705,7 +34705,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="53">
         <v>6</v>
       </c>
@@ -34791,7 +34791,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="53">
         <v>7</v>
       </c>
@@ -34877,7 +34877,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="53">
         <v>8</v>
       </c>
@@ -34963,7 +34963,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="53">
         <v>9</v>
       </c>
@@ -35049,7 +35049,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="53">
         <v>3</v>
       </c>
@@ -35129,7 +35129,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="53">
         <v>10</v>
       </c>
@@ -35215,7 +35215,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53">
         <v>11</v>
       </c>
@@ -35301,7 +35301,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -35347,7 +35347,7 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -35379,7 +35379,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="21" customHeight="1">
+    <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>134</v>
       </c>
@@ -35465,7 +35465,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="48" customHeight="1">
+    <row r="2" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -35551,7 +35551,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -35637,7 +35637,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>27</v>
       </c>
@@ -35738,7 +35738,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -35770,7 +35770,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="227" t="s">
         <v>109</v>
       </c>
@@ -35856,7 +35856,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -35942,7 +35942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -36028,7 +36028,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -36114,7 +36114,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -36200,7 +36200,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -36286,7 +36286,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -36372,7 +36372,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -36458,7 +36458,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -36544,7 +36544,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -36630,7 +36630,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -36716,7 +36716,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -36802,7 +36802,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -36888,7 +36888,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
@@ -36989,7 +36989,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -37021,7 +37021,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>723</v>
       </c>
@@ -37107,7 +37107,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1">
+    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -37193,7 +37193,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -37279,7 +37279,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -37365,7 +37365,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -37451,7 +37451,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="185">
         <v>5</v>
       </c>
@@ -37537,7 +37537,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -37635,7 +37635,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5AF4CA-00D7-4A30-8F64-AC13CDBB2809}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -37667,7 +37667,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>710</v>
       </c>
@@ -37753,7 +37753,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54" customHeight="1">
+    <row r="2" spans="1:28" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -37839,7 +37839,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -37925,7 +37925,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -38011,7 +38011,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -38097,7 +38097,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -38183,7 +38183,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -38280,7 +38280,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15B73F0-D53E-458D-8A18-622E142F07EE}">
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -38312,7 +38312,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>702</v>
       </c>
@@ -38398,7 +38398,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="42.6" customHeight="1">
+    <row r="2" spans="1:28" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -38484,7 +38484,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -38570,7 +38570,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="200">
         <v>2</v>
       </c>
@@ -38656,7 +38656,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="200">
         <v>3</v>
       </c>
@@ -38742,7 +38742,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="200">
         <v>4</v>
       </c>
@@ -38828,7 +38828,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -38914,7 +38914,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -39000,7 +39000,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -39086,7 +39086,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -39172,7 +39172,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -39258,7 +39258,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -39344,7 +39344,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -39430,7 +39430,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -39516,7 +39516,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -39602,7 +39602,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -39688,7 +39688,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -39774,7 +39774,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -39860,7 +39860,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -39946,7 +39946,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>27</v>
       </c>
@@ -40044,7 +40044,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C03CE4-617A-4EF9-89C8-ADAA1610BB0C}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -40074,7 +40074,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>681</v>
       </c>
@@ -40160,7 +40160,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="60.6" customHeight="1">
+    <row r="2" spans="1:28" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -40246,7 +40246,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="19.2" customHeight="1">
+    <row r="3" spans="1:28" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -40332,7 +40332,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="110" t="s">
         <v>27</v>
       </c>
@@ -40429,7 +40429,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41716D2-EB8A-4484-83AF-D7868E55628C}">
   <dimension ref="A1:AB17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -40459,93 +40459,93 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
-      <c r="A1" s="218" t="s">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="221" t="s">
         <v>669</v>
       </c>
-      <c r="B1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="218" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+      <c r="B1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="221" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -40631,7 +40631,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -40717,7 +40717,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -40801,7 +40801,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -40881,7 +40881,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -40961,7 +40961,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="161">
         <v>5</v>
       </c>
@@ -41041,7 +41041,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="161">
         <v>6</v>
       </c>
@@ -41121,7 +41121,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="161">
         <v>7</v>
       </c>
@@ -41201,7 +41201,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="161">
         <v>8</v>
       </c>
@@ -41281,7 +41281,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="161">
         <v>9</v>
       </c>
@@ -41361,7 +41361,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="161">
         <v>10</v>
       </c>
@@ -41441,7 +41441,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="161">
         <v>11</v>
       </c>
@@ -41521,7 +41521,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="161">
         <v>12</v>
       </c>
@@ -41601,7 +41601,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="161">
         <v>13</v>
       </c>
@@ -41681,7 +41681,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="161">
         <v>14</v>
       </c>
@@ -41761,7 +41761,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="168" t="s">
         <v>27</v>
       </c>
@@ -41854,13 +41854,14 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BFDD7F-F2DE-484D-858D-A0AEE46D68A8}">
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.88671875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -41891,7 +41892,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>665</v>
       </c>
@@ -41977,7 +41978,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1">
+    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -42063,7 +42064,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="184" customFormat="1">
+    <row r="3" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="178">
         <v>1</v>
       </c>
@@ -42149,7 +42150,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="184" customFormat="1">
+    <row r="4" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="178">
         <v>2</v>
       </c>
@@ -42235,7 +42236,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="184" customFormat="1">
+    <row r="5" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="178">
         <v>3</v>
       </c>
@@ -42321,7 +42322,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="184" customFormat="1">
+    <row r="6" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="178">
         <v>4</v>
       </c>
@@ -42407,7 +42408,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="184" customFormat="1">
+    <row r="7" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="178">
         <v>5</v>
       </c>
@@ -42493,7 +42494,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="184" customFormat="1">
+    <row r="8" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="178">
         <v>6</v>
       </c>
@@ -42579,7 +42580,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="184" customFormat="1">
+    <row r="9" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="178">
         <v>7</v>
       </c>
@@ -42665,7 +42666,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="184" customFormat="1">
+    <row r="10" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="178">
         <v>8</v>
       </c>
@@ -42751,7 +42752,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="184" customFormat="1">
+    <row r="11" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="178">
         <v>9</v>
       </c>
@@ -42837,7 +42838,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="168" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (17/09/2026 17:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22AD3A92-004C-4894-9B78-E13B00D1E951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC89F820-FBF7-41E8-8495-5B7388F390DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1213" sheetId="159" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (18/09/2026 09:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC89F820-FBF7-41E8-8495-5B7388F390DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC6427C-5D44-4843-BB0B-65635E67B5C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1213" sheetId="159" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7375" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7382" uniqueCount="790">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2454,7 +2454,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2674,7 +2674,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="228">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3325,6 +3325,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3549,7 +3552,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCDEA62-D4C1-4F97-B5A0-F9D378B5F3A6}">
   <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5546875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -3581,7 +3584,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>789</v>
       </c>
@@ -3667,7 +3670,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="52.8" customHeight="1">
+    <row r="2" spans="1:28" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -3753,7 +3756,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1">
+    <row r="3" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -3839,7 +3842,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1">
+    <row r="4" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -3925,7 +3928,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1">
+    <row r="5" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="150">
         <v>3</v>
       </c>
@@ -4011,7 +4014,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1">
+    <row r="6" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="157" t="s">
         <v>27</v>
       </c>
@@ -4108,7 +4111,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BFDD7F-F2DE-484D-858D-A0AEE46D68A8}">
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.88671875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -4139,7 +4142,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>665</v>
       </c>
@@ -4225,7 +4228,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1">
+    <row r="2" spans="1:28" s="167" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -4311,7 +4314,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="184" customFormat="1">
+    <row r="3" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="178">
         <v>1</v>
       </c>
@@ -4397,7 +4400,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="184" customFormat="1">
+    <row r="4" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="178">
         <v>2</v>
       </c>
@@ -4483,7 +4486,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="184" customFormat="1">
+    <row r="5" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="178">
         <v>3</v>
       </c>
@@ -4569,7 +4572,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="184" customFormat="1">
+    <row r="6" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="178">
         <v>4</v>
       </c>
@@ -4655,7 +4658,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="184" customFormat="1">
+    <row r="7" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="178">
         <v>5</v>
       </c>
@@ -4741,7 +4744,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="184" customFormat="1">
+    <row r="8" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="178">
         <v>6</v>
       </c>
@@ -4827,7 +4830,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="184" customFormat="1">
+    <row r="9" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="178">
         <v>7</v>
       </c>
@@ -4913,7 +4916,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="184" customFormat="1">
+    <row r="10" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="178">
         <v>8</v>
       </c>
@@ -4999,7 +5002,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="184" customFormat="1">
+    <row r="11" spans="1:28" s="184" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="178">
         <v>9</v>
       </c>
@@ -5085,7 +5088,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="168" t="s">
         <v>27</v>
       </c>
@@ -5185,7 +5188,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB29"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -5216,7 +5219,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>652</v>
       </c>
@@ -5302,7 +5305,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -5388,7 +5391,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -5474,7 +5477,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -5560,7 +5563,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="150">
         <v>3</v>
       </c>
@@ -5646,7 +5649,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="150">
         <v>4</v>
       </c>
@@ -5732,7 +5735,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="150">
         <v>5</v>
       </c>
@@ -5818,7 +5821,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -5904,7 +5907,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -5990,7 +5993,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -6076,7 +6079,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -6162,7 +6165,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -6248,7 +6251,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -6334,7 +6337,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -6420,7 +6423,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="150">
         <v>13</v>
       </c>
@@ -6506,7 +6509,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="150">
         <v>14</v>
       </c>
@@ -6592,7 +6595,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="150">
         <v>15</v>
       </c>
@@ -6678,7 +6681,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="150">
         <v>16</v>
       </c>
@@ -6764,7 +6767,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="150">
         <v>17</v>
       </c>
@@ -6850,7 +6853,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="150">
         <v>18</v>
       </c>
@@ -6936,7 +6939,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="21" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="150">
         <v>19</v>
       </c>
@@ -7022,7 +7025,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="22" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="150">
         <v>20</v>
       </c>
@@ -7102,7 +7105,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="23" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="150">
         <v>21</v>
       </c>
@@ -7188,7 +7191,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="24" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="150">
         <v>22</v>
       </c>
@@ -7274,7 +7277,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="25" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="150">
         <v>23</v>
       </c>
@@ -7360,7 +7363,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="26" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="150">
         <v>24</v>
       </c>
@@ -7446,7 +7449,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="27" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="150">
         <v>25</v>
       </c>
@@ -7532,7 +7535,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="28" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="157" t="s">
         <v>27</v>
       </c>
@@ -7618,7 +7621,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:28">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B29" s="206"/>
     </row>
   </sheetData>
@@ -7636,7 +7639,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -7667,7 +7670,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>618</v>
       </c>
@@ -7753,7 +7756,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -7839,7 +7842,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -7925,7 +7928,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -8011,7 +8014,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -8097,7 +8100,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -8183,7 +8186,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="168" t="s">
         <v>27</v>
       </c>
@@ -8284,7 +8287,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.21875" style="108" customWidth="1"/>
     <col min="2" max="2" width="15.109375" style="108" customWidth="1"/>
@@ -8316,7 +8319,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>606</v>
       </c>
@@ -8402,7 +8405,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -8488,7 +8491,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="170">
         <v>1</v>
       </c>
@@ -8574,7 +8577,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="170">
         <v>2</v>
       </c>
@@ -8660,7 +8663,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="170">
         <v>3</v>
       </c>
@@ -8746,7 +8749,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="170">
         <v>4</v>
       </c>
@@ -8832,7 +8835,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="170">
         <v>5</v>
       </c>
@@ -8918,7 +8921,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="170">
         <v>6</v>
       </c>
@@ -9004,7 +9007,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="170">
         <v>7</v>
       </c>
@@ -9090,7 +9093,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="170">
         <v>8</v>
       </c>
@@ -9176,7 +9179,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="157" t="s">
         <v>27</v>
       </c>
@@ -9277,7 +9280,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.5546875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -9307,7 +9310,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>599</v>
       </c>
@@ -9393,7 +9396,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -9479,7 +9482,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="150">
         <v>1</v>
       </c>
@@ -9565,7 +9568,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -9651,7 +9654,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="150">
         <v>3</v>
       </c>
@@ -9731,7 +9734,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="157" t="s">
         <v>27</v>
       </c>
@@ -9819,7 +9822,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:28">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="D8" s="158"/>
       <c r="J8" s="159"/>
       <c r="L8" s="159"/>
@@ -9839,7 +9842,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -9867,7 +9870,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>592</v>
       </c>
@@ -9953,7 +9956,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1">
+    <row r="2" spans="1:28" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -10039,7 +10042,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -10125,7 +10128,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -10211,7 +10214,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -10297,7 +10300,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -10377,7 +10380,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -10457,7 +10460,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -10543,7 +10546,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -10629,7 +10632,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -10715,7 +10718,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -10801,7 +10804,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -10902,7 +10905,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -10933,7 +10936,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="222" t="s">
         <v>554</v>
       </c>
@@ -11019,7 +11022,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -11105,7 +11108,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="193">
         <v>1</v>
       </c>
@@ -11191,7 +11194,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="150">
         <v>2</v>
       </c>
@@ -11277,7 +11280,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="193">
         <v>3</v>
       </c>
@@ -11363,7 +11366,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="193">
         <v>4</v>
       </c>
@@ -11449,7 +11452,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="192" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="193">
         <v>5</v>
       </c>
@@ -11535,7 +11538,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="150">
         <v>6</v>
       </c>
@@ -11621,7 +11624,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="150">
         <v>7</v>
       </c>
@@ -11707,7 +11710,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="150">
         <v>8</v>
       </c>
@@ -11793,7 +11796,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="150">
         <v>9</v>
       </c>
@@ -11879,7 +11882,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="150">
         <v>10</v>
       </c>
@@ -11965,7 +11968,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="150">
         <v>11</v>
       </c>
@@ -12051,7 +12054,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="150">
         <v>12</v>
       </c>
@@ -12137,7 +12140,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="157" t="s">
         <v>27</v>
       </c>
@@ -12238,7 +12241,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -12270,7 +12273,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>539</v>
       </c>
@@ -12356,7 +12359,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -12442,7 +12445,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="126">
         <v>1</v>
       </c>
@@ -12528,7 +12531,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -12614,7 +12617,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="132" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="126">
         <v>2</v>
       </c>
@@ -12700,7 +12703,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>3</v>
       </c>
@@ -12786,7 +12789,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -12872,7 +12875,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -12958,7 +12961,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -13044,7 +13047,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="10" spans="1:28">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>27</v>
       </c>
@@ -13142,7 +13145,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
   <dimension ref="A1:AB5"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13174,7 +13177,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>535</v>
       </c>
@@ -13260,7 +13263,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13346,7 +13349,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -13432,7 +13435,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -13518,7 +13521,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
         <v>27</v>
       </c>
@@ -13618,7 +13621,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13650,7 +13653,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="223" t="s">
         <v>523</v>
       </c>
@@ -13736,7 +13739,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="43.2" customHeight="1">
+    <row r="2" spans="1:28" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="107" t="s">
         <v>0</v>
       </c>
@@ -13822,7 +13825,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="90">
         <v>1</v>
       </c>
@@ -13908,7 +13911,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="90">
         <v>2</v>
       </c>
@@ -13994,7 +13997,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="90">
         <v>3</v>
       </c>
@@ -14080,7 +14083,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="90">
         <v>4</v>
       </c>
@@ -14166,7 +14169,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="106" t="s">
         <v>27</v>
       </c>
@@ -14263,8 +14266,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00EADB3A-C171-49AE-8471-729057A3A740}">
-  <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:AB9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -14296,7 +14299,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>781</v>
       </c>
@@ -14382,7 +14385,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="61.2" customHeight="1">
+    <row r="2" spans="1:28" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -14468,7 +14471,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -14554,7 +14557,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -14640,7 +14643,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -14726,7 +14729,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -14812,7 +14815,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -14898,89 +14901,169 @@
         <v>770</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="110">
-        <v>11000</v>
-      </c>
-      <c r="I8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="N8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="O8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="109">
-        <v>4902.7</v>
-      </c>
-      <c r="Q8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="R8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="T8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="V8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="W8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="X8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB8" s="109" t="s">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="116"/>
+      <c r="B8" s="118" t="s">
+        <v>444</v>
+      </c>
+      <c r="C8" s="116" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="228">
+        <v>46282</v>
+      </c>
+      <c r="E8" s="116"/>
+      <c r="F8" s="116">
+        <v>262643</v>
+      </c>
+      <c r="G8" s="116">
+        <v>1748</v>
+      </c>
+      <c r="H8" s="116">
+        <v>600</v>
+      </c>
+      <c r="I8" s="117">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="J8" s="117">
+        <v>1.536</v>
+      </c>
+      <c r="K8" s="116" t="s">
+        <v>587</v>
+      </c>
+      <c r="L8" s="113">
+        <v>874.59799999999996</v>
+      </c>
+      <c r="M8" s="115">
+        <v>921.6</v>
+      </c>
+      <c r="N8" s="112">
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="O8" s="114">
+        <v>15.36</v>
+      </c>
+      <c r="P8" s="111">
+        <v>275.5</v>
+      </c>
+      <c r="Q8" s="111">
+        <v>1</v>
+      </c>
+      <c r="R8" s="111">
+        <v>1000</v>
+      </c>
+      <c r="S8" s="113">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="T8" s="111">
+        <v>51</v>
+      </c>
+      <c r="U8" s="112">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="V8" s="111" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="111" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="111" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="111"/>
+      <c r="Z8" s="111"/>
+      <c r="AA8" s="111">
+        <v>2</v>
+      </c>
+      <c r="AB8" s="111" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="110">
+        <f>SUM(H3:H8)</f>
+        <v>11600</v>
+      </c>
+      <c r="I9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="P9" s="109">
+        <f>SUM(P3:P8)</f>
+        <v>5178.1999999999989</v>
+      </c>
+      <c r="Q9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="R9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="S9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="T9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="U9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="V9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="W9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="X9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB9" s="109" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14998,7 +15081,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" style="3" hidden="1" customWidth="1"/>
@@ -15030,7 +15113,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>512</v>
       </c>
@@ -15116,7 +15199,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -15202,7 +15285,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" customFormat="1">
+    <row r="3" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="120">
         <v>1</v>
       </c>
@@ -15288,7 +15371,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="4" spans="1:28" customFormat="1">
+    <row r="4" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="120">
         <v>2</v>
       </c>
@@ -15374,7 +15457,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:28" customFormat="1">
+    <row r="5" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="120">
         <v>3</v>
       </c>
@@ -15460,7 +15543,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="6" spans="1:28" customFormat="1">
+    <row r="6" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -15546,7 +15629,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="7" spans="1:28" customFormat="1">
+    <row r="7" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="120">
         <v>5</v>
       </c>
@@ -15632,7 +15715,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="8" spans="1:28" customFormat="1">
+    <row r="8" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="47">
         <v>6</v>
       </c>
@@ -15718,7 +15801,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="9" spans="1:28" customFormat="1">
+    <row r="9" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>7</v>
       </c>
@@ -15804,7 +15887,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="10" spans="1:28" customFormat="1">
+    <row r="10" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="120">
         <v>8</v>
       </c>
@@ -15890,7 +15973,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>9</v>
       </c>
@@ -15976,7 +16059,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="45" customFormat="1">
+    <row r="12" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="46" t="s">
         <v>27</v>
       </c>
@@ -16074,7 +16157,7 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -16105,7 +16188,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>531</v>
       </c>
@@ -16191,7 +16274,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39" customHeight="1">
+    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -16277,7 +16360,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -16363,7 +16446,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -16449,7 +16532,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -16535,7 +16618,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -16621,7 +16704,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -16707,7 +16790,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="110" t="s">
         <v>27</v>
       </c>
@@ -16808,7 +16891,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -16840,7 +16923,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>496</v>
       </c>
@@ -16926,7 +17009,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -17012,7 +17095,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="133">
         <v>1</v>
       </c>
@@ -17098,7 +17181,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="133">
         <v>2</v>
       </c>
@@ -17182,7 +17265,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="133">
         <v>3</v>
       </c>
@@ -17268,7 +17351,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="207">
         <v>4</v>
       </c>
@@ -17352,7 +17435,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="214" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="207">
         <v>5</v>
       </c>
@@ -17436,7 +17519,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="133">
         <v>6</v>
       </c>
@@ -17522,7 +17605,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="207">
         <v>7</v>
       </c>
@@ -17606,7 +17689,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="133">
         <v>8</v>
       </c>
@@ -17692,7 +17775,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="207">
         <v>9</v>
       </c>
@@ -17776,7 +17859,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="133">
         <v>10</v>
       </c>
@@ -17862,7 +17945,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="133">
         <v>11</v>
       </c>
@@ -17948,7 +18031,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="133">
         <v>12</v>
       </c>
@@ -18034,7 +18117,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="133">
         <v>13</v>
       </c>
@@ -18120,7 +18203,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="133">
         <v>14</v>
       </c>
@@ -18206,7 +18289,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>27</v>
       </c>
@@ -18309,7 +18392,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -18339,7 +18422,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>486</v>
       </c>
@@ -18425,7 +18508,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -18511,7 +18594,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -18597,7 +18680,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="139">
         <v>2</v>
       </c>
@@ -18683,7 +18766,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="139"/>
       <c r="B5" s="140" t="s">
         <v>480</v>
@@ -18761,7 +18844,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="104" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="139"/>
       <c r="B6" s="140" t="s">
         <v>480</v>
@@ -18839,7 +18922,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34">
         <v>3</v>
       </c>
@@ -18925,7 +19008,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="28" t="s">
         <v>27</v>
       </c>
@@ -19028,7 +19111,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -19058,7 +19141,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>475</v>
       </c>
@@ -19144,7 +19227,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -19230,7 +19313,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="97">
         <v>1</v>
       </c>
@@ -19316,7 +19399,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="97">
         <v>2</v>
       </c>
@@ -19402,7 +19485,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="97">
         <v>3</v>
       </c>
@@ -19488,7 +19571,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="97">
         <v>4</v>
       </c>
@@ -19574,7 +19657,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="97">
         <v>5</v>
       </c>
@@ -19660,7 +19743,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="97">
         <v>6</v>
       </c>
@@ -19746,7 +19829,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="97">
         <v>7</v>
       </c>
@@ -19832,7 +19915,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="97">
         <v>8</v>
       </c>
@@ -19918,7 +20001,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="97">
         <v>9</v>
       </c>
@@ -20004,7 +20087,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="97">
         <v>10</v>
       </c>
@@ -20090,7 +20173,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>27</v>
       </c>
@@ -20191,7 +20274,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -20223,7 +20306,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>454</v>
       </c>
@@ -20309,7 +20392,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="50.4" customHeight="1">
+    <row r="2" spans="1:28" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20395,7 +20478,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -20481,7 +20564,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -20567,7 +20650,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -20653,7 +20736,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -20739,7 +20822,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -20825,7 +20908,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -20926,7 +21009,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -20958,7 +21041,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="33" customHeight="1">
+    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>440</v>
       </c>
@@ -21044,7 +21127,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -21130,7 +21213,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -21216,7 +21299,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -21302,7 +21385,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -21388,7 +21471,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -21474,7 +21557,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -21560,7 +21643,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -21646,7 +21729,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -21732,7 +21815,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
@@ -21833,7 +21916,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -21864,7 +21947,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>403</v>
       </c>
@@ -21950,7 +22033,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1">
+    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -22036,7 +22119,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -22122,7 +22205,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -22206,7 +22289,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -22292,7 +22375,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -22378,7 +22461,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -22462,7 +22545,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -22546,7 +22629,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
@@ -22647,7 +22730,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" customWidth="1"/>
@@ -22677,7 +22760,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="225" t="s">
         <v>380</v>
       </c>
@@ -22763,7 +22846,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="89" t="s">
         <v>0</v>
       </c>
@@ -22849,7 +22932,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14">
         <v>1</v>
       </c>
@@ -22935,7 +23018,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14">
         <v>2</v>
       </c>
@@ -23021,7 +23104,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14">
         <v>3</v>
       </c>
@@ -23107,7 +23190,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14">
         <v>4</v>
       </c>
@@ -23193,7 +23276,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>5</v>
       </c>
@@ -23279,7 +23362,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>6</v>
       </c>
@@ -23365,7 +23448,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>7</v>
       </c>
@@ -23451,7 +23534,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>8</v>
       </c>
@@ -23537,7 +23620,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>9</v>
       </c>
@@ -23623,7 +23706,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>10</v>
       </c>
@@ -23709,7 +23792,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>11</v>
       </c>
@@ -23795,7 +23878,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
         <v>12</v>
       </c>
@@ -23881,7 +23964,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>13</v>
       </c>
@@ -23967,7 +24050,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
         <v>14</v>
       </c>
@@ -24053,7 +24136,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14">
         <v>15</v>
       </c>
@@ -24139,7 +24222,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14">
         <v>16</v>
       </c>
@@ -24225,7 +24308,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14">
         <v>17</v>
       </c>
@@ -24311,7 +24394,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14">
         <v>18</v>
       </c>
@@ -24397,7 +24480,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="25.05" customHeight="1">
+    <row r="21" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="14">
         <v>19</v>
       </c>
@@ -24483,7 +24566,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.05" customHeight="1">
+    <row r="22" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14">
         <v>20</v>
       </c>
@@ -24569,7 +24652,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.05" customHeight="1">
+    <row r="23" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14">
         <v>21</v>
       </c>
@@ -24655,7 +24738,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.05" customHeight="1">
+    <row r="24" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14">
         <v>22</v>
       </c>
@@ -24741,7 +24824,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.05" customHeight="1">
+    <row r="25" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14">
         <v>23</v>
       </c>
@@ -24827,7 +24910,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.05" customHeight="1">
+    <row r="26" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14">
         <v>24</v>
       </c>
@@ -24913,7 +24996,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="90">
         <v>10</v>
       </c>
@@ -24999,7 +25082,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.05" customHeight="1">
+    <row r="28" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="20" t="s">
         <v>27</v>
       </c>
@@ -25100,7 +25183,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" style="3" customWidth="1"/>
@@ -25132,7 +25215,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>332</v>
       </c>
@@ -25218,7 +25301,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -25304,7 +25387,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -25390,7 +25473,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -25476,7 +25559,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -25562,7 +25645,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -25648,7 +25731,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -25734,7 +25817,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:28">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="F14" s="3" t="s">
         <v>395</v>
       </c>
@@ -25751,7 +25834,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A45B5AC-557E-4203-8DD1-DFBBC7E9A9E0}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.77734375" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -25781,7 +25864,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>768</v>
       </c>
@@ -25867,7 +25950,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -25953,7 +26036,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -26039,7 +26122,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -26125,7 +26208,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -26211,7 +26294,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="6" spans="1:28">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -26297,7 +26380,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:28">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="110" t="s">
         <v>27</v>
       </c>
@@ -26397,7 +26480,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -26428,7 +26511,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>329</v>
       </c>
@@ -26514,7 +26597,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -26600,7 +26683,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="81">
         <v>1</v>
       </c>
@@ -26686,7 +26769,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="81">
         <v>2</v>
       </c>
@@ -26772,7 +26855,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37" t="s">
         <v>27</v>
       </c>
@@ -26858,8 +26941,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
-    <row r="8" spans="1:28">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="D8" s="160"/>
     </row>
   </sheetData>
@@ -26877,7 +26960,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
@@ -26907,7 +26990,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>324</v>
       </c>
@@ -26993,7 +27076,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -27079,7 +27162,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -27165,7 +27248,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="34">
         <v>2</v>
       </c>
@@ -27251,7 +27334,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -27337,7 +27420,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34">
         <v>4</v>
       </c>
@@ -27423,7 +27506,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34">
         <v>5</v>
       </c>
@@ -27509,7 +27592,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="34">
         <v>6</v>
       </c>
@@ -27595,7 +27678,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="28" t="s">
         <v>27</v>
       </c>
@@ -27696,7 +27779,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -27727,7 +27810,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="224" t="s">
         <v>281</v>
       </c>
@@ -27813,7 +27896,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1">
+    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -27899,7 +27982,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -27985,7 +28068,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -28071,7 +28154,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -28157,7 +28240,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -28243,7 +28326,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -28344,7 +28427,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB27"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -28375,7 +28458,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>258</v>
       </c>
@@ -28461,7 +28544,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -28547,7 +28630,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -28633,7 +28716,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -28719,7 +28802,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -28805,7 +28888,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -28891,7 +28974,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -28977,7 +29060,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -29063,7 +29146,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -29149,7 +29232,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -29235,7 +29318,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -29321,7 +29404,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -29407,7 +29490,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -29493,7 +29576,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -29577,7 +29660,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -29663,7 +29746,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -29749,7 +29832,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -29835,7 +29918,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -29921,7 +30004,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>27</v>
       </c>
@@ -30007,7 +30090,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:28">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
       <c r="K27" s="1" t="s">
         <v>259</v>
       </c>
@@ -30027,7 +30110,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB18"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -30059,7 +30142,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>240</v>
       </c>
@@ -30145,7 +30228,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -30231,7 +30314,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -30317,7 +30400,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -30403,7 +30486,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -30487,7 +30570,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -30573,7 +30656,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -30657,7 +30740,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -30737,7 +30820,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -30817,7 +30900,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -30897,7 +30980,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -30977,7 +31060,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -31063,7 +31146,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -31149,7 +31232,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -31235,7 +31318,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -31321,7 +31404,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -31407,7 +31490,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -31493,7 +31576,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>27</v>
       </c>
@@ -31594,7 +31677,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -31624,7 +31707,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>202</v>
       </c>
@@ -31710,7 +31793,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -31796,7 +31879,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21">
         <v>1</v>
       </c>
@@ -31882,7 +31965,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="185">
         <v>1</v>
       </c>
@@ -31968,7 +32051,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21">
         <v>2</v>
       </c>
@@ -32054,7 +32137,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21">
         <v>3</v>
       </c>
@@ -32140,7 +32223,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -32226,7 +32309,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -32327,7 +32410,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -32357,7 +32440,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>192</v>
       </c>
@@ -32443,7 +32526,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -32529,7 +32612,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -32615,7 +32698,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -32701,7 +32784,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -32787,7 +32870,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -32873,7 +32956,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -32959,7 +33042,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -33045,7 +33128,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -33131,7 +33214,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -33217,7 +33300,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -33303,7 +33386,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -33404,7 +33487,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" style="3" hidden="1" customWidth="1"/>
@@ -33436,7 +33519,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="226" t="s">
         <v>155</v>
       </c>
@@ -33522,7 +33605,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -33608,7 +33691,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="47">
         <v>1</v>
       </c>
@@ -33694,7 +33777,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="47">
         <v>2</v>
       </c>
@@ -33780,7 +33863,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="47">
         <v>3</v>
       </c>
@@ -33866,7 +33949,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -33952,7 +34035,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>1</v>
       </c>
@@ -34038,7 +34121,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21">
         <v>2</v>
       </c>
@@ -34124,7 +34207,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>5</v>
       </c>
@@ -34210,7 +34293,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="47">
         <v>6</v>
       </c>
@@ -34296,7 +34379,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>7</v>
       </c>
@@ -34382,7 +34465,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="47">
         <v>8</v>
       </c>
@@ -34468,7 +34551,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="47">
         <v>9</v>
       </c>
@@ -34554,7 +34637,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="46" t="s">
         <v>27</v>
       </c>
@@ -34655,7 +34738,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="1" hidden="1" customWidth="1"/>
@@ -34687,7 +34770,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>79</v>
       </c>
@@ -34773,7 +34856,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="63.6" customHeight="1">
+    <row r="2" spans="1:28" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -34859,7 +34942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="53">
         <v>1</v>
       </c>
@@ -34945,7 +35028,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="53">
         <v>2</v>
       </c>
@@ -35031,7 +35114,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="53">
         <v>4</v>
       </c>
@@ -35117,7 +35200,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="53">
         <v>5</v>
       </c>
@@ -35203,7 +35286,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="53">
         <v>6</v>
       </c>
@@ -35289,7 +35372,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="53">
         <v>7</v>
       </c>
@@ -35375,7 +35458,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="53">
         <v>8</v>
       </c>
@@ -35461,7 +35544,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="53">
         <v>9</v>
       </c>
@@ -35547,7 +35630,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="53">
         <v>3</v>
       </c>
@@ -35627,7 +35710,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="53">
         <v>10</v>
       </c>
@@ -35713,7 +35796,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53">
         <v>11</v>
       </c>
@@ -35799,7 +35882,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -35845,7 +35928,7 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -35877,7 +35960,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="21" customHeight="1">
+    <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>134</v>
       </c>
@@ -35963,7 +36046,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="48" customHeight="1">
+    <row r="2" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -36049,7 +36132,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -36135,7 +36218,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>27</v>
       </c>
@@ -36233,7 +36316,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E182FEA0-9E29-45AE-8927-1BAD28B275F4}">
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -36264,7 +36347,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>758</v>
       </c>
@@ -36350,7 +36433,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -36436,7 +36519,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -36522,7 +36605,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -36608,7 +36691,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -36694,7 +36777,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -36780,7 +36863,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -36866,7 +36949,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="116">
         <v>6</v>
       </c>
@@ -36952,7 +37035,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="116">
         <v>7</v>
       </c>
@@ -37038,7 +37121,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="116">
         <v>8</v>
       </c>
@@ -37124,7 +37207,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="116">
         <v>9</v>
       </c>
@@ -37210,7 +37293,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="116">
         <v>10</v>
       </c>
@@ -37296,7 +37379,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="110" t="s">
         <v>27</v>
       </c>
@@ -37396,7 +37479,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -37428,7 +37511,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="227" t="s">
         <v>109</v>
       </c>
@@ -37514,7 +37597,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -37600,7 +37683,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -37686,7 +37769,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -37772,7 +37855,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -37858,7 +37941,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -37944,7 +38027,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -38030,7 +38113,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -38116,7 +38199,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -38202,7 +38285,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -38288,7 +38371,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -38374,7 +38457,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -38460,7 +38543,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -38546,7 +38629,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
@@ -38647,7 +38730,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -38679,7 +38762,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
         <v>723</v>
       </c>
@@ -38765,7 +38848,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1">
+    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -38851,7 +38934,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -38937,7 +39020,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -39023,7 +39106,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -39109,7 +39192,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="185">
         <v>5</v>
       </c>
@@ -39195,7 +39278,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -39293,7 +39376,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5AF4CA-00D7-4A30-8F64-AC13CDBB2809}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -39325,7 +39408,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>710</v>
       </c>
@@ -39411,7 +39494,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54" customHeight="1">
+    <row r="2" spans="1:28" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -39497,7 +39580,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -39583,7 +39666,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -39669,7 +39752,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -39755,7 +39838,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -39841,7 +39924,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -39938,7 +40021,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15B73F0-D53E-458D-8A18-622E142F07EE}">
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -39970,7 +40053,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
         <v>702</v>
       </c>
@@ -40056,7 +40139,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="42.6" customHeight="1">
+    <row r="2" spans="1:28" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -40142,7 +40225,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -40228,7 +40311,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="200">
         <v>2</v>
       </c>
@@ -40314,7 +40397,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="200">
         <v>3</v>
       </c>
@@ -40400,7 +40483,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="200">
         <v>4</v>
       </c>
@@ -40486,7 +40569,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -40572,7 +40655,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -40658,7 +40741,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -40744,7 +40827,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -40830,7 +40913,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -40916,7 +40999,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -41002,7 +41085,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -41088,7 +41171,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -41174,7 +41257,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -41260,7 +41343,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -41346,7 +41429,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -41432,7 +41515,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -41518,7 +41601,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -41604,7 +41687,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>27</v>
       </c>
@@ -41702,7 +41785,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C03CE4-617A-4EF9-89C8-ADAA1610BB0C}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -41732,7 +41815,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
         <v>681</v>
       </c>
@@ -41818,7 +41901,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="60.6" customHeight="1">
+    <row r="2" spans="1:28" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -41904,7 +41987,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="19.2" customHeight="1">
+    <row r="3" spans="1:28" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -41990,7 +42073,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="110" t="s">
         <v>27</v>
       </c>
@@ -42090,7 +42173,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB17"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
@@ -42120,7 +42203,7 @@
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
         <v>669</v>
       </c>
@@ -42206,7 +42289,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -42292,7 +42375,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="161">
         <v>1</v>
       </c>
@@ -42378,7 +42461,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="161">
         <v>2</v>
       </c>
@@ -42462,7 +42545,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="161">
         <v>3</v>
       </c>
@@ -42542,7 +42625,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="161">
         <v>4</v>
       </c>
@@ -42622,7 +42705,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="161">
         <v>5</v>
       </c>
@@ -42702,7 +42785,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="161">
         <v>6</v>
       </c>
@@ -42782,7 +42865,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="161">
         <v>7</v>
       </c>
@@ -42862,7 +42945,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="161">
         <v>8</v>
       </c>
@@ -42942,7 +43025,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="161">
         <v>9</v>
       </c>
@@ -43022,7 +43105,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="161">
         <v>10</v>
       </c>
@@ -43102,7 +43185,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="161">
         <v>11</v>
       </c>
@@ -43182,7 +43265,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="161">
         <v>12</v>
       </c>
@@ -43262,7 +43345,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="161">
         <v>13</v>
       </c>
@@ -43342,7 +43425,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="161">
         <v>14</v>
       </c>
@@ -43422,7 +43505,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="168" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (18/09/2026 09:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DA1775-30B5-4802-8DD2-D56CF376098F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E780A14A-BCEA-4AF9-ADEE-74A55A9E420C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1213" sheetId="159" r:id="rId1"/>
     <sheet name="IPE - PCBOX 1212" sheetId="158" r:id="rId2"/>
     <sheet name="Z4A EMBALAGENS LTDA 1210" sheetId="157" r:id="rId3"/>
-    <sheet name="RM Embalagens 1209" sheetId="156" r:id="rId4"/>
+    <sheet name="RM Embalagens 1209 P" sheetId="156" r:id="rId4"/>
     <sheet name="IPE - PC BOX 1203P" sheetId="154" r:id="rId5"/>
     <sheet name="ABAPEL 1201" sheetId="153" r:id="rId6"/>
     <sheet name="HARMONY EMBALAGENS 1200" sheetId="152" r:id="rId7"/>
@@ -36348,88 +36348,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="218" t="s">
+      <c r="A1" s="221" t="s">
         <v>758</v>
       </c>
-      <c r="B1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="218" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="218" t="s">
+      <c r="B1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="221" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="221" t="s">
         <v>27</v>
       </c>
     </row>
@@ -37470,6 +37470,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (18/09/2026 09:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E780A14A-BCEA-4AF9-ADEE-74A55A9E420C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C3E448-47D2-4F68-A050-978EEBF9E2E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2295,9 +2295,6 @@
     <t>1115x2100</t>
   </si>
   <si>
-    <t>RM Embalagens (Daiane Marques Canossa ME)</t>
-  </si>
-  <si>
     <t>990x1440</t>
   </si>
   <si>
@@ -2349,9 +2346,6 @@
     <t>166x347x166</t>
   </si>
   <si>
-    <t>PROGRAMAÇÃO ONDULADEIRA - RM Embalagens (Daiane Marques Canossa ME)  —  OF: 001209</t>
-  </si>
-  <si>
     <t>2095</t>
   </si>
   <si>
@@ -2443,6 +2437,12 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - ABAPEL COMERCIO DE EMBALAGENS LTDA  —  OF: 001213</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - RM Embalagens   —  OF: 001209</t>
+  </si>
+  <si>
+    <t>RM Embalagens</t>
   </si>
 </sst>
 </file>
@@ -3586,7 +3586,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="B1" s="218" t="s">
         <v>27</v>
@@ -3767,7 +3767,7 @@
         <v>65</v>
       </c>
       <c r="D3" s="150" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E3" s="150" t="s">
         <v>27</v>
@@ -3776,7 +3776,7 @@
         <v>262640</v>
       </c>
       <c r="G3" s="150" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="H3" s="150">
         <v>800</v>
@@ -3788,7 +3788,7 @@
         <v>1.6739999999999999</v>
       </c>
       <c r="K3" s="150" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="L3" s="152">
         <v>980.29399999999998</v>
@@ -3839,7 +3839,7 @@
         <v>30</v>
       </c>
       <c r="AB3" s="150" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
@@ -3853,7 +3853,7 @@
         <v>65</v>
       </c>
       <c r="D4" s="150" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E4" s="150" t="s">
         <v>27</v>
@@ -3862,7 +3862,7 @@
         <v>262641</v>
       </c>
       <c r="G4" s="150" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="H4" s="150">
         <v>1150</v>
@@ -3874,7 +3874,7 @@
         <v>1.44</v>
       </c>
       <c r="K4" s="150" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="L4" s="152">
         <v>905.83199999999999</v>
@@ -3925,7 +3925,7 @@
         <v>33</v>
       </c>
       <c r="AB4" s="150" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
@@ -3939,7 +3939,7 @@
         <v>36</v>
       </c>
       <c r="D5" s="150" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E5" s="150" t="s">
         <v>27</v>
@@ -3948,7 +3948,7 @@
         <v>262642</v>
       </c>
       <c r="G5" s="150" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="H5" s="150">
         <v>1000</v>
@@ -3960,7 +3960,7 @@
         <v>1.58</v>
       </c>
       <c r="K5" s="150" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="L5" s="152">
         <v>917.98</v>
@@ -4011,7 +4011,7 @@
         <v>33</v>
       </c>
       <c r="AB5" s="150" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
@@ -14301,7 +14301,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="B1" s="218" t="s">
         <v>27</v>
@@ -14482,7 +14482,7 @@
         <v>45</v>
       </c>
       <c r="D3" s="116" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E3" s="116" t="s">
         <v>27</v>
@@ -14491,7 +14491,7 @@
         <v>262639</v>
       </c>
       <c r="G3" s="116" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="H3" s="116">
         <v>300</v>
@@ -14503,7 +14503,7 @@
         <v>1.5229999999999999</v>
       </c>
       <c r="K3" s="116" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="L3" s="113">
         <v>307.95100000000002</v>
@@ -14554,7 +14554,7 @@
         <v>33</v>
       </c>
       <c r="AB3" s="111" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14568,7 +14568,7 @@
         <v>45</v>
       </c>
       <c r="D4" s="116" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E4" s="116" t="s">
         <v>27</v>
@@ -14577,7 +14577,7 @@
         <v>262637</v>
       </c>
       <c r="G4" s="116" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="H4" s="116">
         <v>500</v>
@@ -14589,7 +14589,7 @@
         <v>1.4630000000000001</v>
       </c>
       <c r="K4" s="116" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="L4" s="113">
         <v>414.029</v>
@@ -14640,7 +14640,7 @@
         <v>33</v>
       </c>
       <c r="AB4" s="111" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14654,7 +14654,7 @@
         <v>45</v>
       </c>
       <c r="D5" s="116" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E5" s="116" t="s">
         <v>27</v>
@@ -14663,7 +14663,7 @@
         <v>262635</v>
       </c>
       <c r="G5" s="116" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="H5" s="116">
         <v>5000</v>
@@ -14740,7 +14740,7 @@
         <v>45</v>
       </c>
       <c r="D6" s="116" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E6" s="116" t="s">
         <v>27</v>
@@ -14749,7 +14749,7 @@
         <v>262636</v>
       </c>
       <c r="G6" s="116" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="H6" s="116">
         <v>5000</v>
@@ -14826,7 +14826,7 @@
         <v>26</v>
       </c>
       <c r="D7" s="116" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="E7" s="116" t="s">
         <v>27</v>
@@ -14835,7 +14835,7 @@
         <v>262638</v>
       </c>
       <c r="G7" s="116" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="H7" s="116">
         <v>200</v>
@@ -14847,7 +14847,7 @@
         <v>1.423</v>
       </c>
       <c r="K7" s="116" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="L7" s="113">
         <v>153.11500000000001</v>
@@ -14898,7 +14898,7 @@
         <v>39</v>
       </c>
       <c r="AB7" s="111" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -25866,7 +25866,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="218" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="B1" s="218" t="s">
         <v>27</v>
@@ -26056,7 +26056,7 @@
         <v>262633</v>
       </c>
       <c r="G3" s="116" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="H3" s="116">
         <v>7200</v>
@@ -26068,7 +26068,7 @@
         <v>1.843</v>
       </c>
       <c r="K3" s="116" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="L3" s="113">
         <v>8572.1620000000003</v>
@@ -26116,10 +26116,10 @@
         <v>27</v>
       </c>
       <c r="AA3" s="111" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="AB3" s="111" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -26142,7 +26142,7 @@
         <v>262630</v>
       </c>
       <c r="G4" s="116" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="H4" s="116">
         <v>11100</v>
@@ -26202,7 +26202,7 @@
         <v>27</v>
       </c>
       <c r="AA4" s="111" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="AB4" s="111" t="s">
         <v>47</v>
@@ -26228,7 +26228,7 @@
         <v>262632</v>
       </c>
       <c r="G5" s="116" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="H5" s="116">
         <v>3600</v>
@@ -26291,7 +26291,7 @@
         <v>33</v>
       </c>
       <c r="AB5" s="111" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
@@ -26314,7 +26314,7 @@
         <v>262631</v>
       </c>
       <c r="G6" s="116" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="H6" s="116">
         <v>5550</v>
@@ -36315,11 +36315,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E182FEA0-9E29-45AE-8927-1BAD28B275F4}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" style="108" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" style="108" customWidth="1"/>
     <col min="3" max="3" width="5.88671875" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.21875" style="108" customWidth="1"/>
@@ -36349,7 +36352,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="221" t="s">
-        <v>758</v>
+        <v>788</v>
       </c>
       <c r="B1" s="221" t="s">
         <v>27</v>
@@ -36524,7 +36527,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C3" s="116" t="s">
         <v>26</v>
@@ -36551,7 +36554,7 @@
         <v>1.35</v>
       </c>
       <c r="K3" s="116" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="L3" s="113">
         <v>1833.3</v>
@@ -36602,7 +36605,7 @@
         <v>72</v>
       </c>
       <c r="AB3" s="111" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -36610,7 +36613,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C4" s="116" t="s">
         <v>26</v>
@@ -36688,7 +36691,7 @@
         <v>33</v>
       </c>
       <c r="AB4" s="111" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -36696,7 +36699,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C5" s="116" t="s">
         <v>26</v>
@@ -36723,7 +36726,7 @@
         <v>2.36</v>
       </c>
       <c r="K5" s="116" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="L5" s="113">
         <v>559.32000000000005</v>
@@ -36774,7 +36777,7 @@
         <v>33</v>
       </c>
       <c r="AB5" s="111" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -36782,7 +36785,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C6" s="116" t="s">
         <v>26</v>
@@ -36809,7 +36812,7 @@
         <v>2.1</v>
       </c>
       <c r="K6" s="116" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="L6" s="113">
         <v>561.79200000000003</v>
@@ -36860,7 +36863,7 @@
         <v>33</v>
       </c>
       <c r="AB6" s="111" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -36868,7 +36871,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C7" s="116" t="s">
         <v>36</v>
@@ -36895,7 +36898,7 @@
         <v>0.96</v>
       </c>
       <c r="K7" s="116" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="L7" s="113">
         <v>681.6</v>
@@ -36946,7 +36949,7 @@
         <v>39</v>
       </c>
       <c r="AB7" s="111" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -36954,7 +36957,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C8" s="116" t="s">
         <v>36</v>
@@ -36981,7 +36984,7 @@
         <v>1.44</v>
       </c>
       <c r="K8" s="116" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="L8" s="113">
         <v>934.56</v>
@@ -37032,7 +37035,7 @@
         <v>33</v>
       </c>
       <c r="AB8" s="111" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37040,7 +37043,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C9" s="116" t="s">
         <v>296</v>
@@ -37067,7 +37070,7 @@
         <v>1.8</v>
       </c>
       <c r="K9" s="116" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="L9" s="113">
         <v>5395.5</v>
@@ -37118,7 +37121,7 @@
         <v>57</v>
       </c>
       <c r="AB9" s="111" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37126,7 +37129,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C10" s="116" t="s">
         <v>296</v>
@@ -37153,7 +37156,7 @@
         <v>1.03</v>
       </c>
       <c r="K10" s="116" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="L10" s="113">
         <v>2683.15</v>
@@ -37204,7 +37207,7 @@
         <v>32</v>
       </c>
       <c r="AB10" s="111" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37212,7 +37215,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C11" s="116" t="s">
         <v>36</v>
@@ -37239,7 +37242,7 @@
         <v>1.42</v>
       </c>
       <c r="K11" s="116" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="L11" s="113">
         <v>964.18</v>
@@ -37290,7 +37293,7 @@
         <v>33</v>
       </c>
       <c r="AB11" s="111" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -37298,7 +37301,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="118" t="s">
-        <v>740</v>
+        <v>789</v>
       </c>
       <c r="C12" s="116" t="s">
         <v>36</v>
@@ -37470,7 +37473,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="86" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -42863,7 +42866,7 @@
         <v>7</v>
       </c>
       <c r="AB8" s="161" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="167" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (18/09/2026 13:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C3E448-47D2-4F68-A050-978EEBF9E2E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11FBEAED-7F2A-4FA6-B22C-B8E592A71E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="15" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1213" sheetId="159" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7382" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7369" uniqueCount="790">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -13144,7 +13144,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
@@ -13435,175 +13435,89 @@
         <v>532</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
-        <v>2</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>326</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="5">
-        <v>262488</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="H4" s="5">
-        <v>2100</v>
-      </c>
-      <c r="I4" s="7">
-        <v>0.59499999999999997</v>
-      </c>
-      <c r="J4" s="7">
-        <v>0.78600000000000003</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="7">
-        <v>982.10699999999997</v>
-      </c>
-      <c r="M4" s="9">
-        <v>825.3</v>
-      </c>
-      <c r="N4" s="6">
-        <v>0.11459999999999999</v>
-      </c>
-      <c r="O4" s="8">
-        <v>6.88</v>
-      </c>
-      <c r="P4" s="5">
-        <v>358.5</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>2</v>
-      </c>
-      <c r="R4" s="5">
-        <v>1250</v>
-      </c>
-      <c r="S4" s="7">
-        <v>1.19</v>
-      </c>
-      <c r="T4" s="5">
-        <v>60</v>
-      </c>
-      <c r="U4" s="6">
-        <v>4.8000000000000001E-2</v>
-      </c>
-      <c r="V4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB4" s="5" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="28">
-        <v>10350</v>
-      </c>
-      <c r="I5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P5" s="27">
-        <v>1766.7</v>
-      </c>
-      <c r="Q5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB5" s="27" t="s">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="28">
+        <v>8250</v>
+      </c>
+      <c r="I4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" s="27">
+        <v>1408</v>
+      </c>
+      <c r="Q4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB4" s="27" t="s">
         <v>27</v>
       </c>
     </row>
@@ -36322,7 +36236,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" style="108" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" style="108" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" style="108" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="5.88671875" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.21875" style="108" customWidth="1"/>
@@ -37473,7 +37387,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="86" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="96" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (18/09/2026 17:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8E4C91-10E0-477D-93B0-0FCA98AEFF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C919F1-8FE7-45D8-B862-A22A06103335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1217" sheetId="162" r:id="rId1"/>
@@ -6967,7 +6967,7 @@
     <col min="5" max="5" width="9.6640625" style="108" customWidth="1"/>
     <col min="6" max="6" width="8.44140625" style="108" customWidth="1"/>
     <col min="7" max="7" width="4.44140625" style="108" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" style="108" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" style="108" customWidth="1"/>
     <col min="9" max="9" width="6.109375" style="108" customWidth="1"/>
     <col min="10" max="10" width="6.44140625" style="108" customWidth="1"/>
     <col min="11" max="11" width="13.77734375" style="108" customWidth="1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/09/2026 10:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0406AE26-0BE5-4042-B67E-78AEB65AB325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3E1988-2409-4AE6-A02E-ABFABBEB103D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1217" sheetId="162" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7863" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7863" uniqueCount="820">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2385,9 +2385,6 @@
     <t>1096x1443</t>
   </si>
   <si>
-    <t>87x364x87</t>
-  </si>
-  <si>
     <t>1746</t>
   </si>
   <si>
@@ -2400,18 +2397,12 @@
     <t>1152x1483</t>
   </si>
   <si>
-    <t>182x202x182</t>
-  </si>
-  <si>
     <t>1745</t>
   </si>
   <si>
     <t>694x1543</t>
   </si>
   <si>
-    <t>135x404x135</t>
-  </si>
-  <si>
     <t>1747</t>
   </si>
   <si>
@@ -2538,19 +2529,10 @@
     <t>PROGRAMAÇÃO ONDULADEIRA - HARMONY EMBALAGENS  —  OF: 001217</t>
   </si>
   <si>
-    <t>267x960x267</t>
-  </si>
-  <si>
     <t>1514x2583</t>
   </si>
   <si>
-    <t>297x850x297</t>
-  </si>
-  <si>
     <t>1464x2403</t>
-  </si>
-  <si>
-    <t>187x1014x187</t>
   </si>
   <si>
     <t>1408x1523</t>
@@ -2565,7 +2547,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2706,6 +2688,11 @@
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -3697,7 +3684,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="B1" s="219" t="s">
         <v>27</v>
@@ -3878,7 +3865,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E3" s="150" t="s">
         <v>27</v>
@@ -3887,7 +3874,7 @@
         <v>262658</v>
       </c>
       <c r="G3" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H3" s="150">
         <v>300</v>
@@ -3964,7 +3951,7 @@
         <v>36</v>
       </c>
       <c r="D4" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E4" s="150" t="s">
         <v>27</v>
@@ -3973,7 +3960,7 @@
         <v>262656</v>
       </c>
       <c r="G4" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H4" s="150">
         <v>1000</v>
@@ -3985,7 +3972,7 @@
         <v>0.69299999999999995</v>
       </c>
       <c r="K4" s="150" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="L4" s="152">
         <v>528.06600000000003</v>
@@ -4036,7 +4023,7 @@
         <v>39</v>
       </c>
       <c r="AB4" s="150" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4050,7 +4037,7 @@
         <v>36</v>
       </c>
       <c r="D5" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E5" s="150" t="s">
         <v>27</v>
@@ -4059,7 +4046,7 @@
         <v>262651</v>
       </c>
       <c r="G5" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H5" s="150">
         <v>400</v>
@@ -4122,7 +4109,7 @@
         <v>39</v>
       </c>
       <c r="AB5" s="150" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4136,7 +4123,7 @@
         <v>36</v>
       </c>
       <c r="D6" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E6" s="150" t="s">
         <v>27</v>
@@ -4145,7 +4132,7 @@
         <v>262653</v>
       </c>
       <c r="G6" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H6" s="150">
         <v>400</v>
@@ -4208,7 +4195,7 @@
         <v>39</v>
       </c>
       <c r="AB6" s="150" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4222,7 +4209,7 @@
         <v>36</v>
       </c>
       <c r="D7" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E7" s="150" t="s">
         <v>27</v>
@@ -4231,7 +4218,7 @@
         <v>262654</v>
       </c>
       <c r="G7" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H7" s="150">
         <v>600</v>
@@ -4243,7 +4230,7 @@
         <v>1.2490000000000001</v>
       </c>
       <c r="K7" s="150" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="L7" s="152">
         <v>497.60199999999998</v>
@@ -4294,7 +4281,7 @@
         <v>33</v>
       </c>
       <c r="AB7" s="150" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4308,7 +4295,7 @@
         <v>36</v>
       </c>
       <c r="D8" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E8" s="150" t="s">
         <v>27</v>
@@ -4317,7 +4304,7 @@
         <v>262657</v>
       </c>
       <c r="G8" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H8" s="150">
         <v>600</v>
@@ -4329,7 +4316,7 @@
         <v>0.69299999999999995</v>
       </c>
       <c r="K8" s="150" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="L8" s="152">
         <v>479.00200000000001</v>
@@ -4380,7 +4367,7 @@
         <v>39</v>
       </c>
       <c r="AB8" s="150" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4394,7 +4381,7 @@
         <v>36</v>
       </c>
       <c r="D9" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E9" s="150" t="s">
         <v>27</v>
@@ -4403,7 +4390,7 @@
         <v>262655</v>
       </c>
       <c r="G9" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H9" s="150">
         <v>2500</v>
@@ -4466,7 +4453,7 @@
         <v>39</v>
       </c>
       <c r="AB9" s="150" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4480,7 +4467,7 @@
         <v>36</v>
       </c>
       <c r="D10" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E10" s="150" t="s">
         <v>27</v>
@@ -4489,7 +4476,7 @@
         <v>262652</v>
       </c>
       <c r="G10" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H10" s="150">
         <v>400</v>
@@ -4552,7 +4539,7 @@
         <v>39</v>
       </c>
       <c r="AB10" s="150" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4566,7 +4553,7 @@
         <v>36</v>
       </c>
       <c r="D11" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E11" s="150" t="s">
         <v>27</v>
@@ -4575,7 +4562,7 @@
         <v>262660</v>
       </c>
       <c r="G11" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H11" s="150">
         <v>1500</v>
@@ -4587,7 +4574,7 @@
         <v>0.78900000000000003</v>
       </c>
       <c r="K11" s="150" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="L11" s="152">
         <v>501.80399999999997</v>
@@ -4638,7 +4625,7 @@
         <v>39</v>
       </c>
       <c r="AB11" s="150" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4652,7 +4639,7 @@
         <v>36</v>
       </c>
       <c r="D12" s="150" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="E12" s="150" t="s">
         <v>27</v>
@@ -4661,7 +4648,7 @@
         <v>262659</v>
       </c>
       <c r="G12" s="150" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="H12" s="150">
         <v>3000</v>
@@ -4673,7 +4660,7 @@
         <v>0.72899999999999998</v>
       </c>
       <c r="K12" s="150" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="L12" s="152">
         <v>804.81600000000003</v>
@@ -4724,7 +4711,7 @@
         <v>33</v>
       </c>
       <c r="AB12" s="150" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16570,7 +16557,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="B1" s="219" t="s">
         <v>27</v>
@@ -16751,7 +16738,7 @@
         <v>296</v>
       </c>
       <c r="D3" s="116" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="E3" s="116" t="s">
         <v>27</v>
@@ -16760,7 +16747,7 @@
         <v>262649</v>
       </c>
       <c r="G3" s="116" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="H3" s="116">
         <v>2600</v>
@@ -16772,7 +16759,7 @@
         <v>1.2629999999999999</v>
       </c>
       <c r="K3" s="116" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="L3" s="113">
         <v>1615.63</v>
@@ -16823,7 +16810,7 @@
         <v>32</v>
       </c>
       <c r="AB3" s="111" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -16837,7 +16824,7 @@
         <v>296</v>
       </c>
       <c r="D4" s="116" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="E4" s="116" t="s">
         <v>27</v>
@@ -16846,7 +16833,7 @@
         <v>262650</v>
       </c>
       <c r="G4" s="116" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="H4" s="116">
         <v>2300</v>
@@ -16858,7 +16845,7 @@
         <v>1.393</v>
       </c>
       <c r="K4" s="116" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="L4" s="113">
         <v>1464.182</v>
@@ -16909,7 +16896,7 @@
         <v>30</v>
       </c>
       <c r="AB4" s="111" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -18034,7 +18021,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -25820,7 +25807,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="B1" s="219" t="s">
         <v>27</v>
@@ -26001,7 +25988,7 @@
         <v>60</v>
       </c>
       <c r="D3" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E3" s="116" t="s">
         <v>27</v>
@@ -26010,7 +25997,7 @@
         <v>262645</v>
       </c>
       <c r="G3" s="116" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="H3" s="116">
         <v>2740</v>
@@ -26073,7 +26060,7 @@
         <v>32</v>
       </c>
       <c r="AB3" s="111" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -26087,7 +26074,7 @@
         <v>60</v>
       </c>
       <c r="D4" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E4" s="116" t="s">
         <v>27</v>
@@ -26096,7 +26083,7 @@
         <v>262644</v>
       </c>
       <c r="G4" s="116" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="H4" s="116">
         <v>1662</v>
@@ -26159,7 +26146,7 @@
         <v>33</v>
       </c>
       <c r="AB4" s="111" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -26173,7 +26160,7 @@
         <v>60</v>
       </c>
       <c r="D5" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E5" s="116" t="s">
         <v>27</v>
@@ -26182,7 +26169,7 @@
         <v>262646</v>
       </c>
       <c r="G5" s="116" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="H5" s="116">
         <v>1140</v>
@@ -26245,7 +26232,7 @@
         <v>33</v>
       </c>
       <c r="AB5" s="111" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -26259,7 +26246,7 @@
         <v>50</v>
       </c>
       <c r="D6" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E6" s="116" t="s">
         <v>27</v>
@@ -26268,7 +26255,7 @@
         <v>262647</v>
       </c>
       <c r="G6" s="116" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="H6" s="116">
         <v>3052</v>
@@ -26345,7 +26332,7 @@
         <v>50</v>
       </c>
       <c r="D7" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E7" s="116" t="s">
         <v>27</v>
@@ -26354,7 +26341,7 @@
         <v>262648</v>
       </c>
       <c r="G7" s="116" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="H7" s="116">
         <v>3317</v>
@@ -37480,7 +37467,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="B1" s="219" t="s">
         <v>27</v>
@@ -37661,7 +37648,7 @@
         <v>65</v>
       </c>
       <c r="D3" s="150" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E3" s="150" t="s">
         <v>27</v>
@@ -37670,7 +37657,7 @@
         <v>262640</v>
       </c>
       <c r="G3" s="150" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="H3" s="150">
         <v>800</v>
@@ -37682,7 +37669,7 @@
         <v>1.6739999999999999</v>
       </c>
       <c r="K3" s="150" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="L3" s="152">
         <v>980.29399999999998</v>
@@ -37733,7 +37720,7 @@
         <v>30</v>
       </c>
       <c r="AB3" s="150" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
@@ -37747,7 +37734,7 @@
         <v>65</v>
       </c>
       <c r="D4" s="150" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E4" s="150" t="s">
         <v>27</v>
@@ -37756,7 +37743,7 @@
         <v>262641</v>
       </c>
       <c r="G4" s="150" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="H4" s="150">
         <v>1150</v>
@@ -37768,7 +37755,7 @@
         <v>1.44</v>
       </c>
       <c r="K4" s="150" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="L4" s="152">
         <v>905.83199999999999</v>
@@ -37819,7 +37806,7 @@
         <v>33</v>
       </c>
       <c r="AB4" s="150" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
@@ -37833,7 +37820,7 @@
         <v>36</v>
       </c>
       <c r="D5" s="150" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E5" s="150" t="s">
         <v>27</v>
@@ -37842,7 +37829,7 @@
         <v>262642</v>
       </c>
       <c r="G5" s="150" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="H5" s="150">
         <v>1000</v>
@@ -37854,7 +37841,7 @@
         <v>1.58</v>
       </c>
       <c r="K5" s="150" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="L5" s="152">
         <v>917.98</v>
@@ -37905,7 +37892,7 @@
         <v>33</v>
       </c>
       <c r="AB5" s="150" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
@@ -42122,7 +42109,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="219" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="B1" s="219" t="s">
         <v>27</v>
@@ -42321,7 +42308,7 @@
         <v>2.5630000000000002</v>
       </c>
       <c r="K3" t="s">
-        <v>820</v>
+        <v>34</v>
       </c>
       <c r="L3">
         <v>1914.5609999999999</v>
@@ -42372,7 +42359,7 @@
         <v>3</v>
       </c>
       <c r="AB3" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
     </row>
     <row r="4" spans="1:28" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -42404,7 +42391,7 @@
         <v>2.383</v>
       </c>
       <c r="K4" t="s">
-        <v>822</v>
+        <v>34</v>
       </c>
       <c r="L4">
         <v>1720.5260000000001</v>
@@ -42455,7 +42442,7 @@
         <v>3</v>
       </c>
       <c r="AB4" t="s">
-        <v>823</v>
+        <v>818</v>
       </c>
     </row>
     <row r="5" spans="1:28" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -42487,7 +42474,7 @@
         <v>1.5029999999999999</v>
       </c>
       <c r="K5" t="s">
-        <v>824</v>
+        <v>34</v>
       </c>
       <c r="L5">
         <v>834.46600000000001</v>
@@ -42538,7 +42525,7 @@
         <v>3</v>
       </c>
       <c r="AB5" t="s">
-        <v>825</v>
+        <v>819</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -42552,7 +42539,7 @@
         <v>45</v>
       </c>
       <c r="D6" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E6" s="116" t="s">
         <v>27</v>
@@ -42561,7 +42548,7 @@
         <v>262639</v>
       </c>
       <c r="G6" s="116" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="H6" s="116">
         <v>300</v>
@@ -42572,8 +42559,8 @@
       <c r="J6" s="117">
         <v>1.5229999999999999</v>
       </c>
-      <c r="K6" s="116" t="s">
-        <v>777</v>
+      <c r="K6" t="s">
+        <v>34</v>
       </c>
       <c r="L6" s="113">
         <v>307.95100000000002</v>
@@ -42624,7 +42611,7 @@
         <v>33</v>
       </c>
       <c r="AB6" s="111" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -42638,7 +42625,7 @@
         <v>45</v>
       </c>
       <c r="D7" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E7" s="116" t="s">
         <v>27</v>
@@ -42647,7 +42634,7 @@
         <v>262637</v>
       </c>
       <c r="G7" s="116" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="H7" s="116">
         <v>500</v>
@@ -42658,8 +42645,8 @@
       <c r="J7" s="117">
         <v>1.4630000000000001</v>
       </c>
-      <c r="K7" s="116" t="s">
-        <v>774</v>
+      <c r="K7" t="s">
+        <v>34</v>
       </c>
       <c r="L7" s="113">
         <v>414.029</v>
@@ -42710,7 +42697,7 @@
         <v>33</v>
       </c>
       <c r="AB7" s="111" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -42724,7 +42711,7 @@
         <v>45</v>
       </c>
       <c r="D8" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E8" s="116" t="s">
         <v>27</v>
@@ -42733,7 +42720,7 @@
         <v>262635</v>
       </c>
       <c r="G8" s="116" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H8" s="116">
         <v>5000</v>
@@ -42744,8 +42731,8 @@
       <c r="J8" s="117">
         <v>1.389</v>
       </c>
-      <c r="K8" s="116" t="s">
-        <v>446</v>
+      <c r="K8" t="s">
+        <v>34</v>
       </c>
       <c r="L8" s="113">
         <v>3882.2550000000001</v>
@@ -42810,7 +42797,7 @@
         <v>45</v>
       </c>
       <c r="D9" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E9" s="116" t="s">
         <v>27</v>
@@ -42819,7 +42806,7 @@
         <v>262636</v>
       </c>
       <c r="G9" s="116" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H9" s="116">
         <v>5000</v>
@@ -42830,8 +42817,8 @@
       <c r="J9" s="117">
         <v>1.389</v>
       </c>
-      <c r="K9" s="116" t="s">
-        <v>446</v>
+      <c r="K9" t="s">
+        <v>34</v>
       </c>
       <c r="L9" s="113">
         <v>3882.2550000000001</v>
@@ -42896,7 +42883,7 @@
         <v>26</v>
       </c>
       <c r="D10" s="116" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="E10" s="116" t="s">
         <v>27</v>
@@ -42905,7 +42892,7 @@
         <v>262638</v>
       </c>
       <c r="G10" s="116" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="H10" s="116">
         <v>200</v>
@@ -42916,8 +42903,8 @@
       <c r="J10" s="117">
         <v>1.423</v>
       </c>
-      <c r="K10" s="116" t="s">
-        <v>769</v>
+      <c r="K10" t="s">
+        <v>34</v>
       </c>
       <c r="L10" s="113">
         <v>153.11500000000001</v>
@@ -43000,8 +42987,8 @@
       <c r="J11" s="117">
         <v>1.536</v>
       </c>
-      <c r="K11" s="116" t="s">
-        <v>587</v>
+      <c r="K11" t="s">
+        <v>34</v>
       </c>
       <c r="L11" s="113">
         <v>874.59799999999996</v>
@@ -43074,8 +43061,8 @@
         <v>27</v>
       </c>
       <c r="H12" s="110">
-        <f>SUM(H6:H11)</f>
-        <v>11600</v>
+        <f>SUM(H3:H11)</f>
+        <v>13000</v>
       </c>
       <c r="I12" s="110" t="s">
         <v>27</v>
@@ -43099,8 +43086,8 @@
         <v>27</v>
       </c>
       <c r="P12" s="109">
-        <f>SUM(P6:P11)</f>
-        <v>5178.1999999999989</v>
+        <f>SUM(P3:P11)</f>
+        <v>7717</v>
       </c>
       <c r="Q12" s="109" t="s">
         <v>27</v>
@@ -43143,6 +43130,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
+  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
@@ -43829,7 +43817,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="220" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="B1" s="220" t="s">
         <v>27</v>
@@ -44004,7 +43992,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C3" s="116" t="s">
         <v>26</v>
@@ -44090,7 +44078,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C4" s="116" t="s">
         <v>26</v>
@@ -44176,7 +44164,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C5" s="116" t="s">
         <v>26</v>
@@ -44262,7 +44250,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C6" s="116" t="s">
         <v>26</v>
@@ -44348,7 +44336,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C7" s="116" t="s">
         <v>36</v>
@@ -44434,7 +44422,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C8" s="116" t="s">
         <v>36</v>
@@ -44520,7 +44508,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C9" s="116" t="s">
         <v>296</v>
@@ -44606,7 +44594,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C10" s="116" t="s">
         <v>296</v>
@@ -44692,7 +44680,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C11" s="116" t="s">
         <v>36</v>
@@ -44778,7 +44766,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="118" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C12" s="116" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/09/2026 17:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3E1988-2409-4AE6-A02E-ABFABBEB103D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A92C3B-A727-4E7B-8B50-3CC13EB61F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1217" sheetId="162" r:id="rId1"/>
@@ -5103,7 +5103,7 @@
       </c>
     </row>
     <row r="4" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="200">
+      <c r="A4" s="5">
         <v>2</v>
       </c>
       <c r="B4" s="205" t="s">
@@ -5189,7 +5189,7 @@
       </c>
     </row>
     <row r="5" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="200">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
       <c r="B5" s="205" t="s">
@@ -5275,7 +5275,7 @@
       </c>
     </row>
     <row r="6" spans="1:28" s="199" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="200">
+      <c r="A6" s="5">
         <v>4</v>
       </c>
       <c r="B6" s="205" t="s">
@@ -5362,7 +5362,7 @@
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>66</v>
@@ -5448,7 +5448,7 @@
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>66</v>
@@ -5534,7 +5534,7 @@
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>66</v>
@@ -5620,7 +5620,7 @@
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>66</v>
@@ -5706,7 +5706,7 @@
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>66</v>
@@ -5792,7 +5792,7 @@
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>66</v>
@@ -5878,7 +5878,7 @@
     </row>
     <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>66</v>
@@ -5964,7 +5964,7 @@
     </row>
     <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>66</v>
@@ -6050,7 +6050,7 @@
     </row>
     <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>66</v>
@@ -6136,7 +6136,7 @@
     </row>
     <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>66</v>
@@ -6222,7 +6222,7 @@
     </row>
     <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>66</v>
@@ -6308,7 +6308,7 @@
     </row>
     <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>66</v>
@@ -6394,7 +6394,7 @@
     </row>
     <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>66</v>
@@ -6501,6 +6501,7 @@
         <v>27</v>
       </c>
       <c r="H20" s="11">
+        <f>SUM(H3:H19)</f>
         <v>24720</v>
       </c>
       <c r="I20" s="11" t="s">
@@ -6525,7 +6526,8 @@
         <v>27</v>
       </c>
       <c r="P20" s="11">
-        <v>11647.9</v>
+        <f>SUM(P3:P19)</f>
+        <v>11648</v>
       </c>
       <c r="Q20" s="11" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/09/2026 17:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F51DCBF-C3B0-44D2-9DCD-665944775938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534DDD7A-C0F6-461E-ABEE-0B7F43BADB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="18" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1217" sheetId="162" r:id="rId1"/>
@@ -33,7 +33,7 @@
     <sheet name="PCBOX - IPE 1187 P" sheetId="142" r:id="rId18"/>
     <sheet name="RM Embalagens 1184 P" sheetId="141" r:id="rId19"/>
     <sheet name="CARTOMIL EMBALAGENS LTDA 1183 P" sheetId="140" r:id="rId20"/>
-    <sheet name="Z4A EMBALAGENS LTDA 1182" sheetId="139" r:id="rId21"/>
+    <sheet name="Z4A EMBALAGENS LTDA 1182P" sheetId="139" r:id="rId21"/>
     <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId22"/>
     <sheet name="RM Embalagens 1179 P" sheetId="136" r:id="rId23"/>
     <sheet name="Tolecaixas 1181 P" sheetId="138" r:id="rId24"/>
@@ -17942,88 +17942,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="223" t="s">
+      <c r="A1" s="222" t="s">
         <v>535</v>
       </c>
-      <c r="B1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="223" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="223" t="s">
+      <c r="B1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="222" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="222" t="s">
         <v>27</v>
       </c>
     </row>
@@ -18290,6 +18290,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -43143,6 +43144,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A45B5AC-557E-4203-8DD1-DFBBC7E9A9E0}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -43781,7 +43785,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="98" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (22/09/2026 08:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534DDD7A-C0F6-461E-ABEE-0B7F43BADB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E856209B-59A8-4DED-9F55-E7009EEFDF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="18" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1217" sheetId="162" r:id="rId1"/>
@@ -4811,6 +4811,9 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15B73F0-D53E-458D-8A18-622E142F07EE}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6571,7 +6574,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup scale="82" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -17908,6 +17911,9 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -18290,7 +18296,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="95" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (22/09/2026 11:15)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DC19D9-B070-4411-AB41-9D97A3535E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E87694-D54C-41D2-8C87-58343E1A99B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORBOX 1220" sheetId="163" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7984" uniqueCount="831">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8049" uniqueCount="841">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2570,6 +2570,36 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - FORBOX Soluções em Caixas de Papelão LTDA  —  OF: 001220</t>
+  </si>
+  <si>
+    <t>276x800x276</t>
+  </si>
+  <si>
+    <t>8253</t>
+  </si>
+  <si>
+    <t>1172x2360</t>
+  </si>
+  <si>
+    <t>276x600x276</t>
+  </si>
+  <si>
+    <t>1392x2400</t>
+  </si>
+  <si>
+    <t>276x820x276</t>
+  </si>
+  <si>
+    <t>780x2200</t>
+  </si>
+  <si>
+    <t>8260</t>
+  </si>
+  <si>
+    <t>191x210x191</t>
+  </si>
+  <si>
+    <t>612x1639</t>
   </si>
 </sst>
 </file>
@@ -42762,7 +42792,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCDEA62-D4C1-4F97-B5A0-F9D378B5F3A6}">
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AB11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5546875" style="108" customWidth="1"/>
@@ -42967,347 +42997,779 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="150">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="133">
         <v>1</v>
       </c>
-      <c r="B3" s="151" t="s">
+      <c r="B3" s="134" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="150" t="s">
+      <c r="C3" s="133" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="133" t="s">
+        <v>803</v>
+      </c>
+      <c r="E3" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="133">
+        <v>262674</v>
+      </c>
+      <c r="G3" s="133" t="s">
+        <v>832</v>
+      </c>
+      <c r="H3" s="133">
+        <v>400</v>
+      </c>
+      <c r="I3" s="135">
+        <v>1.3720000000000001</v>
+      </c>
+      <c r="J3" s="135">
+        <v>2.38</v>
+      </c>
+      <c r="K3" s="133" t="s">
+        <v>836</v>
+      </c>
+      <c r="L3" s="135">
+        <v>1306.144</v>
+      </c>
+      <c r="M3" s="136">
+        <v>952</v>
+      </c>
+      <c r="N3" s="137">
+        <v>0.26440000000000002</v>
+      </c>
+      <c r="O3" s="138">
+        <v>15.87</v>
+      </c>
+      <c r="P3" s="133">
+        <v>702.7</v>
+      </c>
+      <c r="Q3" s="133">
+        <v>1</v>
+      </c>
+      <c r="R3" s="133">
+        <v>1400</v>
+      </c>
+      <c r="S3" s="135">
+        <v>1.3720000000000001</v>
+      </c>
+      <c r="T3" s="133">
+        <v>28</v>
+      </c>
+      <c r="U3" s="137">
+        <v>0.02</v>
+      </c>
+      <c r="V3" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="133" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="133" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB3" s="133" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="133">
+        <v>2</v>
+      </c>
+      <c r="B4" s="134" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="133" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="133" t="s">
+        <v>803</v>
+      </c>
+      <c r="E4" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="133">
+        <v>262672</v>
+      </c>
+      <c r="G4" s="133" t="s">
+        <v>832</v>
+      </c>
+      <c r="H4" s="133">
+        <v>400</v>
+      </c>
+      <c r="I4" s="135">
+        <v>1.1519999999999999</v>
+      </c>
+      <c r="J4" s="135">
+        <v>2.34</v>
+      </c>
+      <c r="K4" s="133" t="s">
+        <v>834</v>
+      </c>
+      <c r="L4" s="135">
+        <v>1078.2719999999999</v>
+      </c>
+      <c r="M4" s="136">
+        <v>936</v>
+      </c>
+      <c r="N4" s="137">
+        <v>0.26</v>
+      </c>
+      <c r="O4" s="138">
+        <v>15.6</v>
+      </c>
+      <c r="P4" s="133">
+        <v>580.1</v>
+      </c>
+      <c r="Q4" s="133">
+        <v>1</v>
+      </c>
+      <c r="R4" s="133">
+        <v>1200</v>
+      </c>
+      <c r="S4" s="135">
+        <v>1.1519999999999999</v>
+      </c>
+      <c r="T4" s="133">
+        <v>48</v>
+      </c>
+      <c r="U4" s="137">
+        <v>0.04</v>
+      </c>
+      <c r="V4" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="133" t="s">
+        <v>29</v>
+      </c>
+      <c r="X4" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="133" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="133" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="133">
+        <v>3</v>
+      </c>
+      <c r="B5" s="134" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="133" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="133" t="s">
+        <v>803</v>
+      </c>
+      <c r="E5" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="133">
+        <v>262671</v>
+      </c>
+      <c r="G5" s="133" t="s">
+        <v>832</v>
+      </c>
+      <c r="H5" s="133">
+        <v>400</v>
+      </c>
+      <c r="I5" s="135">
+        <v>1.3520000000000001</v>
+      </c>
+      <c r="J5" s="135">
+        <v>2.339</v>
+      </c>
+      <c r="K5" s="133" t="s">
+        <v>831</v>
+      </c>
+      <c r="L5" s="135">
+        <v>1264.931</v>
+      </c>
+      <c r="M5" s="136">
+        <v>467.8</v>
+      </c>
+      <c r="N5" s="137">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="O5" s="138">
+        <v>3.9</v>
+      </c>
+      <c r="P5" s="133">
+        <v>680.5</v>
+      </c>
+      <c r="Q5" s="133">
+        <v>2</v>
+      </c>
+      <c r="R5" s="133">
+        <v>1200</v>
+      </c>
+      <c r="S5" s="135">
+        <v>2.7040000000000002</v>
+      </c>
+      <c r="T5" s="133">
+        <v>-1504</v>
+      </c>
+      <c r="U5" s="137">
+        <v>-1.2533000000000001</v>
+      </c>
+      <c r="V5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="133" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="133" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB5" s="133" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="150">
+        <v>1</v>
+      </c>
+      <c r="B6" s="151" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="150" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="150" t="s">
+      <c r="D6" s="150" t="s">
         <v>770</v>
       </c>
-      <c r="E3" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="150">
+      <c r="E6" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="150">
         <v>262640</v>
       </c>
-      <c r="G3" s="150" t="s">
+      <c r="G6" s="150" t="s">
         <v>779</v>
       </c>
-      <c r="H3" s="150">
+      <c r="H6" s="150">
         <v>800</v>
       </c>
-      <c r="I3" s="152">
+      <c r="I6" s="152">
         <v>0.73199999999999998</v>
       </c>
-      <c r="J3" s="152">
+      <c r="J6" s="152">
         <v>1.6739999999999999</v>
       </c>
-      <c r="K3" s="150" t="s">
+      <c r="K6" s="150" t="s">
         <v>783</v>
       </c>
-      <c r="L3" s="152">
+      <c r="L6" s="152">
         <v>980.29399999999998</v>
       </c>
-      <c r="M3" s="153">
+      <c r="M6" s="153">
         <v>669.6</v>
       </c>
-      <c r="N3" s="154">
+      <c r="N6" s="154">
         <v>9.2999999999999999E-2</v>
       </c>
-      <c r="O3" s="155">
+      <c r="O6" s="155">
         <v>5.58</v>
       </c>
-      <c r="P3" s="150">
+      <c r="P6" s="150">
         <v>317.60000000000002</v>
       </c>
-      <c r="Q3" s="150">
+      <c r="Q6" s="150">
         <v>2</v>
       </c>
-      <c r="R3" s="150">
+      <c r="R6" s="150">
         <v>1500</v>
       </c>
-      <c r="S3" s="152">
+      <c r="S6" s="152">
         <v>1.464</v>
       </c>
-      <c r="T3" s="150">
+      <c r="T6" s="150">
         <v>36</v>
       </c>
-      <c r="U3" s="154">
+      <c r="U6" s="154">
         <v>2.4E-2</v>
       </c>
-      <c r="V3" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="150" t="s">
+      <c r="V6" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="150" t="s">
         <v>30</v>
       </c>
-      <c r="AB3" s="150" t="s">
+      <c r="AB6" s="150" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="150">
+    <row r="7" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="150">
         <v>2</v>
       </c>
-      <c r="B4" s="151" t="s">
+      <c r="B7" s="151" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="150" t="s">
+      <c r="C7" s="150" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="150" t="s">
+      <c r="D7" s="150" t="s">
         <v>770</v>
       </c>
-      <c r="E4" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="150">
+      <c r="E7" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="150">
         <v>262641</v>
       </c>
-      <c r="G4" s="150" t="s">
+      <c r="G7" s="150" t="s">
         <v>779</v>
       </c>
-      <c r="H4" s="150">
+      <c r="H7" s="150">
         <v>1150</v>
       </c>
-      <c r="I4" s="152">
+      <c r="I7" s="152">
         <v>0.54700000000000004</v>
       </c>
-      <c r="J4" s="152">
+      <c r="J7" s="152">
         <v>1.44</v>
       </c>
-      <c r="K4" s="150" t="s">
+      <c r="K7" s="150" t="s">
         <v>781</v>
       </c>
-      <c r="L4" s="152">
+      <c r="L7" s="152">
         <v>905.83199999999999</v>
       </c>
-      <c r="M4" s="153">
+      <c r="M7" s="153">
         <v>828</v>
       </c>
-      <c r="N4" s="154">
+      <c r="N7" s="154">
         <v>0.115</v>
       </c>
-      <c r="O4" s="155">
+      <c r="O7" s="155">
         <v>6.9</v>
       </c>
-      <c r="P4" s="150">
+      <c r="P7" s="150">
         <v>293.5</v>
       </c>
-      <c r="Q4" s="150">
+      <c r="Q7" s="150">
         <v>2</v>
       </c>
-      <c r="R4" s="150">
+      <c r="R7" s="150">
         <v>1150</v>
       </c>
-      <c r="S4" s="152">
+      <c r="S7" s="152">
         <v>1.0940000000000001</v>
       </c>
-      <c r="T4" s="150">
+      <c r="T7" s="150">
         <v>56</v>
       </c>
-      <c r="U4" s="154">
+      <c r="U7" s="154">
         <v>4.87E-2</v>
       </c>
-      <c r="V4" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="150" t="s">
+      <c r="V7" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB4" s="150" t="s">
+      <c r="AB7" s="150" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="150">
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="133">
+        <v>4</v>
+      </c>
+      <c r="B8" s="134" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="133" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="133" t="s">
+        <v>803</v>
+      </c>
+      <c r="E8" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="133">
+        <v>262673</v>
+      </c>
+      <c r="G8" s="133" t="s">
+        <v>832</v>
+      </c>
+      <c r="H8" s="133">
+        <v>1000</v>
+      </c>
+      <c r="I8" s="135">
+        <v>0.76</v>
+      </c>
+      <c r="J8" s="135">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="K8" s="133" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" s="135">
+        <v>828.4</v>
+      </c>
+      <c r="M8" s="136">
+        <v>545</v>
+      </c>
+      <c r="N8" s="137">
+        <v>7.5700000000000003E-2</v>
+      </c>
+      <c r="O8" s="138">
+        <v>4.54</v>
+      </c>
+      <c r="P8" s="133">
+        <v>260.89999999999998</v>
+      </c>
+      <c r="Q8" s="133">
+        <v>2</v>
+      </c>
+      <c r="R8" s="133">
+        <v>1550</v>
+      </c>
+      <c r="S8" s="135">
+        <v>1.52</v>
+      </c>
+      <c r="T8" s="133">
+        <v>30</v>
+      </c>
+      <c r="U8" s="137">
+        <v>1.9400000000000001E-2</v>
+      </c>
+      <c r="V8" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="133" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB8" s="133" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="133">
+        <v>5</v>
+      </c>
+      <c r="B9" s="134" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="133" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="133" t="s">
+        <v>824</v>
+      </c>
+      <c r="E9" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="133">
+        <v>262675</v>
+      </c>
+      <c r="G9" s="133" t="s">
+        <v>838</v>
+      </c>
+      <c r="H9" s="133">
+        <v>1350</v>
+      </c>
+      <c r="I9" s="135">
+        <v>0.59199999999999997</v>
+      </c>
+      <c r="J9" s="135">
+        <v>1.619</v>
+      </c>
+      <c r="K9" s="133" t="s">
+        <v>839</v>
+      </c>
+      <c r="L9" s="135">
+        <v>1293.905</v>
+      </c>
+      <c r="M9" s="136">
+        <v>1092.8</v>
+      </c>
+      <c r="N9" s="137">
+        <v>0.15179999999999999</v>
+      </c>
+      <c r="O9" s="138">
+        <v>9.11</v>
+      </c>
+      <c r="P9" s="133">
+        <v>407.6</v>
+      </c>
+      <c r="Q9" s="133">
+        <v>2</v>
+      </c>
+      <c r="R9" s="133">
+        <v>1250</v>
+      </c>
+      <c r="S9" s="135">
+        <v>1.1839999999999999</v>
+      </c>
+      <c r="T9" s="133">
+        <v>66</v>
+      </c>
+      <c r="U9" s="137">
+        <v>5.28E-2</v>
+      </c>
+      <c r="V9" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="133" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB9" s="133" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="156" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="150">
         <v>3</v>
       </c>
-      <c r="B5" s="151" t="s">
+      <c r="B10" s="151" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="150" t="s">
+      <c r="C10" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="150" t="s">
+      <c r="D10" s="150" t="s">
         <v>770</v>
       </c>
-      <c r="E5" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="150">
+      <c r="E10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="150">
         <v>262642</v>
       </c>
-      <c r="G5" s="150" t="s">
+      <c r="G10" s="150" t="s">
         <v>779</v>
       </c>
-      <c r="H5" s="150">
+      <c r="H10" s="150">
         <v>1000</v>
       </c>
-      <c r="I5" s="152">
+      <c r="I10" s="152">
         <v>0.58099999999999996</v>
       </c>
-      <c r="J5" s="152">
+      <c r="J10" s="152">
         <v>1.58</v>
       </c>
-      <c r="K5" s="150" t="s">
+      <c r="K10" s="150" t="s">
         <v>778</v>
       </c>
-      <c r="L5" s="152">
+      <c r="L10" s="152">
         <v>917.98</v>
       </c>
-      <c r="M5" s="153">
+      <c r="M10" s="153">
         <v>790</v>
       </c>
-      <c r="N5" s="154">
+      <c r="N10" s="154">
         <v>0.10970000000000001</v>
       </c>
-      <c r="O5" s="155">
+      <c r="O10" s="155">
         <v>6.58</v>
       </c>
-      <c r="P5" s="150">
+      <c r="P10" s="150">
         <v>289.2</v>
       </c>
-      <c r="Q5" s="150">
+      <c r="Q10" s="150">
         <v>2</v>
       </c>
-      <c r="R5" s="150">
+      <c r="R10" s="150">
         <v>1200</v>
       </c>
-      <c r="S5" s="152">
+      <c r="S10" s="152">
         <v>1.1619999999999999</v>
       </c>
-      <c r="T5" s="150">
+      <c r="T10" s="150">
         <v>38</v>
       </c>
-      <c r="U5" s="154">
+      <c r="U10" s="154">
         <v>3.1699999999999999E-2</v>
       </c>
-      <c r="V5" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="150" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="150" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="150" t="s">
+      <c r="V10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="150" t="s">
         <v>33</v>
       </c>
-      <c r="AB5" s="150" t="s">
+      <c r="AB10" s="150" t="s">
         <v>777</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="157">
-        <v>2950</v>
-      </c>
-      <c r="I6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="O6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" s="157">
-        <v>900.3</v>
-      </c>
-      <c r="Q6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="R6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="S6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="T6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="U6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="V6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="W6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="X6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="157" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB6" s="157" t="s">
+    <row r="11" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="157">
+        <f>SUM(H3:H10)</f>
+        <v>6500</v>
+      </c>
+      <c r="I11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="O11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="P11" s="157">
+        <f>SUM(P3:P10)</f>
+        <v>3532.1</v>
+      </c>
+      <c r="Q11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="R11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="S11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="T11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="U11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="V11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="W11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="X11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB11" s="157" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (22/09/2026 14:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804C317C-881D-4E11-80A3-52B1967C472C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F510F66A-1E3A-4254-9693-4B736CA28D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45115,7 +45115,7 @@
     <col min="8" max="8" width="6" style="108" customWidth="1"/>
     <col min="9" max="9" width="7.21875" style="108" customWidth="1"/>
     <col min="10" max="10" width="6.5546875" style="108" customWidth="1"/>
-    <col min="11" max="11" width="9" style="108" customWidth="1"/>
+    <col min="11" max="11" width="6" style="108" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="108" hidden="1" customWidth="1"/>
@@ -45130,7 +45130,7 @@
     <col min="24" max="24" width="7.44140625" style="108" customWidth="1"/>
     <col min="25" max="25" width="7.77734375" style="108" customWidth="1"/>
     <col min="26" max="26" width="7.44140625" style="108" customWidth="1"/>
-    <col min="27" max="27" width="4.88671875" style="108" customWidth="1"/>
+    <col min="27" max="27" width="4.21875" style="108" customWidth="1"/>
     <col min="28" max="28" width="11.33203125" style="108" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (23/09/2026 08:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D147D9F-282C-404A-AEB8-BFEBB234C189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EE718D-169E-4DE8-8DCC-68CDFCA40164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId1"/>
@@ -1168,7 +1168,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1437,7 +1437,6 @@
     <xf numFmtId="14" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1446,6 +1445,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1703,88 +1708,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>302</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2348,88 +2353,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="94" t="s">
         <v>183</v>
       </c>
-      <c r="B1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="95" t="s">
+      <c r="B1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="94" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2996,88 +3001,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="94" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="95" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="95" t="s">
+      <c r="B1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="94" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4763,88 +4768,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="93" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="94" t="s">
+      <c r="B1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="93" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6196,88 +6201,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -7273,88 +7278,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="95" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="96" t="s">
+      <c r="B1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="95" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="95" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8610,88 +8615,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="96" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="97" t="s">
+      <c r="B1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="96" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="96" t="s">
         <v>27</v>
       </c>
     </row>
@@ -9258,88 +9263,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -9901,88 +9906,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>284</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -10543,88 +10548,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11705,88 +11710,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>253</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -12177,88 +12182,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>245</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -12909,88 +12914,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>238</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13900,88 +13905,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="93" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="93" t="s">
+      <c r="B1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="92" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="92" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14071,850 +14076,850 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="3" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="98">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="98" t="s">
         <v>90</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="98" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="92">
+      <c r="D3" s="99">
         <v>46283</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="98">
         <v>262665</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="98">
         <v>1749</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="98">
         <v>500</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="98">
         <v>1.494</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="98">
         <v>2.5630000000000002</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="98">
         <v>1914.5609999999999</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="98">
         <v>1281.5</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="98">
         <v>0.35599999999999998</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="98">
         <v>21.36</v>
       </c>
-      <c r="P3">
+      <c r="P3" s="98">
         <v>1087.5</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="98">
         <v>1</v>
       </c>
-      <c r="R3">
+      <c r="R3" s="98">
         <v>1550</v>
       </c>
-      <c r="S3">
+      <c r="S3" s="98">
         <v>1.494</v>
       </c>
-      <c r="T3">
+      <c r="T3" s="98">
         <v>56</v>
       </c>
-      <c r="U3">
+      <c r="U3" s="98">
         <v>3.61E-2</v>
       </c>
-      <c r="V3" t="s">
+      <c r="V3" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="98" t="s">
         <v>39</v>
       </c>
-      <c r="X3" t="s">
+      <c r="X3" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Y3" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="Z3" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="AA3">
+      <c r="AA3" s="98">
         <v>3</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AB3" s="98" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="4" spans="1:28" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="98">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="98" t="s">
         <v>90</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="98" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="92">
+      <c r="D4" s="99">
         <v>46283</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="98">
         <v>262666</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="98">
         <v>1749</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="98">
         <v>500</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="98">
         <v>1.444</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="98">
         <v>2.383</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="98">
         <v>1720.5260000000001</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="98">
         <v>1191.5</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="98">
         <v>0.33100000000000002</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="98">
         <v>19.86</v>
       </c>
-      <c r="P4">
+      <c r="P4" s="98">
         <v>977.3</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="98">
         <v>1</v>
       </c>
-      <c r="R4">
+      <c r="R4" s="98">
         <v>1500</v>
       </c>
-      <c r="S4">
+      <c r="S4" s="98">
         <v>1.444</v>
       </c>
-      <c r="T4">
+      <c r="T4" s="98">
         <v>56</v>
       </c>
-      <c r="U4">
+      <c r="U4" s="98">
         <v>3.73E-2</v>
       </c>
-      <c r="V4" t="s">
+      <c r="V4" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="W4" t="s">
+      <c r="W4" s="98" t="s">
         <v>39</v>
       </c>
-      <c r="X4" t="s">
+      <c r="X4" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Y4" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="Z4" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="AA4">
+      <c r="AA4" s="98">
         <v>3</v>
       </c>
-      <c r="AB4" t="s">
+      <c r="AB4" s="98" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="5" spans="1:28" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="5" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="98">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="98" t="s">
         <v>90</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="98" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="92">
+      <c r="D5" s="99">
         <v>46283</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="98">
         <v>262667</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="98">
         <v>1751</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="98">
         <v>400</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="98">
         <v>1.3879999999999999</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="98">
         <v>1.5029999999999999</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="98">
         <v>834.46600000000001</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="98">
         <v>601.20000000000005</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="98">
         <v>0.16700000000000001</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="98">
         <v>10.02</v>
       </c>
-      <c r="P5">
+      <c r="P5" s="98">
         <v>474</v>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="98">
         <v>1</v>
       </c>
-      <c r="R5">
+      <c r="R5" s="98">
         <v>1450</v>
       </c>
-      <c r="S5">
+      <c r="S5" s="98">
         <v>1.3879999999999999</v>
       </c>
-      <c r="T5">
+      <c r="T5" s="98">
         <v>62</v>
       </c>
-      <c r="U5">
+      <c r="U5" s="98">
         <v>4.2799999999999998E-2</v>
       </c>
-      <c r="V5" t="s">
+      <c r="V5" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="W5" t="s">
+      <c r="W5" s="98" t="s">
         <v>39</v>
       </c>
-      <c r="X5" t="s">
+      <c r="X5" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Y5" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="Z5" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="AA5">
+      <c r="AA5" s="98">
         <v>3</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="AB5" s="98" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="98">
         <v>4</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="42" t="s">
+      <c r="D6" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="E6" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="42">
+      <c r="E6" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="52">
         <v>262639</v>
       </c>
-      <c r="G6" s="42" t="s">
+      <c r="G6" s="52" t="s">
         <v>229</v>
       </c>
-      <c r="H6" s="42">
+      <c r="H6" s="52">
         <v>300</v>
       </c>
-      <c r="I6" s="43">
+      <c r="I6" s="54">
         <v>0.67400000000000004</v>
       </c>
-      <c r="J6" s="43">
+      <c r="J6" s="54">
         <v>1.5229999999999999</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="39">
+      <c r="L6" s="54">
         <v>307.95100000000002</v>
       </c>
-      <c r="M6" s="41">
+      <c r="M6" s="55">
         <v>228.4</v>
       </c>
-      <c r="N6" s="38">
+      <c r="N6" s="56">
         <v>3.1699999999999999E-2</v>
       </c>
-      <c r="O6" s="40">
+      <c r="O6" s="57">
         <v>1.9</v>
       </c>
-      <c r="P6" s="37">
+      <c r="P6" s="52">
         <v>174.9</v>
       </c>
-      <c r="Q6" s="37">
+      <c r="Q6" s="52">
         <v>2</v>
       </c>
-      <c r="R6" s="37">
+      <c r="R6" s="52">
         <v>1400</v>
       </c>
-      <c r="S6" s="39">
+      <c r="S6" s="54">
         <v>1.3480000000000001</v>
       </c>
-      <c r="T6" s="37">
+      <c r="T6" s="52">
         <v>52</v>
       </c>
-      <c r="U6" s="38">
+      <c r="U6" s="56">
         <v>3.7100000000000001E-2</v>
       </c>
-      <c r="V6" s="37" t="s">
+      <c r="V6" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="W6" s="37" t="s">
+      <c r="W6" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="X6" s="37" t="s">
+      <c r="X6" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Y6" s="37" t="s">
+      <c r="Y6" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Z6" s="37" t="s">
+      <c r="Z6" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="AA6" s="37" t="s">
+      <c r="AA6" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB6" s="37" t="s">
+      <c r="AB6" s="52" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="98">
         <v>5</v>
       </c>
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="42" t="s">
+      <c r="D7" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="E7" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="42">
+      <c r="E7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="52">
         <v>262637</v>
       </c>
-      <c r="G7" s="42" t="s">
+      <c r="G7" s="52" t="s">
         <v>227</v>
       </c>
-      <c r="H7" s="42">
+      <c r="H7" s="52">
         <v>500</v>
       </c>
-      <c r="I7" s="43">
+      <c r="I7" s="54">
         <v>0.56599999999999995</v>
       </c>
-      <c r="J7" s="43">
+      <c r="J7" s="54">
         <v>1.4630000000000001</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L7" s="39">
+      <c r="L7" s="54">
         <v>414.029</v>
       </c>
-      <c r="M7" s="41">
+      <c r="M7" s="55">
         <v>365.8</v>
       </c>
-      <c r="N7" s="38">
+      <c r="N7" s="56">
         <v>5.0799999999999998E-2</v>
       </c>
-      <c r="O7" s="40">
+      <c r="O7" s="57">
         <v>3.05</v>
       </c>
-      <c r="P7" s="37">
+      <c r="P7" s="52">
         <v>235.2</v>
       </c>
-      <c r="Q7" s="37">
+      <c r="Q7" s="52">
         <v>2</v>
       </c>
-      <c r="R7" s="37">
+      <c r="R7" s="52">
         <v>1200</v>
       </c>
-      <c r="S7" s="39">
+      <c r="S7" s="54">
         <v>1.1319999999999999</v>
       </c>
-      <c r="T7" s="37">
+      <c r="T7" s="52">
         <v>68</v>
       </c>
-      <c r="U7" s="38">
+      <c r="U7" s="56">
         <v>5.67E-2</v>
       </c>
-      <c r="V7" s="37" t="s">
+      <c r="V7" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="W7" s="37" t="s">
+      <c r="W7" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="X7" s="37" t="s">
+      <c r="X7" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Y7" s="37" t="s">
+      <c r="Y7" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Z7" s="37" t="s">
+      <c r="Z7" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="AA7" s="37" t="s">
+      <c r="AA7" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="37" t="s">
+      <c r="AB7" s="52" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8">
+    <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="98">
         <v>6</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="42" t="s">
+      <c r="D8" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="E8" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="42">
+      <c r="E8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="52">
         <v>262635</v>
       </c>
-      <c r="G8" s="42" t="s">
+      <c r="G8" s="52" t="s">
         <v>225</v>
       </c>
-      <c r="H8" s="42">
+      <c r="H8" s="52">
         <v>5000</v>
       </c>
-      <c r="I8" s="43">
+      <c r="I8" s="54">
         <v>0.55900000000000005</v>
       </c>
-      <c r="J8" s="43">
+      <c r="J8" s="54">
         <v>1.389</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L8" s="39">
+      <c r="L8" s="54">
         <v>3882.2550000000001</v>
       </c>
-      <c r="M8" s="41">
+      <c r="M8" s="55">
         <v>3472.5</v>
       </c>
-      <c r="N8" s="38">
+      <c r="N8" s="56">
         <v>0.48230000000000001</v>
       </c>
-      <c r="O8" s="40">
+      <c r="O8" s="57">
         <v>28.94</v>
       </c>
-      <c r="P8" s="37">
+      <c r="P8" s="52">
         <v>2205.1</v>
       </c>
-      <c r="Q8" s="37">
+      <c r="Q8" s="52">
         <v>2</v>
       </c>
-      <c r="R8" s="37">
+      <c r="R8" s="52">
         <v>1150</v>
       </c>
-      <c r="S8" s="39">
+      <c r="S8" s="54">
         <v>1.1180000000000001</v>
       </c>
-      <c r="T8" s="37">
+      <c r="T8" s="52">
         <v>32</v>
       </c>
-      <c r="U8" s="38">
+      <c r="U8" s="56">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="V8" s="37" t="s">
+      <c r="V8" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="W8" s="37" t="s">
+      <c r="W8" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="X8" s="37" t="s">
+      <c r="X8" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Y8" s="37" t="s">
+      <c r="Y8" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Z8" s="37" t="s">
+      <c r="Z8" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="AA8" s="37" t="s">
+      <c r="AA8" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="AB8" s="37" t="s">
+      <c r="AB8" s="52" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9">
+    <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="98">
         <v>7</v>
       </c>
-      <c r="B9" s="44" t="s">
+      <c r="B9" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="C9" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="42" t="s">
+      <c r="D9" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="E9" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="42">
+      <c r="E9" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="52">
         <v>262636</v>
       </c>
-      <c r="G9" s="42" t="s">
+      <c r="G9" s="52" t="s">
         <v>225</v>
       </c>
-      <c r="H9" s="42">
+      <c r="H9" s="52">
         <v>5000</v>
       </c>
-      <c r="I9" s="43">
+      <c r="I9" s="54">
         <v>0.55900000000000005</v>
       </c>
-      <c r="J9" s="43">
+      <c r="J9" s="54">
         <v>1.389</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L9" s="39">
+      <c r="L9" s="54">
         <v>3882.2550000000001</v>
       </c>
-      <c r="M9" s="41">
+      <c r="M9" s="55">
         <v>3472.5</v>
       </c>
-      <c r="N9" s="38">
+      <c r="N9" s="56">
         <v>0.48230000000000001</v>
       </c>
-      <c r="O9" s="40">
+      <c r="O9" s="57">
         <v>28.94</v>
       </c>
-      <c r="P9" s="37">
+      <c r="P9" s="52">
         <v>2205.1</v>
       </c>
-      <c r="Q9" s="37">
+      <c r="Q9" s="52">
         <v>2</v>
       </c>
-      <c r="R9" s="37">
+      <c r="R9" s="52">
         <v>1150</v>
       </c>
-      <c r="S9" s="39">
+      <c r="S9" s="54">
         <v>1.1180000000000001</v>
       </c>
-      <c r="T9" s="37">
+      <c r="T9" s="52">
         <v>32</v>
       </c>
-      <c r="U9" s="38">
+      <c r="U9" s="56">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="V9" s="37" t="s">
+      <c r="V9" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="W9" s="37" t="s">
+      <c r="W9" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="X9" s="37" t="s">
+      <c r="X9" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Y9" s="37" t="s">
+      <c r="Y9" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="Z9" s="37" t="s">
+      <c r="Z9" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="AA9" s="37" t="s">
+      <c r="AA9" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="AB9" s="37" t="s">
+      <c r="AB9" s="52" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10">
+    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="98">
         <v>8</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="42" t="s">
+      <c r="D10" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="E10" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="42">
+      <c r="E10" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="52">
         <v>262638</v>
       </c>
-      <c r="G10" s="42" t="s">
+      <c r="G10" s="52" t="s">
         <v>223</v>
       </c>
-      <c r="H10" s="42">
+      <c r="H10" s="52">
         <v>200</v>
       </c>
-      <c r="I10" s="43">
+      <c r="I10" s="54">
         <v>0.53800000000000003</v>
       </c>
-      <c r="J10" s="43">
+      <c r="J10" s="54">
         <v>1.423</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L10" s="39">
+      <c r="L10" s="54">
         <v>153.11500000000001</v>
       </c>
-      <c r="M10" s="41">
+      <c r="M10" s="55">
         <v>142.30000000000001</v>
       </c>
-      <c r="N10" s="38">
+      <c r="N10" s="56">
         <v>1.9800000000000002E-2</v>
       </c>
-      <c r="O10" s="40">
+      <c r="O10" s="57">
         <v>1.19</v>
       </c>
-      <c r="P10" s="37">
+      <c r="P10" s="52">
         <v>82.4</v>
       </c>
-      <c r="Q10" s="37">
+      <c r="Q10" s="52">
         <v>2</v>
       </c>
-      <c r="R10" s="37">
+      <c r="R10" s="52">
         <v>1100</v>
       </c>
-      <c r="S10" s="39">
+      <c r="S10" s="54">
         <v>1.0760000000000001</v>
       </c>
-      <c r="T10" s="37">
+      <c r="T10" s="52">
         <v>24</v>
       </c>
-      <c r="U10" s="38">
+      <c r="U10" s="56">
         <v>2.18E-2</v>
       </c>
-      <c r="V10" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="37" t="s">
+      <c r="V10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="X10" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z10" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA10" s="37" t="s">
+      <c r="X10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA10" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="AB10" s="37" t="s">
+      <c r="AB10" s="52" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11">
+    <row r="11" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="98">
         <v>9</v>
       </c>
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="91">
+      <c r="D11" s="68">
         <v>46282</v>
       </c>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42">
+      <c r="E11" s="52"/>
+      <c r="F11" s="52">
         <v>262643</v>
       </c>
-      <c r="G11" s="42">
+      <c r="G11" s="52">
         <v>1748</v>
       </c>
-      <c r="H11" s="42">
+      <c r="H11" s="52">
         <v>600</v>
       </c>
-      <c r="I11" s="43">
+      <c r="I11" s="54">
         <v>0.94899999999999995</v>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="54">
         <v>1.536</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="L11" s="39">
+      <c r="L11" s="54">
         <v>874.59799999999996</v>
       </c>
-      <c r="M11" s="41">
+      <c r="M11" s="55">
         <v>921.6</v>
       </c>
-      <c r="N11" s="38">
+      <c r="N11" s="56">
         <v>0.25600000000000001</v>
       </c>
-      <c r="O11" s="40">
+      <c r="O11" s="57">
         <v>15.36</v>
       </c>
-      <c r="P11" s="37">
+      <c r="P11" s="52">
         <v>275.5</v>
       </c>
-      <c r="Q11" s="37">
+      <c r="Q11" s="52">
         <v>1</v>
       </c>
-      <c r="R11" s="37">
+      <c r="R11" s="52">
         <v>1000</v>
       </c>
-      <c r="S11" s="39">
+      <c r="S11" s="54">
         <v>0.94899999999999995</v>
       </c>
-      <c r="T11" s="37">
+      <c r="T11" s="52">
         <v>51</v>
       </c>
-      <c r="U11" s="38">
+      <c r="U11" s="56">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="V11" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="37"/>
-      <c r="Z11" s="37"/>
-      <c r="AA11" s="37">
+      <c r="V11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="52"/>
+      <c r="Z11" s="52"/>
+      <c r="AA11" s="52">
         <v>2</v>
       </c>
-      <c r="AB11" s="37" t="s">
+      <c r="AB11" s="52" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="36">
+    <row r="12" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="59">
         <f>SUM(H3:H11)</f>
         <v>13000</v>
       </c>
-      <c r="I12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="35">
+      <c r="I12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="59">
         <f>SUM(P3:P11)</f>
         <v>7717</v>
       </c>
-      <c r="Q12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="35" t="s">
+      <c r="Q12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB12" s="59" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14964,88 +14969,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="93" t="s">
         <v>220</v>
       </c>
-      <c r="B1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="94" t="s">
+      <c r="B1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="93" t="s">
         <v>27</v>
       </c>
     </row>
@@ -15612,88 +15617,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="93" t="s">
         <v>239</v>
       </c>
-      <c r="B1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="94" t="s">
+      <c r="B1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="93" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (23/09/2026 09:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EE718D-169E-4DE8-8DCC-68CDFCA40164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D599C30-3F8D-4D3C-A89E-27CAEAF954B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="9" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Z4A EMBALAGENS LTDA 1216" sheetId="161" r:id="rId4"/>
     <sheet name="Tolecaixas 1215" sheetId="160" r:id="rId5"/>
     <sheet name="ABAPEL 1213" sheetId="159" r:id="rId6"/>
-    <sheet name="IPE - PCBOX 1212" sheetId="158" r:id="rId7"/>
+    <sheet name="IPE - PCBOX 1212 P" sheetId="158" r:id="rId7"/>
     <sheet name="Z4A EMBALAGENS LTDA 1210 P" sheetId="157" r:id="rId8"/>
     <sheet name="RM Embalagens 1209 P" sheetId="156" r:id="rId9"/>
     <sheet name="ABAPEL 1201" sheetId="153" r:id="rId10"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2774" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2783" uniqueCount="307">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -964,6 +964,12 @@
   </si>
   <si>
     <t>750x2000</t>
+  </si>
+  <si>
+    <t>ABAPEL COMERCIO DE EMBALAOENS LTDA</t>
+  </si>
+  <si>
+    <t>940x1240</t>
   </si>
 </sst>
 </file>
@@ -975,7 +981,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1102,6 +1108,13 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1168,7 +1181,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1451,6 +1464,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2319,7 +2336,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5AF4CA-00D7-4A30-8F64-AC13CDBB2809}">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
@@ -2869,88 +2886,174 @@
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="11">
-        <v>2900</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="11">
-        <v>2419.3000000000002</v>
-      </c>
-      <c r="Q7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB7" s="11" t="s">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>305</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="101">
+        <v>46288</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5">
+        <v>262681</v>
+      </c>
+      <c r="G7" s="5">
+        <v>8207</v>
+      </c>
+      <c r="H7" s="5">
+        <v>410</v>
+      </c>
+      <c r="I7" s="7">
+        <v>0.92</v>
+      </c>
+      <c r="J7" s="7">
+        <v>1.22</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L7" s="7">
+        <v>460.18400000000003</v>
+      </c>
+      <c r="M7" s="9">
+        <v>500.2</v>
+      </c>
+      <c r="N7" s="6">
+        <v>0.1389</v>
+      </c>
+      <c r="O7" s="8">
+        <v>8.34</v>
+      </c>
+      <c r="P7" s="5">
+        <v>247.6</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>1</v>
+      </c>
+      <c r="R7" s="5">
+        <v>950</v>
+      </c>
+      <c r="S7" s="7">
+        <v>0.92</v>
+      </c>
+      <c r="T7" s="5">
+        <v>30</v>
+      </c>
+      <c r="U7" s="6">
+        <v>3.1600000000000003E-2</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="5">
+        <v>3</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="11">
+        <f>SUM(H3:H7)</f>
+        <v>3310</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="11">
+        <f>SUM(P3:P7)</f>
+        <v>2667</v>
+      </c>
+      <c r="Q8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6201,88 +6304,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="100" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="92" t="s">
+      <c r="B1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="100" t="s">
         <v>27</v>
       </c>
     </row>
@@ -7237,6 +7340,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13871,6 +13975,9 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00EADB3A-C171-49AE-8471-729057A3A740}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -13905,88 +14012,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="93" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="92" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="92" t="s">
+      <c r="B1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="93" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14929,6 +15036,7 @@
   </mergeCells>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (23/09/2026 09:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D599C30-3F8D-4D3C-A89E-27CAEAF954B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74321D3-D5E0-44C4-A731-8B62523DFA73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="9" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="ABAPEL 1201" sheetId="153" r:id="rId10"/>
     <sheet name="HARMONY EMBALAGENS 1200" sheetId="152" r:id="rId11"/>
     <sheet name="FAVINCO EMBALAGENS 1197 P" sheetId="150" r:id="rId12"/>
-    <sheet name="ABAPEL 1196" sheetId="149" r:id="rId13"/>
+    <sheet name="ABAPEL 1196 P" sheetId="149" r:id="rId13"/>
     <sheet name="RM Embalagens 1184 P" sheetId="141" r:id="rId14"/>
     <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId15"/>
     <sheet name="Carpel 1158 P" sheetId="119" r:id="rId16"/>
@@ -981,7 +981,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1108,13 +1108,6 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1181,7 +1174,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1464,7 +1457,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="14" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2895,7 +2887,7 @@
       <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="101">
+      <c r="D7" s="100">
         <v>46288</v>
       </c>
       <c r="E7" s="5"/>
@@ -6271,6 +6263,9 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BFDD7F-F2DE-484D-858D-A0AEE46D68A8}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6304,88 +6299,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="93" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="100" t="s">
+      <c r="B1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="93" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6475,7 +6470,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="69">
         <v>1</v>
       </c>
@@ -6561,7 +6556,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="69">
         <v>2</v>
       </c>
@@ -6647,7 +6642,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="69">
         <v>3</v>
       </c>
@@ -6733,7 +6728,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="69">
         <v>4</v>
       </c>
@@ -6819,7 +6814,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="69">
         <v>5</v>
       </c>
@@ -6905,7 +6900,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="69">
         <v>6</v>
       </c>
@@ -6991,7 +6986,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="69">
         <v>7</v>
       </c>
@@ -7077,7 +7072,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="69">
         <v>8</v>
       </c>
@@ -7163,7 +7158,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="75" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="69">
         <v>9</v>
       </c>
@@ -7249,7 +7244,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="67" t="s">
         <v>27</v>
       </c>
@@ -7339,8 +7334,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.72" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup scale="75" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (23/09/2026 10:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74321D3-D5E0-44C4-A731-8B62523DFA73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{165E8C47-23F5-401B-8B0E-31A40344A5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <sheet name="IPE - PCBOX 1212 P" sheetId="158" r:id="rId7"/>
     <sheet name="Z4A EMBALAGENS LTDA 1210 P" sheetId="157" r:id="rId8"/>
     <sheet name="RM Embalagens 1209 P" sheetId="156" r:id="rId9"/>
-    <sheet name="ABAPEL 1201" sheetId="153" r:id="rId10"/>
+    <sheet name="ABAPEL 1201 P" sheetId="153" r:id="rId10"/>
     <sheet name="HARMONY EMBALAGENS 1200" sheetId="152" r:id="rId11"/>
     <sheet name="FAVINCO EMBALAGENS 1197 P" sheetId="150" r:id="rId12"/>
     <sheet name="ABAPEL 1196 P" sheetId="149" r:id="rId13"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2783" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2780" uniqueCount="307">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -468,12 +468,6 @@
     <t>873x2125</t>
   </si>
   <si>
-    <t>1175x2150</t>
-  </si>
-  <si>
-    <t>70x70x75x70x400x75x335x60</t>
-  </si>
-  <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - ABAPEL COMERCIO DE EMBALAGENS LTDA  —  OF: 001196</t>
   </si>
   <si>
@@ -970,6 +964,12 @@
   </si>
   <si>
     <t>940x1240</t>
+  </si>
+  <si>
+    <t>W55R23</t>
+  </si>
+  <si>
+    <t>1185x2150</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1174,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1460,6 +1460,10 @@
     <xf numFmtId="14" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="15" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1718,7 +1722,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="92" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B1" s="92" t="s">
         <v>27</v>
@@ -1899,7 +1903,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E3" s="42" t="s">
         <v>27</v>
@@ -1908,7 +1912,7 @@
         <v>262676</v>
       </c>
       <c r="G3" s="42" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H3" s="42">
         <v>200</v>
@@ -1971,7 +1975,7 @@
         <v>32</v>
       </c>
       <c r="AB3" s="37" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -1985,7 +1989,7 @@
         <v>35</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E4" s="42" t="s">
         <v>27</v>
@@ -1994,7 +1998,7 @@
         <v>262678</v>
       </c>
       <c r="G4" s="42" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="H4" s="42">
         <v>250</v>
@@ -2057,7 +2061,7 @@
         <v>38</v>
       </c>
       <c r="AB4" s="37" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -2071,7 +2075,7 @@
         <v>35</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E5" s="42" t="s">
         <v>27</v>
@@ -2080,7 +2084,7 @@
         <v>262679</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="H5" s="42">
         <v>150</v>
@@ -2143,7 +2147,7 @@
         <v>38</v>
       </c>
       <c r="AB5" s="37" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
@@ -2157,7 +2161,7 @@
         <v>42</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E6" s="42" t="s">
         <v>27</v>
@@ -2166,7 +2170,7 @@
         <v>262677</v>
       </c>
       <c r="G6" s="42" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="H6" s="42">
         <v>1000</v>
@@ -2229,7 +2233,7 @@
         <v>32</v>
       </c>
       <c r="AB6" s="37" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
@@ -2328,6 +2332,9 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5AF4CA-00D7-4A30-8F64-AC13CDBB2809}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2362,88 +2369,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="94" t="s">
-        <v>183</v>
-      </c>
-      <c r="B1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="94" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="94" t="s">
+      <c r="A1" s="101" t="s">
+        <v>181</v>
+      </c>
+      <c r="B1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="101" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2544,7 +2551,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>27</v>
@@ -2553,7 +2560,7 @@
         <v>262601</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H3" s="5">
         <v>1000</v>
@@ -2565,7 +2572,7 @@
         <v>2.19</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="L3" s="7">
         <v>1559.28</v>
@@ -2616,7 +2623,7 @@
         <v>40</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2630,7 +2637,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>27</v>
@@ -2639,7 +2646,7 @@
         <v>262600</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H4" s="5">
         <v>900</v>
@@ -2702,7 +2709,7 @@
         <v>48</v>
       </c>
       <c r="AB4" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2716,7 +2723,7 @@
         <v>26</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>27</v>
@@ -2725,7 +2732,7 @@
         <v>262599</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H5" s="5">
         <v>450</v>
@@ -2737,7 +2744,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="L5" s="7">
         <v>615.78</v>
@@ -2788,7 +2795,7 @@
         <v>30</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2802,7 +2809,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>27</v>
@@ -2811,7 +2818,7 @@
         <v>262598</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H6" s="5">
         <v>550</v>
@@ -2874,7 +2881,7 @@
         <v>30</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2882,7 +2889,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>26</v>
@@ -2958,7 +2965,7 @@
         <v>3</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3053,7 +3060,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.39" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="94" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3097,7 +3105,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="94" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B1" s="94" t="s">
         <v>27</v>
@@ -3278,7 +3286,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>27</v>
@@ -3287,7 +3295,7 @@
         <v>262591</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H3" s="5">
         <v>1250</v>
@@ -3350,7 +3358,7 @@
         <v>31</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="84" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3364,7 +3372,7 @@
         <v>57</v>
       </c>
       <c r="D4" s="85" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E4" s="85" t="s">
         <v>27</v>
@@ -3373,7 +3381,7 @@
         <v>262597</v>
       </c>
       <c r="G4" s="85" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H4" s="85">
         <v>600</v>
@@ -3450,7 +3458,7 @@
         <v>57</v>
       </c>
       <c r="D5" s="85" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E5" s="85" t="s">
         <v>27</v>
@@ -3459,7 +3467,7 @@
         <v>262596</v>
       </c>
       <c r="G5" s="85" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H5" s="85">
         <v>2000</v>
@@ -3536,7 +3544,7 @@
         <v>44</v>
       </c>
       <c r="D6" s="85" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E6" s="85" t="s">
         <v>27</v>
@@ -3545,7 +3553,7 @@
         <v>262595</v>
       </c>
       <c r="G6" s="85" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H6" s="85">
         <v>1400</v>
@@ -3622,7 +3630,7 @@
         <v>26</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>27</v>
@@ -3631,7 +3639,7 @@
         <v>262589</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H7" s="5">
         <v>1250</v>
@@ -3694,7 +3702,7 @@
         <v>54</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3708,7 +3716,7 @@
         <v>26</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>27</v>
@@ -3717,7 +3725,7 @@
         <v>262590</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H8" s="5">
         <v>5000</v>
@@ -3780,7 +3788,7 @@
         <v>66</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3794,7 +3802,7 @@
         <v>35</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>27</v>
@@ -3803,7 +3811,7 @@
         <v>262588</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H9" s="5">
         <v>3000</v>
@@ -3866,7 +3874,7 @@
         <v>32</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3880,7 +3888,7 @@
         <v>35</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>27</v>
@@ -3889,7 +3897,7 @@
         <v>262586</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H10" s="5">
         <v>3000</v>
@@ -3952,7 +3960,7 @@
         <v>38</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3966,7 +3974,7 @@
         <v>35</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>27</v>
@@ -3975,7 +3983,7 @@
         <v>262587</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H11" s="5">
         <v>2000</v>
@@ -4038,7 +4046,7 @@
         <v>38</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4052,7 +4060,7 @@
         <v>42</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>27</v>
@@ -4061,7 +4069,7 @@
         <v>262583</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H12" s="5">
         <v>450</v>
@@ -4073,7 +4081,7 @@
         <v>1.169</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="L12" s="7">
         <v>270.39</v>
@@ -4124,7 +4132,7 @@
         <v>38</v>
       </c>
       <c r="AB12" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4138,7 +4146,7 @@
         <v>42</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>27</v>
@@ -4147,7 +4155,7 @@
         <v>262592</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H13" s="5">
         <v>270</v>
@@ -4210,7 +4218,7 @@
         <v>38</v>
       </c>
       <c r="AB13" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4224,7 +4232,7 @@
         <v>35</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>27</v>
@@ -4233,7 +4241,7 @@
         <v>262593</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H14" s="5">
         <v>500</v>
@@ -4296,7 +4304,7 @@
         <v>38</v>
       </c>
       <c r="AB14" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4310,7 +4318,7 @@
         <v>42</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>27</v>
@@ -4319,7 +4327,7 @@
         <v>262584</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H15" s="5">
         <v>550</v>
@@ -4331,7 +4339,7 @@
         <v>1.0489999999999999</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="L15" s="7">
         <v>256.166</v>
@@ -4382,7 +4390,7 @@
         <v>38</v>
       </c>
       <c r="AB15" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4396,7 +4404,7 @@
         <v>35</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>27</v>
@@ -4405,7 +4413,7 @@
         <v>262585</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H16" s="5">
         <v>550</v>
@@ -4468,7 +4476,7 @@
         <v>38</v>
       </c>
       <c r="AB16" s="5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4482,7 +4490,7 @@
         <v>35</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>27</v>
@@ -4491,7 +4499,7 @@
         <v>262594</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H17" s="5">
         <v>600</v>
@@ -4554,7 +4562,7 @@
         <v>32</v>
       </c>
       <c r="AB17" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4568,7 +4576,7 @@
         <v>49</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>27</v>
@@ -4577,7 +4585,7 @@
         <v>262581</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H18" s="5">
         <v>1000</v>
@@ -4589,7 +4597,7 @@
         <v>0.94899999999999995</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="L18" s="7">
         <v>317.91500000000002</v>
@@ -4640,7 +4648,7 @@
         <v>38</v>
       </c>
       <c r="AB18" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4654,7 +4662,7 @@
         <v>35</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>27</v>
@@ -4663,7 +4671,7 @@
         <v>262582</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H19" s="5">
         <v>1300</v>
@@ -4675,7 +4683,7 @@
         <v>0.78900000000000003</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="L19" s="7">
         <v>342.584</v>
@@ -4726,7 +4734,7 @@
         <v>38</v>
       </c>
       <c r="AB19" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4864,7 +4872,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="93" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B1" s="93" t="s">
         <v>27</v>
@@ -5054,7 +5062,7 @@
         <v>262575</v>
       </c>
       <c r="G3" s="60" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H3" s="60">
         <v>600</v>
@@ -5066,7 +5074,7 @@
         <v>0.95</v>
       </c>
       <c r="K3" s="60" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="L3" s="62">
         <v>309.51</v>
@@ -5117,7 +5125,7 @@
         <v>38</v>
       </c>
       <c r="AB3" s="60" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5150,7 +5158,7 @@
         <v>2.41</v>
       </c>
       <c r="K4" s="60" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L4" s="62">
         <v>804.69899999999996</v>
@@ -5201,7 +5209,7 @@
         <v>2</v>
       </c>
       <c r="AB4" s="60" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5212,7 +5220,7 @@
         <v>93</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D5" s="76">
         <v>46279</v>
@@ -5234,7 +5242,7 @@
         <v>1.29</v>
       </c>
       <c r="K5" s="60" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="L5" s="62">
         <v>677.25</v>
@@ -5281,7 +5289,7 @@
         <v>2</v>
       </c>
       <c r="AB5" s="60" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5292,7 +5300,7 @@
         <v>93</v>
       </c>
       <c r="C6" s="60" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D6" s="76">
         <v>46279</v>
@@ -5314,7 +5322,7 @@
         <v>1.59</v>
       </c>
       <c r="K6" s="60" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L6" s="62">
         <v>357.75</v>
@@ -5361,7 +5369,7 @@
         <v>1</v>
       </c>
       <c r="AB6" s="60" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5372,7 +5380,7 @@
         <v>93</v>
       </c>
       <c r="C7" s="60" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D7" s="76">
         <v>46279</v>
@@ -5394,7 +5402,7 @@
         <v>1.41</v>
       </c>
       <c r="K7" s="60" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L7" s="62">
         <v>461.916</v>
@@ -5441,7 +5449,7 @@
         <v>1</v>
       </c>
       <c r="AB7" s="60" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5521,7 +5529,7 @@
         <v>7</v>
       </c>
       <c r="AB8" s="60" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5601,7 +5609,7 @@
         <v>1</v>
       </c>
       <c r="AB9" s="60" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5681,7 +5689,7 @@
         <v>1</v>
       </c>
       <c r="AB10" s="60" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5761,7 +5769,7 @@
         <v>1</v>
       </c>
       <c r="AB11" s="60" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5794,7 +5802,7 @@
         <v>1.3420000000000001</v>
       </c>
       <c r="K12" s="60" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="L12" s="62">
         <v>1379.576</v>
@@ -5841,7 +5849,7 @@
         <v>3</v>
       </c>
       <c r="AB12" s="60" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5921,7 +5929,7 @@
         <v>2</v>
       </c>
       <c r="AB13" s="60" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5954,7 +5962,7 @@
         <v>1.002</v>
       </c>
       <c r="K14" s="60" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="L14" s="62">
         <v>559.11599999999999</v>
@@ -6001,7 +6009,7 @@
         <v>1</v>
       </c>
       <c r="AB14" s="60" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6034,7 +6042,7 @@
         <v>1.04</v>
       </c>
       <c r="K15" s="60" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="L15" s="62">
         <v>2277.6</v>
@@ -6081,7 +6089,7 @@
         <v>3</v>
       </c>
       <c r="AB15" s="60" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6114,7 +6122,7 @@
         <v>1.004</v>
       </c>
       <c r="K16" s="52" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="L16" s="54">
         <v>840.34799999999996</v>
@@ -6300,7 +6308,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="93" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B1" s="93" t="s">
         <v>27</v>
@@ -6480,32 +6488,30 @@
       <c r="C3" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="69" t="s">
-        <v>125</v>
-      </c>
-      <c r="E3" s="69" t="s">
-        <v>27</v>
-      </c>
+      <c r="D3" s="102">
+        <v>46288</v>
+      </c>
+      <c r="E3" s="69"/>
       <c r="F3" s="69">
-        <v>262566</v>
+        <v>262682</v>
       </c>
       <c r="G3" s="69" t="s">
-        <v>130</v>
+        <v>305</v>
       </c>
       <c r="H3" s="69">
         <v>450</v>
       </c>
       <c r="I3" s="71">
-        <v>1.155</v>
+        <v>1.165</v>
       </c>
       <c r="J3" s="71">
         <v>2.13</v>
       </c>
       <c r="K3" s="69" t="s">
-        <v>140</v>
+        <v>33</v>
       </c>
       <c r="L3" s="71">
-        <v>1107.068</v>
+        <v>1116.653</v>
       </c>
       <c r="M3" s="72">
         <v>958.5</v>
@@ -6517,7 +6523,7 @@
         <v>15.97</v>
       </c>
       <c r="P3" s="69">
-        <v>656.5</v>
+        <v>600.79999999999995</v>
       </c>
       <c r="Q3" s="69">
         <v>1</v>
@@ -6526,13 +6532,13 @@
         <v>1200</v>
       </c>
       <c r="S3" s="71">
-        <v>1.155</v>
+        <v>1.165</v>
       </c>
       <c r="T3" s="69">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="U3" s="73">
-        <v>3.7499999999999999E-2</v>
+        <v>2.92E-2</v>
       </c>
       <c r="V3" s="69" t="s">
         <v>28</v>
@@ -6549,11 +6555,11 @@
       <c r="Z3" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="AA3" s="69" t="s">
-        <v>30</v>
+      <c r="AA3" s="69">
+        <v>3</v>
       </c>
       <c r="AB3" s="69" t="s">
-        <v>139</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="75" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -10006,7 +10012,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="92" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B1" s="92" t="s">
         <v>27</v>
@@ -10181,13 +10187,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C3" s="42" t="s">
         <v>44</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E3" s="42" t="s">
         <v>27</v>
@@ -10196,7 +10202,7 @@
         <v>262670</v>
       </c>
       <c r="G3" s="42" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H3" s="42">
         <v>1050</v>
@@ -10208,7 +10214,7 @@
         <v>1.33</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="L3" s="39">
         <v>794.60799999999995</v>
@@ -10259,7 +10265,7 @@
         <v>30</v>
       </c>
       <c r="AB3" s="37" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -10267,13 +10273,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C4" s="42" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E4" s="42" t="s">
         <v>27</v>
@@ -10282,7 +10288,7 @@
         <v>262669</v>
       </c>
       <c r="G4" s="42" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H4" s="42">
         <v>3100</v>
@@ -10294,7 +10300,7 @@
         <v>1.67</v>
       </c>
       <c r="K4" s="42" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="L4" s="39">
         <v>5793.0630000000001</v>
@@ -10345,7 +10351,7 @@
         <v>64</v>
       </c>
       <c r="AB4" s="37" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -10353,13 +10359,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E5" s="42" t="s">
         <v>27</v>
@@ -10368,7 +10374,7 @@
         <v>262668</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H5" s="42">
         <v>4200</v>
@@ -10380,7 +10386,7 @@
         <v>1.48</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="L5" s="39">
         <v>5463.8639999999996</v>
@@ -10428,10 +10434,10 @@
         <v>34</v>
       </c>
       <c r="AA5" s="37" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="AB5" s="37" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
@@ -10439,7 +10445,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C6" s="42" t="s">
         <v>26</v>
@@ -10515,7 +10521,7 @@
         <v>3</v>
       </c>
       <c r="AB6" s="37" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
@@ -10648,7 +10654,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="92" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B1" s="92" t="s">
         <v>27</v>
@@ -10829,7 +10835,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E3" s="52" t="s">
         <v>27</v>
@@ -10838,7 +10844,7 @@
         <v>262658</v>
       </c>
       <c r="G3" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H3" s="52">
         <v>300</v>
@@ -10915,7 +10921,7 @@
         <v>35</v>
       </c>
       <c r="D4" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E4" s="52" t="s">
         <v>27</v>
@@ -10924,7 +10930,7 @@
         <v>262656</v>
       </c>
       <c r="G4" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H4" s="52">
         <v>1000</v>
@@ -10936,7 +10942,7 @@
         <v>0.69299999999999995</v>
       </c>
       <c r="K4" s="52" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="L4" s="54">
         <v>528.06600000000003</v>
@@ -10987,7 +10993,7 @@
         <v>38</v>
       </c>
       <c r="AB4" s="52" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11001,7 +11007,7 @@
         <v>35</v>
       </c>
       <c r="D5" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E5" s="52" t="s">
         <v>27</v>
@@ -11010,7 +11016,7 @@
         <v>262651</v>
       </c>
       <c r="G5" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H5" s="52">
         <v>400</v>
@@ -11073,7 +11079,7 @@
         <v>38</v>
       </c>
       <c r="AB5" s="52" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11087,7 +11093,7 @@
         <v>35</v>
       </c>
       <c r="D6" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E6" s="52" t="s">
         <v>27</v>
@@ -11096,7 +11102,7 @@
         <v>262653</v>
       </c>
       <c r="G6" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H6" s="52">
         <v>400</v>
@@ -11159,7 +11165,7 @@
         <v>38</v>
       </c>
       <c r="AB6" s="52" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11173,7 +11179,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E7" s="52" t="s">
         <v>27</v>
@@ -11182,7 +11188,7 @@
         <v>262654</v>
       </c>
       <c r="G7" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H7" s="52">
         <v>600</v>
@@ -11194,7 +11200,7 @@
         <v>1.2490000000000001</v>
       </c>
       <c r="K7" s="52" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="L7" s="54">
         <v>497.60199999999998</v>
@@ -11245,7 +11251,7 @@
         <v>32</v>
       </c>
       <c r="AB7" s="52" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11259,7 +11265,7 @@
         <v>35</v>
       </c>
       <c r="D8" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E8" s="52" t="s">
         <v>27</v>
@@ -11268,7 +11274,7 @@
         <v>262657</v>
       </c>
       <c r="G8" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H8" s="52">
         <v>600</v>
@@ -11280,7 +11286,7 @@
         <v>0.69299999999999995</v>
       </c>
       <c r="K8" s="52" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="L8" s="54">
         <v>479.00200000000001</v>
@@ -11331,7 +11337,7 @@
         <v>38</v>
       </c>
       <c r="AB8" s="52" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11345,7 +11351,7 @@
         <v>35</v>
       </c>
       <c r="D9" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E9" s="52" t="s">
         <v>27</v>
@@ -11354,7 +11360,7 @@
         <v>262655</v>
       </c>
       <c r="G9" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H9" s="52">
         <v>2500</v>
@@ -11417,7 +11423,7 @@
         <v>38</v>
       </c>
       <c r="AB9" s="52" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11431,7 +11437,7 @@
         <v>35</v>
       </c>
       <c r="D10" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E10" s="52" t="s">
         <v>27</v>
@@ -11440,7 +11446,7 @@
         <v>262652</v>
       </c>
       <c r="G10" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H10" s="52">
         <v>400</v>
@@ -11503,7 +11509,7 @@
         <v>38</v>
       </c>
       <c r="AB10" s="52" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11517,7 +11523,7 @@
         <v>35</v>
       </c>
       <c r="D11" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E11" s="52" t="s">
         <v>27</v>
@@ -11526,7 +11532,7 @@
         <v>262660</v>
       </c>
       <c r="G11" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H11" s="52">
         <v>1500</v>
@@ -11538,7 +11544,7 @@
         <v>0.78900000000000003</v>
       </c>
       <c r="K11" s="52" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L11" s="54">
         <v>501.80399999999997</v>
@@ -11589,7 +11595,7 @@
         <v>38</v>
       </c>
       <c r="AB11" s="52" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11603,7 +11609,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="52" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E12" s="52" t="s">
         <v>27</v>
@@ -11612,7 +11618,7 @@
         <v>262659</v>
       </c>
       <c r="G12" s="52" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H12" s="52">
         <v>3000</v>
@@ -11624,7 +11630,7 @@
         <v>0.72899999999999998</v>
       </c>
       <c r="K12" s="52" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L12" s="54">
         <v>804.81600000000003</v>
@@ -11675,7 +11681,7 @@
         <v>32</v>
       </c>
       <c r="AB12" s="52" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11810,7 +11816,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="92" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B1" s="92" t="s">
         <v>27</v>
@@ -11991,7 +11997,7 @@
         <v>81</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E3" s="42" t="s">
         <v>27</v>
@@ -12000,7 +12006,7 @@
         <v>262649</v>
       </c>
       <c r="G3" s="42" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H3" s="42">
         <v>2600</v>
@@ -12012,7 +12018,7 @@
         <v>1.2629999999999999</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="L3" s="39">
         <v>1615.63</v>
@@ -12063,7 +12069,7 @@
         <v>31</v>
       </c>
       <c r="AB3" s="37" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -12077,7 +12083,7 @@
         <v>81</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E4" s="42" t="s">
         <v>27</v>
@@ -12086,7 +12092,7 @@
         <v>262650</v>
       </c>
       <c r="G4" s="42" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H4" s="42">
         <v>2300</v>
@@ -12098,7 +12104,7 @@
         <v>1.393</v>
       </c>
       <c r="K4" s="42" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L4" s="39">
         <v>1464.182</v>
@@ -12149,7 +12155,7 @@
         <v>30</v>
       </c>
       <c r="AB4" s="37" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -12282,7 +12288,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="92" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B1" s="92" t="s">
         <v>27</v>
@@ -12463,7 +12469,7 @@
         <v>55</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E3" s="42" t="s">
         <v>27</v>
@@ -12472,7 +12478,7 @@
         <v>262645</v>
       </c>
       <c r="G3" s="42" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H3" s="42">
         <v>2740</v>
@@ -12535,7 +12541,7 @@
         <v>31</v>
       </c>
       <c r="AB3" s="37" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12549,7 +12555,7 @@
         <v>55</v>
       </c>
       <c r="D4" s="42" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E4" s="42" t="s">
         <v>27</v>
@@ -12558,7 +12564,7 @@
         <v>262644</v>
       </c>
       <c r="G4" s="42" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H4" s="42">
         <v>1662</v>
@@ -12621,7 +12627,7 @@
         <v>32</v>
       </c>
       <c r="AB4" s="37" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12635,7 +12641,7 @@
         <v>55</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E5" s="42" t="s">
         <v>27</v>
@@ -12644,7 +12650,7 @@
         <v>262646</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H5" s="42">
         <v>1140</v>
@@ -12707,7 +12713,7 @@
         <v>32</v>
       </c>
       <c r="AB5" s="37" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -12721,7 +12727,7 @@
         <v>49</v>
       </c>
       <c r="D6" s="42" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E6" s="42" t="s">
         <v>27</v>
@@ -12730,7 +12736,7 @@
         <v>262647</v>
       </c>
       <c r="G6" s="42" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H6" s="42">
         <v>3052</v>
@@ -12807,7 +12813,7 @@
         <v>49</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E7" s="42" t="s">
         <v>27</v>
@@ -12816,7 +12822,7 @@
         <v>262648</v>
       </c>
       <c r="G7" s="42" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H7" s="42">
         <v>3317</v>
@@ -13014,7 +13020,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="92" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B1" s="92" t="s">
         <v>27</v>
@@ -13195,7 +13201,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="46" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E3" s="46" t="s">
         <v>27</v>
@@ -13204,7 +13210,7 @@
         <v>262674</v>
       </c>
       <c r="G3" s="46" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H3" s="46">
         <v>400</v>
@@ -13216,7 +13222,7 @@
         <v>2.38</v>
       </c>
       <c r="K3" s="46" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="L3" s="48">
         <v>1306.144</v>
@@ -13267,7 +13273,7 @@
         <v>30</v>
       </c>
       <c r="AB3" s="46" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13281,7 +13287,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="46" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E4" s="46" t="s">
         <v>27</v>
@@ -13290,7 +13296,7 @@
         <v>262672</v>
       </c>
       <c r="G4" s="46" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H4" s="46">
         <v>400</v>
@@ -13302,7 +13308,7 @@
         <v>2.34</v>
       </c>
       <c r="K4" s="46" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="L4" s="48">
         <v>1078.2719999999999</v>
@@ -13353,7 +13359,7 @@
         <v>30</v>
       </c>
       <c r="AB4" s="46" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13367,7 +13373,7 @@
         <v>26</v>
       </c>
       <c r="D5" s="46" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E5" s="46" t="s">
         <v>27</v>
@@ -13376,7 +13382,7 @@
         <v>262671</v>
       </c>
       <c r="G5" s="46" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H5" s="46">
         <v>400</v>
@@ -13388,7 +13394,7 @@
         <v>2.339</v>
       </c>
       <c r="K5" s="46" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="L5" s="48">
         <v>1264.931</v>
@@ -13439,7 +13445,7 @@
         <v>30</v>
       </c>
       <c r="AB5" s="46" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13453,7 +13459,7 @@
         <v>59</v>
       </c>
       <c r="D6" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E6" s="52" t="s">
         <v>27</v>
@@ -13462,7 +13468,7 @@
         <v>262640</v>
       </c>
       <c r="G6" s="52" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H6" s="52">
         <v>800</v>
@@ -13474,7 +13480,7 @@
         <v>1.6739999999999999</v>
       </c>
       <c r="K6" s="52" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="L6" s="54">
         <v>980.29399999999998</v>
@@ -13525,7 +13531,7 @@
         <v>30</v>
       </c>
       <c r="AB6" s="52" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13539,7 +13545,7 @@
         <v>59</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E7" s="52" t="s">
         <v>27</v>
@@ -13548,7 +13554,7 @@
         <v>262641</v>
       </c>
       <c r="G7" s="52" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H7" s="52">
         <v>1150</v>
@@ -13560,7 +13566,7 @@
         <v>1.44</v>
       </c>
       <c r="K7" s="52" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L7" s="54">
         <v>905.83199999999999</v>
@@ -13611,7 +13617,7 @@
         <v>32</v>
       </c>
       <c r="AB7" s="52" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13625,7 +13631,7 @@
         <v>35</v>
       </c>
       <c r="D8" s="46" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E8" s="46" t="s">
         <v>27</v>
@@ -13634,7 +13640,7 @@
         <v>262673</v>
       </c>
       <c r="G8" s="46" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H8" s="46">
         <v>1000</v>
@@ -13697,7 +13703,7 @@
         <v>32</v>
       </c>
       <c r="AB8" s="46" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13711,7 +13717,7 @@
         <v>35</v>
       </c>
       <c r="D9" s="46" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E9" s="46" t="s">
         <v>27</v>
@@ -13720,7 +13726,7 @@
         <v>262675</v>
       </c>
       <c r="G9" s="46" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="H9" s="46">
         <v>1350</v>
@@ -13732,7 +13738,7 @@
         <v>1.619</v>
       </c>
       <c r="K9" s="46" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="L9" s="48">
         <v>1293.905</v>
@@ -13783,7 +13789,7 @@
         <v>31</v>
       </c>
       <c r="AB9" s="46" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13797,7 +13803,7 @@
         <v>35</v>
       </c>
       <c r="D10" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E10" s="52" t="s">
         <v>27</v>
@@ -13806,7 +13812,7 @@
         <v>262642</v>
       </c>
       <c r="G10" s="52" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H10" s="52">
         <v>1000</v>
@@ -13818,7 +13824,7 @@
         <v>1.58</v>
       </c>
       <c r="K10" s="52" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="L10" s="54">
         <v>917.98</v>
@@ -13869,7 +13875,7 @@
         <v>32</v>
       </c>
       <c r="AB10" s="52" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="58" customFormat="1" x14ac:dyDescent="0.3">
@@ -14008,7 +14014,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="93" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B1" s="93" t="s">
         <v>27</v>
@@ -14258,7 +14264,7 @@
         <v>3</v>
       </c>
       <c r="AB3" s="98" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14341,7 +14347,7 @@
         <v>3</v>
       </c>
       <c r="AB4" s="98" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14424,7 +14430,7 @@
         <v>3</v>
       </c>
       <c r="AB5" s="98" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14438,7 +14444,7 @@
         <v>44</v>
       </c>
       <c r="D6" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E6" s="52" t="s">
         <v>27</v>
@@ -14447,7 +14453,7 @@
         <v>262639</v>
       </c>
       <c r="G6" s="52" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H6" s="52">
         <v>300</v>
@@ -14510,7 +14516,7 @@
         <v>32</v>
       </c>
       <c r="AB6" s="52" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14524,7 +14530,7 @@
         <v>44</v>
       </c>
       <c r="D7" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E7" s="52" t="s">
         <v>27</v>
@@ -14533,7 +14539,7 @@
         <v>262637</v>
       </c>
       <c r="G7" s="52" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H7" s="52">
         <v>500</v>
@@ -14596,7 +14602,7 @@
         <v>32</v>
       </c>
       <c r="AB7" s="52" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14610,7 +14616,7 @@
         <v>44</v>
       </c>
       <c r="D8" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E8" s="52" t="s">
         <v>27</v>
@@ -14619,7 +14625,7 @@
         <v>262635</v>
       </c>
       <c r="G8" s="52" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H8" s="52">
         <v>5000</v>
@@ -14696,7 +14702,7 @@
         <v>44</v>
       </c>
       <c r="D9" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E9" s="52" t="s">
         <v>27</v>
@@ -14705,7 +14711,7 @@
         <v>262636</v>
       </c>
       <c r="G9" s="52" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H9" s="52">
         <v>5000</v>
@@ -14782,7 +14788,7 @@
         <v>26</v>
       </c>
       <c r="D10" s="52" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E10" s="52" t="s">
         <v>27</v>
@@ -14791,7 +14797,7 @@
         <v>262638</v>
       </c>
       <c r="G10" s="52" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H10" s="52">
         <v>200</v>
@@ -14854,7 +14860,7 @@
         <v>38</v>
       </c>
       <c r="AB10" s="52" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -15073,7 +15079,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="93" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B1" s="93" t="s">
         <v>27</v>
@@ -15263,7 +15269,7 @@
         <v>262633</v>
       </c>
       <c r="G3" s="42" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="H3" s="42">
         <v>7200</v>
@@ -15275,7 +15281,7 @@
         <v>1.843</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="L3" s="39">
         <v>8572.1620000000003</v>
@@ -15323,10 +15329,10 @@
         <v>27</v>
       </c>
       <c r="AA3" s="37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AB3" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -15349,7 +15355,7 @@
         <v>262630</v>
       </c>
       <c r="G4" s="42" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H4" s="42">
         <v>11100</v>
@@ -15409,7 +15415,7 @@
         <v>27</v>
       </c>
       <c r="AA4" s="37" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="AB4" s="37" t="s">
         <v>46</v>
@@ -15435,7 +15441,7 @@
         <v>262632</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="H5" s="42">
         <v>3600</v>
@@ -15498,7 +15504,7 @@
         <v>32</v>
       </c>
       <c r="AB5" s="37" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
@@ -15521,7 +15527,7 @@
         <v>262631</v>
       </c>
       <c r="G6" s="42" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H6" s="42">
         <v>5550</v>
@@ -15721,7 +15727,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="93" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B1" s="93" t="s">
         <v>27</v>
@@ -15896,7 +15902,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C3" s="42" t="s">
         <v>26</v>
@@ -15923,7 +15929,7 @@
         <v>1.35</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L3" s="39">
         <v>1833.3</v>
@@ -15974,7 +15980,7 @@
         <v>65</v>
       </c>
       <c r="AB3" s="37" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -15982,7 +15988,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C4" s="42" t="s">
         <v>26</v>
@@ -16060,7 +16066,7 @@
         <v>32</v>
       </c>
       <c r="AB4" s="37" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16068,7 +16074,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C5" s="42" t="s">
         <v>26</v>
@@ -16095,7 +16101,7 @@
         <v>2.36</v>
       </c>
       <c r="K5" s="42" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L5" s="39">
         <v>559.32000000000005</v>
@@ -16146,7 +16152,7 @@
         <v>32</v>
       </c>
       <c r="AB5" s="37" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16154,7 +16160,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C6" s="42" t="s">
         <v>26</v>
@@ -16181,7 +16187,7 @@
         <v>2.1</v>
       </c>
       <c r="K6" s="42" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L6" s="39">
         <v>561.79200000000003</v>
@@ -16232,7 +16238,7 @@
         <v>32</v>
       </c>
       <c r="AB6" s="37" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16240,7 +16246,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C7" s="42" t="s">
         <v>35</v>
@@ -16267,7 +16273,7 @@
         <v>0.96</v>
       </c>
       <c r="K7" s="42" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L7" s="39">
         <v>681.6</v>
@@ -16318,7 +16324,7 @@
         <v>38</v>
       </c>
       <c r="AB7" s="37" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16326,7 +16332,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C8" s="42" t="s">
         <v>35</v>
@@ -16353,7 +16359,7 @@
         <v>1.44</v>
       </c>
       <c r="K8" s="42" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L8" s="39">
         <v>934.56</v>
@@ -16404,7 +16410,7 @@
         <v>32</v>
       </c>
       <c r="AB8" s="37" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16412,7 +16418,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C9" s="42" t="s">
         <v>81</v>
@@ -16439,7 +16445,7 @@
         <v>1.8</v>
       </c>
       <c r="K9" s="42" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="L9" s="39">
         <v>5395.5</v>
@@ -16490,7 +16496,7 @@
         <v>54</v>
       </c>
       <c r="AB9" s="37" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16498,7 +16504,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C10" s="42" t="s">
         <v>81</v>
@@ -16525,7 +16531,7 @@
         <v>1.03</v>
       </c>
       <c r="K10" s="42" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="L10" s="39">
         <v>2683.15</v>
@@ -16576,7 +16582,7 @@
         <v>31</v>
       </c>
       <c r="AB10" s="37" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16584,7 +16590,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C11" s="42" t="s">
         <v>35</v>
@@ -16611,7 +16617,7 @@
         <v>1.42</v>
       </c>
       <c r="K11" s="42" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="L11" s="39">
         <v>964.18</v>
@@ -16662,7 +16668,7 @@
         <v>32</v>
       </c>
       <c r="AB11" s="37" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16670,7 +16676,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="44" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C12" s="42" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (23/09/2026 16:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8681A2D3-6B57-40CA-A43A-091A8101E793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BC09C0-A779-460C-9BC4-34767F88F857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3083" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3097" uniqueCount="330">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1028,6 +1028,18 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - RM Embalagens ( Daiane Marques Canossa ME  —  OF: 001226</t>
+  </si>
+  <si>
+    <t>96x130x96</t>
+  </si>
+  <si>
+    <t>986x1900</t>
+  </si>
+  <si>
+    <t>181x230x181</t>
+  </si>
+  <si>
+    <t>612x1640</t>
   </si>
 </sst>
 </file>
@@ -1232,7 +1244,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1522,6 +1534,9 @@
     <xf numFmtId="14" fontId="15" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1745,6 +1760,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CFEEFF-BB40-454C-844D-5753B7370662}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3502,7 +3520,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="93" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -15970,7 +15988,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCDEA62-D4C1-4F97-B5A0-F9D378B5F3A6}">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5546875" style="34" customWidth="1"/>
@@ -16433,95 +16451,89 @@
         <v>280</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="52">
-        <v>1</v>
-      </c>
-      <c r="B6" s="53" t="s">
+    <row r="6" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="46">
+        <v>4</v>
+      </c>
+      <c r="B6" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="52">
-        <v>262640</v>
-      </c>
-      <c r="G6" s="52" t="s">
-        <v>231</v>
-      </c>
-      <c r="H6" s="52">
-        <v>800</v>
-      </c>
-      <c r="I6" s="54">
-        <v>0.73199999999999998</v>
-      </c>
-      <c r="J6" s="54">
-        <v>1.6739999999999999</v>
-      </c>
-      <c r="K6" s="52" t="s">
-        <v>235</v>
-      </c>
-      <c r="L6" s="54">
-        <v>980.29399999999998</v>
-      </c>
-      <c r="M6" s="55">
-        <v>669.6</v>
-      </c>
-      <c r="N6" s="56">
-        <v>9.2999999999999999E-2</v>
-      </c>
-      <c r="O6" s="57">
-        <v>5.58</v>
-      </c>
-      <c r="P6" s="52">
-        <v>317.60000000000002</v>
-      </c>
-      <c r="Q6" s="52">
+      <c r="D6" s="103">
+        <v>46287</v>
+      </c>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46">
+        <v>262701</v>
+      </c>
+      <c r="G6" s="46">
+        <v>8263</v>
+      </c>
+      <c r="H6" s="46">
+        <v>930</v>
+      </c>
+      <c r="I6" s="48">
+        <v>0.59199999999999997</v>
+      </c>
+      <c r="J6" s="48">
+        <v>1.62</v>
+      </c>
+      <c r="K6" s="46" t="s">
+        <v>328</v>
+      </c>
+      <c r="L6" s="48">
+        <v>891.90700000000004</v>
+      </c>
+      <c r="M6" s="49">
+        <v>753.3</v>
+      </c>
+      <c r="N6" s="50">
+        <v>0.1046</v>
+      </c>
+      <c r="O6" s="51">
+        <v>6.28</v>
+      </c>
+      <c r="P6" s="46">
+        <v>289</v>
+      </c>
+      <c r="Q6" s="46">
         <v>2</v>
       </c>
-      <c r="R6" s="52">
-        <v>1500</v>
-      </c>
-      <c r="S6" s="54">
-        <v>1.464</v>
-      </c>
-      <c r="T6" s="52">
-        <v>36</v>
-      </c>
-      <c r="U6" s="56">
-        <v>2.4E-2</v>
-      </c>
-      <c r="V6" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="52" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB6" s="52" t="s">
-        <v>234</v>
+      <c r="R6" s="46">
+        <v>1250</v>
+      </c>
+      <c r="S6" s="48">
+        <v>1.1839999999999999</v>
+      </c>
+      <c r="T6" s="46">
+        <v>66</v>
+      </c>
+      <c r="U6" s="50">
+        <v>5.28E-2</v>
+      </c>
+      <c r="V6" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="46"/>
+      <c r="Z6" s="46"/>
+      <c r="AA6" s="46">
+        <v>3</v>
+      </c>
+      <c r="AB6" s="46" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="52">
-        <v>2</v>
+      <c r="A7" s="46">
+        <v>5</v>
       </c>
       <c r="B7" s="53" t="s">
         <v>58</v>
@@ -16536,418 +16548,584 @@
         <v>27</v>
       </c>
       <c r="F7" s="52">
-        <v>262641</v>
+        <v>262640</v>
       </c>
       <c r="G7" s="52" t="s">
         <v>231</v>
       </c>
       <c r="H7" s="52">
-        <v>1150</v>
+        <v>800</v>
       </c>
       <c r="I7" s="54">
-        <v>0.54700000000000004</v>
+        <v>0.73199999999999998</v>
       </c>
       <c r="J7" s="54">
-        <v>1.44</v>
+        <v>1.6739999999999999</v>
       </c>
       <c r="K7" s="52" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="L7" s="54">
-        <v>905.83199999999999</v>
+        <v>980.29399999999998</v>
       </c>
       <c r="M7" s="55">
-        <v>828</v>
+        <v>669.6</v>
       </c>
       <c r="N7" s="56">
-        <v>0.115</v>
+        <v>9.2999999999999999E-2</v>
       </c>
       <c r="O7" s="57">
-        <v>6.9</v>
+        <v>5.58</v>
       </c>
       <c r="P7" s="52">
-        <v>293.5</v>
+        <v>317.60000000000002</v>
       </c>
       <c r="Q7" s="52">
         <v>2</v>
       </c>
       <c r="R7" s="52">
+        <v>1500</v>
+      </c>
+      <c r="S7" s="54">
+        <v>1.464</v>
+      </c>
+      <c r="T7" s="52">
+        <v>36</v>
+      </c>
+      <c r="U7" s="56">
+        <v>2.4E-2</v>
+      </c>
+      <c r="V7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="52" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB7" s="52" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="46">
+        <v>6</v>
+      </c>
+      <c r="B8" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="52">
+        <v>262641</v>
+      </c>
+      <c r="G8" s="52" t="s">
+        <v>231</v>
+      </c>
+      <c r="H8" s="52">
         <v>1150</v>
       </c>
-      <c r="S7" s="54">
+      <c r="I8" s="54">
+        <v>0.54700000000000004</v>
+      </c>
+      <c r="J8" s="54">
+        <v>1.44</v>
+      </c>
+      <c r="K8" s="52" t="s">
+        <v>233</v>
+      </c>
+      <c r="L8" s="54">
+        <v>905.83199999999999</v>
+      </c>
+      <c r="M8" s="55">
+        <v>828</v>
+      </c>
+      <c r="N8" s="56">
+        <v>0.115</v>
+      </c>
+      <c r="O8" s="57">
+        <v>6.9</v>
+      </c>
+      <c r="P8" s="52">
+        <v>293.5</v>
+      </c>
+      <c r="Q8" s="52">
+        <v>2</v>
+      </c>
+      <c r="R8" s="52">
+        <v>1150</v>
+      </c>
+      <c r="S8" s="54">
         <v>1.0940000000000001</v>
       </c>
-      <c r="T7" s="52">
+      <c r="T8" s="52">
         <v>56</v>
       </c>
-      <c r="U7" s="56">
+      <c r="U8" s="56">
         <v>4.87E-2</v>
       </c>
-      <c r="V7" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="52" t="s">
+      <c r="V8" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="52" t="s">
+      <c r="AB8" s="52" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="46">
-        <v>4</v>
-      </c>
-      <c r="B8" s="47" t="s">
+    <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="46">
+        <v>7</v>
+      </c>
+      <c r="B9" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C9" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="68">
+        <v>46287</v>
+      </c>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52">
+        <v>262700</v>
+      </c>
+      <c r="G9" s="52">
+        <v>8263</v>
+      </c>
+      <c r="H9" s="52">
+        <v>9500</v>
+      </c>
+      <c r="I9" s="54">
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="J9" s="54">
+        <v>0.94</v>
+      </c>
+      <c r="K9" s="52" t="s">
+        <v>326</v>
+      </c>
+      <c r="L9" s="54">
+        <v>2875.46</v>
+      </c>
+      <c r="M9" s="55">
+        <v>4465</v>
+      </c>
+      <c r="N9" s="56">
+        <v>0.62009999999999998</v>
+      </c>
+      <c r="O9" s="57">
+        <v>37.21</v>
+      </c>
+      <c r="P9" s="52">
+        <v>931.6</v>
+      </c>
+      <c r="Q9" s="52">
+        <v>2</v>
+      </c>
+      <c r="R9" s="52">
+        <v>700</v>
+      </c>
+      <c r="S9" s="54">
+        <v>0.64400000000000002</v>
+      </c>
+      <c r="T9" s="52">
+        <v>56</v>
+      </c>
+      <c r="U9" s="56">
+        <v>0.08</v>
+      </c>
+      <c r="V9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="52"/>
+      <c r="Z9" s="52"/>
+      <c r="AA9" s="52">
+        <v>5</v>
+      </c>
+      <c r="AB9" s="52" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="46">
+        <v>8</v>
+      </c>
+      <c r="B10" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D10" s="46" t="s">
         <v>255</v>
       </c>
-      <c r="E8" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="46">
+      <c r="E10" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="46">
         <v>262673</v>
       </c>
-      <c r="G8" s="46" t="s">
+      <c r="G10" s="46" t="s">
         <v>284</v>
       </c>
-      <c r="H8" s="46">
+      <c r="H10" s="46">
         <v>1000</v>
       </c>
-      <c r="I8" s="48">
+      <c r="I10" s="48">
         <v>0.76</v>
       </c>
-      <c r="J8" s="48">
+      <c r="J10" s="48">
         <v>1.0900000000000001</v>
       </c>
-      <c r="K8" s="46" t="s">
+      <c r="K10" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="L8" s="48">
+      <c r="L10" s="48">
         <v>828.4</v>
       </c>
-      <c r="M8" s="49">
+      <c r="M10" s="49">
         <v>545</v>
       </c>
-      <c r="N8" s="50">
+      <c r="N10" s="50">
         <v>7.5700000000000003E-2</v>
       </c>
-      <c r="O8" s="51">
+      <c r="O10" s="51">
         <v>4.54</v>
       </c>
-      <c r="P8" s="46">
+      <c r="P10" s="46">
         <v>260.89999999999998</v>
       </c>
-      <c r="Q8" s="46">
+      <c r="Q10" s="46">
         <v>2</v>
       </c>
-      <c r="R8" s="46">
+      <c r="R10" s="46">
         <v>1550</v>
       </c>
-      <c r="S8" s="48">
+      <c r="S10" s="48">
         <v>1.52</v>
       </c>
-      <c r="T8" s="46">
+      <c r="T10" s="46">
         <v>30</v>
       </c>
-      <c r="U8" s="50">
+      <c r="U10" s="50">
         <v>1.9400000000000001E-2</v>
       </c>
-      <c r="V8" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="46" t="s">
+      <c r="V10" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="AB8" s="46" t="s">
+      <c r="AB10" s="46" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="46">
-        <v>5</v>
-      </c>
-      <c r="B9" s="47" t="s">
+    <row r="11" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="46">
+        <v>9</v>
+      </c>
+      <c r="B11" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="46" t="s">
+      <c r="C11" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D11" s="46" t="s">
         <v>276</v>
       </c>
-      <c r="E9" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="46">
+      <c r="E11" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="46">
         <v>262675</v>
       </c>
-      <c r="G9" s="46" t="s">
+      <c r="G11" s="46" t="s">
         <v>290</v>
       </c>
-      <c r="H9" s="46">
+      <c r="H11" s="46">
         <v>1350</v>
       </c>
-      <c r="I9" s="48">
+      <c r="I11" s="48">
         <v>0.59199999999999997</v>
       </c>
-      <c r="J9" s="48">
+      <c r="J11" s="48">
         <v>1.619</v>
       </c>
-      <c r="K9" s="46" t="s">
+      <c r="K11" s="46" t="s">
         <v>291</v>
       </c>
-      <c r="L9" s="48">
+      <c r="L11" s="48">
         <v>1293.905</v>
       </c>
-      <c r="M9" s="49">
+      <c r="M11" s="49">
         <v>1092.8</v>
       </c>
-      <c r="N9" s="50">
+      <c r="N11" s="50">
         <v>0.15179999999999999</v>
       </c>
-      <c r="O9" s="51">
+      <c r="O11" s="51">
         <v>9.11</v>
       </c>
-      <c r="P9" s="46">
+      <c r="P11" s="46">
         <v>407.6</v>
       </c>
-      <c r="Q9" s="46">
+      <c r="Q11" s="46">
         <v>2</v>
       </c>
-      <c r="R9" s="46">
+      <c r="R11" s="46">
         <v>1250</v>
       </c>
-      <c r="S9" s="48">
+      <c r="S11" s="48">
         <v>1.1839999999999999</v>
       </c>
-      <c r="T9" s="46">
+      <c r="T11" s="46">
         <v>66</v>
       </c>
-      <c r="U9" s="50">
+      <c r="U11" s="50">
         <v>5.28E-2</v>
       </c>
-      <c r="V9" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="46" t="s">
+      <c r="V11" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="AB9" s="46" t="s">
+      <c r="AB11" s="46" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="52">
-        <v>3</v>
-      </c>
-      <c r="B10" s="53" t="s">
+    <row r="12" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="46">
+        <v>10</v>
+      </c>
+      <c r="B12" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="52" t="s">
+      <c r="C12" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="52" t="s">
+      <c r="D12" s="52" t="s">
         <v>222</v>
       </c>
-      <c r="E10" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="52">
+      <c r="E12" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="52">
         <v>262642</v>
       </c>
-      <c r="G10" s="52" t="s">
+      <c r="G12" s="52" t="s">
         <v>231</v>
       </c>
-      <c r="H10" s="52">
+      <c r="H12" s="52">
         <v>1000</v>
       </c>
-      <c r="I10" s="54">
+      <c r="I12" s="54">
         <v>0.58099999999999996</v>
       </c>
-      <c r="J10" s="54">
+      <c r="J12" s="54">
         <v>1.58</v>
       </c>
-      <c r="K10" s="52" t="s">
+      <c r="K12" s="52" t="s">
         <v>230</v>
       </c>
-      <c r="L10" s="54">
+      <c r="L12" s="54">
         <v>917.98</v>
       </c>
-      <c r="M10" s="55">
+      <c r="M12" s="55">
         <v>790</v>
       </c>
-      <c r="N10" s="56">
+      <c r="N12" s="56">
         <v>0.10970000000000001</v>
       </c>
-      <c r="O10" s="57">
+      <c r="O12" s="57">
         <v>6.58</v>
       </c>
-      <c r="P10" s="52">
+      <c r="P12" s="52">
         <v>289.2</v>
       </c>
-      <c r="Q10" s="52">
+      <c r="Q12" s="52">
         <v>2</v>
       </c>
-      <c r="R10" s="52">
+      <c r="R12" s="52">
         <v>1200</v>
       </c>
-      <c r="S10" s="54">
+      <c r="S12" s="54">
         <v>1.1619999999999999</v>
       </c>
-      <c r="T10" s="52">
+      <c r="T12" s="52">
         <v>38</v>
       </c>
-      <c r="U10" s="56">
+      <c r="U12" s="56">
         <v>3.1699999999999999E-2</v>
       </c>
-      <c r="V10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="52" t="s">
+      <c r="V12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB10" s="52" t="s">
+      <c r="AB12" s="52" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="58" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="59">
-        <f>SUM(H3:H10)</f>
-        <v>6500</v>
-      </c>
-      <c r="I11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="K11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="L11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="M11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="N11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="O11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="P11" s="59">
-        <f>SUM(P3:P10)</f>
-        <v>3532.1</v>
-      </c>
-      <c r="Q11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="R11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="S11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="T11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="U11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="V11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="W11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="X11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB11" s="59" t="s">
+    <row r="13" spans="1:28" s="58" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="59">
+        <f>SUM(H3:H12)</f>
+        <v>16930</v>
+      </c>
+      <c r="I13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P13" s="59">
+        <f>SUM(P3:P12)</f>
+        <v>4752.7</v>
+      </c>
+      <c r="Q13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB13" s="59" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (23/09/2026 16:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BC09C0-A779-460C-9BC4-34767F88F857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F317127A-A57A-4524-A69E-E286745A52C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3097" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3113" uniqueCount="332">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1040,6 +1040,12 @@
   </si>
   <si>
     <t>612x1640</t>
+  </si>
+  <si>
+    <t>894x1403</t>
+  </si>
+  <si>
+    <t>1171x1839</t>
   </si>
 </sst>
 </file>
@@ -12338,7 +12344,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B791AA56-47E9-44C0-8D6D-1F61C5308578}">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="34" customWidth="1"/>
@@ -12543,433 +12549,593 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="42">
+    <row r="3" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="98" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="98" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="99">
+        <v>46288</v>
+      </c>
+      <c r="F3" s="98">
+        <v>262703</v>
+      </c>
+      <c r="G3" s="98">
+        <v>1767</v>
+      </c>
+      <c r="H3" s="98">
+        <v>200</v>
+      </c>
+      <c r="I3" s="98">
+        <v>1.151</v>
+      </c>
+      <c r="J3" s="98">
+        <v>1.819</v>
+      </c>
+      <c r="K3" s="98" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="98">
+        <v>418.73399999999998</v>
+      </c>
+      <c r="M3" s="98">
+        <v>363.8</v>
+      </c>
+      <c r="N3" s="98">
+        <v>0.1011</v>
+      </c>
+      <c r="O3" s="98">
+        <v>6.06</v>
+      </c>
+      <c r="P3" s="98">
+        <v>237.8</v>
+      </c>
+      <c r="Q3" s="98">
         <v>1</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="R3" s="98">
+        <v>1200</v>
+      </c>
+      <c r="S3" s="98">
+        <v>1.151</v>
+      </c>
+      <c r="T3" s="98">
+        <v>49</v>
+      </c>
+      <c r="U3" s="98">
+        <v>4.0800000000000003E-2</v>
+      </c>
+      <c r="V3" s="98" t="s">
+        <v>34</v>
+      </c>
+      <c r="W3" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3" s="98" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y3" s="98" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z3" s="98" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="98">
+        <v>2</v>
+      </c>
+      <c r="AB3" s="98" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="52">
+        <v>1</v>
+      </c>
+      <c r="B4" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="42" t="s">
+      <c r="C4" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="42" t="s">
+      <c r="D4" s="52" t="s">
         <v>276</v>
       </c>
-      <c r="E3" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="42">
+      <c r="E4" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="52">
         <v>262676</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="G4" s="52" t="s">
         <v>299</v>
       </c>
-      <c r="H3" s="42">
+      <c r="H4" s="52">
         <v>200</v>
       </c>
-      <c r="I3" s="43">
+      <c r="I4" s="54">
         <v>1.026</v>
       </c>
-      <c r="J3" s="43">
+      <c r="J4" s="54">
         <v>2.0630000000000002</v>
       </c>
-      <c r="K3" s="42" t="s">
+      <c r="K4" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="39">
+      <c r="L4" s="54">
         <v>423.32799999999997</v>
       </c>
-      <c r="M3" s="41">
+      <c r="M4" s="55">
         <v>412.6</v>
       </c>
-      <c r="N3" s="38">
+      <c r="N4" s="56">
         <v>0.11459999999999999</v>
       </c>
-      <c r="O3" s="40">
+      <c r="O4" s="57">
         <v>6.88</v>
       </c>
-      <c r="P3" s="37">
+      <c r="P4" s="52">
         <v>227.8</v>
       </c>
-      <c r="Q3" s="37">
+      <c r="Q4" s="52">
         <v>1</v>
       </c>
-      <c r="R3" s="37">
+      <c r="R4" s="52">
         <v>1050</v>
       </c>
-      <c r="S3" s="39">
+      <c r="S4" s="54">
         <v>1.026</v>
       </c>
-      <c r="T3" s="37">
+      <c r="T4" s="52">
         <v>24</v>
       </c>
-      <c r="U3" s="38">
+      <c r="U4" s="56">
         <v>2.29E-2</v>
       </c>
-      <c r="V3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="37" t="s">
+      <c r="V4" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="37" t="s">
+      <c r="X4" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB3" s="37" t="s">
+      <c r="AB4" s="52" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="42">
+    <row r="5" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="52">
         <v>2</v>
       </c>
-      <c r="B4" s="44" t="s">
+      <c r="B5" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C5" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="42" t="s">
+      <c r="D5" s="52" t="s">
         <v>276</v>
       </c>
-      <c r="E4" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="42">
+      <c r="E5" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="52">
         <v>262678</v>
       </c>
-      <c r="G4" s="42" t="s">
+      <c r="G5" s="52" t="s">
         <v>296</v>
       </c>
-      <c r="H4" s="42">
+      <c r="H5" s="52">
         <v>250</v>
       </c>
-      <c r="I4" s="43">
+      <c r="I5" s="54">
         <v>1.4890000000000001</v>
       </c>
-      <c r="J4" s="43">
+      <c r="J5" s="54">
         <v>1.9890000000000001</v>
       </c>
-      <c r="K4" s="42" t="s">
+      <c r="K5" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="39">
+      <c r="L5" s="54">
         <v>740.40499999999997</v>
       </c>
-      <c r="M4" s="41">
+      <c r="M5" s="55">
         <v>497.3</v>
       </c>
-      <c r="N4" s="38">
+      <c r="N5" s="56">
         <v>0.1381</v>
       </c>
-      <c r="O4" s="40">
+      <c r="O5" s="57">
         <v>8.2899999999999991</v>
       </c>
-      <c r="P4" s="37">
+      <c r="P5" s="52">
         <v>233.2</v>
       </c>
-      <c r="Q4" s="37">
+      <c r="Q5" s="52">
         <v>1</v>
       </c>
-      <c r="R4" s="37">
+      <c r="R5" s="52">
         <v>1550</v>
       </c>
-      <c r="S4" s="39">
+      <c r="S5" s="54">
         <v>1.4890000000000001</v>
       </c>
-      <c r="T4" s="37">
+      <c r="T5" s="52">
         <v>61</v>
       </c>
-      <c r="U4" s="38">
+      <c r="U5" s="56">
         <v>3.9399999999999998E-2</v>
       </c>
-      <c r="V4" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="37" t="s">
+      <c r="V5" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="AB4" s="37" t="s">
+      <c r="AB5" s="52" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="42">
+    <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="52"/>
+      <c r="B6" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="68">
+        <v>46287</v>
+      </c>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52">
+        <v>262702</v>
+      </c>
+      <c r="G6" s="52">
+        <v>1765</v>
+      </c>
+      <c r="H6" s="52">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="54">
+        <v>0.437</v>
+      </c>
+      <c r="J6" s="54">
+        <v>1.383</v>
+      </c>
+      <c r="K6" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="L6" s="54">
+        <v>604.37099999999998</v>
+      </c>
+      <c r="M6" s="55">
+        <v>461</v>
+      </c>
+      <c r="N6" s="56">
+        <v>4.2700000000000002E-2</v>
+      </c>
+      <c r="O6" s="57">
+        <v>2.56</v>
+      </c>
+      <c r="P6" s="52">
+        <v>190.4</v>
+      </c>
+      <c r="Q6" s="52">
         <v>3</v>
       </c>
-      <c r="B5" s="44" t="s">
+      <c r="R6" s="52">
+        <v>1350</v>
+      </c>
+      <c r="S6" s="54">
+        <v>1.3109999999999999</v>
+      </c>
+      <c r="T6" s="52">
+        <v>39</v>
+      </c>
+      <c r="U6" s="56">
+        <v>2.8899999999999999E-2</v>
+      </c>
+      <c r="V6" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="52"/>
+      <c r="Z6" s="52"/>
+      <c r="AA6" s="52">
+        <v>2</v>
+      </c>
+      <c r="AB6" s="52" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="52">
+        <v>3</v>
+      </c>
+      <c r="B7" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C7" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="42" t="s">
+      <c r="D7" s="52" t="s">
         <v>276</v>
       </c>
-      <c r="E5" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="42">
+      <c r="E7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="52">
         <v>262679</v>
       </c>
-      <c r="G5" s="42" t="s">
+      <c r="G7" s="52" t="s">
         <v>296</v>
       </c>
-      <c r="H5" s="42">
+      <c r="H7" s="52">
         <v>150</v>
       </c>
-      <c r="I5" s="43">
+      <c r="I7" s="54">
         <v>1.19</v>
       </c>
-      <c r="J5" s="43">
+      <c r="J7" s="54">
         <v>1.417</v>
       </c>
-      <c r="K5" s="42" t="s">
+      <c r="K7" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="L5" s="39">
+      <c r="L7" s="54">
         <v>252.934</v>
       </c>
-      <c r="M5" s="41">
+      <c r="M7" s="55">
         <v>212.6</v>
       </c>
-      <c r="N5" s="38">
+      <c r="N7" s="56">
         <v>5.8999999999999997E-2</v>
       </c>
-      <c r="O5" s="40">
+      <c r="O7" s="57">
         <v>3.54</v>
       </c>
-      <c r="P5" s="37">
+      <c r="P7" s="52">
         <v>79.7</v>
       </c>
-      <c r="Q5" s="37">
+      <c r="Q7" s="52">
         <v>1</v>
       </c>
-      <c r="R5" s="37">
+      <c r="R7" s="52">
         <v>1250</v>
       </c>
-      <c r="S5" s="39">
+      <c r="S7" s="54">
         <v>1.19</v>
       </c>
-      <c r="T5" s="37">
+      <c r="T7" s="52">
         <v>60</v>
       </c>
-      <c r="U5" s="38">
+      <c r="U7" s="56">
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="V5" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="37" t="s">
+      <c r="V7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="AB5" s="37" t="s">
+      <c r="AB7" s="52" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="42">
+    <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="52">
         <v>4</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B8" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C8" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="42" t="s">
+      <c r="D8" s="52" t="s">
         <v>276</v>
       </c>
-      <c r="E6" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="42">
+      <c r="E8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="52">
         <v>262677</v>
       </c>
-      <c r="G6" s="42" t="s">
+      <c r="G8" s="52" t="s">
         <v>294</v>
       </c>
-      <c r="H6" s="42">
+      <c r="H8" s="52">
         <v>1000</v>
       </c>
-      <c r="I6" s="43">
+      <c r="I8" s="54">
         <v>0.8</v>
       </c>
-      <c r="J6" s="43">
+      <c r="J8" s="54">
         <v>1.171</v>
       </c>
-      <c r="K6" s="42" t="s">
+      <c r="K8" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="39">
+      <c r="L8" s="54">
         <v>936.8</v>
       </c>
-      <c r="M6" s="41">
+      <c r="M8" s="55">
         <v>1171</v>
       </c>
-      <c r="N6" s="38">
+      <c r="N8" s="56">
         <v>0.32529999999999998</v>
       </c>
-      <c r="O6" s="40">
+      <c r="O8" s="57">
         <v>19.52</v>
       </c>
-      <c r="P6" s="37">
+      <c r="P8" s="52">
         <v>323.2</v>
       </c>
-      <c r="Q6" s="37">
+      <c r="Q8" s="52">
         <v>1</v>
       </c>
-      <c r="R6" s="37">
+      <c r="R8" s="52">
         <v>850</v>
       </c>
-      <c r="S6" s="39">
+      <c r="S8" s="54">
         <v>0.8</v>
       </c>
-      <c r="T6" s="37">
+      <c r="T8" s="52">
         <v>50</v>
       </c>
-      <c r="U6" s="38">
+      <c r="U8" s="56">
         <v>5.8799999999999998E-2</v>
       </c>
-      <c r="V6" s="37" t="s">
+      <c r="V8" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="W6" s="37" t="s">
+      <c r="W8" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="37" t="s">
+      <c r="X8" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB6" s="37" t="s">
+      <c r="AB8" s="52" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="36">
-        <v>1600</v>
-      </c>
-      <c r="I7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="35">
-        <v>863.8</v>
-      </c>
-      <c r="Q7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="U7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB7" s="35" t="s">
+    <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="59">
+        <f>SUM(H3:H8)</f>
+        <v>2800</v>
+      </c>
+      <c r="I9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P9" s="59">
+        <f>SUM(P3:P8)</f>
+        <v>1292.0999999999999</v>
+      </c>
+      <c r="Q9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB9" s="59" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (23/09/2026 17:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F317127A-A57A-4524-A69E-E286745A52C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB79B808-4D13-4374-97EA-474316AF377D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId1"/>
@@ -18380,7 +18380,7 @@
   <cols>
     <col min="1" max="1" width="2.77734375" style="34" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" style="34" customWidth="1"/>
+    <col min="3" max="3" width="7.44140625" style="34" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="34" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8.77734375" style="34" customWidth="1"/>
     <col min="6" max="6" width="7.109375" style="34" customWidth="1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (24/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF618506-4F09-4B5F-83D5-280BE7E07D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F6E116C-9FEA-4897-8663-3B2AD6D7C9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId1"/>
     <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId2"/>
     <sheet name="FORBOX 1220" sheetId="163" r:id="rId3"/>
-    <sheet name="HARMONY EMBALAGENS 1217" sheetId="162" r:id="rId4"/>
+    <sheet name="HARMONY EMBALAGENS 1217 P" sheetId="162" r:id="rId4"/>
     <sheet name="Z4A EMBALAGENS LTDA 1216" sheetId="161" r:id="rId5"/>
     <sheet name="Tolecaixas 1215" sheetId="160" r:id="rId6"/>
     <sheet name="ABAPEL 1213" sheetId="159" r:id="rId7"/>
@@ -24,7 +24,7 @@
     <sheet name="Z4A EMBALAGENS LTDA 1210 P" sheetId="157" r:id="rId9"/>
     <sheet name="RM Embalagens 1209 P" sheetId="156" r:id="rId10"/>
     <sheet name="ABAPEL 1201 P" sheetId="153" r:id="rId11"/>
-    <sheet name="HARMONY EMBALAGENS 1200" sheetId="152" r:id="rId12"/>
+    <sheet name="HARMONY EMBALAGENS 1200 P" sheetId="152" r:id="rId12"/>
     <sheet name="FAVINCO EMBALAGENS 1197 P" sheetId="150" r:id="rId13"/>
     <sheet name="ABAPEL 1196 P" sheetId="149" r:id="rId14"/>
     <sheet name="RM Embalagens 1184 P" sheetId="141" r:id="rId15"/>
@@ -1051,19 +1051,12 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color rgb="FF0F1E2E"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1240,277 +1233,277 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="13" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="15" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1519,24 +1512,23 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="15" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="14" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5462,88 +5454,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="99" t="s">
         <v>173</v>
       </c>
-      <c r="B1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="100" t="s">
+      <c r="B1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="99" t="s">
         <v>27</v>
       </c>
     </row>
@@ -9741,88 +9733,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="100" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="101" t="s">
+      <c r="B1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="100" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11078,88 +11070,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="101" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="102" t="s">
+      <c r="B1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="101" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11726,88 +11718,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="102" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="103" t="s">
+      <c r="B1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="102" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13816,88 +13808,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>266</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -18272,7 +18264,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/09/2026 11:05)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55634912-F294-4A7C-8692-850E5F5D69A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BD993C-AF93-47CA-AFFD-FF59B084F013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANSELMO E FILHOS LTDA. 1229" sheetId="167" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3195" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3202" uniqueCount="335">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1053,6 +1053,9 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - ANSELMO E FILHOS LTDA.  —  OF: 001229</t>
+  </si>
+  <si>
+    <t>817x1507</t>
   </si>
 </sst>
 </file>
@@ -13378,7 +13381,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B791AA56-47E9-44C0-8D6D-1F61C5308578}">
-  <dimension ref="A1:AB9"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="34" customWidth="1"/>
@@ -13584,6 +13587,9 @@
       </c>
     </row>
     <row r="3" spans="1:28" s="92" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="92">
+        <v>1</v>
+      </c>
       <c r="B3" s="92" t="s">
         <v>90</v>
       </c>
@@ -13664,8 +13670,8 @@
       </c>
     </row>
     <row r="4" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52">
-        <v>1</v>
+      <c r="A4" s="92">
+        <v>2</v>
       </c>
       <c r="B4" s="53" t="s">
         <v>90</v>
@@ -13750,8 +13756,8 @@
       </c>
     </row>
     <row r="5" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="52">
-        <v>2</v>
+      <c r="A5" s="92">
+        <v>3</v>
       </c>
       <c r="B5" s="53" t="s">
         <v>90</v>
@@ -13836,7 +13842,9 @@
       </c>
     </row>
     <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="52"/>
+      <c r="A6" s="92">
+        <v>4</v>
+      </c>
       <c r="B6" s="53" t="s">
         <v>90</v>
       </c>
@@ -13914,8 +13922,8 @@
       </c>
     </row>
     <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="52">
-        <v>3</v>
+      <c r="A7" s="92">
+        <v>5</v>
       </c>
       <c r="B7" s="53" t="s">
         <v>90</v>
@@ -14000,8 +14008,8 @@
       </c>
     </row>
     <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="52">
-        <v>4</v>
+      <c r="A8" s="92">
+        <v>6</v>
       </c>
       <c r="B8" s="53" t="s">
         <v>90</v>
@@ -14086,90 +14094,170 @@
       </c>
     </row>
     <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="59">
-        <f>SUM(H3:H8)</f>
-        <v>2800</v>
-      </c>
-      <c r="I9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="J9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="K9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="M9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="N9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="O9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="P9" s="59">
-        <f>SUM(P3:P8)</f>
-        <v>1292.0999999999999</v>
-      </c>
-      <c r="Q9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="R9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="S9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="T9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="U9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="V9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="W9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="X9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB9" s="59" t="s">
+      <c r="A9" s="92">
+        <v>7</v>
+      </c>
+      <c r="B9" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="68">
+        <v>46288</v>
+      </c>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52">
+        <v>262705</v>
+      </c>
+      <c r="G9" s="52">
+        <v>1768</v>
+      </c>
+      <c r="H9" s="52">
+        <v>200</v>
+      </c>
+      <c r="I9" s="54">
+        <v>0.79700000000000004</v>
+      </c>
+      <c r="J9" s="54">
+        <v>1.4870000000000001</v>
+      </c>
+      <c r="K9" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="L9" s="54">
+        <v>237.02799999999999</v>
+      </c>
+      <c r="M9" s="55">
+        <v>297.39999999999998</v>
+      </c>
+      <c r="N9" s="56">
+        <v>8.2600000000000007E-2</v>
+      </c>
+      <c r="O9" s="57">
+        <v>4.96</v>
+      </c>
+      <c r="P9" s="52">
+        <v>74.7</v>
+      </c>
+      <c r="Q9" s="52">
+        <v>1</v>
+      </c>
+      <c r="R9" s="52">
+        <v>850</v>
+      </c>
+      <c r="S9" s="54">
+        <v>0.79700000000000004</v>
+      </c>
+      <c r="T9" s="52">
+        <v>53</v>
+      </c>
+      <c r="U9" s="56">
+        <v>6.2399999999999997E-2</v>
+      </c>
+      <c r="V9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="52"/>
+      <c r="Z9" s="52"/>
+      <c r="AA9" s="52">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="52" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="59">
+        <f>SUM(H3:H9)</f>
+        <v>3000</v>
+      </c>
+      <c r="I10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P10" s="59">
+        <f>SUM(P3:P9)</f>
+        <v>1366.8</v>
+      </c>
+      <c r="Q10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB10" s="59" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/09/2026 11:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BD993C-AF93-47CA-AFFD-FF59B084F013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE13FED0-CE4B-4021-B8E2-4E1EF4107851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ANSELMO E FILHOS LTDA. 1229" sheetId="167" r:id="rId1"/>
+    <sheet name="FAVINCO 1229" sheetId="167" r:id="rId1"/>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId2"/>
     <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId3"/>
     <sheet name="FORBOX 1220" sheetId="163" r:id="rId4"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3202" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3202" uniqueCount="334">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1049,13 +1049,10 @@
     <t>24/09/2026</t>
   </si>
   <si>
-    <t>ANSELMO E FILHOS LTDA.</t>
-  </si>
-  <si>
-    <t>PROGRAMAÇÃO ONDULADEIRA - ANSELMO E FILHOS LTDA.  —  OF: 001229</t>
-  </si>
-  <si>
     <t>817x1507</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - FAVINCO  —  OF: 001229</t>
   </si>
 </sst>
 </file>
@@ -1772,7 +1769,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="34" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="34" customWidth="1"/>
     <col min="3" max="3" width="5.77734375" style="34" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="34" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9" style="34" customWidth="1"/>
@@ -1978,7 +1975,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>332</v>
+        <v>126</v>
       </c>
       <c r="C3" s="42" t="s">
         <v>35</v>
@@ -14170,7 +14167,7 @@
         <v>1</v>
       </c>
       <c r="AB9" s="52" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/09/2026 11:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE13FED0-CE4B-4021-B8E2-4E1EF4107851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CCD6D7A-5294-4E4D-ABF3-9A25BF761622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FAVINCO 1229" sheetId="167" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3202" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3209" uniqueCount="335">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1053,6 +1053,9 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - FAVINCO  —  OF: 001229</t>
+  </si>
+  <si>
+    <t>870x1427</t>
   </si>
 </sst>
 </file>
@@ -13378,7 +13381,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B791AA56-47E9-44C0-8D6D-1F61C5308578}">
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AB11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="34" customWidth="1"/>
@@ -14012,82 +14015,76 @@
         <v>90</v>
       </c>
       <c r="C8" s="52" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" s="52" t="s">
-        <v>274</v>
-      </c>
-      <c r="E8" s="52" t="s">
-        <v>27</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="D8" s="68">
+        <v>46289</v>
+      </c>
+      <c r="E8" s="52"/>
       <c r="F8" s="52">
-        <v>262677</v>
-      </c>
-      <c r="G8" s="52" t="s">
-        <v>292</v>
+        <v>262706</v>
+      </c>
+      <c r="G8" s="52">
+        <v>1770</v>
       </c>
       <c r="H8" s="52">
-        <v>1000</v>
+        <v>220</v>
       </c>
       <c r="I8" s="54">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="J8" s="54">
-        <v>1.171</v>
+        <v>1.407</v>
       </c>
       <c r="K8" s="52" t="s">
         <v>33</v>
       </c>
       <c r="L8" s="54">
-        <v>936.8</v>
+        <v>263.10899999999998</v>
       </c>
       <c r="M8" s="55">
-        <v>1171</v>
+        <v>309.5</v>
       </c>
       <c r="N8" s="56">
-        <v>0.32529999999999998</v>
+        <v>8.5999999999999993E-2</v>
       </c>
       <c r="O8" s="57">
-        <v>19.52</v>
+        <v>5.16</v>
       </c>
       <c r="P8" s="52">
-        <v>323.2</v>
+        <v>82.9</v>
       </c>
       <c r="Q8" s="52">
         <v>1</v>
       </c>
       <c r="R8" s="52">
-        <v>850</v>
+        <v>900</v>
       </c>
       <c r="S8" s="54">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="T8" s="52">
         <v>50</v>
       </c>
       <c r="U8" s="56">
-        <v>5.8799999999999998E-2</v>
+        <v>5.5599999999999997E-2</v>
       </c>
       <c r="V8" s="52" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W8" s="52" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X8" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="Y8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="52" t="s">
-        <v>32</v>
+      <c r="Y8" s="52"/>
+      <c r="Z8" s="52"/>
+      <c r="AA8" s="52">
+        <v>1</v>
       </c>
       <c r="AB8" s="52" t="s">
-        <v>291</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14098,44 +14095,46 @@
         <v>90</v>
       </c>
       <c r="C9" s="52" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="68">
-        <v>46288</v>
-      </c>
-      <c r="E9" s="52"/>
+        <v>42</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>274</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>27</v>
+      </c>
       <c r="F9" s="52">
-        <v>262705</v>
-      </c>
-      <c r="G9" s="52">
-        <v>1768</v>
+        <v>262677</v>
+      </c>
+      <c r="G9" s="52" t="s">
+        <v>292</v>
       </c>
       <c r="H9" s="52">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="I9" s="54">
-        <v>0.79700000000000004</v>
+        <v>0.8</v>
       </c>
       <c r="J9" s="54">
-        <v>1.4870000000000001</v>
+        <v>1.171</v>
       </c>
       <c r="K9" s="52" t="s">
         <v>33</v>
       </c>
       <c r="L9" s="54">
-        <v>237.02799999999999</v>
+        <v>936.8</v>
       </c>
       <c r="M9" s="55">
-        <v>297.39999999999998</v>
+        <v>1171</v>
       </c>
       <c r="N9" s="56">
-        <v>8.2600000000000007E-2</v>
+        <v>0.32529999999999998</v>
       </c>
       <c r="O9" s="57">
-        <v>4.96</v>
+        <v>19.52</v>
       </c>
       <c r="P9" s="52">
-        <v>74.7</v>
+        <v>323.2</v>
       </c>
       <c r="Q9" s="52">
         <v>1</v>
@@ -14144,117 +14143,201 @@
         <v>850</v>
       </c>
       <c r="S9" s="54">
+        <v>0.8</v>
+      </c>
+      <c r="T9" s="52">
+        <v>50</v>
+      </c>
+      <c r="U9" s="56">
+        <v>5.8799999999999998E-2</v>
+      </c>
+      <c r="V9" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="W9" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB9" s="52" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="92">
+        <v>8</v>
+      </c>
+      <c r="B10" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="68">
+        <v>46288</v>
+      </c>
+      <c r="E10" s="52"/>
+      <c r="F10" s="52">
+        <v>262705</v>
+      </c>
+      <c r="G10" s="52">
+        <v>1768</v>
+      </c>
+      <c r="H10" s="52">
+        <v>200</v>
+      </c>
+      <c r="I10" s="54">
         <v>0.79700000000000004</v>
       </c>
-      <c r="T9" s="52">
+      <c r="J10" s="54">
+        <v>1.4870000000000001</v>
+      </c>
+      <c r="K10" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="L10" s="54">
+        <v>237.02799999999999</v>
+      </c>
+      <c r="M10" s="55">
+        <v>297.39999999999998</v>
+      </c>
+      <c r="N10" s="56">
+        <v>8.2600000000000007E-2</v>
+      </c>
+      <c r="O10" s="57">
+        <v>4.96</v>
+      </c>
+      <c r="P10" s="52">
+        <v>74.7</v>
+      </c>
+      <c r="Q10" s="52">
+        <v>1</v>
+      </c>
+      <c r="R10" s="52">
+        <v>850</v>
+      </c>
+      <c r="S10" s="54">
+        <v>0.79700000000000004</v>
+      </c>
+      <c r="T10" s="52">
         <v>53</v>
       </c>
-      <c r="U9" s="56">
+      <c r="U10" s="56">
         <v>6.2399999999999997E-2</v>
       </c>
-      <c r="V9" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="52"/>
-      <c r="Z9" s="52"/>
-      <c r="AA9" s="52">
+      <c r="V10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="52"/>
+      <c r="Z10" s="52"/>
+      <c r="AA10" s="52">
         <v>1</v>
       </c>
-      <c r="AB9" s="52" t="s">
+      <c r="AB10" s="52" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="59">
-        <f>SUM(H3:H9)</f>
-        <v>3000</v>
-      </c>
-      <c r="I10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="K10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="M10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="O10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="P10" s="59">
-        <f>SUM(P3:P9)</f>
-        <v>1366.8</v>
-      </c>
-      <c r="Q10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="R10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="S10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="T10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="U10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="V10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="W10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="X10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB10" s="59" t="s">
+    <row r="11" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="59">
+        <f>SUM(H3:H10)</f>
+        <v>3220</v>
+      </c>
+      <c r="I11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P11" s="59">
+        <f>SUM(P3:P10)</f>
+        <v>1449.7</v>
+      </c>
+      <c r="Q11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB11" s="59" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/09/2026 14:05)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,29 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CCD6D7A-5294-4E4D-ABF3-9A25BF761622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5483660-88EE-43E5-84B7-D88F65CF0517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="FAVINCO 1229" sheetId="167" r:id="rId1"/>
-    <sheet name="RM Embalagens P" sheetId="166" r:id="rId2"/>
-    <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId3"/>
-    <sheet name="FORBOX 1220" sheetId="163" r:id="rId4"/>
-    <sheet name="HARMONY EMBALAGENS 1217 P" sheetId="162" r:id="rId5"/>
-    <sheet name="Z4A EMBALAGENS LTDA 1216" sheetId="161" r:id="rId6"/>
-    <sheet name="Tolecaixas 1215" sheetId="160" r:id="rId7"/>
-    <sheet name="ABAPEL 1213" sheetId="159" r:id="rId8"/>
-    <sheet name="IPE - PCBOX 1212 P" sheetId="158" r:id="rId9"/>
-    <sheet name="Z4A EMBALAGENS LTDA 1210 P" sheetId="157" r:id="rId10"/>
-    <sheet name="RM Embalagens 1209 P" sheetId="156" r:id="rId11"/>
-    <sheet name="ABAPEL 1201 P" sheetId="153" r:id="rId12"/>
-    <sheet name="HARMONY EMBALAGENS 1200 P" sheetId="152" r:id="rId13"/>
-    <sheet name="FAVINCO EMBALAGENS 1197 P" sheetId="150" r:id="rId14"/>
-    <sheet name="ABAPEL 1196 P" sheetId="149" r:id="rId15"/>
-    <sheet name="RM Embalagens 1184 P" sheetId="141" r:id="rId16"/>
-    <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId17"/>
-    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId18"/>
+    <sheet name="HARMONY EMBALAGENS 1231" sheetId="168" r:id="rId1"/>
+    <sheet name="FAVINCO 1229" sheetId="167" r:id="rId2"/>
+    <sheet name="RM Embalagens P" sheetId="166" r:id="rId3"/>
+    <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId4"/>
+    <sheet name="FORBOX 1220" sheetId="163" r:id="rId5"/>
+    <sheet name="HARMONY EMBALAGENS 1217 P" sheetId="162" r:id="rId6"/>
+    <sheet name="Z4A EMBALAGENS LTDA 1216" sheetId="161" r:id="rId7"/>
+    <sheet name="Tolecaixas 1215" sheetId="160" r:id="rId8"/>
+    <sheet name="ABAPEL 1213" sheetId="159" r:id="rId9"/>
+    <sheet name="IPE - PCBOX 1212 P" sheetId="158" r:id="rId10"/>
+    <sheet name="Z4A EMBALAGENS LTDA 1210 P" sheetId="157" r:id="rId11"/>
+    <sheet name="RM Embalagens 1209 P" sheetId="156" r:id="rId12"/>
+    <sheet name="ABAPEL 1201 P" sheetId="153" r:id="rId13"/>
+    <sheet name="HARMONY EMBALAGENS 1200 P" sheetId="152" r:id="rId14"/>
+    <sheet name="FAVINCO EMBALAGENS 1197 P" sheetId="150" r:id="rId15"/>
+    <sheet name="ABAPEL 1196 P" sheetId="149" r:id="rId16"/>
+    <sheet name="RM Embalagens 1184 P" sheetId="141" r:id="rId17"/>
+    <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId18"/>
+    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3209" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3512" uniqueCount="370">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1056,6 +1057,111 @@
   </si>
   <si>
     <t>870x1427</t>
+  </si>
+  <si>
+    <t>995x1966</t>
+  </si>
+  <si>
+    <t>89x147x89</t>
+  </si>
+  <si>
+    <t>23-09-26</t>
+  </si>
+  <si>
+    <t>23/09/2026</t>
+  </si>
+  <si>
+    <t>932x1838</t>
+  </si>
+  <si>
+    <t>93x118x93</t>
+  </si>
+  <si>
+    <t>950x1658</t>
+  </si>
+  <si>
+    <t>78x154x78</t>
+  </si>
+  <si>
+    <t>1096x1758</t>
+  </si>
+  <si>
+    <t>820x1640</t>
+  </si>
+  <si>
+    <t>1040x2174</t>
+  </si>
+  <si>
+    <t>132x246x132</t>
+  </si>
+  <si>
+    <t>992x1938</t>
+  </si>
+  <si>
+    <t>105x114x105</t>
+  </si>
+  <si>
+    <t>1014x1859</t>
+  </si>
+  <si>
+    <t>330x334x330</t>
+  </si>
+  <si>
+    <t>1078x1856</t>
+  </si>
+  <si>
+    <t>90x349x90</t>
+  </si>
+  <si>
+    <t>1118x1936</t>
+  </si>
+  <si>
+    <t>40x469x40</t>
+  </si>
+  <si>
+    <t>938x1529</t>
+  </si>
+  <si>
+    <t>230x109x120</t>
+  </si>
+  <si>
+    <t>699x1549</t>
+  </si>
+  <si>
+    <t>170x339x170</t>
+  </si>
+  <si>
+    <t>720x1979</t>
+  </si>
+  <si>
+    <t>243x214x243</t>
+  </si>
+  <si>
+    <t>1000x1439</t>
+  </si>
+  <si>
+    <t>168x154x168</t>
+  </si>
+  <si>
+    <t>784x1339</t>
+  </si>
+  <si>
+    <t>270x224x270</t>
+  </si>
+  <si>
+    <t>769x1759</t>
+  </si>
+  <si>
+    <t>185x379x185</t>
+  </si>
+  <si>
+    <t>794x1569</t>
+  </si>
+  <si>
+    <t>230x314x230</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - HARMONY EMBALAGENS  —  OF: 001231</t>
   </si>
 </sst>
 </file>
@@ -1253,7 +1359,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1545,6 +1651,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1767,127 +1876,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5961B2D-99FA-47E1-921A-0764410641DC}">
-  <dimension ref="A1:AB4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1138A384-FB07-407A-A271-F489A21E653B}">
+  <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="34" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="34" customWidth="1"/>
-    <col min="3" max="3" width="5.77734375" style="34" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" style="34" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="9" style="34" customWidth="1"/>
-    <col min="6" max="6" width="6.77734375" style="34" customWidth="1"/>
-    <col min="7" max="7" width="4.5546875" style="34" customWidth="1"/>
-    <col min="8" max="8" width="5.109375" style="34" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" style="34" customWidth="1"/>
-    <col min="10" max="10" width="6.33203125" style="34" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" style="34" customWidth="1"/>
+    <col min="5" max="5" width="7.88671875" style="34" customWidth="1"/>
+    <col min="6" max="6" width="7.21875" style="34" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" style="34" customWidth="1"/>
+    <col min="8" max="8" width="5.5546875" style="34" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" style="34" customWidth="1"/>
+    <col min="10" max="10" width="7.5546875" style="34" customWidth="1"/>
+    <col min="11" max="11" width="13.21875" style="34" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="34" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="34" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.5546875" style="34" customWidth="1"/>
-    <col min="17" max="17" width="3.33203125" style="34" customWidth="1"/>
-    <col min="18" max="18" width="5.109375" style="34" customWidth="1"/>
-    <col min="19" max="19" width="5.88671875" style="34" customWidth="1"/>
+    <col min="16" max="16" width="8.77734375" style="34" customWidth="1"/>
+    <col min="17" max="17" width="4.33203125" style="34" customWidth="1"/>
+    <col min="18" max="18" width="5.77734375" style="34" customWidth="1"/>
+    <col min="19" max="19" width="6.33203125" style="34" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="34" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="6.44140625" style="34" customWidth="1"/>
-    <col min="23" max="23" width="8.21875" style="34" customWidth="1"/>
-    <col min="24" max="24" width="8.5546875" style="34" customWidth="1"/>
-    <col min="25" max="25" width="10.44140625" style="34" customWidth="1"/>
-    <col min="26" max="26" width="10.109375" style="34" customWidth="1"/>
-    <col min="27" max="27" width="4.5546875" style="34" customWidth="1"/>
-    <col min="28" max="28" width="11.109375" style="34" customWidth="1"/>
+    <col min="22" max="22" width="8.21875" style="34" customWidth="1"/>
+    <col min="23" max="23" width="7.77734375" style="34" customWidth="1"/>
+    <col min="24" max="24" width="8" style="34" customWidth="1"/>
+    <col min="25" max="25" width="7.109375" style="34" customWidth="1"/>
+    <col min="26" max="26" width="8" style="34" customWidth="1"/>
+    <col min="27" max="27" width="5.21875" style="34" customWidth="1"/>
+    <col min="28" max="28" width="9.5546875" style="34" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
-        <v>333</v>
-      </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="103" t="s">
+        <v>369</v>
+      </c>
+      <c r="B1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="103" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
         <v>0</v>
       </c>
@@ -1973,175 +2082,1551 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="42">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="52">
         <v>1</v>
       </c>
-      <c r="B3" s="44" t="s">
-        <v>126</v>
-      </c>
-      <c r="C3" s="42" t="s">
+      <c r="B3" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E3" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="52">
+        <v>262714</v>
+      </c>
+      <c r="G3" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H3" s="52">
+        <v>200</v>
+      </c>
+      <c r="I3" s="54">
+        <v>0.77400000000000002</v>
+      </c>
+      <c r="J3" s="54">
+        <v>1.5489999999999999</v>
+      </c>
+      <c r="K3" s="52" t="s">
+        <v>368</v>
+      </c>
+      <c r="L3" s="54">
+        <v>239.785</v>
+      </c>
+      <c r="M3" s="55">
+        <v>154.9</v>
+      </c>
+      <c r="N3" s="56">
+        <v>2.1499999999999998E-2</v>
+      </c>
+      <c r="O3" s="57">
+        <v>1.29</v>
+      </c>
+      <c r="P3" s="52">
+        <v>129</v>
+      </c>
+      <c r="Q3" s="52">
+        <v>2</v>
+      </c>
+      <c r="R3" s="52">
+        <v>1600</v>
+      </c>
+      <c r="S3" s="54">
+        <v>1.548</v>
+      </c>
+      <c r="T3" s="52">
+        <v>52</v>
+      </c>
+      <c r="U3" s="56">
+        <v>3.2500000000000001E-2</v>
+      </c>
+      <c r="V3" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB3" s="52" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="52">
+        <v>2</v>
+      </c>
+      <c r="B4" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E4" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="52">
+        <v>262708</v>
+      </c>
+      <c r="G4" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H4" s="52">
+        <v>330</v>
+      </c>
+      <c r="I4" s="54">
+        <v>0.749</v>
+      </c>
+      <c r="J4" s="54">
+        <v>1.7390000000000001</v>
+      </c>
+      <c r="K4" s="52" t="s">
+        <v>366</v>
+      </c>
+      <c r="L4" s="54">
+        <v>429.82900000000001</v>
+      </c>
+      <c r="M4" s="55">
+        <v>286.89999999999998</v>
+      </c>
+      <c r="N4" s="56">
+        <v>3.9899999999999998E-2</v>
+      </c>
+      <c r="O4" s="57">
+        <v>2.39</v>
+      </c>
+      <c r="P4" s="52">
+        <v>244.1</v>
+      </c>
+      <c r="Q4" s="52">
+        <v>2</v>
+      </c>
+      <c r="R4" s="52">
+        <v>1550</v>
+      </c>
+      <c r="S4" s="54">
+        <v>1.498</v>
+      </c>
+      <c r="T4" s="52">
+        <v>52</v>
+      </c>
+      <c r="U4" s="56">
+        <v>3.3500000000000002E-2</v>
+      </c>
+      <c r="V4" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="W4" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="X4" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y4" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z4" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA4" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB4" s="52" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="52">
+        <v>3</v>
+      </c>
+      <c r="B5" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E5" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="52">
+        <v>262718</v>
+      </c>
+      <c r="G5" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H5" s="52">
+        <v>200</v>
+      </c>
+      <c r="I5" s="54">
+        <v>0.76400000000000001</v>
+      </c>
+      <c r="J5" s="54">
+        <v>1.319</v>
+      </c>
+      <c r="K5" s="52" t="s">
+        <v>364</v>
+      </c>
+      <c r="L5" s="54">
+        <v>201.54300000000001</v>
+      </c>
+      <c r="M5" s="55">
+        <v>131.9</v>
+      </c>
+      <c r="N5" s="56">
+        <v>1.83E-2</v>
+      </c>
+      <c r="O5" s="57">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="P5" s="52">
+        <v>108.4</v>
+      </c>
+      <c r="Q5" s="52">
+        <v>2</v>
+      </c>
+      <c r="R5" s="52">
+        <v>1550</v>
+      </c>
+      <c r="S5" s="54">
+        <v>1.528</v>
+      </c>
+      <c r="T5" s="52">
+        <v>22</v>
+      </c>
+      <c r="U5" s="56">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="V5" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB5" s="52" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="52">
+        <v>4</v>
+      </c>
+      <c r="B6" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E6" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="52">
+        <v>262715</v>
+      </c>
+      <c r="G6" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H6" s="52">
+        <v>300</v>
+      </c>
+      <c r="I6" s="54">
+        <v>0.49</v>
+      </c>
+      <c r="J6" s="54">
+        <v>1.419</v>
+      </c>
+      <c r="K6" s="52" t="s">
+        <v>362</v>
+      </c>
+      <c r="L6" s="54">
+        <v>208.59299999999999</v>
+      </c>
+      <c r="M6" s="55">
+        <v>141.9</v>
+      </c>
+      <c r="N6" s="56">
+        <v>1.3100000000000001E-2</v>
+      </c>
+      <c r="O6" s="57">
+        <v>0.79</v>
+      </c>
+      <c r="P6" s="52">
+        <v>112.2</v>
+      </c>
+      <c r="Q6" s="52">
+        <v>3</v>
+      </c>
+      <c r="R6" s="52">
+        <v>1500</v>
+      </c>
+      <c r="S6" s="54">
+        <v>1.47</v>
+      </c>
+      <c r="T6" s="52">
+        <v>30</v>
+      </c>
+      <c r="U6" s="56">
+        <v>0.02</v>
+      </c>
+      <c r="V6" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB6" s="52" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="52">
+        <v>5</v>
+      </c>
+      <c r="B7" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="52">
+        <v>262712</v>
+      </c>
+      <c r="G7" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H7" s="52">
+        <v>150</v>
+      </c>
+      <c r="I7" s="54">
+        <v>0.7</v>
+      </c>
+      <c r="J7" s="54">
+        <v>1.9590000000000001</v>
+      </c>
+      <c r="K7" s="52" t="s">
+        <v>360</v>
+      </c>
+      <c r="L7" s="54">
+        <v>205.69499999999999</v>
+      </c>
+      <c r="M7" s="55">
+        <v>146.9</v>
+      </c>
+      <c r="N7" s="56">
+        <v>2.0400000000000001E-2</v>
+      </c>
+      <c r="O7" s="57">
+        <v>1.22</v>
+      </c>
+      <c r="P7" s="52">
+        <v>110.7</v>
+      </c>
+      <c r="Q7" s="52">
+        <v>2</v>
+      </c>
+      <c r="R7" s="52">
+        <v>1450</v>
+      </c>
+      <c r="S7" s="54">
+        <v>1.4</v>
+      </c>
+      <c r="T7" s="52">
+        <v>50</v>
+      </c>
+      <c r="U7" s="56">
+        <v>3.4500000000000003E-2</v>
+      </c>
+      <c r="V7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB7" s="52" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="52">
+        <v>6</v>
+      </c>
+      <c r="B8" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="52">
+        <v>262707</v>
+      </c>
+      <c r="G8" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H8" s="52">
+        <v>330</v>
+      </c>
+      <c r="I8" s="54">
+        <v>0.67900000000000005</v>
+      </c>
+      <c r="J8" s="54">
+        <v>1.5289999999999999</v>
+      </c>
+      <c r="K8" s="52" t="s">
+        <v>358</v>
+      </c>
+      <c r="L8" s="54">
+        <v>342.60300000000001</v>
+      </c>
+      <c r="M8" s="55">
+        <v>252.3</v>
+      </c>
+      <c r="N8" s="56">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="O8" s="57">
+        <v>2.1</v>
+      </c>
+      <c r="P8" s="52">
+        <v>194.6</v>
+      </c>
+      <c r="Q8" s="52">
+        <v>2</v>
+      </c>
+      <c r="R8" s="52">
+        <v>1400</v>
+      </c>
+      <c r="S8" s="54">
+        <v>1.3580000000000001</v>
+      </c>
+      <c r="T8" s="52">
+        <v>42</v>
+      </c>
+      <c r="U8" s="56">
+        <v>0.03</v>
+      </c>
+      <c r="V8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="W8" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="X8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA8" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB8" s="52" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="52">
+        <v>7</v>
+      </c>
+      <c r="B9" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="52">
+        <v>262711</v>
+      </c>
+      <c r="G9" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H9" s="52">
+        <v>250</v>
+      </c>
+      <c r="I9" s="54">
+        <v>0.45900000000000002</v>
+      </c>
+      <c r="J9" s="54">
+        <v>1.5089999999999999</v>
+      </c>
+      <c r="K9" s="52" t="s">
+        <v>356</v>
+      </c>
+      <c r="L9" s="54">
+        <v>173.15799999999999</v>
+      </c>
+      <c r="M9" s="55">
+        <v>125.8</v>
+      </c>
+      <c r="N9" s="56">
+        <v>1.1599999999999999E-2</v>
+      </c>
+      <c r="O9" s="57">
+        <v>0.7</v>
+      </c>
+      <c r="P9" s="52">
+        <v>93.2</v>
+      </c>
+      <c r="Q9" s="52">
+        <v>3</v>
+      </c>
+      <c r="R9" s="52">
+        <v>1400</v>
+      </c>
+      <c r="S9" s="54">
+        <v>1.377</v>
+      </c>
+      <c r="T9" s="52">
+        <v>23</v>
+      </c>
+      <c r="U9" s="56">
+        <v>1.6400000000000001E-2</v>
+      </c>
+      <c r="V9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z9" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA9" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB9" s="52" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="52">
+        <v>8</v>
+      </c>
+      <c r="B10" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E10" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="52">
+        <v>262719</v>
+      </c>
+      <c r="G10" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H10" s="52">
+        <v>700</v>
+      </c>
+      <c r="I10" s="54">
+        <v>0.54900000000000004</v>
+      </c>
+      <c r="J10" s="54">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="K10" s="52" t="s">
+        <v>354</v>
+      </c>
+      <c r="L10" s="54">
+        <v>184.08</v>
+      </c>
+      <c r="M10" s="55">
+        <v>167.7</v>
+      </c>
+      <c r="N10" s="56">
+        <v>2.3300000000000001E-2</v>
+      </c>
+      <c r="O10" s="57">
+        <v>1.4</v>
+      </c>
+      <c r="P10" s="52">
+        <v>99</v>
+      </c>
+      <c r="Q10" s="52">
+        <v>2</v>
+      </c>
+      <c r="R10" s="52">
+        <v>1150</v>
+      </c>
+      <c r="S10" s="54">
+        <v>1.0980000000000001</v>
+      </c>
+      <c r="T10" s="52">
+        <v>52</v>
+      </c>
+      <c r="U10" s="56">
+        <v>4.5199999999999997E-2</v>
+      </c>
+      <c r="V10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA10" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB10" s="52" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="52">
+        <v>9</v>
+      </c>
+      <c r="B11" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E11" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="52">
+        <v>262716</v>
+      </c>
+      <c r="G11" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H11" s="52">
+        <v>700</v>
+      </c>
+      <c r="I11" s="54">
+        <v>0.52900000000000003</v>
+      </c>
+      <c r="J11" s="54">
+        <v>0.45900000000000002</v>
+      </c>
+      <c r="K11" s="52" t="s">
+        <v>352</v>
+      </c>
+      <c r="L11" s="54">
+        <v>169.96799999999999</v>
+      </c>
+      <c r="M11" s="55">
+        <v>160.69999999999999</v>
+      </c>
+      <c r="N11" s="56">
+        <v>2.23E-2</v>
+      </c>
+      <c r="O11" s="57">
+        <v>1.34</v>
+      </c>
+      <c r="P11" s="52">
+        <v>91.4</v>
+      </c>
+      <c r="Q11" s="52">
+        <v>2</v>
+      </c>
+      <c r="R11" s="52">
+        <v>1100</v>
+      </c>
+      <c r="S11" s="54">
+        <v>1.0580000000000001</v>
+      </c>
+      <c r="T11" s="52">
+        <v>42</v>
+      </c>
+      <c r="U11" s="56">
+        <v>3.8199999999999998E-2</v>
+      </c>
+      <c r="V11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA11" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB11" s="52" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="52">
+        <v>10</v>
+      </c>
+      <c r="B12" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E12" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="52">
+        <v>262717</v>
+      </c>
+      <c r="G12" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H12" s="52">
+        <v>100</v>
+      </c>
+      <c r="I12" s="54">
+        <v>0.99399999999999999</v>
+      </c>
+      <c r="J12" s="54">
+        <v>1.839</v>
+      </c>
+      <c r="K12" s="52" t="s">
+        <v>350</v>
+      </c>
+      <c r="L12" s="54">
+        <v>182.797</v>
+      </c>
+      <c r="M12" s="55">
+        <v>183.9</v>
+      </c>
+      <c r="N12" s="56">
+        <v>5.11E-2</v>
+      </c>
+      <c r="O12" s="57">
+        <v>3.06</v>
+      </c>
+      <c r="P12" s="52">
+        <v>98.3</v>
+      </c>
+      <c r="Q12" s="52">
+        <v>1</v>
+      </c>
+      <c r="R12" s="52">
+        <v>1050</v>
+      </c>
+      <c r="S12" s="54">
+        <v>0.99399999999999999</v>
+      </c>
+      <c r="T12" s="52">
+        <v>56</v>
+      </c>
+      <c r="U12" s="56">
+        <v>5.33E-2</v>
+      </c>
+      <c r="V12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z12" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA12" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB12" s="52" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="52">
+        <v>11</v>
+      </c>
+      <c r="B13" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E13" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="52">
+        <v>262713</v>
+      </c>
+      <c r="G13" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H13" s="52">
+        <v>500</v>
+      </c>
+      <c r="I13" s="54">
+        <v>0.32400000000000001</v>
+      </c>
+      <c r="J13" s="54">
+        <v>0.95899999999999996</v>
+      </c>
+      <c r="K13" s="52" t="s">
+        <v>348</v>
+      </c>
+      <c r="L13" s="54">
+        <v>155.358</v>
+      </c>
+      <c r="M13" s="55">
+        <v>239.8</v>
+      </c>
+      <c r="N13" s="56">
+        <v>3.3300000000000003E-2</v>
+      </c>
+      <c r="O13" s="57">
+        <v>2</v>
+      </c>
+      <c r="P13" s="52">
+        <v>83.6</v>
+      </c>
+      <c r="Q13" s="52">
+        <v>2</v>
+      </c>
+      <c r="R13" s="52">
+        <v>700</v>
+      </c>
+      <c r="S13" s="54">
+        <v>0.64800000000000002</v>
+      </c>
+      <c r="T13" s="52">
+        <v>52</v>
+      </c>
+      <c r="U13" s="56">
+        <v>7.4300000000000005E-2</v>
+      </c>
+      <c r="V13" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X13" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z13" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA13" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB13" s="52" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="52">
+        <v>12</v>
+      </c>
+      <c r="B14" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="42" t="s">
-        <v>331</v>
-      </c>
-      <c r="E3" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="42">
-        <v>262704</v>
-      </c>
-      <c r="G3" s="42" t="s">
-        <v>330</v>
-      </c>
-      <c r="H3" s="42">
-        <v>4000</v>
-      </c>
-      <c r="I3" s="43">
-        <v>0.27900000000000003</v>
-      </c>
-      <c r="J3" s="43">
-        <v>1.002</v>
-      </c>
-      <c r="K3" s="42" t="s">
-        <v>188</v>
-      </c>
-      <c r="L3" s="39">
-        <v>1118.232</v>
-      </c>
-      <c r="M3" s="41">
-        <v>1336</v>
-      </c>
-      <c r="N3" s="38">
-        <v>0.1237</v>
-      </c>
-      <c r="O3" s="40">
-        <v>7.42</v>
-      </c>
-      <c r="P3" s="37">
-        <v>352.2</v>
-      </c>
-      <c r="Q3" s="37">
+      <c r="D14" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E14" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="52">
+        <v>262710</v>
+      </c>
+      <c r="G14" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H14" s="52">
+        <v>500</v>
+      </c>
+      <c r="I14" s="54">
+        <v>0.51</v>
+      </c>
+      <c r="J14" s="54">
+        <v>1.077</v>
+      </c>
+      <c r="K14" s="52" t="s">
+        <v>346</v>
+      </c>
+      <c r="L14" s="54">
+        <v>274.63499999999999</v>
+      </c>
+      <c r="M14" s="55">
+        <v>179.5</v>
+      </c>
+      <c r="N14" s="56">
+        <v>1.66E-2</v>
+      </c>
+      <c r="O14" s="57">
+        <v>1</v>
+      </c>
+      <c r="P14" s="52">
+        <v>86.5</v>
+      </c>
+      <c r="Q14" s="52">
         <v>3</v>
       </c>
-      <c r="R3" s="37">
-        <v>900</v>
-      </c>
-      <c r="S3" s="39">
-        <v>0.83699999999999997</v>
-      </c>
-      <c r="T3" s="37">
-        <v>63</v>
-      </c>
-      <c r="U3" s="38">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="V3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB3" s="37" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="36">
-        <v>4000</v>
-      </c>
-      <c r="I4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="L4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="P4" s="35">
-        <v>352.2</v>
-      </c>
-      <c r="Q4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="R4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="S4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="T4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="U4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="V4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="W4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="X4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB4" s="35" t="s">
+      <c r="R14" s="52">
+        <v>1550</v>
+      </c>
+      <c r="S14" s="54">
+        <v>1.53</v>
+      </c>
+      <c r="T14" s="52">
+        <v>20</v>
+      </c>
+      <c r="U14" s="56">
+        <v>1.29E-2</v>
+      </c>
+      <c r="V14" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB14" s="52" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="52">
+        <v>13</v>
+      </c>
+      <c r="B15" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E15" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="52">
+        <v>262720</v>
+      </c>
+      <c r="G15" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H15" s="52">
+        <v>1000</v>
+      </c>
+      <c r="I15" s="54">
+        <v>0.4</v>
+      </c>
+      <c r="J15" s="54">
+        <v>0.81</v>
+      </c>
+      <c r="K15" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="L15" s="54">
+        <v>324</v>
+      </c>
+      <c r="M15" s="55">
+        <v>270</v>
+      </c>
+      <c r="N15" s="56">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="O15" s="57">
+        <v>1.5</v>
+      </c>
+      <c r="P15" s="52">
+        <v>102.1</v>
+      </c>
+      <c r="Q15" s="52">
+        <v>3</v>
+      </c>
+      <c r="R15" s="52">
+        <v>1250</v>
+      </c>
+      <c r="S15" s="54">
+        <v>1.2</v>
+      </c>
+      <c r="T15" s="52">
+        <v>50</v>
+      </c>
+      <c r="U15" s="56">
+        <v>0.04</v>
+      </c>
+      <c r="V15" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB15" s="52" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="52">
+        <v>14</v>
+      </c>
+      <c r="B16" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E16" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="52">
+        <v>262721</v>
+      </c>
+      <c r="G16" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H16" s="52">
+        <v>275</v>
+      </c>
+      <c r="I16" s="54">
+        <v>1.0760000000000001</v>
+      </c>
+      <c r="J16" s="54">
+        <v>0.86899999999999999</v>
+      </c>
+      <c r="K16" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="L16" s="54">
+        <v>257.137</v>
+      </c>
+      <c r="M16" s="55">
+        <v>239</v>
+      </c>
+      <c r="N16" s="56">
+        <v>6.6400000000000001E-2</v>
+      </c>
+      <c r="O16" s="57">
+        <v>3.98</v>
+      </c>
+      <c r="P16" s="52">
+        <v>81</v>
+      </c>
+      <c r="Q16" s="52">
+        <v>1</v>
+      </c>
+      <c r="R16" s="52">
+        <v>1100</v>
+      </c>
+      <c r="S16" s="54">
+        <v>1.0760000000000001</v>
+      </c>
+      <c r="T16" s="52">
+        <v>24</v>
+      </c>
+      <c r="U16" s="56">
+        <v>2.18E-2</v>
+      </c>
+      <c r="V16" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y16" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z16" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA16" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB16" s="52" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="52">
+        <v>15</v>
+      </c>
+      <c r="B17" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E17" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="52">
+        <v>262709</v>
+      </c>
+      <c r="G17" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H17" s="52">
+        <v>1100</v>
+      </c>
+      <c r="I17" s="54">
+        <v>0.31</v>
+      </c>
+      <c r="J17" s="54">
+        <v>0.81899999999999995</v>
+      </c>
+      <c r="K17" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="L17" s="54">
+        <v>279.279</v>
+      </c>
+      <c r="M17" s="55">
+        <v>300.3</v>
+      </c>
+      <c r="N17" s="56">
+        <v>2.7799999999999998E-2</v>
+      </c>
+      <c r="O17" s="57">
+        <v>1.67</v>
+      </c>
+      <c r="P17" s="52">
+        <v>88</v>
+      </c>
+      <c r="Q17" s="52">
+        <v>3</v>
+      </c>
+      <c r="R17" s="52">
+        <v>950</v>
+      </c>
+      <c r="S17" s="54">
+        <v>0.93</v>
+      </c>
+      <c r="T17" s="52">
+        <v>20</v>
+      </c>
+      <c r="U17" s="56">
+        <v>2.1100000000000001E-2</v>
+      </c>
+      <c r="V17" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W17" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X17" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y17" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB17" s="52" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="52">
+        <v>16</v>
+      </c>
+      <c r="B18" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="52">
+        <v>262722</v>
+      </c>
+      <c r="G18" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H18" s="52">
+        <v>1000</v>
+      </c>
+      <c r="I18" s="54">
+        <v>0.30399999999999999</v>
+      </c>
+      <c r="J18" s="54">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="K18" s="52" t="s">
+        <v>340</v>
+      </c>
+      <c r="L18" s="54">
+        <v>276.33600000000001</v>
+      </c>
+      <c r="M18" s="55">
+        <v>303</v>
+      </c>
+      <c r="N18" s="56">
+        <v>2.81E-2</v>
+      </c>
+      <c r="O18" s="57">
+        <v>1.68</v>
+      </c>
+      <c r="P18" s="52">
+        <v>87</v>
+      </c>
+      <c r="Q18" s="52">
+        <v>3</v>
+      </c>
+      <c r="R18" s="52">
+        <v>950</v>
+      </c>
+      <c r="S18" s="54">
+        <v>0.91200000000000003</v>
+      </c>
+      <c r="T18" s="52">
+        <v>38</v>
+      </c>
+      <c r="U18" s="56">
+        <v>0.04</v>
+      </c>
+      <c r="V18" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W18" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X18" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB18" s="52" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="52">
+        <v>17</v>
+      </c>
+      <c r="B19" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="E19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="52">
+        <v>262723</v>
+      </c>
+      <c r="G19" s="52" t="s">
+        <v>337</v>
+      </c>
+      <c r="H19" s="52">
+        <v>1000</v>
+      </c>
+      <c r="I19" s="54">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="J19" s="54">
+        <v>0.97299999999999998</v>
+      </c>
+      <c r="K19" s="52" t="s">
+        <v>336</v>
+      </c>
+      <c r="L19" s="54">
+        <v>316.22500000000002</v>
+      </c>
+      <c r="M19" s="55">
+        <v>486.5</v>
+      </c>
+      <c r="N19" s="56">
+        <v>6.7599999999999993E-2</v>
+      </c>
+      <c r="O19" s="57">
+        <v>4.05</v>
+      </c>
+      <c r="P19" s="52">
+        <v>99.6</v>
+      </c>
+      <c r="Q19" s="52">
+        <v>2</v>
+      </c>
+      <c r="R19" s="52">
+        <v>700</v>
+      </c>
+      <c r="S19" s="54">
+        <v>0.65</v>
+      </c>
+      <c r="T19" s="52">
+        <v>50</v>
+      </c>
+      <c r="U19" s="56">
+        <v>7.1400000000000005E-2</v>
+      </c>
+      <c r="V19" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W19" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X19" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB19" s="52" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" s="59">
+        <v>8635</v>
+      </c>
+      <c r="I20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P20" s="59">
+        <v>1908.8</v>
+      </c>
+      <c r="Q20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA20" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB20" s="59" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2150,11 +3635,1077 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00EADB3A-C171-49AE-8471-729057A3A740}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.33203125" style="34" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="34" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" style="34" customWidth="1"/>
+    <col min="6" max="6" width="7.109375" style="34" customWidth="1"/>
+    <col min="7" max="7" width="5.77734375" style="34" customWidth="1"/>
+    <col min="8" max="8" width="6" style="34" customWidth="1"/>
+    <col min="9" max="9" width="7.21875" style="34" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" style="34" customWidth="1"/>
+    <col min="11" max="11" width="6" style="34" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.44140625" style="34" customWidth="1"/>
+    <col min="17" max="17" width="4.21875" style="34" customWidth="1"/>
+    <col min="18" max="18" width="6.44140625" style="34" customWidth="1"/>
+    <col min="19" max="19" width="5.77734375" style="34" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.77734375" style="34" customWidth="1"/>
+    <col min="23" max="23" width="7.6640625" style="34" customWidth="1"/>
+    <col min="24" max="24" width="7.44140625" style="34" customWidth="1"/>
+    <col min="25" max="25" width="7.77734375" style="34" customWidth="1"/>
+    <col min="26" max="26" width="7.44140625" style="34" customWidth="1"/>
+    <col min="27" max="27" width="4.21875" style="34" customWidth="1"/>
+    <col min="28" max="28" width="11.33203125" style="34" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="34"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="97" t="s">
+        <v>228</v>
+      </c>
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="45" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="45" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="45" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="45" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="45" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="45" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" s="92" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="92">
+        <v>1</v>
+      </c>
+      <c r="B3" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="92" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="93">
+        <v>46283</v>
+      </c>
+      <c r="F3" s="92">
+        <v>262665</v>
+      </c>
+      <c r="G3" s="92">
+        <v>1749</v>
+      </c>
+      <c r="H3" s="92">
+        <v>500</v>
+      </c>
+      <c r="I3" s="92">
+        <v>1.494</v>
+      </c>
+      <c r="J3" s="92">
+        <v>2.5630000000000002</v>
+      </c>
+      <c r="K3" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="92">
+        <v>1914.5609999999999</v>
+      </c>
+      <c r="M3" s="92">
+        <v>1281.5</v>
+      </c>
+      <c r="N3" s="92">
+        <v>0.35599999999999998</v>
+      </c>
+      <c r="O3" s="92">
+        <v>21.36</v>
+      </c>
+      <c r="P3" s="92">
+        <v>1087.5</v>
+      </c>
+      <c r="Q3" s="92">
+        <v>1</v>
+      </c>
+      <c r="R3" s="92">
+        <v>1550</v>
+      </c>
+      <c r="S3" s="92">
+        <v>1.494</v>
+      </c>
+      <c r="T3" s="92">
+        <v>56</v>
+      </c>
+      <c r="U3" s="92">
+        <v>3.61E-2</v>
+      </c>
+      <c r="V3" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="W3" s="92" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y3" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z3" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="92">
+        <v>3</v>
+      </c>
+      <c r="AB3" s="92" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="92" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="92">
+        <v>2</v>
+      </c>
+      <c r="B4" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="92" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="93">
+        <v>46283</v>
+      </c>
+      <c r="F4" s="92">
+        <v>262666</v>
+      </c>
+      <c r="G4" s="92">
+        <v>1749</v>
+      </c>
+      <c r="H4" s="92">
+        <v>500</v>
+      </c>
+      <c r="I4" s="92">
+        <v>1.444</v>
+      </c>
+      <c r="J4" s="92">
+        <v>2.383</v>
+      </c>
+      <c r="K4" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="92">
+        <v>1720.5260000000001</v>
+      </c>
+      <c r="M4" s="92">
+        <v>1191.5</v>
+      </c>
+      <c r="N4" s="92">
+        <v>0.33100000000000002</v>
+      </c>
+      <c r="O4" s="92">
+        <v>19.86</v>
+      </c>
+      <c r="P4" s="92">
+        <v>977.3</v>
+      </c>
+      <c r="Q4" s="92">
+        <v>1</v>
+      </c>
+      <c r="R4" s="92">
+        <v>1500</v>
+      </c>
+      <c r="S4" s="92">
+        <v>1.444</v>
+      </c>
+      <c r="T4" s="92">
+        <v>56</v>
+      </c>
+      <c r="U4" s="92">
+        <v>3.73E-2</v>
+      </c>
+      <c r="V4" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="W4" s="92" t="s">
+        <v>39</v>
+      </c>
+      <c r="X4" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y4" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z4" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA4" s="92">
+        <v>3</v>
+      </c>
+      <c r="AB4" s="92" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="92" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="92">
+        <v>3</v>
+      </c>
+      <c r="B5" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="92" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="93">
+        <v>46283</v>
+      </c>
+      <c r="F5" s="92">
+        <v>262667</v>
+      </c>
+      <c r="G5" s="92">
+        <v>1751</v>
+      </c>
+      <c r="H5" s="92">
+        <v>400</v>
+      </c>
+      <c r="I5" s="92">
+        <v>1.3879999999999999</v>
+      </c>
+      <c r="J5" s="92">
+        <v>1.5029999999999999</v>
+      </c>
+      <c r="K5" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L5" s="92">
+        <v>834.46600000000001</v>
+      </c>
+      <c r="M5" s="92">
+        <v>601.20000000000005</v>
+      </c>
+      <c r="N5" s="92">
+        <v>0.16700000000000001</v>
+      </c>
+      <c r="O5" s="92">
+        <v>10.02</v>
+      </c>
+      <c r="P5" s="92">
+        <v>474</v>
+      </c>
+      <c r="Q5" s="92">
+        <v>1</v>
+      </c>
+      <c r="R5" s="92">
+        <v>1450</v>
+      </c>
+      <c r="S5" s="92">
+        <v>1.3879999999999999</v>
+      </c>
+      <c r="T5" s="92">
+        <v>62</v>
+      </c>
+      <c r="U5" s="92">
+        <v>4.2799999999999998E-2</v>
+      </c>
+      <c r="V5" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="W5" s="92" t="s">
+        <v>39</v>
+      </c>
+      <c r="X5" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y5" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z5" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA5" s="92">
+        <v>3</v>
+      </c>
+      <c r="AB5" s="92" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="92">
+        <v>4</v>
+      </c>
+      <c r="B6" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E6" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="52">
+        <v>262639</v>
+      </c>
+      <c r="G6" s="52" t="s">
+        <v>227</v>
+      </c>
+      <c r="H6" s="52">
+        <v>300</v>
+      </c>
+      <c r="I6" s="54">
+        <v>0.67400000000000004</v>
+      </c>
+      <c r="J6" s="54">
+        <v>1.5229999999999999</v>
+      </c>
+      <c r="K6" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L6" s="54">
+        <v>307.95100000000002</v>
+      </c>
+      <c r="M6" s="55">
+        <v>228.4</v>
+      </c>
+      <c r="N6" s="56">
+        <v>3.1699999999999999E-2</v>
+      </c>
+      <c r="O6" s="57">
+        <v>1.9</v>
+      </c>
+      <c r="P6" s="52">
+        <v>174.9</v>
+      </c>
+      <c r="Q6" s="52">
+        <v>2</v>
+      </c>
+      <c r="R6" s="52">
+        <v>1400</v>
+      </c>
+      <c r="S6" s="54">
+        <v>1.3480000000000001</v>
+      </c>
+      <c r="T6" s="52">
+        <v>52</v>
+      </c>
+      <c r="U6" s="56">
+        <v>3.7100000000000001E-2</v>
+      </c>
+      <c r="V6" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="W6" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="X6" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y6" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z6" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA6" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB6" s="52" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="92">
+        <v>5</v>
+      </c>
+      <c r="B7" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E7" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="52">
+        <v>262637</v>
+      </c>
+      <c r="G7" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="H7" s="52">
+        <v>500</v>
+      </c>
+      <c r="I7" s="54">
+        <v>0.56599999999999995</v>
+      </c>
+      <c r="J7" s="54">
+        <v>1.4630000000000001</v>
+      </c>
+      <c r="K7" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L7" s="54">
+        <v>414.029</v>
+      </c>
+      <c r="M7" s="55">
+        <v>365.8</v>
+      </c>
+      <c r="N7" s="56">
+        <v>5.0799999999999998E-2</v>
+      </c>
+      <c r="O7" s="57">
+        <v>3.05</v>
+      </c>
+      <c r="P7" s="52">
+        <v>235.2</v>
+      </c>
+      <c r="Q7" s="52">
+        <v>2</v>
+      </c>
+      <c r="R7" s="52">
+        <v>1200</v>
+      </c>
+      <c r="S7" s="54">
+        <v>1.1319999999999999</v>
+      </c>
+      <c r="T7" s="52">
+        <v>68</v>
+      </c>
+      <c r="U7" s="56">
+        <v>5.67E-2</v>
+      </c>
+      <c r="V7" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="W7" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="X7" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y7" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z7" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA7" s="52" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB7" s="52" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="92">
+        <v>6</v>
+      </c>
+      <c r="B8" s="53" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="52">
+        <v>262635</v>
+      </c>
+      <c r="G8" s="52" t="s">
+        <v>223</v>
+      </c>
+      <c r="H8" s="52">
+        <v>5000</v>
+      </c>
+      <c r="I8" s="54">
+        <v>0.55900000000000005</v>
+      </c>
+      <c r="J8" s="54">
+        <v>1.389</v>
+      </c>
+      <c r="K8" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L8" s="54">
+        <v>3882.2550000000001</v>
+      </c>
+      <c r="M8" s="55">
+        <v>3472.5</v>
+      </c>
+      <c r="N8" s="56">
+        <v>0.48230000000000001</v>
+      </c>
+      <c r="O8" s="57">
+        <v>28.94</v>
+      </c>
+      <c r="P8" s="52">
+        <v>2205.1</v>
+      </c>
+      <c r="Q8" s="52">
+        <v>2</v>
+      </c>
+      <c r="R8" s="52">
+        <v>1150</v>
+      </c>
+      <c r="S8" s="54">
+        <v>1.1180000000000001</v>
+      </c>
+      <c r="T8" s="52">
+        <v>32</v>
+      </c>
+      <c r="U8" s="56">
+        <v>2.7799999999999998E-2</v>
+      </c>
+      <c r="V8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="W8" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="X8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z8" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA8" s="52" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB8" s="52" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="92">
+        <v>7</v>
+      </c>
+      <c r="B9" s="53" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="52">
+        <v>262636</v>
+      </c>
+      <c r="G9" s="52" t="s">
+        <v>223</v>
+      </c>
+      <c r="H9" s="52">
+        <v>5000</v>
+      </c>
+      <c r="I9" s="54">
+        <v>0.55900000000000005</v>
+      </c>
+      <c r="J9" s="54">
+        <v>1.389</v>
+      </c>
+      <c r="K9" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L9" s="54">
+        <v>3882.2550000000001</v>
+      </c>
+      <c r="M9" s="55">
+        <v>3472.5</v>
+      </c>
+      <c r="N9" s="56">
+        <v>0.48230000000000001</v>
+      </c>
+      <c r="O9" s="57">
+        <v>28.94</v>
+      </c>
+      <c r="P9" s="52">
+        <v>2205.1</v>
+      </c>
+      <c r="Q9" s="52">
+        <v>2</v>
+      </c>
+      <c r="R9" s="52">
+        <v>1150</v>
+      </c>
+      <c r="S9" s="54">
+        <v>1.1180000000000001</v>
+      </c>
+      <c r="T9" s="52">
+        <v>32</v>
+      </c>
+      <c r="U9" s="56">
+        <v>2.7799999999999998E-2</v>
+      </c>
+      <c r="V9" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="W9" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="X9" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y9" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z9" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA9" s="52" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB9" s="52" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="92">
+        <v>8</v>
+      </c>
+      <c r="B10" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E10" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="52">
+        <v>262638</v>
+      </c>
+      <c r="G10" s="52" t="s">
+        <v>221</v>
+      </c>
+      <c r="H10" s="52">
+        <v>200</v>
+      </c>
+      <c r="I10" s="54">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="J10" s="54">
+        <v>1.423</v>
+      </c>
+      <c r="K10" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L10" s="54">
+        <v>153.11500000000001</v>
+      </c>
+      <c r="M10" s="55">
+        <v>142.30000000000001</v>
+      </c>
+      <c r="N10" s="56">
+        <v>1.9800000000000002E-2</v>
+      </c>
+      <c r="O10" s="57">
+        <v>1.19</v>
+      </c>
+      <c r="P10" s="52">
+        <v>82.4</v>
+      </c>
+      <c r="Q10" s="52">
+        <v>2</v>
+      </c>
+      <c r="R10" s="52">
+        <v>1100</v>
+      </c>
+      <c r="S10" s="54">
+        <v>1.0760000000000001</v>
+      </c>
+      <c r="T10" s="52">
+        <v>24</v>
+      </c>
+      <c r="U10" s="56">
+        <v>2.18E-2</v>
+      </c>
+      <c r="V10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="X10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA10" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB10" s="52" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="92">
+        <v>9</v>
+      </c>
+      <c r="B11" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="68">
+        <v>46282</v>
+      </c>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52">
+        <v>262643</v>
+      </c>
+      <c r="G11" s="52">
+        <v>1748</v>
+      </c>
+      <c r="H11" s="52">
+        <v>600</v>
+      </c>
+      <c r="I11" s="54">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="J11" s="54">
+        <v>1.536</v>
+      </c>
+      <c r="K11" s="92" t="s">
+        <v>33</v>
+      </c>
+      <c r="L11" s="54">
+        <v>874.59799999999996</v>
+      </c>
+      <c r="M11" s="55">
+        <v>921.6</v>
+      </c>
+      <c r="N11" s="56">
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="O11" s="57">
+        <v>15.36</v>
+      </c>
+      <c r="P11" s="52">
+        <v>275.5</v>
+      </c>
+      <c r="Q11" s="52">
+        <v>1</v>
+      </c>
+      <c r="R11" s="52">
+        <v>1000</v>
+      </c>
+      <c r="S11" s="54">
+        <v>0.94899999999999995</v>
+      </c>
+      <c r="T11" s="52">
+        <v>51</v>
+      </c>
+      <c r="U11" s="56">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="V11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="52"/>
+      <c r="Z11" s="52"/>
+      <c r="AA11" s="52">
+        <v>2</v>
+      </c>
+      <c r="AB11" s="52" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="59">
+        <f>SUM(H3:H11)</f>
+        <v>13000</v>
+      </c>
+      <c r="I12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="59">
+        <f>SUM(P3:P11)</f>
+        <v>7717</v>
+      </c>
+      <c r="Q12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB12" s="59" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <phoneticPr fontId="19" type="noConversion"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A45B5AC-557E-4203-8DD1-DFBBC7E9A9E0}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -2801,7 +5352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E182FEA0-9E29-45AE-8927-1BAD28B275F4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3965,7 +6516,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5AF4CA-00D7-4A30-8F64-AC13CDBB2809}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4700,7 +7251,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15B73F0-D53E-458D-8A18-622E142F07EE}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -6469,7 +9020,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41716D2-EB8A-4484-83AF-D7868E55628C}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7904,7 +10455,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BFDD7F-F2DE-484D-858D-A0AEE46D68A8}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -8980,7 +11531,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC1CA626-F30A-4671-8B85-D3FC298D272A}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -10316,7 +12867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF67A62F-5FE1-4200-9945-6FEF51449597}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -10965,7 +13516,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F92D4A50-F39E-46BC-B44A-89840FB14E42}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -11614,6 +14165,394 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5961B2D-99FA-47E1-921A-0764410641DC}">
+  <dimension ref="A1:AB4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.77734375" style="34" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="34" customWidth="1"/>
+    <col min="3" max="3" width="5.77734375" style="34" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="9" style="34" customWidth="1"/>
+    <col min="6" max="6" width="6.77734375" style="34" customWidth="1"/>
+    <col min="7" max="7" width="4.5546875" style="34" customWidth="1"/>
+    <col min="8" max="8" width="5.109375" style="34" customWidth="1"/>
+    <col min="9" max="9" width="6.5546875" style="34" customWidth="1"/>
+    <col min="10" max="10" width="6.33203125" style="34" customWidth="1"/>
+    <col min="11" max="11" width="10.77734375" style="34" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" style="34" customWidth="1"/>
+    <col min="17" max="17" width="3.33203125" style="34" customWidth="1"/>
+    <col min="18" max="18" width="5.109375" style="34" customWidth="1"/>
+    <col min="19" max="19" width="5.88671875" style="34" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="34" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="6.44140625" style="34" customWidth="1"/>
+    <col min="23" max="23" width="8.21875" style="34" customWidth="1"/>
+    <col min="24" max="24" width="8.5546875" style="34" customWidth="1"/>
+    <col min="25" max="25" width="10.44140625" style="34" customWidth="1"/>
+    <col min="26" max="26" width="10.109375" style="34" customWidth="1"/>
+    <col min="27" max="27" width="4.5546875" style="34" customWidth="1"/>
+    <col min="28" max="28" width="11.109375" style="34" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="34"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="98" t="s">
+        <v>333</v>
+      </c>
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="45" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="45" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="45" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="45" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="45" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="45" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A3" s="42">
+        <v>1</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>331</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="42">
+        <v>262704</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>330</v>
+      </c>
+      <c r="H3" s="42">
+        <v>4000</v>
+      </c>
+      <c r="I3" s="43">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="J3" s="43">
+        <v>1.002</v>
+      </c>
+      <c r="K3" s="42" t="s">
+        <v>188</v>
+      </c>
+      <c r="L3" s="39">
+        <v>1118.232</v>
+      </c>
+      <c r="M3" s="41">
+        <v>1336</v>
+      </c>
+      <c r="N3" s="38">
+        <v>0.1237</v>
+      </c>
+      <c r="O3" s="40">
+        <v>7.42</v>
+      </c>
+      <c r="P3" s="37">
+        <v>352.2</v>
+      </c>
+      <c r="Q3" s="37">
+        <v>3</v>
+      </c>
+      <c r="R3" s="37">
+        <v>900</v>
+      </c>
+      <c r="S3" s="39">
+        <v>0.83699999999999997</v>
+      </c>
+      <c r="T3" s="37">
+        <v>63</v>
+      </c>
+      <c r="U3" s="38">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V3" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB3" s="37" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="36">
+        <v>4000</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" s="35">
+        <v>352.2</v>
+      </c>
+      <c r="Q4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="R4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="T4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="U4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="V4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="W4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB4" s="35" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CFEEFF-BB40-454C-844D-5753B7370662}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -13379,7 +16318,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B791AA56-47E9-44C0-8D6D-1F61C5308578}">
   <dimension ref="A1:AB11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14349,7 +17288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD2CB328-92D9-4132-AB19-3AEA902CFC6F}">
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14989,7 +17928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{108C031E-2A12-45DB-84D8-2B63EF3B2F74}">
   <dimension ref="A1:AB14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -16150,7 +19089,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EF77729-461D-4869-88D8-71569C5BCEE0}">
   <dimension ref="A1:AB5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -16623,7 +19562,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED6A221D-BD7D-4C5D-A432-527A12F5B88A}">
   <dimension ref="A1:AB9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -17354,7 +20293,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCDEA62-D4C1-4F97-B5A0-F9D378B5F3A6}">
   <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -18417,1071 +21356,4 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00EADB3A-C171-49AE-8471-729057A3A740}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="3.33203125" style="34" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" style="34" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" style="34" customWidth="1"/>
-    <col min="6" max="6" width="7.109375" style="34" customWidth="1"/>
-    <col min="7" max="7" width="5.77734375" style="34" customWidth="1"/>
-    <col min="8" max="8" width="6" style="34" customWidth="1"/>
-    <col min="9" max="9" width="7.21875" style="34" customWidth="1"/>
-    <col min="10" max="10" width="6.5546875" style="34" customWidth="1"/>
-    <col min="11" max="11" width="6" style="34" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="7.44140625" style="34" customWidth="1"/>
-    <col min="17" max="17" width="4.21875" style="34" customWidth="1"/>
-    <col min="18" max="18" width="6.44140625" style="34" customWidth="1"/>
-    <col min="19" max="19" width="5.77734375" style="34" customWidth="1"/>
-    <col min="20" max="20" width="11.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="34" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7.77734375" style="34" customWidth="1"/>
-    <col min="23" max="23" width="7.6640625" style="34" customWidth="1"/>
-    <col min="24" max="24" width="7.44140625" style="34" customWidth="1"/>
-    <col min="25" max="25" width="7.77734375" style="34" customWidth="1"/>
-    <col min="26" max="26" width="7.44140625" style="34" customWidth="1"/>
-    <col min="27" max="27" width="4.21875" style="34" customWidth="1"/>
-    <col min="28" max="28" width="11.33203125" style="34" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="34"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="97" t="s">
-        <v>228</v>
-      </c>
-      <c r="B1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="97" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="45" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="45" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="45" t="s">
-        <v>53</v>
-      </c>
-      <c r="G2" s="45" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="45" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="45" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="45" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="45" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" s="45" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="V2" s="45" t="s">
-        <v>19</v>
-      </c>
-      <c r="W2" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="X2" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y2" s="45" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z2" s="45" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA2" s="45" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="45" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" s="92" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="92">
-        <v>1</v>
-      </c>
-      <c r="B3" s="92" t="s">
-        <v>90</v>
-      </c>
-      <c r="C3" s="92" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="93">
-        <v>46283</v>
-      </c>
-      <c r="F3" s="92">
-        <v>262665</v>
-      </c>
-      <c r="G3" s="92">
-        <v>1749</v>
-      </c>
-      <c r="H3" s="92">
-        <v>500</v>
-      </c>
-      <c r="I3" s="92">
-        <v>1.494</v>
-      </c>
-      <c r="J3" s="92">
-        <v>2.5630000000000002</v>
-      </c>
-      <c r="K3" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" s="92">
-        <v>1914.5609999999999</v>
-      </c>
-      <c r="M3" s="92">
-        <v>1281.5</v>
-      </c>
-      <c r="N3" s="92">
-        <v>0.35599999999999998</v>
-      </c>
-      <c r="O3" s="92">
-        <v>21.36</v>
-      </c>
-      <c r="P3" s="92">
-        <v>1087.5</v>
-      </c>
-      <c r="Q3" s="92">
-        <v>1</v>
-      </c>
-      <c r="R3" s="92">
-        <v>1550</v>
-      </c>
-      <c r="S3" s="92">
-        <v>1.494</v>
-      </c>
-      <c r="T3" s="92">
-        <v>56</v>
-      </c>
-      <c r="U3" s="92">
-        <v>3.61E-2</v>
-      </c>
-      <c r="V3" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="W3" s="92" t="s">
-        <v>39</v>
-      </c>
-      <c r="X3" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y3" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z3" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA3" s="92">
-        <v>3</v>
-      </c>
-      <c r="AB3" s="92" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" s="92" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="92">
-        <v>2</v>
-      </c>
-      <c r="B4" s="92" t="s">
-        <v>90</v>
-      </c>
-      <c r="C4" s="92" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="93">
-        <v>46283</v>
-      </c>
-      <c r="F4" s="92">
-        <v>262666</v>
-      </c>
-      <c r="G4" s="92">
-        <v>1749</v>
-      </c>
-      <c r="H4" s="92">
-        <v>500</v>
-      </c>
-      <c r="I4" s="92">
-        <v>1.444</v>
-      </c>
-      <c r="J4" s="92">
-        <v>2.383</v>
-      </c>
-      <c r="K4" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L4" s="92">
-        <v>1720.5260000000001</v>
-      </c>
-      <c r="M4" s="92">
-        <v>1191.5</v>
-      </c>
-      <c r="N4" s="92">
-        <v>0.33100000000000002</v>
-      </c>
-      <c r="O4" s="92">
-        <v>19.86</v>
-      </c>
-      <c r="P4" s="92">
-        <v>977.3</v>
-      </c>
-      <c r="Q4" s="92">
-        <v>1</v>
-      </c>
-      <c r="R4" s="92">
-        <v>1500</v>
-      </c>
-      <c r="S4" s="92">
-        <v>1.444</v>
-      </c>
-      <c r="T4" s="92">
-        <v>56</v>
-      </c>
-      <c r="U4" s="92">
-        <v>3.73E-2</v>
-      </c>
-      <c r="V4" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="W4" s="92" t="s">
-        <v>39</v>
-      </c>
-      <c r="X4" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y4" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z4" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA4" s="92">
-        <v>3</v>
-      </c>
-      <c r="AB4" s="92" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" s="92" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="92">
-        <v>3</v>
-      </c>
-      <c r="B5" s="92" t="s">
-        <v>90</v>
-      </c>
-      <c r="C5" s="92" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="93">
-        <v>46283</v>
-      </c>
-      <c r="F5" s="92">
-        <v>262667</v>
-      </c>
-      <c r="G5" s="92">
-        <v>1751</v>
-      </c>
-      <c r="H5" s="92">
-        <v>400</v>
-      </c>
-      <c r="I5" s="92">
-        <v>1.3879999999999999</v>
-      </c>
-      <c r="J5" s="92">
-        <v>1.5029999999999999</v>
-      </c>
-      <c r="K5" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L5" s="92">
-        <v>834.46600000000001</v>
-      </c>
-      <c r="M5" s="92">
-        <v>601.20000000000005</v>
-      </c>
-      <c r="N5" s="92">
-        <v>0.16700000000000001</v>
-      </c>
-      <c r="O5" s="92">
-        <v>10.02</v>
-      </c>
-      <c r="P5" s="92">
-        <v>474</v>
-      </c>
-      <c r="Q5" s="92">
-        <v>1</v>
-      </c>
-      <c r="R5" s="92">
-        <v>1450</v>
-      </c>
-      <c r="S5" s="92">
-        <v>1.3879999999999999</v>
-      </c>
-      <c r="T5" s="92">
-        <v>62</v>
-      </c>
-      <c r="U5" s="92">
-        <v>4.2799999999999998E-2</v>
-      </c>
-      <c r="V5" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="W5" s="92" t="s">
-        <v>39</v>
-      </c>
-      <c r="X5" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y5" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z5" s="92" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA5" s="92">
-        <v>3</v>
-      </c>
-      <c r="AB5" s="92" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="92">
-        <v>4</v>
-      </c>
-      <c r="B6" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="C6" s="52" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="52">
-        <v>262639</v>
-      </c>
-      <c r="G6" s="52" t="s">
-        <v>227</v>
-      </c>
-      <c r="H6" s="52">
-        <v>300</v>
-      </c>
-      <c r="I6" s="54">
-        <v>0.67400000000000004</v>
-      </c>
-      <c r="J6" s="54">
-        <v>1.5229999999999999</v>
-      </c>
-      <c r="K6" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L6" s="54">
-        <v>307.95100000000002</v>
-      </c>
-      <c r="M6" s="55">
-        <v>228.4</v>
-      </c>
-      <c r="N6" s="56">
-        <v>3.1699999999999999E-2</v>
-      </c>
-      <c r="O6" s="57">
-        <v>1.9</v>
-      </c>
-      <c r="P6" s="52">
-        <v>174.9</v>
-      </c>
-      <c r="Q6" s="52">
-        <v>2</v>
-      </c>
-      <c r="R6" s="52">
-        <v>1400</v>
-      </c>
-      <c r="S6" s="54">
-        <v>1.3480000000000001</v>
-      </c>
-      <c r="T6" s="52">
-        <v>52</v>
-      </c>
-      <c r="U6" s="56">
-        <v>3.7100000000000001E-2</v>
-      </c>
-      <c r="V6" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="W6" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="X6" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y6" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z6" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA6" s="52" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB6" s="52" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="92">
-        <v>5</v>
-      </c>
-      <c r="B7" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="52" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="52">
-        <v>262637</v>
-      </c>
-      <c r="G7" s="52" t="s">
-        <v>225</v>
-      </c>
-      <c r="H7" s="52">
-        <v>500</v>
-      </c>
-      <c r="I7" s="54">
-        <v>0.56599999999999995</v>
-      </c>
-      <c r="J7" s="54">
-        <v>1.4630000000000001</v>
-      </c>
-      <c r="K7" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L7" s="54">
-        <v>414.029</v>
-      </c>
-      <c r="M7" s="55">
-        <v>365.8</v>
-      </c>
-      <c r="N7" s="56">
-        <v>5.0799999999999998E-2</v>
-      </c>
-      <c r="O7" s="57">
-        <v>3.05</v>
-      </c>
-      <c r="P7" s="52">
-        <v>235.2</v>
-      </c>
-      <c r="Q7" s="52">
-        <v>2</v>
-      </c>
-      <c r="R7" s="52">
-        <v>1200</v>
-      </c>
-      <c r="S7" s="54">
-        <v>1.1319999999999999</v>
-      </c>
-      <c r="T7" s="52">
-        <v>68</v>
-      </c>
-      <c r="U7" s="56">
-        <v>5.67E-2</v>
-      </c>
-      <c r="V7" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="W7" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="X7" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y7" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z7" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA7" s="52" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB7" s="52" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="92">
-        <v>6</v>
-      </c>
-      <c r="B8" s="53" t="s">
-        <v>92</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="52">
-        <v>262635</v>
-      </c>
-      <c r="G8" s="52" t="s">
-        <v>223</v>
-      </c>
-      <c r="H8" s="52">
-        <v>5000</v>
-      </c>
-      <c r="I8" s="54">
-        <v>0.55900000000000005</v>
-      </c>
-      <c r="J8" s="54">
-        <v>1.389</v>
-      </c>
-      <c r="K8" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L8" s="54">
-        <v>3882.2550000000001</v>
-      </c>
-      <c r="M8" s="55">
-        <v>3472.5</v>
-      </c>
-      <c r="N8" s="56">
-        <v>0.48230000000000001</v>
-      </c>
-      <c r="O8" s="57">
-        <v>28.94</v>
-      </c>
-      <c r="P8" s="52">
-        <v>2205.1</v>
-      </c>
-      <c r="Q8" s="52">
-        <v>2</v>
-      </c>
-      <c r="R8" s="52">
-        <v>1150</v>
-      </c>
-      <c r="S8" s="54">
-        <v>1.1180000000000001</v>
-      </c>
-      <c r="T8" s="52">
-        <v>32</v>
-      </c>
-      <c r="U8" s="56">
-        <v>2.7799999999999998E-2</v>
-      </c>
-      <c r="V8" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="W8" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="X8" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y8" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z8" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA8" s="52" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB8" s="52" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="92">
-        <v>7</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>92</v>
-      </c>
-      <c r="C9" s="52" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E9" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="52">
-        <v>262636</v>
-      </c>
-      <c r="G9" s="52" t="s">
-        <v>223</v>
-      </c>
-      <c r="H9" s="52">
-        <v>5000</v>
-      </c>
-      <c r="I9" s="54">
-        <v>0.55900000000000005</v>
-      </c>
-      <c r="J9" s="54">
-        <v>1.389</v>
-      </c>
-      <c r="K9" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L9" s="54">
-        <v>3882.2550000000001</v>
-      </c>
-      <c r="M9" s="55">
-        <v>3472.5</v>
-      </c>
-      <c r="N9" s="56">
-        <v>0.48230000000000001</v>
-      </c>
-      <c r="O9" s="57">
-        <v>28.94</v>
-      </c>
-      <c r="P9" s="52">
-        <v>2205.1</v>
-      </c>
-      <c r="Q9" s="52">
-        <v>2</v>
-      </c>
-      <c r="R9" s="52">
-        <v>1150</v>
-      </c>
-      <c r="S9" s="54">
-        <v>1.1180000000000001</v>
-      </c>
-      <c r="T9" s="52">
-        <v>32</v>
-      </c>
-      <c r="U9" s="56">
-        <v>2.7799999999999998E-2</v>
-      </c>
-      <c r="V9" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="W9" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="X9" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y9" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z9" s="52" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA9" s="52" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB9" s="52" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="92">
-        <v>8</v>
-      </c>
-      <c r="B10" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" s="52" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E10" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="52">
-        <v>262638</v>
-      </c>
-      <c r="G10" s="52" t="s">
-        <v>221</v>
-      </c>
-      <c r="H10" s="52">
-        <v>200</v>
-      </c>
-      <c r="I10" s="54">
-        <v>0.53800000000000003</v>
-      </c>
-      <c r="J10" s="54">
-        <v>1.423</v>
-      </c>
-      <c r="K10" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L10" s="54">
-        <v>153.11500000000001</v>
-      </c>
-      <c r="M10" s="55">
-        <v>142.30000000000001</v>
-      </c>
-      <c r="N10" s="56">
-        <v>1.9800000000000002E-2</v>
-      </c>
-      <c r="O10" s="57">
-        <v>1.19</v>
-      </c>
-      <c r="P10" s="52">
-        <v>82.4</v>
-      </c>
-      <c r="Q10" s="52">
-        <v>2</v>
-      </c>
-      <c r="R10" s="52">
-        <v>1100</v>
-      </c>
-      <c r="S10" s="54">
-        <v>1.0760000000000001</v>
-      </c>
-      <c r="T10" s="52">
-        <v>24</v>
-      </c>
-      <c r="U10" s="56">
-        <v>2.18E-2</v>
-      </c>
-      <c r="V10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="52" t="s">
-        <v>29</v>
-      </c>
-      <c r="X10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA10" s="52" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB10" s="52" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="92">
-        <v>9</v>
-      </c>
-      <c r="B11" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" s="52" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="68">
-        <v>46282</v>
-      </c>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52">
-        <v>262643</v>
-      </c>
-      <c r="G11" s="52">
-        <v>1748</v>
-      </c>
-      <c r="H11" s="52">
-        <v>600</v>
-      </c>
-      <c r="I11" s="54">
-        <v>0.94899999999999995</v>
-      </c>
-      <c r="J11" s="54">
-        <v>1.536</v>
-      </c>
-      <c r="K11" s="92" t="s">
-        <v>33</v>
-      </c>
-      <c r="L11" s="54">
-        <v>874.59799999999996</v>
-      </c>
-      <c r="M11" s="55">
-        <v>921.6</v>
-      </c>
-      <c r="N11" s="56">
-        <v>0.25600000000000001</v>
-      </c>
-      <c r="O11" s="57">
-        <v>15.36</v>
-      </c>
-      <c r="P11" s="52">
-        <v>275.5</v>
-      </c>
-      <c r="Q11" s="52">
-        <v>1</v>
-      </c>
-      <c r="R11" s="52">
-        <v>1000</v>
-      </c>
-      <c r="S11" s="54">
-        <v>0.94899999999999995</v>
-      </c>
-      <c r="T11" s="52">
-        <v>51</v>
-      </c>
-      <c r="U11" s="56">
-        <v>5.0999999999999997E-2</v>
-      </c>
-      <c r="V11" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="52"/>
-      <c r="Z11" s="52"/>
-      <c r="AA11" s="52">
-        <v>2</v>
-      </c>
-      <c r="AB11" s="52" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="59">
-        <f>SUM(H3:H11)</f>
-        <v>13000</v>
-      </c>
-      <c r="I12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="59">
-        <f>SUM(P3:P11)</f>
-        <v>7717</v>
-      </c>
-      <c r="Q12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="59" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AB1"/>
-  </mergeCells>
-  <phoneticPr fontId="19" type="noConversion"/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (28/09/2026 09:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F37965F-0ABA-4CE7-A989-93EE2C7A8F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43464021-31F0-4194-800C-21AF3318E528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX EMBALAGENS LTDA 1233" sheetId="170" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3884" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3923" uniqueCount="407">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1260,6 +1260,21 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - PCBOX EMBALAGENS LTDA  —  OF: 001233</t>
+  </si>
+  <si>
+    <t>176x355x176</t>
+  </si>
+  <si>
+    <t>8275</t>
+  </si>
+  <si>
+    <t>733x2119</t>
+  </si>
+  <si>
+    <t>184x345x184</t>
+  </si>
+  <si>
+    <t>982x2138</t>
   </si>
 </sst>
 </file>
@@ -3781,7 +3796,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BCDEA62-D4C1-4F97-B5A0-F9D378B5F3A6}">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5546875" style="34" customWidth="1"/>
@@ -3997,58 +4012,58 @@
         <v>26</v>
       </c>
       <c r="D3" s="46" t="s">
-        <v>253</v>
+        <v>385</v>
       </c>
       <c r="E3" s="46" t="s">
         <v>27</v>
       </c>
       <c r="F3" s="46">
-        <v>262674</v>
+        <v>262740</v>
       </c>
       <c r="G3" s="46" t="s">
-        <v>282</v>
+        <v>403</v>
       </c>
       <c r="H3" s="46">
-        <v>400</v>
+        <v>550</v>
       </c>
       <c r="I3" s="48">
-        <v>1.3720000000000001</v>
+        <v>0.70699999999999996</v>
       </c>
       <c r="J3" s="48">
-        <v>2.38</v>
+        <v>1.4990000000000001</v>
       </c>
       <c r="K3" s="46" t="s">
-        <v>286</v>
+        <v>402</v>
       </c>
       <c r="L3" s="48">
-        <v>1306.144</v>
+        <v>582.88599999999997</v>
       </c>
       <c r="M3" s="49">
-        <v>952</v>
+        <v>412.2</v>
       </c>
       <c r="N3" s="50">
-        <v>0.26440000000000002</v>
+        <v>5.7299999999999997E-2</v>
       </c>
       <c r="O3" s="51">
-        <v>15.87</v>
+        <v>3.44</v>
       </c>
       <c r="P3" s="46">
-        <v>702.7</v>
+        <v>313.60000000000002</v>
       </c>
       <c r="Q3" s="46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R3" s="46">
-        <v>1400</v>
+        <v>1450</v>
       </c>
       <c r="S3" s="48">
-        <v>1.3720000000000001</v>
+        <v>1.4139999999999999</v>
       </c>
       <c r="T3" s="46">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="U3" s="50">
-        <v>0.02</v>
+        <v>2.4799999999999999E-2</v>
       </c>
       <c r="V3" s="46" t="s">
         <v>28</v>
@@ -4066,10 +4081,10 @@
         <v>28</v>
       </c>
       <c r="AA3" s="46" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="AB3" s="46" t="s">
-        <v>285</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4083,58 +4098,58 @@
         <v>26</v>
       </c>
       <c r="D4" s="46" t="s">
-        <v>253</v>
+        <v>385</v>
       </c>
       <c r="E4" s="46" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="46">
-        <v>262672</v>
+        <v>262741</v>
       </c>
       <c r="G4" s="46" t="s">
-        <v>282</v>
+        <v>403</v>
       </c>
       <c r="H4" s="46">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="I4" s="48">
-        <v>1.1519999999999999</v>
+        <v>0.71299999999999997</v>
       </c>
       <c r="J4" s="48">
-        <v>2.34</v>
+        <v>2.0990000000000002</v>
       </c>
       <c r="K4" s="46" t="s">
-        <v>284</v>
+        <v>405</v>
       </c>
       <c r="L4" s="48">
-        <v>1078.2719999999999</v>
+        <v>576.18600000000004</v>
       </c>
       <c r="M4" s="49">
-        <v>936</v>
+        <v>404.1</v>
       </c>
       <c r="N4" s="50">
-        <v>0.26</v>
+        <v>5.6099999999999997E-2</v>
       </c>
       <c r="O4" s="51">
-        <v>15.6</v>
+        <v>3.37</v>
       </c>
       <c r="P4" s="46">
-        <v>580.1</v>
+        <v>310</v>
       </c>
       <c r="Q4" s="46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R4" s="46">
-        <v>1200</v>
+        <v>1450</v>
       </c>
       <c r="S4" s="48">
-        <v>1.1519999999999999</v>
+        <v>1.4259999999999999</v>
       </c>
       <c r="T4" s="46">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="U4" s="50">
-        <v>0.04</v>
+        <v>1.66E-2</v>
       </c>
       <c r="V4" s="46" t="s">
         <v>28</v>
@@ -4152,15 +4167,15 @@
         <v>28</v>
       </c>
       <c r="AA4" s="46" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AB4" s="46" t="s">
-        <v>283</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="46">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" s="47" t="s">
         <v>58</v>
@@ -4175,7 +4190,7 @@
         <v>27</v>
       </c>
       <c r="F5" s="46">
-        <v>262671</v>
+        <v>262674</v>
       </c>
       <c r="G5" s="46" t="s">
         <v>282</v>
@@ -4184,43 +4199,43 @@
         <v>400</v>
       </c>
       <c r="I5" s="48">
-        <v>1.3520000000000001</v>
+        <v>1.3720000000000001</v>
       </c>
       <c r="J5" s="48">
-        <v>2.339</v>
+        <v>2.38</v>
       </c>
       <c r="K5" s="46" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="L5" s="48">
-        <v>1264.931</v>
+        <v>1306.144</v>
       </c>
       <c r="M5" s="49">
-        <v>467.8</v>
+        <v>952</v>
       </c>
       <c r="N5" s="50">
-        <v>6.5000000000000002E-2</v>
+        <v>0.26440000000000002</v>
       </c>
       <c r="O5" s="51">
-        <v>3.9</v>
+        <v>15.87</v>
       </c>
       <c r="P5" s="46">
-        <v>680.5</v>
+        <v>702.7</v>
       </c>
       <c r="Q5" s="46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R5" s="46">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="S5" s="48">
-        <v>2.7040000000000002</v>
+        <v>1.3720000000000001</v>
       </c>
       <c r="T5" s="46">
-        <v>-1504</v>
+        <v>28</v>
       </c>
       <c r="U5" s="50">
-        <v>-1.2533000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="V5" s="46" t="s">
         <v>28</v>
@@ -4241,318 +4256,328 @@
         <v>30</v>
       </c>
       <c r="AB5" s="46" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="46">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" s="47" t="s">
         <v>58</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" s="96">
-        <v>46287</v>
-      </c>
-      <c r="E6" s="46"/>
+        <v>26</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>253</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>27</v>
+      </c>
       <c r="F6" s="46">
-        <v>262701</v>
-      </c>
-      <c r="G6" s="46">
-        <v>8263</v>
+        <v>262672</v>
+      </c>
+      <c r="G6" s="46" t="s">
+        <v>282</v>
       </c>
       <c r="H6" s="46">
-        <v>930</v>
+        <v>400</v>
       </c>
       <c r="I6" s="48">
-        <v>0.59199999999999997</v>
+        <v>1.1519999999999999</v>
       </c>
       <c r="J6" s="48">
-        <v>1.62</v>
+        <v>2.34</v>
       </c>
       <c r="K6" s="46" t="s">
-        <v>326</v>
+        <v>284</v>
       </c>
       <c r="L6" s="48">
-        <v>891.90700000000004</v>
+        <v>1078.2719999999999</v>
       </c>
       <c r="M6" s="49">
-        <v>753.3</v>
+        <v>936</v>
       </c>
       <c r="N6" s="50">
-        <v>0.1046</v>
+        <v>0.26</v>
       </c>
       <c r="O6" s="51">
-        <v>6.28</v>
+        <v>15.6</v>
       </c>
       <c r="P6" s="46">
-        <v>289</v>
+        <v>580.1</v>
       </c>
       <c r="Q6" s="46">
+        <v>1</v>
+      </c>
+      <c r="R6" s="46">
+        <v>1200</v>
+      </c>
+      <c r="S6" s="48">
+        <v>1.1519999999999999</v>
+      </c>
+      <c r="T6" s="46">
+        <v>48</v>
+      </c>
+      <c r="U6" s="50">
+        <v>0.04</v>
+      </c>
+      <c r="V6" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB6" s="46" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="46">
+        <v>3</v>
+      </c>
+      <c r="B7" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>253</v>
+      </c>
+      <c r="E7" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="46">
+        <v>262671</v>
+      </c>
+      <c r="G7" s="46" t="s">
+        <v>282</v>
+      </c>
+      <c r="H7" s="46">
+        <v>400</v>
+      </c>
+      <c r="I7" s="48">
+        <v>1.3520000000000001</v>
+      </c>
+      <c r="J7" s="48">
+        <v>2.339</v>
+      </c>
+      <c r="K7" s="46" t="s">
+        <v>281</v>
+      </c>
+      <c r="L7" s="48">
+        <v>1264.931</v>
+      </c>
+      <c r="M7" s="49">
+        <v>467.8</v>
+      </c>
+      <c r="N7" s="50">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="O7" s="51">
+        <v>3.9</v>
+      </c>
+      <c r="P7" s="46">
+        <v>680.5</v>
+      </c>
+      <c r="Q7" s="46">
         <v>2</v>
       </c>
-      <c r="R6" s="46">
-        <v>1250</v>
-      </c>
-      <c r="S6" s="48">
-        <v>1.1839999999999999</v>
-      </c>
-      <c r="T6" s="46">
-        <v>66</v>
-      </c>
-      <c r="U6" s="50">
-        <v>5.28E-2</v>
-      </c>
-      <c r="V6" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="46"/>
-      <c r="Z6" s="46"/>
-      <c r="AA6" s="46">
+      <c r="R7" s="46">
+        <v>1200</v>
+      </c>
+      <c r="S7" s="48">
+        <v>2.7040000000000002</v>
+      </c>
+      <c r="T7" s="46">
+        <v>-1504</v>
+      </c>
+      <c r="U7" s="50">
+        <v>-1.2533000000000001</v>
+      </c>
+      <c r="V7" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB7" s="46" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="46">
         <v>3</v>
       </c>
-      <c r="AB6" s="46" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="46">
-        <v>6</v>
-      </c>
-      <c r="B7" s="53" t="s">
+      <c r="B8" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="52" t="s">
-        <v>59</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="52">
-        <v>262641</v>
-      </c>
-      <c r="G7" s="52" t="s">
-        <v>231</v>
-      </c>
-      <c r="H7" s="52">
-        <v>1150</v>
-      </c>
-      <c r="I7" s="54">
-        <v>0.54700000000000004</v>
-      </c>
-      <c r="J7" s="54">
-        <v>1.44</v>
-      </c>
-      <c r="K7" s="52" t="s">
-        <v>233</v>
-      </c>
-      <c r="L7" s="54">
-        <v>905.83199999999999</v>
-      </c>
-      <c r="M7" s="55">
-        <v>828</v>
-      </c>
-      <c r="N7" s="56">
-        <v>0.115</v>
-      </c>
-      <c r="O7" s="57">
-        <v>6.9</v>
-      </c>
-      <c r="P7" s="52">
-        <v>293.5</v>
-      </c>
-      <c r="Q7" s="52">
-        <v>2</v>
-      </c>
-      <c r="R7" s="52">
-        <v>1150</v>
-      </c>
-      <c r="S7" s="54">
-        <v>1.0940000000000001</v>
-      </c>
-      <c r="T7" s="52">
-        <v>56</v>
-      </c>
-      <c r="U7" s="56">
-        <v>4.87E-2</v>
-      </c>
-      <c r="V7" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="52" t="s">
+      <c r="C8" s="46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>385</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="46">
+        <v>262742</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>403</v>
+      </c>
+      <c r="H8" s="46">
+        <v>285</v>
+      </c>
+      <c r="I8" s="48">
+        <v>0.96199999999999997</v>
+      </c>
+      <c r="J8" s="48">
+        <v>2.1179999999999999</v>
+      </c>
+      <c r="K8" s="46" t="s">
+        <v>70</v>
+      </c>
+      <c r="L8" s="48">
+        <v>580.69200000000001</v>
+      </c>
+      <c r="M8" s="49">
+        <v>603.6</v>
+      </c>
+      <c r="N8" s="50">
+        <v>0.16769999999999999</v>
+      </c>
+      <c r="O8" s="51">
+        <v>10.06</v>
+      </c>
+      <c r="P8" s="46">
+        <v>312.39999999999998</v>
+      </c>
+      <c r="Q8" s="46">
+        <v>1</v>
+      </c>
+      <c r="R8" s="46">
+        <v>1000</v>
+      </c>
+      <c r="S8" s="48">
+        <v>0.96199999999999997</v>
+      </c>
+      <c r="T8" s="46">
+        <v>38</v>
+      </c>
+      <c r="U8" s="50">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="V8" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="X8" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="52" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="46">
-        <v>7</v>
-      </c>
-      <c r="B8" s="53" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="68">
-        <v>46287</v>
-      </c>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52">
-        <v>262700</v>
-      </c>
-      <c r="G8" s="52">
-        <v>8263</v>
-      </c>
-      <c r="H8" s="52">
-        <v>9500</v>
-      </c>
-      <c r="I8" s="54">
-        <v>0.32200000000000001</v>
-      </c>
-      <c r="J8" s="54">
-        <v>0.94</v>
-      </c>
-      <c r="K8" s="52" t="s">
-        <v>324</v>
-      </c>
-      <c r="L8" s="54">
-        <v>2875.46</v>
-      </c>
-      <c r="M8" s="55">
-        <v>4465</v>
-      </c>
-      <c r="N8" s="56">
-        <v>0.62009999999999998</v>
-      </c>
-      <c r="O8" s="57">
-        <v>37.21</v>
-      </c>
-      <c r="P8" s="52">
-        <v>931.6</v>
-      </c>
-      <c r="Q8" s="52">
-        <v>2</v>
-      </c>
-      <c r="R8" s="52">
-        <v>700</v>
-      </c>
-      <c r="S8" s="54">
-        <v>0.64400000000000002</v>
-      </c>
-      <c r="T8" s="52">
-        <v>56</v>
-      </c>
-      <c r="U8" s="56">
-        <v>0.08</v>
-      </c>
-      <c r="V8" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="52"/>
-      <c r="Z8" s="52"/>
-      <c r="AA8" s="52">
-        <v>5</v>
-      </c>
-      <c r="AB8" s="52" t="s">
-        <v>325</v>
+      <c r="AB8" s="46" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="46">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B9" s="47" t="s">
         <v>58</v>
       </c>
       <c r="C9" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="46" t="s">
-        <v>253</v>
-      </c>
-      <c r="E9" s="46" t="s">
-        <v>27</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="D9" s="96">
+        <v>46287</v>
+      </c>
+      <c r="E9" s="46"/>
       <c r="F9" s="46">
-        <v>262673</v>
-      </c>
-      <c r="G9" s="46" t="s">
-        <v>282</v>
+        <v>262701</v>
+      </c>
+      <c r="G9" s="46">
+        <v>8263</v>
       </c>
       <c r="H9" s="46">
-        <v>1000</v>
+        <v>930</v>
       </c>
       <c r="I9" s="48">
-        <v>0.76</v>
+        <v>0.59199999999999997</v>
       </c>
       <c r="J9" s="48">
-        <v>1.0900000000000001</v>
+        <v>1.62</v>
       </c>
       <c r="K9" s="46" t="s">
-        <v>33</v>
+        <v>326</v>
       </c>
       <c r="L9" s="48">
-        <v>828.4</v>
+        <v>891.90700000000004</v>
       </c>
       <c r="M9" s="49">
-        <v>545</v>
+        <v>753.3</v>
       </c>
       <c r="N9" s="50">
-        <v>7.5700000000000003E-2</v>
+        <v>0.1046</v>
       </c>
       <c r="O9" s="51">
-        <v>4.54</v>
+        <v>6.28</v>
       </c>
       <c r="P9" s="46">
-        <v>260.89999999999998</v>
+        <v>289</v>
       </c>
       <c r="Q9" s="46">
         <v>2</v>
       </c>
       <c r="R9" s="46">
-        <v>1550</v>
+        <v>1250</v>
       </c>
       <c r="S9" s="48">
-        <v>1.52</v>
+        <v>1.1839999999999999</v>
       </c>
       <c r="T9" s="46">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="U9" s="50">
-        <v>1.9400000000000001E-2</v>
+        <v>5.28E-2</v>
       </c>
       <c r="V9" s="46" t="s">
         <v>28</v>
@@ -4563,279 +4588,528 @@
       <c r="X9" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="Y9" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="46" t="s">
+      <c r="Y9" s="46"/>
+      <c r="Z9" s="46"/>
+      <c r="AA9" s="46">
+        <v>3</v>
+      </c>
+      <c r="AB9" s="46" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="46">
+        <v>6</v>
+      </c>
+      <c r="B10" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E10" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="52">
+        <v>262641</v>
+      </c>
+      <c r="G10" s="52" t="s">
+        <v>231</v>
+      </c>
+      <c r="H10" s="52">
+        <v>1150</v>
+      </c>
+      <c r="I10" s="54">
+        <v>0.54700000000000004</v>
+      </c>
+      <c r="J10" s="54">
+        <v>1.44</v>
+      </c>
+      <c r="K10" s="52" t="s">
+        <v>233</v>
+      </c>
+      <c r="L10" s="54">
+        <v>905.83199999999999</v>
+      </c>
+      <c r="M10" s="55">
+        <v>828</v>
+      </c>
+      <c r="N10" s="56">
+        <v>0.115</v>
+      </c>
+      <c r="O10" s="57">
+        <v>6.9</v>
+      </c>
+      <c r="P10" s="52">
+        <v>293.5</v>
+      </c>
+      <c r="Q10" s="52">
+        <v>2</v>
+      </c>
+      <c r="R10" s="52">
+        <v>1150</v>
+      </c>
+      <c r="S10" s="54">
+        <v>1.0940000000000001</v>
+      </c>
+      <c r="T10" s="52">
+        <v>56</v>
+      </c>
+      <c r="U10" s="56">
+        <v>4.87E-2</v>
+      </c>
+      <c r="V10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB9" s="46" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="46">
-        <v>9</v>
-      </c>
-      <c r="B10" s="47" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="46" t="s">
-        <v>274</v>
-      </c>
-      <c r="E10" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="46">
-        <v>262675</v>
-      </c>
-      <c r="G10" s="46" t="s">
-        <v>288</v>
-      </c>
-      <c r="H10" s="46">
-        <v>1350</v>
-      </c>
-      <c r="I10" s="48">
-        <v>0.59199999999999997</v>
-      </c>
-      <c r="J10" s="48">
-        <v>1.619</v>
-      </c>
-      <c r="K10" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="L10" s="48">
-        <v>1293.905</v>
-      </c>
-      <c r="M10" s="49">
-        <v>1092.8</v>
-      </c>
-      <c r="N10" s="50">
-        <v>0.15179999999999999</v>
-      </c>
-      <c r="O10" s="51">
-        <v>9.11</v>
-      </c>
-      <c r="P10" s="46">
-        <v>407.6</v>
-      </c>
-      <c r="Q10" s="46">
-        <v>2</v>
-      </c>
-      <c r="R10" s="46">
-        <v>1250</v>
-      </c>
-      <c r="S10" s="48">
-        <v>1.1839999999999999</v>
-      </c>
-      <c r="T10" s="46">
-        <v>66</v>
-      </c>
-      <c r="U10" s="50">
-        <v>5.28E-2</v>
-      </c>
-      <c r="V10" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="46" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB10" s="46" t="s">
-        <v>290</v>
+      <c r="AB10" s="52" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="46">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B11" s="53" t="s">
         <v>58</v>
       </c>
       <c r="C11" s="52" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="52" t="s">
-        <v>222</v>
-      </c>
-      <c r="E11" s="52" t="s">
-        <v>27</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="D11" s="68">
+        <v>46287</v>
+      </c>
+      <c r="E11" s="52"/>
       <c r="F11" s="52">
-        <v>262642</v>
-      </c>
-      <c r="G11" s="52" t="s">
-        <v>231</v>
+        <v>262700</v>
+      </c>
+      <c r="G11" s="52">
+        <v>8263</v>
       </c>
       <c r="H11" s="52">
-        <v>1000</v>
+        <v>9500</v>
       </c>
       <c r="I11" s="54">
-        <v>0.58099999999999996</v>
+        <v>0.32200000000000001</v>
       </c>
       <c r="J11" s="54">
-        <v>1.58</v>
+        <v>0.94</v>
       </c>
       <c r="K11" s="52" t="s">
-        <v>230</v>
+        <v>324</v>
       </c>
       <c r="L11" s="54">
-        <v>917.98</v>
+        <v>2875.46</v>
       </c>
       <c r="M11" s="55">
-        <v>790</v>
+        <v>4465</v>
       </c>
       <c r="N11" s="56">
-        <v>0.10970000000000001</v>
+        <v>0.62009999999999998</v>
       </c>
       <c r="O11" s="57">
-        <v>6.58</v>
+        <v>37.21</v>
       </c>
       <c r="P11" s="52">
-        <v>289.2</v>
+        <v>931.6</v>
       </c>
       <c r="Q11" s="52">
         <v>2</v>
       </c>
       <c r="R11" s="52">
+        <v>700</v>
+      </c>
+      <c r="S11" s="54">
+        <v>0.64400000000000002</v>
+      </c>
+      <c r="T11" s="52">
+        <v>56</v>
+      </c>
+      <c r="U11" s="56">
+        <v>0.08</v>
+      </c>
+      <c r="V11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="52"/>
+      <c r="Z11" s="52"/>
+      <c r="AA11" s="52">
+        <v>5</v>
+      </c>
+      <c r="AB11" s="52" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="46">
+        <v>8</v>
+      </c>
+      <c r="B12" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>253</v>
+      </c>
+      <c r="E12" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="46">
+        <v>262673</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>282</v>
+      </c>
+      <c r="H12" s="46">
+        <v>1000</v>
+      </c>
+      <c r="I12" s="48">
+        <v>0.76</v>
+      </c>
+      <c r="J12" s="48">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="K12" s="46" t="s">
+        <v>33</v>
+      </c>
+      <c r="L12" s="48">
+        <v>828.4</v>
+      </c>
+      <c r="M12" s="49">
+        <v>545</v>
+      </c>
+      <c r="N12" s="50">
+        <v>7.5700000000000003E-2</v>
+      </c>
+      <c r="O12" s="51">
+        <v>4.54</v>
+      </c>
+      <c r="P12" s="46">
+        <v>260.89999999999998</v>
+      </c>
+      <c r="Q12" s="46">
+        <v>2</v>
+      </c>
+      <c r="R12" s="46">
+        <v>1550</v>
+      </c>
+      <c r="S12" s="48">
+        <v>1.52</v>
+      </c>
+      <c r="T12" s="46">
+        <v>30</v>
+      </c>
+      <c r="U12" s="50">
+        <v>1.9400000000000001E-2</v>
+      </c>
+      <c r="V12" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB12" s="46" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="13" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="46">
+        <v>9</v>
+      </c>
+      <c r="B13" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>274</v>
+      </c>
+      <c r="E13" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="46">
+        <v>262675</v>
+      </c>
+      <c r="G13" s="46" t="s">
+        <v>288</v>
+      </c>
+      <c r="H13" s="46">
+        <v>1350</v>
+      </c>
+      <c r="I13" s="48">
+        <v>0.59199999999999997</v>
+      </c>
+      <c r="J13" s="48">
+        <v>1.619</v>
+      </c>
+      <c r="K13" s="46" t="s">
+        <v>289</v>
+      </c>
+      <c r="L13" s="48">
+        <v>1293.905</v>
+      </c>
+      <c r="M13" s="49">
+        <v>1092.8</v>
+      </c>
+      <c r="N13" s="50">
+        <v>0.15179999999999999</v>
+      </c>
+      <c r="O13" s="51">
+        <v>9.11</v>
+      </c>
+      <c r="P13" s="46">
+        <v>407.6</v>
+      </c>
+      <c r="Q13" s="46">
+        <v>2</v>
+      </c>
+      <c r="R13" s="46">
+        <v>1250</v>
+      </c>
+      <c r="S13" s="48">
+        <v>1.1839999999999999</v>
+      </c>
+      <c r="T13" s="46">
+        <v>66</v>
+      </c>
+      <c r="U13" s="50">
+        <v>5.28E-2</v>
+      </c>
+      <c r="V13" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB13" s="46" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="46">
+        <v>10</v>
+      </c>
+      <c r="B14" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E14" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="52">
+        <v>262642</v>
+      </c>
+      <c r="G14" s="52" t="s">
+        <v>231</v>
+      </c>
+      <c r="H14" s="52">
+        <v>1000</v>
+      </c>
+      <c r="I14" s="54">
+        <v>0.58099999999999996</v>
+      </c>
+      <c r="J14" s="54">
+        <v>1.58</v>
+      </c>
+      <c r="K14" s="52" t="s">
+        <v>230</v>
+      </c>
+      <c r="L14" s="54">
+        <v>917.98</v>
+      </c>
+      <c r="M14" s="55">
+        <v>790</v>
+      </c>
+      <c r="N14" s="56">
+        <v>0.10970000000000001</v>
+      </c>
+      <c r="O14" s="57">
+        <v>6.58</v>
+      </c>
+      <c r="P14" s="52">
+        <v>289.2</v>
+      </c>
+      <c r="Q14" s="52">
+        <v>2</v>
+      </c>
+      <c r="R14" s="52">
         <v>1200</v>
       </c>
-      <c r="S11" s="54">
+      <c r="S14" s="54">
         <v>1.1619999999999999</v>
       </c>
-      <c r="T11" s="52">
+      <c r="T14" s="52">
         <v>38</v>
       </c>
-      <c r="U11" s="56">
+      <c r="U14" s="56">
         <v>3.1699999999999999E-2</v>
       </c>
-      <c r="V11" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="52" t="s">
+      <c r="V14" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="AB11" s="52" t="s">
+      <c r="AB14" s="52" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="58" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="59">
-        <f>SUM(H3:H11)</f>
-        <v>16130</v>
-      </c>
-      <c r="I12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="59">
-        <f>SUM(P3:P11)</f>
-        <v>4435.1000000000004</v>
-      </c>
-      <c r="Q12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="59" t="s">
-        <v>27</v>
-      </c>
-    </row>
+    <row r="15" spans="1:28" s="58" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="59">
+        <f>SUM(H3:H14)</f>
+        <v>17350</v>
+      </c>
+      <c r="I15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="J15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="M15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="O15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="P15" s="59">
+        <f>SUM(P3:P14)</f>
+        <v>5371.1</v>
+      </c>
+      <c r="Q15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="R15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="S15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="T15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="U15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="V15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="W15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="X15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB15" s="59" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (29/09/2026 08:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43464021-31F0-4194-800C-21AF3318E528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11DE0FE7-DE14-4B78-A480-6507128DFBC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX EMBALAGENS LTDA 1233" sheetId="170" r:id="rId1"/>
     <sheet name="RM Embalagens 1232" sheetId="169" r:id="rId2"/>
-    <sheet name="HARMONY EMBALAGENS 1231" sheetId="168" r:id="rId3"/>
+    <sheet name="HARMONY EMBALAGENS 1231 P" sheetId="168" r:id="rId3"/>
     <sheet name="FAVINCO 1229" sheetId="167" r:id="rId4"/>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId5"/>
     <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId6"/>
@@ -1756,9 +1756,6 @@
     <xf numFmtId="14" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1767,6 +1764,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2024,88 +2024,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>401</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3098,88 +3098,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>241</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3830,88 +3830,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5157,88 +5157,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="99" t="s">
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6222,88 +6222,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="99" t="s">
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6870,88 +6870,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>235</v>
       </c>
-      <c r="B1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="99" t="s">
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8035,88 +8035,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="99" t="s">
         <v>181</v>
       </c>
-      <c r="B1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="100" t="s">
+      <c r="B1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="99" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8770,88 +8770,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="99" t="s">
         <v>173</v>
       </c>
-      <c r="B1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="100" t="s">
+      <c r="B1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="99" t="s">
         <v>27</v>
       </c>
     </row>
@@ -10537,88 +10537,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="99" t="s">
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11973,88 +11973,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="99" t="s">
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13049,88 +13049,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="100" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="101" t="s">
+      <c r="B1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="100" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14382,88 +14382,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>381</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -15288,88 +15288,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="101" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="102" t="s">
+      <c r="B1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="101" t="s">
         <v>27</v>
       </c>
     </row>
@@ -15936,88 +15936,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="102" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="103" t="s">
+      <c r="B1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="102" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="102" t="s">
         <v>27</v>
       </c>
     </row>
@@ -16548,6 +16548,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1138A384-FB07-407A-A271-F489A21E653B}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -16582,88 +16585,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="100" t="s">
         <v>369</v>
       </c>
-      <c r="B1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="97" t="s">
+      <c r="B1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="100" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="100" t="s">
         <v>27</v>
       </c>
     </row>
@@ -18205,7 +18208,7 @@
       <c r="Y19" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="Z19" s="52" t="s">
+      <c r="Z19" s="103" t="s">
         <v>27</v>
       </c>
       <c r="AA19" s="52" t="s">
@@ -18306,6 +18309,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="93" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -18345,88 +18349,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>333</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -18735,88 +18739,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>323</v>
       </c>
-      <c r="B1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="99" t="s">
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
         <v>27</v>
       </c>
     </row>
@@ -20499,88 +20503,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>298</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -21466,88 +21470,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>280</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>
@@ -22108,88 +22112,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="98" t="s">
         <v>266</v>
       </c>
-      <c r="B1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="99" t="s">
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
         <v>27</v>
       </c>
     </row>
@@ -23270,88 +23274,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="98" t="s">
+      <c r="A1" s="97" t="s">
         <v>249</v>
       </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (29/09/2026 11:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA008B4-1071-435E-97C1-1F8376F527A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D1B989-022A-45D9-8CE9-1C1982348B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renovapel 1235" sheetId="171" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (30/09/2026 13:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A1DD47-70E2-4881-8914-0AADC4A3E918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BA1D49-75AD-4466-8599-0A5083C3835C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renovapel 1242 P" sheetId="174" r:id="rId1"/>
     <sheet name="Tole. DR EMB. VO CH S. M 1241" sheetId="173" r:id="rId2"/>
-    <sheet name="FAVINCO 1239" sheetId="172" r:id="rId3"/>
+    <sheet name="FAVINCO 1239 P" sheetId="172" r:id="rId3"/>
     <sheet name="PCBOX EMBALAGENS LTDA 1233" sheetId="170" r:id="rId4"/>
     <sheet name="RM Embalagens 1232" sheetId="169" r:id="rId5"/>
     <sheet name="HARMONY EMBALAGENS 1231 P" sheetId="168" r:id="rId6"/>
@@ -19591,88 +19591,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="93" t="s">
         <v>459</v>
       </c>
-      <c r="B1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="91" t="s">
+      <c r="B1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="93" t="s">
         <v>27</v>
       </c>
     </row>
@@ -20450,6 +20450,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (30/09/2026 14:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BA1D49-75AD-4466-8599-0A5083C3835C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F2CC57-836B-4DCF-9A21-0858E0B6AA2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19558,6 +19558,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84ED9CA-CD86-4E4D-8079-E7302B17DD18}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -19586,7 +19589,7 @@
     <col min="25" max="25" width="8.33203125" style="33" customWidth="1"/>
     <col min="26" max="26" width="8.5546875" style="33" customWidth="1"/>
     <col min="27" max="27" width="7.109375" style="33" customWidth="1"/>
-    <col min="28" max="28" width="10.88671875" style="33" customWidth="1"/>
+    <col min="28" max="28" width="12.5546875" style="33" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="33"/>
   </cols>
   <sheetData>
@@ -20449,8 +20452,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.41" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup scale="83" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (30/09/2026 18:05)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F2CC57-836B-4DCF-9A21-0858E0B6AA2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15CF6D90-74BD-43A9-A02F-E51890872692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renovapel 1242 P" sheetId="174" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="RM Embalagens 1232" sheetId="169" r:id="rId5"/>
     <sheet name="HARMONY EMBALAGENS 1231 P" sheetId="168" r:id="rId6"/>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId7"/>
-    <sheet name="PCBOX EMBALAGENS LTDA 1222" sheetId="164" r:id="rId8"/>
+    <sheet name="PCBOX EMBALAGENS LTDA 1222 P" sheetId="164" r:id="rId8"/>
     <sheet name="FORBOX 1220" sheetId="163" r:id="rId9"/>
     <sheet name="HARMONY EMBALAGENS 1217 P" sheetId="162" r:id="rId10"/>
     <sheet name="Z4A EMBALAGENS LTDA 1216" sheetId="161" r:id="rId11"/>
@@ -1692,7 +1692,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1991,6 +1991,9 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -25969,6 +25972,9 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B791AA56-47E9-44C0-8D6D-1F61C5308578}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -26003,88 +26009,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="93" t="s">
         <v>296</v>
       </c>
-      <c r="B1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="91" t="s">
+      <c r="B1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="93" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="93" t="s">
         <v>27</v>
       </c>
     </row>
@@ -26676,88 +26682,88 @@
       </c>
     </row>
     <row r="9" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="85">
+      <c r="A9" s="106">
         <v>7</v>
       </c>
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="72" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="71" t="s">
         <v>272</v>
       </c>
-      <c r="E9" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="45">
+      <c r="E9" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="71">
         <v>262677</v>
       </c>
-      <c r="G9" s="45" t="s">
+      <c r="G9" s="71" t="s">
         <v>290</v>
       </c>
-      <c r="H9" s="45">
+      <c r="H9" s="71">
         <v>1000</v>
       </c>
-      <c r="I9" s="47">
+      <c r="I9" s="73">
         <v>0.8</v>
       </c>
-      <c r="J9" s="47">
+      <c r="J9" s="73">
         <v>1.171</v>
       </c>
-      <c r="K9" s="45" t="s">
+      <c r="K9" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="L9" s="47">
+      <c r="L9" s="73">
         <v>936.8</v>
       </c>
-      <c r="M9" s="48">
+      <c r="M9" s="74">
         <v>1171</v>
       </c>
-      <c r="N9" s="49">
+      <c r="N9" s="75">
         <v>0.32529999999999998</v>
       </c>
-      <c r="O9" s="50">
+      <c r="O9" s="76">
         <v>19.52</v>
       </c>
-      <c r="P9" s="45">
+      <c r="P9" s="71">
         <v>323.2</v>
       </c>
-      <c r="Q9" s="45">
+      <c r="Q9" s="71">
         <v>1</v>
       </c>
-      <c r="R9" s="45">
+      <c r="R9" s="71">
         <v>850</v>
       </c>
-      <c r="S9" s="47">
+      <c r="S9" s="73">
         <v>0.8</v>
       </c>
-      <c r="T9" s="45">
+      <c r="T9" s="71">
         <v>50</v>
       </c>
-      <c r="U9" s="49">
+      <c r="U9" s="75">
         <v>5.8799999999999998E-2</v>
       </c>
-      <c r="V9" s="45" t="s">
+      <c r="V9" s="71" t="s">
         <v>29</v>
       </c>
-      <c r="W9" s="45" t="s">
+      <c r="W9" s="71" t="s">
         <v>29</v>
       </c>
-      <c r="X9" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="45" t="s">
+      <c r="X9" s="71" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="71" t="s">
         <v>32</v>
       </c>
-      <c r="AB9" s="45" t="s">
+      <c r="AB9" s="71" t="s">
         <v>289</v>
       </c>
     </row>
@@ -26934,6 +26940,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="94" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 09:14)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{216F5F63-5EA5-40BC-80F2-F15689C70B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E9A667-1602-47C8-9F7F-3CE679BFF184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FAVINCO 1243 P" sheetId="175" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4626" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4642" uniqueCount="495">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1529,6 +1529,18 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - FAVINCO.  —  OF: 001243</t>
+  </si>
+  <si>
+    <t>W55R02110</t>
+  </si>
+  <si>
+    <t>820x2020</t>
+  </si>
+  <si>
+    <t>W55R0210</t>
+  </si>
+  <si>
+    <t>750x1900</t>
   </si>
 </sst>
 </file>
@@ -1726,7 +1738,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2028,6 +2040,28 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyFill="1"/>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2251,11 +2285,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{130D3884-F477-41AF-855E-4F984E358A9D}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" style="33" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="33" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="6.109375" style="33" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8.21875" style="33" customWidth="1"/>
@@ -2805,8 +2842,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.79" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="90" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -19089,16 +19126,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{320660EC-40AA-4456-8D33-C51008EBC785}">
-  <dimension ref="A1:AB20"/>
+  <dimension ref="A1:AB22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5546875" style="33" customWidth="1"/>
-    <col min="2" max="2" width="27.21875" style="33" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" style="33" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="33" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.44140625" style="33" customWidth="1"/>
     <col min="6" max="6" width="8.77734375" style="33" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="33" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" style="33" customWidth="1"/>
     <col min="8" max="8" width="7.5546875" style="33" customWidth="1"/>
     <col min="9" max="9" width="9.77734375" style="33" customWidth="1"/>
     <col min="10" max="10" width="8" style="33" customWidth="1"/>
@@ -19294,1497 +19331,1655 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="45">
+    <row r="3" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="107">
         <v>1</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="108" t="s">
         <v>107</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="107" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="107" t="s">
         <v>222</v>
       </c>
-      <c r="E3" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="45">
+      <c r="E3" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="107">
         <v>262792</v>
       </c>
-      <c r="G3" s="45" t="s">
+      <c r="G3" s="107" t="s">
         <v>271</v>
       </c>
-      <c r="H3" s="45">
+      <c r="H3" s="107">
         <v>3052</v>
       </c>
-      <c r="I3" s="47">
+      <c r="I3" s="109">
         <v>0.39</v>
       </c>
-      <c r="J3" s="47">
+      <c r="J3" s="109">
         <v>0.71</v>
       </c>
-      <c r="K3" s="45" t="s">
+      <c r="K3" s="107" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="47">
+      <c r="L3" s="109">
         <v>845.09900000000005</v>
       </c>
-      <c r="M3" s="48">
+      <c r="M3" s="110">
         <v>541.70000000000005</v>
       </c>
-      <c r="N3" s="49">
+      <c r="N3" s="111">
         <v>3.7600000000000001E-2</v>
       </c>
-      <c r="O3" s="50">
+      <c r="O3" s="112">
         <v>2.2599999999999998</v>
       </c>
-      <c r="P3" s="45">
+      <c r="P3" s="107">
         <v>300</v>
       </c>
-      <c r="Q3" s="45">
+      <c r="Q3" s="107">
         <v>4</v>
       </c>
-      <c r="R3" s="45">
+      <c r="R3" s="107">
         <v>1600</v>
       </c>
-      <c r="S3" s="47">
+      <c r="S3" s="109">
         <v>1.56</v>
       </c>
-      <c r="T3" s="45">
+      <c r="T3" s="107">
         <v>40</v>
       </c>
-      <c r="U3" s="49">
+      <c r="U3" s="111">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="V3" s="45" t="s">
+      <c r="V3" s="107" t="s">
         <v>29</v>
       </c>
-      <c r="W3" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="45" t="s">
+      <c r="W3" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="107" t="s">
         <v>29</v>
       </c>
-      <c r="Y3" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="45" t="s">
+      <c r="Y3" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="107" t="s">
         <v>38</v>
       </c>
-      <c r="AB3" s="45" t="s">
+      <c r="AB3" s="107" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="45">
+    <row r="4" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="107">
         <v>2</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="108" t="s">
         <v>472</v>
       </c>
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="107" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="107" t="s">
         <v>466</v>
       </c>
-      <c r="E4" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="45">
+      <c r="E4" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="107">
         <v>262800</v>
       </c>
-      <c r="G4" s="45" t="s">
+      <c r="G4" s="107" t="s">
         <v>471</v>
       </c>
-      <c r="H4" s="45">
+      <c r="H4" s="107">
+        <v>1000</v>
+      </c>
+      <c r="I4" s="109">
+        <v>0.495</v>
+      </c>
+      <c r="J4" s="109">
+        <v>0.97</v>
+      </c>
+      <c r="K4" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="109">
+        <v>288.08999999999997</v>
+      </c>
+      <c r="M4" s="110">
+        <v>194</v>
+      </c>
+      <c r="N4" s="111">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="O4" s="112">
+        <v>1.08</v>
+      </c>
+      <c r="P4" s="107">
+        <v>90.7</v>
+      </c>
+      <c r="Q4" s="107">
+        <v>3</v>
+      </c>
+      <c r="R4" s="107">
+        <v>1550</v>
+      </c>
+      <c r="S4" s="109">
+        <v>1.4850000000000001</v>
+      </c>
+      <c r="T4" s="107">
+        <v>65</v>
+      </c>
+      <c r="U4" s="111">
+        <v>4.19E-2</v>
+      </c>
+      <c r="V4" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X4" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="107" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB4" s="107" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="107">
+        <v>3</v>
+      </c>
+      <c r="B5" s="108" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="107" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="107" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="107">
+        <v>262790</v>
+      </c>
+      <c r="G5" s="107" t="s">
+        <v>271</v>
+      </c>
+      <c r="H5" s="107">
+        <v>2740</v>
+      </c>
+      <c r="I5" s="109">
+        <v>0.48</v>
+      </c>
+      <c r="J5" s="109">
+        <v>1.25</v>
+      </c>
+      <c r="K5" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L5" s="109">
+        <v>1644</v>
+      </c>
+      <c r="M5" s="110">
+        <v>1141.7</v>
+      </c>
+      <c r="N5" s="111">
+        <v>0.1057</v>
+      </c>
+      <c r="O5" s="112">
+        <v>6.34</v>
+      </c>
+      <c r="P5" s="107">
+        <v>600.1</v>
+      </c>
+      <c r="Q5" s="107">
+        <v>3</v>
+      </c>
+      <c r="R5" s="107">
+        <v>1500</v>
+      </c>
+      <c r="S5" s="109">
+        <v>1.44</v>
+      </c>
+      <c r="T5" s="107">
+        <v>60</v>
+      </c>
+      <c r="U5" s="111">
+        <v>0.04</v>
+      </c>
+      <c r="V5" s="107" t="s">
+        <v>37</v>
+      </c>
+      <c r="W5" s="107" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="107" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y5" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="107" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB5" s="107" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="107"/>
+      <c r="B6" s="108" t="s">
+        <v>472</v>
+      </c>
+      <c r="C6" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="114">
+        <v>46297</v>
+      </c>
+      <c r="E6" s="107"/>
+      <c r="F6" s="107">
+        <v>262827</v>
+      </c>
+      <c r="G6" s="107" t="s">
+        <v>493</v>
+      </c>
+      <c r="H6" s="107">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="109">
+        <v>0.73</v>
+      </c>
+      <c r="J6" s="109">
+        <v>0.47</v>
+      </c>
+      <c r="K6" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L6" s="109">
+        <v>343.1</v>
+      </c>
+      <c r="M6" s="110">
+        <v>235</v>
+      </c>
+      <c r="N6" s="111">
+        <v>3.2599999999999997E-2</v>
+      </c>
+      <c r="O6" s="112">
+        <v>1.96</v>
+      </c>
+      <c r="P6" s="107">
+        <v>108.1</v>
+      </c>
+      <c r="Q6" s="107">
+        <v>2</v>
+      </c>
+      <c r="R6" s="107">
+        <v>1500</v>
+      </c>
+      <c r="S6" s="109">
+        <v>1.46</v>
+      </c>
+      <c r="T6" s="107">
+        <v>40</v>
+      </c>
+      <c r="U6" s="111">
+        <v>2.6700000000000002E-2</v>
+      </c>
+      <c r="V6" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="107"/>
+      <c r="Z6" s="107"/>
+      <c r="AA6" s="107">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="107" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="107">
+        <v>4</v>
+      </c>
+      <c r="B7" s="108" t="s">
+        <v>467</v>
+      </c>
+      <c r="C7" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="107" t="s">
+        <v>466</v>
+      </c>
+      <c r="E7" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="107">
+        <v>262802</v>
+      </c>
+      <c r="G7" s="107" t="s">
+        <v>465</v>
+      </c>
+      <c r="H7" s="107">
+        <v>2000</v>
+      </c>
+      <c r="I7" s="109">
+        <v>0.35</v>
+      </c>
+      <c r="J7" s="109">
+        <v>0.7</v>
+      </c>
+      <c r="K7" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L7" s="109">
+        <v>490</v>
+      </c>
+      <c r="M7" s="110">
+        <v>350</v>
+      </c>
+      <c r="N7" s="111">
+        <v>2.4299999999999999E-2</v>
+      </c>
+      <c r="O7" s="112">
+        <v>1.46</v>
+      </c>
+      <c r="P7" s="107">
+        <v>154.30000000000001</v>
+      </c>
+      <c r="Q7" s="107">
+        <v>4</v>
+      </c>
+      <c r="R7" s="107">
+        <v>1450</v>
+      </c>
+      <c r="S7" s="109">
+        <v>1.4</v>
+      </c>
+      <c r="T7" s="107">
+        <v>50</v>
+      </c>
+      <c r="U7" s="111">
+        <v>3.4500000000000003E-2</v>
+      </c>
+      <c r="V7" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="107" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB7" s="107" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="107">
+        <v>5</v>
+      </c>
+      <c r="B8" s="108" t="s">
+        <v>463</v>
+      </c>
+      <c r="C8" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="107" t="s">
+        <v>404</v>
+      </c>
+      <c r="E8" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="107">
+        <v>262794</v>
+      </c>
+      <c r="G8" s="107" t="s">
+        <v>462</v>
+      </c>
+      <c r="H8" s="107">
+        <v>5000</v>
+      </c>
+      <c r="I8" s="109">
+        <v>0.46</v>
+      </c>
+      <c r="J8" s="109">
+        <v>0.92</v>
+      </c>
+      <c r="K8" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L8" s="109">
+        <v>2116</v>
+      </c>
+      <c r="M8" s="110">
+        <v>1533.3</v>
+      </c>
+      <c r="N8" s="111">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="O8" s="112">
+        <v>8.52</v>
+      </c>
+      <c r="P8" s="107">
+        <v>666.5</v>
+      </c>
+      <c r="Q8" s="107">
+        <v>3</v>
+      </c>
+      <c r="R8" s="107">
+        <v>1400</v>
+      </c>
+      <c r="S8" s="109">
+        <v>1.38</v>
+      </c>
+      <c r="T8" s="107">
+        <v>20</v>
+      </c>
+      <c r="U8" s="111">
+        <v>1.43E-2</v>
+      </c>
+      <c r="V8" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="107" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB8" s="107" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="107">
+        <v>6</v>
+      </c>
+      <c r="B9" s="108" t="s">
+        <v>467</v>
+      </c>
+      <c r="C9" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="107" t="s">
+        <v>466</v>
+      </c>
+      <c r="E9" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="107">
+        <v>262804</v>
+      </c>
+      <c r="G9" s="107" t="s">
+        <v>465</v>
+      </c>
+      <c r="H9" s="107">
+        <v>2000</v>
+      </c>
+      <c r="I9" s="109">
+        <v>0.46</v>
+      </c>
+      <c r="J9" s="109">
+        <v>0.9</v>
+      </c>
+      <c r="K9" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L9" s="109">
+        <v>828</v>
+      </c>
+      <c r="M9" s="110">
         <v>600</v>
       </c>
-      <c r="I4" s="47">
-        <v>0.495</v>
-      </c>
-      <c r="J4" s="47">
+      <c r="N9" s="111">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="O9" s="112">
+        <v>3.33</v>
+      </c>
+      <c r="P9" s="107">
+        <v>260.8</v>
+      </c>
+      <c r="Q9" s="107">
+        <v>3</v>
+      </c>
+      <c r="R9" s="107">
+        <v>1400</v>
+      </c>
+      <c r="S9" s="109">
+        <v>1.38</v>
+      </c>
+      <c r="T9" s="107">
+        <v>20</v>
+      </c>
+      <c r="U9" s="111">
+        <v>1.43E-2</v>
+      </c>
+      <c r="V9" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="107" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB9" s="107" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="107">
+        <v>7</v>
+      </c>
+      <c r="B10" s="108" t="s">
+        <v>472</v>
+      </c>
+      <c r="C10" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="107" t="s">
+        <v>466</v>
+      </c>
+      <c r="E10" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="107">
+        <v>262799</v>
+      </c>
+      <c r="G10" s="107" t="s">
+        <v>471</v>
+      </c>
+      <c r="H10" s="107">
+        <v>1000</v>
+      </c>
+      <c r="I10" s="109">
+        <v>0.44500000000000001</v>
+      </c>
+      <c r="J10" s="109">
+        <v>0.87</v>
+      </c>
+      <c r="K10" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L10" s="109">
+        <v>232.29</v>
+      </c>
+      <c r="M10" s="110">
+        <v>174</v>
+      </c>
+      <c r="N10" s="111">
+        <v>1.61E-2</v>
+      </c>
+      <c r="O10" s="112">
         <v>0.97</v>
       </c>
-      <c r="K4" s="45" t="s">
+      <c r="P10" s="107">
+        <v>73.2</v>
+      </c>
+      <c r="Q10" s="107">
+        <v>3</v>
+      </c>
+      <c r="R10" s="107">
+        <v>1400</v>
+      </c>
+      <c r="S10" s="109">
+        <v>1.335</v>
+      </c>
+      <c r="T10" s="107">
+        <v>65</v>
+      </c>
+      <c r="U10" s="111">
+        <v>4.6399999999999997E-2</v>
+      </c>
+      <c r="V10" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="107" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB10" s="107" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="107">
+        <v>8</v>
+      </c>
+      <c r="B11" s="108" t="s">
+        <v>463</v>
+      </c>
+      <c r="C11" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="107" t="s">
+        <v>404</v>
+      </c>
+      <c r="E11" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="107">
+        <v>262795</v>
+      </c>
+      <c r="G11" s="107" t="s">
+        <v>462</v>
+      </c>
+      <c r="H11" s="107">
+        <v>1000</v>
+      </c>
+      <c r="I11" s="109">
+        <v>0.66</v>
+      </c>
+      <c r="J11" s="109">
+        <v>0.82</v>
+      </c>
+      <c r="K11" s="107" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="47">
-        <v>288.08999999999997</v>
-      </c>
-      <c r="M4" s="48">
-        <v>194</v>
-      </c>
-      <c r="N4" s="49">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="O4" s="50">
-        <v>1.08</v>
-      </c>
-      <c r="P4" s="45">
-        <v>90.7</v>
-      </c>
-      <c r="Q4" s="45">
+      <c r="L11" s="109">
+        <v>541.20000000000005</v>
+      </c>
+      <c r="M11" s="110">
+        <v>410</v>
+      </c>
+      <c r="N11" s="111">
+        <v>5.6899999999999999E-2</v>
+      </c>
+      <c r="O11" s="112">
+        <v>3.42</v>
+      </c>
+      <c r="P11" s="107">
+        <v>170.5</v>
+      </c>
+      <c r="Q11" s="107">
+        <v>2</v>
+      </c>
+      <c r="R11" s="107">
+        <v>1350</v>
+      </c>
+      <c r="S11" s="109">
+        <v>1.32</v>
+      </c>
+      <c r="T11" s="107">
+        <v>30</v>
+      </c>
+      <c r="U11" s="111">
+        <v>2.2200000000000001E-2</v>
+      </c>
+      <c r="V11" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="107" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB11" s="107" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="107">
+        <v>9</v>
+      </c>
+      <c r="B12" s="108" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="107" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="107" t="s">
+        <v>222</v>
+      </c>
+      <c r="E12" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="107">
+        <v>262789</v>
+      </c>
+      <c r="G12" s="107" t="s">
+        <v>271</v>
+      </c>
+      <c r="H12" s="107">
+        <v>1662</v>
+      </c>
+      <c r="I12" s="109">
+        <v>0.43</v>
+      </c>
+      <c r="J12" s="109">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="K12" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L12" s="109">
+        <v>821.85900000000004</v>
+      </c>
+      <c r="M12" s="110">
+        <v>637.1</v>
+      </c>
+      <c r="N12" s="111">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="O12" s="112">
+        <v>3.54</v>
+      </c>
+      <c r="P12" s="107">
+        <v>300</v>
+      </c>
+      <c r="Q12" s="107">
         <v>3</v>
       </c>
-      <c r="R4" s="45">
-        <v>1550</v>
-      </c>
-      <c r="S4" s="47">
-        <v>1.4850000000000001</v>
-      </c>
-      <c r="T4" s="45">
-        <v>65</v>
-      </c>
-      <c r="U4" s="49">
-        <v>4.19E-2</v>
-      </c>
-      <c r="V4" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="45" t="s">
+      <c r="R12" s="107">
+        <v>1350</v>
+      </c>
+      <c r="S12" s="109">
+        <v>1.29</v>
+      </c>
+      <c r="T12" s="107">
+        <v>60</v>
+      </c>
+      <c r="U12" s="111">
+        <v>4.4400000000000002E-2</v>
+      </c>
+      <c r="V12" s="107" t="s">
+        <v>37</v>
+      </c>
+      <c r="W12" s="107" t="s">
+        <v>29</v>
+      </c>
+      <c r="X12" s="107" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y12" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="107" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB12" s="107" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="107">
+        <v>10</v>
+      </c>
+      <c r="B13" s="108" t="s">
+        <v>472</v>
+      </c>
+      <c r="C13" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="107" t="s">
+        <v>466</v>
+      </c>
+      <c r="E13" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="107">
+        <v>262798</v>
+      </c>
+      <c r="G13" s="107" t="s">
+        <v>471</v>
+      </c>
+      <c r="H13" s="107">
+        <v>300</v>
+      </c>
+      <c r="I13" s="109">
+        <v>0.42</v>
+      </c>
+      <c r="J13" s="109">
+        <v>0.82</v>
+      </c>
+      <c r="K13" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L13" s="109">
+        <v>103.32</v>
+      </c>
+      <c r="M13" s="110">
+        <v>82</v>
+      </c>
+      <c r="N13" s="111">
+        <v>7.6E-3</v>
+      </c>
+      <c r="O13" s="112">
+        <v>0.46</v>
+      </c>
+      <c r="P13" s="107">
+        <v>32.5</v>
+      </c>
+      <c r="Q13" s="107">
+        <v>3</v>
+      </c>
+      <c r="R13" s="107">
+        <v>1300</v>
+      </c>
+      <c r="S13" s="109">
+        <v>1.26</v>
+      </c>
+      <c r="T13" s="107">
+        <v>40</v>
+      </c>
+      <c r="U13" s="111">
+        <v>3.0800000000000001E-2</v>
+      </c>
+      <c r="V13" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="107" t="s">
         <v>38</v>
       </c>
-      <c r="AB4" s="45" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="45">
+      <c r="AB13" s="107" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="107">
+        <v>11</v>
+      </c>
+      <c r="B14" s="108" t="s">
+        <v>467</v>
+      </c>
+      <c r="C14" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="107" t="s">
+        <v>466</v>
+      </c>
+      <c r="E14" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="107">
+        <v>262803</v>
+      </c>
+      <c r="G14" s="107" t="s">
+        <v>465</v>
+      </c>
+      <c r="H14" s="107">
+        <v>2000</v>
+      </c>
+      <c r="I14" s="109">
+        <v>0.4</v>
+      </c>
+      <c r="J14" s="109">
+        <v>0.8</v>
+      </c>
+      <c r="K14" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L14" s="109">
+        <v>640</v>
+      </c>
+      <c r="M14" s="110">
+        <v>533.29999999999995</v>
+      </c>
+      <c r="N14" s="111">
+        <v>4.9399999999999999E-2</v>
+      </c>
+      <c r="O14" s="112">
+        <v>2.96</v>
+      </c>
+      <c r="P14" s="107">
+        <v>201.6</v>
+      </c>
+      <c r="Q14" s="107">
         <v>3</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="R14" s="107">
+        <v>1250</v>
+      </c>
+      <c r="S14" s="109">
+        <v>1.2</v>
+      </c>
+      <c r="T14" s="107">
+        <v>50</v>
+      </c>
+      <c r="U14" s="111">
+        <v>0.04</v>
+      </c>
+      <c r="V14" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="107" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB14" s="107" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="107">
+        <v>12</v>
+      </c>
+      <c r="B15" s="108" t="s">
+        <v>463</v>
+      </c>
+      <c r="C15" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="107" t="s">
+        <v>404</v>
+      </c>
+      <c r="E15" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="107">
+        <v>262797</v>
+      </c>
+      <c r="G15" s="107" t="s">
+        <v>462</v>
+      </c>
+      <c r="H15" s="107">
+        <v>500</v>
+      </c>
+      <c r="I15" s="109">
+        <v>0.59</v>
+      </c>
+      <c r="J15" s="109">
+        <v>0.88</v>
+      </c>
+      <c r="K15" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L15" s="109">
+        <v>259.60000000000002</v>
+      </c>
+      <c r="M15" s="110">
+        <v>220</v>
+      </c>
+      <c r="N15" s="111">
+        <v>3.0599999999999999E-2</v>
+      </c>
+      <c r="O15" s="112">
+        <v>1.83</v>
+      </c>
+      <c r="P15" s="107">
+        <v>81.8</v>
+      </c>
+      <c r="Q15" s="107">
+        <v>2</v>
+      </c>
+      <c r="R15" s="107">
+        <v>1200</v>
+      </c>
+      <c r="S15" s="109">
+        <v>1.18</v>
+      </c>
+      <c r="T15" s="107">
+        <v>20</v>
+      </c>
+      <c r="U15" s="111">
+        <v>1.67E-2</v>
+      </c>
+      <c r="V15" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="107" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB15" s="107" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="107">
+        <v>13</v>
+      </c>
+      <c r="B16" s="108" t="s">
+        <v>467</v>
+      </c>
+      <c r="C16" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="107" t="s">
+        <v>466</v>
+      </c>
+      <c r="E16" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="107">
+        <v>262801</v>
+      </c>
+      <c r="G16" s="107" t="s">
+        <v>465</v>
+      </c>
+      <c r="H16" s="107">
+        <v>1000</v>
+      </c>
+      <c r="I16" s="109">
+        <v>0.59</v>
+      </c>
+      <c r="J16" s="109">
+        <v>1.5</v>
+      </c>
+      <c r="K16" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L16" s="109">
+        <v>885</v>
+      </c>
+      <c r="M16" s="110">
+        <v>750</v>
+      </c>
+      <c r="N16" s="111">
+        <v>0.1042</v>
+      </c>
+      <c r="O16" s="112">
+        <v>6.25</v>
+      </c>
+      <c r="P16" s="107">
+        <v>278.8</v>
+      </c>
+      <c r="Q16" s="107">
+        <v>2</v>
+      </c>
+      <c r="R16" s="107">
+        <v>1200</v>
+      </c>
+      <c r="S16" s="109">
+        <v>1.18</v>
+      </c>
+      <c r="T16" s="107">
+        <v>20</v>
+      </c>
+      <c r="U16" s="111">
+        <v>1.67E-2</v>
+      </c>
+      <c r="V16" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y16" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z16" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA16" s="107" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB16" s="107" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="107">
+        <v>14</v>
+      </c>
+      <c r="B17" s="108" t="s">
+        <v>463</v>
+      </c>
+      <c r="C17" s="107" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="107" t="s">
+        <v>404</v>
+      </c>
+      <c r="E17" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="107">
+        <v>262796</v>
+      </c>
+      <c r="G17" s="107" t="s">
+        <v>462</v>
+      </c>
+      <c r="H17" s="107">
+        <v>1000</v>
+      </c>
+      <c r="I17" s="109">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J17" s="109">
+        <v>0.62</v>
+      </c>
+      <c r="K17" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L17" s="109">
+        <v>347.2</v>
+      </c>
+      <c r="M17" s="110">
+        <v>310</v>
+      </c>
+      <c r="N17" s="111">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="O17" s="112">
+        <v>2.58</v>
+      </c>
+      <c r="P17" s="107">
+        <v>109.4</v>
+      </c>
+      <c r="Q17" s="107">
+        <v>2</v>
+      </c>
+      <c r="R17" s="107">
+        <v>1150</v>
+      </c>
+      <c r="S17" s="109">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="T17" s="107">
+        <v>30</v>
+      </c>
+      <c r="U17" s="111">
+        <v>2.6100000000000002E-2</v>
+      </c>
+      <c r="V17" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W17" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X17" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y17" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="107" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB17" s="107" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="107">
+        <v>15</v>
+      </c>
+      <c r="B18" s="108" t="s">
         <v>107</v>
       </c>
-      <c r="C5" s="45" t="s">
+      <c r="C18" s="107" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="107" t="s">
+        <v>222</v>
+      </c>
+      <c r="E18" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="107">
+        <v>262793</v>
+      </c>
+      <c r="G18" s="107" t="s">
+        <v>271</v>
+      </c>
+      <c r="H18" s="107">
+        <v>3317</v>
+      </c>
+      <c r="I18" s="109">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J18" s="109">
+        <v>0.91</v>
+      </c>
+      <c r="K18" s="107" t="s">
+        <v>33</v>
+      </c>
+      <c r="L18" s="109">
+        <v>1690.3430000000001</v>
+      </c>
+      <c r="M18" s="110">
+        <v>1509.2</v>
+      </c>
+      <c r="N18" s="111">
+        <v>0.20960000000000001</v>
+      </c>
+      <c r="O18" s="112">
+        <v>12.58</v>
+      </c>
+      <c r="P18" s="107">
+        <v>600.1</v>
+      </c>
+      <c r="Q18" s="107">
+        <v>2</v>
+      </c>
+      <c r="R18" s="107">
+        <v>1150</v>
+      </c>
+      <c r="S18" s="109">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="T18" s="107">
+        <v>30</v>
+      </c>
+      <c r="U18" s="111">
+        <v>2.6100000000000002E-2</v>
+      </c>
+      <c r="V18" s="107" t="s">
+        <v>29</v>
+      </c>
+      <c r="W18" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X18" s="107" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y18" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="107" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB18" s="107" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="107">
+        <v>16</v>
+      </c>
+      <c r="B19" s="108" t="s">
+        <v>107</v>
+      </c>
+      <c r="C19" s="107" t="s">
         <v>55</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="D19" s="107" t="s">
         <v>222</v>
       </c>
-      <c r="E5" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="45">
-        <v>262790</v>
-      </c>
-      <c r="G5" s="45" t="s">
+      <c r="E19" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="107">
+        <v>262791</v>
+      </c>
+      <c r="G19" s="107" t="s">
         <v>271</v>
       </c>
-      <c r="H5" s="45">
-        <v>2740</v>
-      </c>
-      <c r="I5" s="47">
-        <v>0.48</v>
-      </c>
-      <c r="J5" s="47">
-        <v>1.25</v>
-      </c>
-      <c r="K5" s="45" t="s">
+      <c r="H19" s="107">
+        <v>1140</v>
+      </c>
+      <c r="I19" s="109">
+        <v>0.53</v>
+      </c>
+      <c r="J19" s="109">
+        <v>1.36</v>
+      </c>
+      <c r="K19" s="107" t="s">
         <v>33</v>
       </c>
-      <c r="L5" s="47">
-        <v>1644</v>
-      </c>
-      <c r="M5" s="48">
-        <v>1141.7</v>
-      </c>
-      <c r="N5" s="49">
-        <v>0.1057</v>
-      </c>
-      <c r="O5" s="50">
-        <v>6.34</v>
-      </c>
-      <c r="P5" s="45">
-        <v>600.1</v>
-      </c>
-      <c r="Q5" s="45">
-        <v>3</v>
-      </c>
-      <c r="R5" s="45">
-        <v>1500</v>
-      </c>
-      <c r="S5" s="47">
-        <v>1.44</v>
-      </c>
-      <c r="T5" s="45">
-        <v>60</v>
-      </c>
-      <c r="U5" s="49">
-        <v>0.04</v>
-      </c>
-      <c r="V5" s="45" t="s">
+      <c r="L19" s="109">
+        <v>821.71199999999999</v>
+      </c>
+      <c r="M19" s="110">
+        <v>775.2</v>
+      </c>
+      <c r="N19" s="111">
+        <v>0.1077</v>
+      </c>
+      <c r="O19" s="112">
+        <v>6.46</v>
+      </c>
+      <c r="P19" s="107">
+        <v>299.89999999999998</v>
+      </c>
+      <c r="Q19" s="107">
+        <v>2</v>
+      </c>
+      <c r="R19" s="107">
+        <v>1100</v>
+      </c>
+      <c r="S19" s="109">
+        <v>1.06</v>
+      </c>
+      <c r="T19" s="107">
+        <v>40</v>
+      </c>
+      <c r="U19" s="111">
+        <v>3.6400000000000002E-2</v>
+      </c>
+      <c r="V19" s="107" t="s">
         <v>37</v>
       </c>
-      <c r="W5" s="45" t="s">
+      <c r="W19" s="107" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="45" t="s">
+      <c r="X19" s="107" t="s">
         <v>34</v>
       </c>
-      <c r="Y5" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="45" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB5" s="45" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="45">
-        <v>4</v>
-      </c>
-      <c r="B6" s="46" t="s">
-        <v>467</v>
-      </c>
-      <c r="C6" s="45" t="s">
+      <c r="Y19" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="107" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB19" s="107" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" s="113" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="107"/>
+      <c r="B20" s="108" t="s">
+        <v>472</v>
+      </c>
+      <c r="C20" s="107" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="45" t="s">
-        <v>466</v>
-      </c>
-      <c r="E6" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="45">
-        <v>262802</v>
-      </c>
-      <c r="G6" s="45" t="s">
-        <v>465</v>
-      </c>
-      <c r="H6" s="45">
-        <v>2000</v>
-      </c>
-      <c r="I6" s="47">
-        <v>0.35</v>
-      </c>
-      <c r="J6" s="47">
-        <v>0.7</v>
-      </c>
-      <c r="K6" s="45" t="s">
+      <c r="D20" s="114">
+        <v>46296</v>
+      </c>
+      <c r="E20" s="107"/>
+      <c r="F20" s="107">
+        <v>262826</v>
+      </c>
+      <c r="G20" s="107" t="s">
+        <v>491</v>
+      </c>
+      <c r="H20" s="107">
+        <v>1000</v>
+      </c>
+      <c r="I20" s="109">
+        <v>0.8</v>
+      </c>
+      <c r="J20" s="109">
+        <v>0.5</v>
+      </c>
+      <c r="K20" s="107" t="s">
         <v>33</v>
       </c>
-      <c r="L6" s="47">
-        <v>490</v>
-      </c>
-      <c r="M6" s="48">
-        <v>350</v>
-      </c>
-      <c r="N6" s="49">
-        <v>2.4299999999999999E-2</v>
-      </c>
-      <c r="O6" s="50">
-        <v>1.46</v>
-      </c>
-      <c r="P6" s="45">
-        <v>154.30000000000001</v>
-      </c>
-      <c r="Q6" s="45">
-        <v>4</v>
-      </c>
-      <c r="R6" s="45">
-        <v>1450</v>
-      </c>
-      <c r="S6" s="47">
-        <v>1.4</v>
-      </c>
-      <c r="T6" s="45">
+      <c r="L20" s="109">
+        <v>400</v>
+      </c>
+      <c r="M20" s="110">
+        <v>500</v>
+      </c>
+      <c r="N20" s="111">
+        <v>0.1389</v>
+      </c>
+      <c r="O20" s="112">
+        <v>8.33</v>
+      </c>
+      <c r="P20" s="107">
+        <v>126</v>
+      </c>
+      <c r="Q20" s="107">
+        <v>1</v>
+      </c>
+      <c r="R20" s="107">
+        <v>850</v>
+      </c>
+      <c r="S20" s="109">
+        <v>0.8</v>
+      </c>
+      <c r="T20" s="107">
         <v>50</v>
       </c>
-      <c r="U6" s="49">
-        <v>3.4500000000000003E-2</v>
-      </c>
-      <c r="V6" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB6" s="45" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="45">
-        <v>5</v>
-      </c>
-      <c r="B7" s="46" t="s">
-        <v>463</v>
-      </c>
-      <c r="C7" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>404</v>
-      </c>
-      <c r="E7" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="45">
-        <v>262794</v>
-      </c>
-      <c r="G7" s="45" t="s">
-        <v>462</v>
-      </c>
-      <c r="H7" s="45">
-        <v>5000</v>
-      </c>
-      <c r="I7" s="47">
-        <v>0.46</v>
-      </c>
-      <c r="J7" s="47">
-        <v>0.92</v>
-      </c>
-      <c r="K7" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L7" s="47">
-        <v>2116</v>
-      </c>
-      <c r="M7" s="48">
-        <v>1533.3</v>
-      </c>
-      <c r="N7" s="49">
-        <v>0.14199999999999999</v>
-      </c>
-      <c r="O7" s="50">
-        <v>8.52</v>
-      </c>
-      <c r="P7" s="45">
-        <v>666.5</v>
-      </c>
-      <c r="Q7" s="45">
-        <v>3</v>
-      </c>
-      <c r="R7" s="45">
-        <v>1400</v>
-      </c>
-      <c r="S7" s="47">
-        <v>1.38</v>
-      </c>
-      <c r="T7" s="45">
-        <v>20</v>
-      </c>
-      <c r="U7" s="49">
-        <v>1.43E-2</v>
-      </c>
-      <c r="V7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="45" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB7" s="45" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="45">
-        <v>6</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>467</v>
-      </c>
-      <c r="C8" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="45" t="s">
-        <v>466</v>
-      </c>
-      <c r="E8" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="45">
-        <v>262804</v>
-      </c>
-      <c r="G8" s="45" t="s">
-        <v>465</v>
-      </c>
-      <c r="H8" s="45">
-        <v>2000</v>
-      </c>
-      <c r="I8" s="47">
-        <v>0.46</v>
-      </c>
-      <c r="J8" s="47">
-        <v>0.9</v>
-      </c>
-      <c r="K8" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L8" s="47">
-        <v>828</v>
-      </c>
-      <c r="M8" s="48">
-        <v>600</v>
-      </c>
-      <c r="N8" s="49">
-        <v>5.5599999999999997E-2</v>
-      </c>
-      <c r="O8" s="50">
-        <v>3.33</v>
-      </c>
-      <c r="P8" s="45">
-        <v>260.8</v>
-      </c>
-      <c r="Q8" s="45">
-        <v>3</v>
-      </c>
-      <c r="R8" s="45">
-        <v>1400</v>
-      </c>
-      <c r="S8" s="47">
-        <v>1.38</v>
-      </c>
-      <c r="T8" s="45">
-        <v>20</v>
-      </c>
-      <c r="U8" s="49">
-        <v>1.43E-2</v>
-      </c>
-      <c r="V8" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="45" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB8" s="45" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A9" s="45">
-        <v>7</v>
-      </c>
-      <c r="B9" s="46" t="s">
-        <v>472</v>
-      </c>
-      <c r="C9" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="45" t="s">
-        <v>466</v>
-      </c>
-      <c r="E9" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="45">
-        <v>262799</v>
-      </c>
-      <c r="G9" s="45" t="s">
-        <v>471</v>
-      </c>
-      <c r="H9" s="45">
-        <v>600</v>
-      </c>
-      <c r="I9" s="47">
-        <v>0.44500000000000001</v>
-      </c>
-      <c r="J9" s="47">
-        <v>0.87</v>
-      </c>
-      <c r="K9" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L9" s="47">
-        <v>232.29</v>
-      </c>
-      <c r="M9" s="48">
-        <v>174</v>
-      </c>
-      <c r="N9" s="49">
-        <v>1.61E-2</v>
-      </c>
-      <c r="O9" s="50">
-        <v>0.97</v>
-      </c>
-      <c r="P9" s="45">
-        <v>73.2</v>
-      </c>
-      <c r="Q9" s="45">
-        <v>3</v>
-      </c>
-      <c r="R9" s="45">
-        <v>1400</v>
-      </c>
-      <c r="S9" s="47">
-        <v>1.335</v>
-      </c>
-      <c r="T9" s="45">
-        <v>65</v>
-      </c>
-      <c r="U9" s="49">
-        <v>4.6399999999999997E-2</v>
-      </c>
-      <c r="V9" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB9" s="45" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A10" s="45">
-        <v>8</v>
-      </c>
-      <c r="B10" s="46" t="s">
-        <v>463</v>
-      </c>
-      <c r="C10" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="45" t="s">
-        <v>404</v>
-      </c>
-      <c r="E10" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="45">
-        <v>262795</v>
-      </c>
-      <c r="G10" s="45" t="s">
-        <v>462</v>
-      </c>
-      <c r="H10" s="45">
-        <v>1000</v>
-      </c>
-      <c r="I10" s="47">
-        <v>0.66</v>
-      </c>
-      <c r="J10" s="47">
-        <v>0.82</v>
-      </c>
-      <c r="K10" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L10" s="47">
-        <v>541.20000000000005</v>
-      </c>
-      <c r="M10" s="48">
-        <v>410</v>
-      </c>
-      <c r="N10" s="49">
-        <v>5.6899999999999999E-2</v>
-      </c>
-      <c r="O10" s="50">
-        <v>3.42</v>
-      </c>
-      <c r="P10" s="45">
-        <v>170.5</v>
-      </c>
-      <c r="Q10" s="45">
-        <v>2</v>
-      </c>
-      <c r="R10" s="45">
-        <v>1350</v>
-      </c>
-      <c r="S10" s="47">
-        <v>1.32</v>
-      </c>
-      <c r="T10" s="45">
-        <v>30</v>
-      </c>
-      <c r="U10" s="49">
-        <v>2.2200000000000001E-2</v>
-      </c>
-      <c r="V10" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB10" s="45" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" s="45">
-        <v>9</v>
-      </c>
-      <c r="B11" s="46" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" s="45" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="45" t="s">
-        <v>222</v>
-      </c>
-      <c r="E11" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="45">
-        <v>262789</v>
-      </c>
-      <c r="G11" s="45" t="s">
-        <v>271</v>
-      </c>
-      <c r="H11" s="45">
-        <v>1662</v>
-      </c>
-      <c r="I11" s="47">
-        <v>0.43</v>
-      </c>
-      <c r="J11" s="47">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="K11" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L11" s="47">
-        <v>821.85900000000004</v>
-      </c>
-      <c r="M11" s="48">
-        <v>637.1</v>
-      </c>
-      <c r="N11" s="49">
-        <v>5.8999999999999997E-2</v>
-      </c>
-      <c r="O11" s="50">
-        <v>3.54</v>
-      </c>
-      <c r="P11" s="45">
-        <v>300</v>
-      </c>
-      <c r="Q11" s="45">
-        <v>3</v>
-      </c>
-      <c r="R11" s="45">
-        <v>1350</v>
-      </c>
-      <c r="S11" s="47">
-        <v>1.29</v>
-      </c>
-      <c r="T11" s="45">
-        <v>60</v>
-      </c>
-      <c r="U11" s="49">
-        <v>4.4400000000000002E-2</v>
-      </c>
-      <c r="V11" s="45" t="s">
-        <v>37</v>
-      </c>
-      <c r="W11" s="45" t="s">
-        <v>29</v>
-      </c>
-      <c r="X11" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y11" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="45" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB11" s="45" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" s="45">
-        <v>10</v>
-      </c>
-      <c r="B12" s="46" t="s">
-        <v>472</v>
-      </c>
-      <c r="C12" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="45" t="s">
-        <v>466</v>
-      </c>
-      <c r="E12" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="45">
-        <v>262798</v>
-      </c>
-      <c r="G12" s="45" t="s">
-        <v>471</v>
-      </c>
-      <c r="H12" s="45">
-        <v>300</v>
-      </c>
-      <c r="I12" s="47">
-        <v>0.42</v>
-      </c>
-      <c r="J12" s="47">
-        <v>0.82</v>
-      </c>
-      <c r="K12" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L12" s="47">
-        <v>103.32</v>
-      </c>
-      <c r="M12" s="48">
-        <v>82</v>
-      </c>
-      <c r="N12" s="49">
-        <v>7.6E-3</v>
-      </c>
-      <c r="O12" s="50">
-        <v>0.46</v>
-      </c>
-      <c r="P12" s="45">
-        <v>32.5</v>
-      </c>
-      <c r="Q12" s="45">
-        <v>3</v>
-      </c>
-      <c r="R12" s="45">
-        <v>1300</v>
-      </c>
-      <c r="S12" s="47">
-        <v>1.26</v>
-      </c>
-      <c r="T12" s="45">
-        <v>40</v>
-      </c>
-      <c r="U12" s="49">
-        <v>3.0800000000000001E-2</v>
-      </c>
-      <c r="V12" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X12" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB12" s="45" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" s="45">
-        <v>11</v>
-      </c>
-      <c r="B13" s="46" t="s">
-        <v>467</v>
-      </c>
-      <c r="C13" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="45" t="s">
-        <v>466</v>
-      </c>
-      <c r="E13" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="45">
-        <v>262803</v>
-      </c>
-      <c r="G13" s="45" t="s">
-        <v>465</v>
-      </c>
-      <c r="H13" s="45">
-        <v>2000</v>
-      </c>
-      <c r="I13" s="47">
-        <v>0.4</v>
-      </c>
-      <c r="J13" s="47">
-        <v>0.8</v>
-      </c>
-      <c r="K13" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L13" s="47">
-        <v>640</v>
-      </c>
-      <c r="M13" s="48">
-        <v>533.29999999999995</v>
-      </c>
-      <c r="N13" s="49">
-        <v>4.9399999999999999E-2</v>
-      </c>
-      <c r="O13" s="50">
-        <v>2.96</v>
-      </c>
-      <c r="P13" s="45">
-        <v>201.6</v>
-      </c>
-      <c r="Q13" s="45">
-        <v>3</v>
-      </c>
-      <c r="R13" s="45">
-        <v>1250</v>
-      </c>
-      <c r="S13" s="47">
-        <v>1.2</v>
-      </c>
-      <c r="T13" s="45">
-        <v>50</v>
-      </c>
-      <c r="U13" s="49">
-        <v>0.04</v>
-      </c>
-      <c r="V13" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W13" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X13" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y13" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="45" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB13" s="45" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A14" s="45">
-        <v>12</v>
-      </c>
-      <c r="B14" s="46" t="s">
-        <v>463</v>
-      </c>
-      <c r="C14" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="45" t="s">
-        <v>404</v>
-      </c>
-      <c r="E14" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="45">
-        <v>262797</v>
-      </c>
-      <c r="G14" s="45" t="s">
-        <v>462</v>
-      </c>
-      <c r="H14" s="45">
-        <v>500</v>
-      </c>
-      <c r="I14" s="47">
-        <v>0.59</v>
-      </c>
-      <c r="J14" s="47">
-        <v>0.88</v>
-      </c>
-      <c r="K14" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L14" s="47">
-        <v>259.60000000000002</v>
-      </c>
-      <c r="M14" s="48">
-        <v>220</v>
-      </c>
-      <c r="N14" s="49">
-        <v>3.0599999999999999E-2</v>
-      </c>
-      <c r="O14" s="50">
-        <v>1.83</v>
-      </c>
-      <c r="P14" s="45">
-        <v>81.8</v>
-      </c>
-      <c r="Q14" s="45">
-        <v>2</v>
-      </c>
-      <c r="R14" s="45">
-        <v>1200</v>
-      </c>
-      <c r="S14" s="47">
-        <v>1.18</v>
-      </c>
-      <c r="T14" s="45">
-        <v>20</v>
-      </c>
-      <c r="U14" s="49">
-        <v>1.67E-2</v>
-      </c>
-      <c r="V14" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W14" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X14" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y14" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z14" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA14" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB14" s="45" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A15" s="45">
-        <v>13</v>
-      </c>
-      <c r="B15" s="46" t="s">
-        <v>467</v>
-      </c>
-      <c r="C15" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="45" t="s">
-        <v>466</v>
-      </c>
-      <c r="E15" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="45">
-        <v>262801</v>
-      </c>
-      <c r="G15" s="45" t="s">
-        <v>465</v>
-      </c>
-      <c r="H15" s="45">
-        <v>1000</v>
-      </c>
-      <c r="I15" s="47">
-        <v>0.59</v>
-      </c>
-      <c r="J15" s="47">
-        <v>1.5</v>
-      </c>
-      <c r="K15" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L15" s="47">
-        <v>885</v>
-      </c>
-      <c r="M15" s="48">
-        <v>750</v>
-      </c>
-      <c r="N15" s="49">
-        <v>0.1042</v>
-      </c>
-      <c r="O15" s="50">
-        <v>6.25</v>
-      </c>
-      <c r="P15" s="45">
-        <v>278.8</v>
-      </c>
-      <c r="Q15" s="45">
-        <v>2</v>
-      </c>
-      <c r="R15" s="45">
-        <v>1200</v>
-      </c>
-      <c r="S15" s="47">
-        <v>1.18</v>
-      </c>
-      <c r="T15" s="45">
-        <v>20</v>
-      </c>
-      <c r="U15" s="49">
-        <v>1.67E-2</v>
-      </c>
-      <c r="V15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="45" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB15" s="45" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A16" s="45">
-        <v>14</v>
-      </c>
-      <c r="B16" s="46" t="s">
-        <v>463</v>
-      </c>
-      <c r="C16" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" s="45" t="s">
-        <v>404</v>
-      </c>
-      <c r="E16" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="45">
-        <v>262796</v>
-      </c>
-      <c r="G16" s="45" t="s">
-        <v>462</v>
-      </c>
-      <c r="H16" s="45">
-        <v>1000</v>
-      </c>
-      <c r="I16" s="47">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="J16" s="47">
-        <v>0.62</v>
-      </c>
-      <c r="K16" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L16" s="47">
-        <v>347.2</v>
-      </c>
-      <c r="M16" s="48">
-        <v>310</v>
-      </c>
-      <c r="N16" s="49">
-        <v>4.3099999999999999E-2</v>
-      </c>
-      <c r="O16" s="50">
-        <v>2.58</v>
-      </c>
-      <c r="P16" s="45">
-        <v>109.4</v>
-      </c>
-      <c r="Q16" s="45">
-        <v>2</v>
-      </c>
-      <c r="R16" s="45">
-        <v>1150</v>
-      </c>
-      <c r="S16" s="47">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="T16" s="45">
-        <v>30</v>
-      </c>
-      <c r="U16" s="49">
-        <v>2.6100000000000002E-2</v>
-      </c>
-      <c r="V16" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W16" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X16" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y16" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z16" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA16" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB16" s="45" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A17" s="45">
-        <v>15</v>
-      </c>
-      <c r="B17" s="46" t="s">
-        <v>107</v>
-      </c>
-      <c r="C17" s="45" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17" s="45" t="s">
-        <v>222</v>
-      </c>
-      <c r="E17" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="45">
-        <v>262793</v>
-      </c>
-      <c r="G17" s="45" t="s">
-        <v>271</v>
-      </c>
-      <c r="H17" s="45">
-        <v>3317</v>
-      </c>
-      <c r="I17" s="47">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="J17" s="47">
-        <v>0.91</v>
-      </c>
-      <c r="K17" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L17" s="47">
-        <v>1690.3430000000001</v>
-      </c>
-      <c r="M17" s="48">
-        <v>1509.2</v>
-      </c>
-      <c r="N17" s="49">
-        <v>0.20960000000000001</v>
-      </c>
-      <c r="O17" s="50">
-        <v>12.58</v>
-      </c>
-      <c r="P17" s="45">
-        <v>600.1</v>
-      </c>
-      <c r="Q17" s="45">
-        <v>2</v>
-      </c>
-      <c r="R17" s="45">
-        <v>1150</v>
-      </c>
-      <c r="S17" s="47">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="T17" s="45">
-        <v>30</v>
-      </c>
-      <c r="U17" s="49">
-        <v>2.6100000000000002E-2</v>
-      </c>
-      <c r="V17" s="45" t="s">
-        <v>29</v>
-      </c>
-      <c r="W17" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X17" s="45" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y17" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z17" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA17" s="45" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB17" s="45" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A18" s="45">
-        <v>16</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>107</v>
-      </c>
-      <c r="C18" s="45" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="45" t="s">
-        <v>222</v>
-      </c>
-      <c r="E18" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="45">
-        <v>262791</v>
-      </c>
-      <c r="G18" s="45" t="s">
-        <v>271</v>
-      </c>
-      <c r="H18" s="45">
-        <v>1140</v>
-      </c>
-      <c r="I18" s="47">
-        <v>0.53</v>
-      </c>
-      <c r="J18" s="47">
-        <v>1.36</v>
-      </c>
-      <c r="K18" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="L18" s="47">
-        <v>821.71199999999999</v>
-      </c>
-      <c r="M18" s="48">
-        <v>775.2</v>
-      </c>
-      <c r="N18" s="49">
-        <v>0.1077</v>
-      </c>
-      <c r="O18" s="50">
-        <v>6.46</v>
-      </c>
-      <c r="P18" s="45">
-        <v>299.89999999999998</v>
-      </c>
-      <c r="Q18" s="45">
-        <v>2</v>
-      </c>
-      <c r="R18" s="45">
-        <v>1100</v>
-      </c>
-      <c r="S18" s="47">
-        <v>1.06</v>
-      </c>
-      <c r="T18" s="45">
-        <v>40</v>
-      </c>
-      <c r="U18" s="49">
-        <v>3.6400000000000002E-2</v>
-      </c>
-      <c r="V18" s="45" t="s">
-        <v>37</v>
-      </c>
-      <c r="W18" s="45" t="s">
-        <v>29</v>
-      </c>
-      <c r="X18" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y18" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z18" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA18" s="45" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB18" s="45" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="G19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="H19" s="52">
-        <v>27911</v>
-      </c>
-      <c r="I19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="J19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="K19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="L19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="M19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="N19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="O19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="P19" s="52">
-        <v>4220.2</v>
-      </c>
-      <c r="Q19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="R19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="S19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="T19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="U19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="V19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="W19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="X19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA19" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB19" s="52" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A20" s="51"/>
-      <c r="B20" s="51"/>
-      <c r="C20" s="51"/>
-      <c r="D20" s="51"/>
-      <c r="E20" s="51"/>
-      <c r="F20" s="51"/>
-      <c r="G20" s="51"/>
-      <c r="H20" s="51"/>
-      <c r="I20" s="51"/>
-      <c r="J20" s="51"/>
-      <c r="K20" s="51"/>
-      <c r="L20" s="51"/>
-      <c r="M20" s="51"/>
-      <c r="N20" s="51"/>
-      <c r="O20" s="51"/>
-      <c r="P20" s="51"/>
-      <c r="Q20" s="51"/>
-      <c r="R20" s="51"/>
-      <c r="S20" s="51"/>
-      <c r="T20" s="51"/>
-      <c r="U20" s="51"/>
-      <c r="V20" s="51"/>
-      <c r="W20" s="51"/>
-      <c r="X20" s="51"/>
-      <c r="Y20" s="51"/>
-      <c r="Z20" s="51"/>
-      <c r="AA20" s="51"/>
-      <c r="AB20" s="51"/>
+      <c r="U20" s="111">
+        <v>5.8799999999999998E-2</v>
+      </c>
+      <c r="V20" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="W20" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="X20" s="107" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y20" s="107"/>
+      <c r="Z20" s="107"/>
+      <c r="AA20" s="107">
+        <v>1</v>
+      </c>
+      <c r="AB20" s="107" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="H21" s="52">
+        <f>SUM(H3:H20)</f>
+        <v>30711</v>
+      </c>
+      <c r="I21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="K21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="M21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="O21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="P21" s="52">
+        <f>SUM(P3:P20)</f>
+        <v>4454.3</v>
+      </c>
+      <c r="Q21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="R21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="S21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="T21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="U21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="V21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="W21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="X21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA21" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB21" s="52" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A22" s="51"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="51"/>
+      <c r="H22" s="51"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="51"/>
+      <c r="K22" s="51"/>
+      <c r="L22" s="51"/>
+      <c r="M22" s="51"/>
+      <c r="N22" s="51"/>
+      <c r="O22" s="51"/>
+      <c r="P22" s="51"/>
+      <c r="Q22" s="51"/>
+      <c r="R22" s="51"/>
+      <c r="S22" s="51"/>
+      <c r="T22" s="51"/>
+      <c r="U22" s="51"/>
+      <c r="V22" s="51"/>
+      <c r="W22" s="51"/>
+      <c r="X22" s="51"/>
+      <c r="Y22" s="51"/>
+      <c r="Z22" s="51"/>
+      <c r="AA22" s="51"/>
+      <c r="AB22" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 09:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BBF9352-E4F6-4818-A129-7F4CF7A4328E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5924DF-FB8B-4CC1-AE14-46BE4C075A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FAVINCO 1243 P" sheetId="175" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4642" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4656" uniqueCount="499">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1541,6 +1541,18 @@
   </si>
   <si>
     <t>750x1900</t>
+  </si>
+  <si>
+    <t>128x138x128</t>
+  </si>
+  <si>
+    <t>808x2160</t>
+  </si>
+  <si>
+    <t>155x230x155</t>
+  </si>
+  <si>
+    <t>1100x1630</t>
   </si>
 </sst>
 </file>
@@ -2285,7 +2297,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" style="33" customWidth="1"/>
@@ -2490,101 +2502,92 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="45">
+    <row r="3" spans="1:28" s="85" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="85">
         <v>1</v>
       </c>
-      <c r="B3" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="C3" s="45" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="45" t="s">
-        <v>483</v>
-      </c>
-      <c r="E3" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="45">
-        <v>262823</v>
-      </c>
-      <c r="G3" s="45" t="s">
-        <v>489</v>
-      </c>
-      <c r="H3" s="45">
-        <v>300</v>
-      </c>
-      <c r="I3" s="47">
-        <v>0.36599999999999999</v>
-      </c>
-      <c r="J3" s="47">
-        <v>1.57</v>
-      </c>
-      <c r="K3" s="45" t="s">
-        <v>488</v>
-      </c>
-      <c r="L3" s="47">
-        <v>172.386</v>
-      </c>
-      <c r="M3" s="48">
-        <v>117.8</v>
-      </c>
-      <c r="N3" s="49">
-        <v>8.2000000000000007E-3</v>
-      </c>
-      <c r="O3" s="50">
-        <v>0.49</v>
-      </c>
-      <c r="P3" s="45">
-        <v>97.9</v>
-      </c>
-      <c r="Q3" s="45">
+      <c r="B3" s="85" t="s">
+        <v>460</v>
+      </c>
+      <c r="C3" s="85" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="86">
+        <v>46297</v>
+      </c>
+      <c r="F3" s="85">
+        <v>262828</v>
+      </c>
+      <c r="G3" s="85">
+        <v>81</v>
+      </c>
+      <c r="H3" s="85">
+        <v>2000</v>
+      </c>
+      <c r="I3" s="85">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="J3" s="85">
+        <v>1.07</v>
+      </c>
+      <c r="K3" s="85" t="s">
+        <v>495</v>
+      </c>
+      <c r="L3" s="85">
+        <v>843.16</v>
+      </c>
+      <c r="M3" s="85">
+        <v>535</v>
+      </c>
+      <c r="N3" s="85">
+        <v>3.7199999999999997E-2</v>
+      </c>
+      <c r="O3" s="85">
+        <v>2.23</v>
+      </c>
+      <c r="P3" s="85">
+        <v>299.3</v>
+      </c>
+      <c r="Q3" s="85">
         <v>4</v>
       </c>
-      <c r="R3" s="45">
-        <v>1500</v>
-      </c>
-      <c r="S3" s="47">
-        <v>1.464</v>
-      </c>
-      <c r="T3" s="45">
-        <v>36</v>
-      </c>
-      <c r="U3" s="49">
-        <v>2.4E-2</v>
-      </c>
-      <c r="V3" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="W3" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="X3" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y3" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z3" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA3" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB3" s="45" t="s">
-        <v>487</v>
+      <c r="R3" s="85">
+        <v>1600</v>
+      </c>
+      <c r="S3" s="85">
+        <v>1.5760000000000001</v>
+      </c>
+      <c r="T3" s="85">
+        <v>24</v>
+      </c>
+      <c r="U3" s="85">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="V3" s="85" t="s">
+        <v>29</v>
+      </c>
+      <c r="W3" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="85" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA3" s="85">
+        <v>2</v>
+      </c>
+      <c r="AB3" s="85" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="45">
+      <c r="A4" s="85">
         <v>2</v>
       </c>
       <c r="B4" s="46" t="s">
         <v>126</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="D4" s="45" t="s">
         <v>483</v>
@@ -2593,77 +2596,77 @@
         <v>27</v>
       </c>
       <c r="F4" s="45">
-        <v>262824</v>
+        <v>262823</v>
       </c>
       <c r="G4" s="45" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="H4" s="45">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="I4" s="47">
-        <v>0.63900000000000001</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="J4" s="47">
-        <v>1.9019999999999999</v>
+        <v>1.57</v>
       </c>
       <c r="K4" s="45" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="L4" s="47">
-        <v>425.38200000000001</v>
+        <v>172.386</v>
       </c>
       <c r="M4" s="48">
-        <v>332.8</v>
+        <v>117.8</v>
       </c>
       <c r="N4" s="49">
-        <v>4.6199999999999998E-2</v>
+        <v>8.2000000000000007E-3</v>
       </c>
       <c r="O4" s="50">
-        <v>2.77</v>
+        <v>0.49</v>
       </c>
       <c r="P4" s="45">
-        <v>134</v>
+        <v>97.9</v>
       </c>
       <c r="Q4" s="45">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R4" s="45">
-        <v>1300</v>
+        <v>1500</v>
       </c>
       <c r="S4" s="47">
-        <v>1.278</v>
+        <v>1.464</v>
       </c>
       <c r="T4" s="45">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="U4" s="49">
-        <v>1.6899999999999998E-2</v>
+        <v>2.4E-2</v>
       </c>
       <c r="V4" s="45" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="W4" s="45" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="X4" s="45" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="Y4" s="45" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="Z4" s="45" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="AA4" s="45" t="s">
         <v>38</v>
       </c>
       <c r="AB4" s="45" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="45">
+      <c r="A5" s="85">
         <v>3</v>
       </c>
       <c r="B5" s="46" t="s">
@@ -2679,52 +2682,52 @@
         <v>27</v>
       </c>
       <c r="F5" s="45">
-        <v>262825</v>
+        <v>262824</v>
       </c>
       <c r="G5" s="45" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="H5" s="45">
-        <v>1175</v>
+        <v>350</v>
       </c>
       <c r="I5" s="47">
-        <v>0.49199999999999999</v>
+        <v>0.63900000000000001</v>
       </c>
       <c r="J5" s="47">
-        <v>0.87</v>
+        <v>1.9019999999999999</v>
       </c>
       <c r="K5" s="45" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="L5" s="47">
-        <v>502.947</v>
+        <v>425.38200000000001</v>
       </c>
       <c r="M5" s="48">
-        <v>511.1</v>
+        <v>332.8</v>
       </c>
       <c r="N5" s="49">
-        <v>7.0999999999999994E-2</v>
+        <v>4.6199999999999998E-2</v>
       </c>
       <c r="O5" s="50">
-        <v>4.26</v>
+        <v>2.77</v>
       </c>
       <c r="P5" s="45">
-        <v>158.4</v>
+        <v>134</v>
       </c>
       <c r="Q5" s="45">
         <v>2</v>
       </c>
       <c r="R5" s="45">
-        <v>1050</v>
+        <v>1300</v>
       </c>
       <c r="S5" s="47">
-        <v>0.98399999999999999</v>
+        <v>1.278</v>
       </c>
       <c r="T5" s="45">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="U5" s="49">
-        <v>6.2899999999999998E-2</v>
+        <v>1.6899999999999998E-2</v>
       </c>
       <c r="V5" s="45" t="s">
         <v>28</v>
@@ -2745,96 +2748,262 @@
         <v>38</v>
       </c>
       <c r="AB5" s="45" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="85">
+        <v>4</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>460</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="61">
+        <v>46297</v>
+      </c>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45">
+        <v>262829</v>
+      </c>
+      <c r="G6" s="45">
+        <v>81</v>
+      </c>
+      <c r="H6" s="45">
+        <v>2000</v>
+      </c>
+      <c r="I6" s="47">
+        <v>0.54</v>
+      </c>
+      <c r="J6" s="47">
+        <v>1.61</v>
+      </c>
+      <c r="K6" s="45" t="s">
+        <v>497</v>
+      </c>
+      <c r="L6" s="47">
+        <v>1738.8</v>
+      </c>
+      <c r="M6" s="48">
+        <v>1610</v>
+      </c>
+      <c r="N6" s="49">
+        <v>0.22359999999999999</v>
+      </c>
+      <c r="O6" s="50">
+        <v>13.42</v>
+      </c>
+      <c r="P6" s="45">
+        <v>617.29999999999995</v>
+      </c>
+      <c r="Q6" s="45">
+        <v>2</v>
+      </c>
+      <c r="R6" s="45">
+        <v>1100</v>
+      </c>
+      <c r="S6" s="47">
+        <v>1.08</v>
+      </c>
+      <c r="T6" s="45">
+        <v>20</v>
+      </c>
+      <c r="U6" s="49">
+        <v>1.8200000000000001E-2</v>
+      </c>
+      <c r="V6" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="W6" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y6" s="45"/>
+      <c r="Z6" s="45"/>
+      <c r="AA6" s="45">
+        <v>3</v>
+      </c>
+      <c r="AB6" s="45" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="85">
+        <v>5</v>
+      </c>
+      <c r="B7" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>483</v>
+      </c>
+      <c r="E7" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="45">
+        <v>262825</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>482</v>
+      </c>
+      <c r="H7" s="45">
+        <v>1175</v>
+      </c>
+      <c r="I7" s="47">
+        <v>0.49199999999999999</v>
+      </c>
+      <c r="J7" s="47">
+        <v>0.87</v>
+      </c>
+      <c r="K7" s="45" t="s">
+        <v>481</v>
+      </c>
+      <c r="L7" s="47">
+        <v>502.947</v>
+      </c>
+      <c r="M7" s="48">
+        <v>511.1</v>
+      </c>
+      <c r="N7" s="49">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="O7" s="50">
+        <v>4.26</v>
+      </c>
+      <c r="P7" s="45">
+        <v>158.4</v>
+      </c>
+      <c r="Q7" s="45">
+        <v>2</v>
+      </c>
+      <c r="R7" s="45">
+        <v>1050</v>
+      </c>
+      <c r="S7" s="47">
+        <v>0.98399999999999999</v>
+      </c>
+      <c r="T7" s="45">
+        <v>66</v>
+      </c>
+      <c r="U7" s="49">
+        <v>6.2899999999999998E-2</v>
+      </c>
+      <c r="V7" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="45" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB7" s="45" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="52">
+    <row r="8" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="52">
         <v>1825</v>
       </c>
-      <c r="I6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="O6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" s="52">
+      <c r="I8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="52">
         <v>390.3</v>
       </c>
-      <c r="Q6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="R6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="S6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="T6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="U6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="V6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="W6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="X6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB6" s="52" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="Q8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="52" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
@@ -19123,6 +19292,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{320660EC-40AA-4456-8D33-C51008EBC785}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -19328,7 +19500,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="106">
         <v>1</v>
       </c>
@@ -19414,7 +19586,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="106">
         <v>2</v>
       </c>
@@ -19500,7 +19672,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="106">
         <v>3</v>
       </c>
@@ -19586,8 +19758,10 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="106"/>
+    <row r="6" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="106">
+        <v>4</v>
+      </c>
       <c r="B6" s="107" t="s">
         <v>472</v>
       </c>
@@ -19664,9 +19838,9 @@
         <v>494</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="106">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="107" t="s">
         <v>467</v>
@@ -19750,9 +19924,9 @@
         <v>476</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="106">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="107" t="s">
         <v>463</v>
@@ -19836,9 +20010,9 @@
         <v>475</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="106">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="107" t="s">
         <v>467</v>
@@ -19922,9 +20096,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="106">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="107" t="s">
         <v>472</v>
@@ -20008,9 +20182,9 @@
         <v>474</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="106">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" s="107" t="s">
         <v>463</v>
@@ -20094,9 +20268,9 @@
         <v>473</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="106">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" s="107" t="s">
         <v>107</v>
@@ -20180,9 +20354,9 @@
         <v>238</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="106">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" s="107" t="s">
         <v>472</v>
@@ -20266,9 +20440,9 @@
         <v>470</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="106">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" s="107" t="s">
         <v>467</v>
@@ -20352,9 +20526,9 @@
         <v>469</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="106">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" s="107" t="s">
         <v>463</v>
@@ -20438,9 +20612,9 @@
         <v>468</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="106">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" s="107" t="s">
         <v>467</v>
@@ -20524,9 +20698,9 @@
         <v>464</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="106">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B17" s="107" t="s">
         <v>463</v>
@@ -20610,9 +20784,9 @@
         <v>461</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="106">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B18" s="107" t="s">
         <v>107</v>
@@ -20696,9 +20870,9 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="106">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B19" s="107" t="s">
         <v>107</v>
@@ -20782,8 +20956,10 @@
         <v>237</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="112" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="106"/>
+    <row r="20" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="106">
+        <v>18</v>
+      </c>
       <c r="B20" s="107" t="s">
         <v>472</v>
       </c>
@@ -20982,8 +21158,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.44" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup scale="65" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 09:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5924DF-FB8B-4CC1-AE14-46BE4C075A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DE2B31-E4EA-434D-8476-F8206CD503D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1564,7 +1564,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1684,6 +1684,38 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1750,7 +1782,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2071,6 +2103,40 @@
     <xf numFmtId="14" fontId="14" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="24" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2307,17 +2373,17 @@
     <col min="5" max="5" width="8.21875" style="33" customWidth="1"/>
     <col min="6" max="6" width="7.5546875" style="33" customWidth="1"/>
     <col min="7" max="7" width="5.109375" style="33" customWidth="1"/>
-    <col min="8" max="8" width="5.5546875" style="33" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" style="33" customWidth="1"/>
+    <col min="8" max="8" width="8" style="33" customWidth="1"/>
+    <col min="9" max="9" width="10.77734375" style="33" customWidth="1"/>
     <col min="10" max="10" width="7.109375" style="33" customWidth="1"/>
-    <col min="11" max="11" width="17" style="33" customWidth="1"/>
+    <col min="11" max="11" width="21" style="33" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="7.77734375" style="33" customWidth="1"/>
     <col min="17" max="17" width="4.77734375" style="33" customWidth="1"/>
     <col min="18" max="18" width="7.33203125" style="33" customWidth="1"/>
-    <col min="19" max="19" width="6.109375" style="33" customWidth="1"/>
+    <col min="19" max="19" width="9.21875" style="33" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="22" max="22" width="7.88671875" style="33" customWidth="1"/>
@@ -2331,675 +2397,678 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="114" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="101" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="101" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="B1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="114" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="114" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="115" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="115" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="44" t="s">
+      <c r="E2" s="115" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="44" t="s">
+      <c r="F2" s="115" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="44" t="s">
+      <c r="G2" s="115" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="44" t="s">
+      <c r="H2" s="115" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="44" t="s">
+      <c r="I2" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="44" t="s">
+      <c r="J2" s="115" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="44" t="s">
+      <c r="K2" s="115" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="44" t="s">
+      <c r="L2" s="115" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="44" t="s">
+      <c r="M2" s="115" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="44" t="s">
+      <c r="N2" s="115" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="44" t="s">
+      <c r="O2" s="115" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="44" t="s">
+      <c r="P2" s="115" t="s">
         <v>13</v>
       </c>
-      <c r="Q2" s="44" t="s">
+      <c r="Q2" s="115" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="44" t="s">
+      <c r="R2" s="115" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="44" t="s">
+      <c r="S2" s="115" t="s">
         <v>16</v>
       </c>
-      <c r="T2" s="44" t="s">
+      <c r="T2" s="115" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="44" t="s">
+      <c r="U2" s="115" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="44" t="s">
+      <c r="V2" s="115" t="s">
         <v>19</v>
       </c>
-      <c r="W2" s="44" t="s">
+      <c r="W2" s="115" t="s">
         <v>20</v>
       </c>
-      <c r="X2" s="44" t="s">
+      <c r="X2" s="115" t="s">
         <v>21</v>
       </c>
-      <c r="Y2" s="44" t="s">
+      <c r="Y2" s="115" t="s">
         <v>22</v>
       </c>
-      <c r="Z2" s="44" t="s">
+      <c r="Z2" s="115" t="s">
         <v>23</v>
       </c>
-      <c r="AA2" s="44" t="s">
+      <c r="AA2" s="115" t="s">
         <v>24</v>
       </c>
-      <c r="AB2" s="44" t="s">
+      <c r="AB2" s="115" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:28" s="85" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="85">
+      <c r="A3" s="116">
         <v>1</v>
       </c>
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="116" t="s">
         <v>460</v>
       </c>
-      <c r="C3" s="85" t="s">
+      <c r="C3" s="116" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="86">
+      <c r="D3" s="117">
         <v>46297</v>
       </c>
-      <c r="F3" s="85">
+      <c r="E3" s="116"/>
+      <c r="F3" s="116">
         <v>262828</v>
       </c>
-      <c r="G3" s="85">
+      <c r="G3" s="116">
         <v>81</v>
       </c>
-      <c r="H3" s="85">
+      <c r="H3" s="116">
         <v>2000</v>
       </c>
-      <c r="I3" s="85">
+      <c r="I3" s="116">
         <v>0.39400000000000002</v>
       </c>
-      <c r="J3" s="85">
+      <c r="J3" s="116">
         <v>1.07</v>
       </c>
-      <c r="K3" s="85" t="s">
+      <c r="K3" s="116" t="s">
         <v>495</v>
       </c>
-      <c r="L3" s="85">
+      <c r="L3" s="116">
         <v>843.16</v>
       </c>
-      <c r="M3" s="85">
+      <c r="M3" s="116">
         <v>535</v>
       </c>
-      <c r="N3" s="85">
+      <c r="N3" s="116">
         <v>3.7199999999999997E-2</v>
       </c>
-      <c r="O3" s="85">
+      <c r="O3" s="116">
         <v>2.23</v>
       </c>
-      <c r="P3" s="85">
+      <c r="P3" s="116">
         <v>299.3</v>
       </c>
-      <c r="Q3" s="85">
+      <c r="Q3" s="116">
         <v>4</v>
       </c>
-      <c r="R3" s="85">
+      <c r="R3" s="116">
         <v>1600</v>
       </c>
-      <c r="S3" s="85">
+      <c r="S3" s="116">
         <v>1.5760000000000001</v>
       </c>
-      <c r="T3" s="85">
+      <c r="T3" s="116">
         <v>24</v>
       </c>
-      <c r="U3" s="85">
+      <c r="U3" s="116">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="V3" s="85" t="s">
+      <c r="V3" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="W3" s="85" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="85" t="s">
+      <c r="W3" s="116" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="AA3" s="85">
+      <c r="Y3" s="116"/>
+      <c r="Z3" s="116"/>
+      <c r="AA3" s="116">
         <v>2</v>
       </c>
-      <c r="AB3" s="85" t="s">
+      <c r="AB3" s="116" t="s">
         <v>496</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="85">
+      <c r="A4" s="116">
         <v>2</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="118" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="119" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="119" t="s">
         <v>483</v>
       </c>
-      <c r="E4" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="45">
+      <c r="E4" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="119">
         <v>262823</v>
       </c>
-      <c r="G4" s="45" t="s">
+      <c r="G4" s="119" t="s">
         <v>489</v>
       </c>
-      <c r="H4" s="45">
+      <c r="H4" s="119">
         <v>300</v>
       </c>
-      <c r="I4" s="47">
+      <c r="I4" s="120">
         <v>0.36599999999999999</v>
       </c>
-      <c r="J4" s="47">
+      <c r="J4" s="120">
         <v>1.57</v>
       </c>
-      <c r="K4" s="45" t="s">
+      <c r="K4" s="119" t="s">
         <v>488</v>
       </c>
-      <c r="L4" s="47">
+      <c r="L4" s="120">
         <v>172.386</v>
       </c>
-      <c r="M4" s="48">
+      <c r="M4" s="121">
         <v>117.8</v>
       </c>
-      <c r="N4" s="49">
+      <c r="N4" s="122">
         <v>8.2000000000000007E-3</v>
       </c>
-      <c r="O4" s="50">
+      <c r="O4" s="123">
         <v>0.49</v>
       </c>
-      <c r="P4" s="45">
+      <c r="P4" s="119">
         <v>97.9</v>
       </c>
-      <c r="Q4" s="45">
+      <c r="Q4" s="119">
         <v>4</v>
       </c>
-      <c r="R4" s="45">
+      <c r="R4" s="119">
         <v>1500</v>
       </c>
-      <c r="S4" s="47">
+      <c r="S4" s="120">
         <v>1.464</v>
       </c>
-      <c r="T4" s="45">
+      <c r="T4" s="119">
         <v>36</v>
       </c>
-      <c r="U4" s="49">
+      <c r="U4" s="122">
         <v>2.4E-2</v>
       </c>
-      <c r="V4" s="45" t="s">
+      <c r="V4" s="119" t="s">
         <v>34</v>
       </c>
-      <c r="W4" s="45" t="s">
+      <c r="W4" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="X4" s="45" t="s">
+      <c r="X4" s="119" t="s">
         <v>34</v>
       </c>
-      <c r="Y4" s="45" t="s">
+      <c r="Y4" s="119" t="s">
         <v>34</v>
       </c>
-      <c r="Z4" s="45" t="s">
+      <c r="Z4" s="119" t="s">
         <v>34</v>
       </c>
-      <c r="AA4" s="45" t="s">
+      <c r="AA4" s="119" t="s">
         <v>38</v>
       </c>
-      <c r="AB4" s="45" t="s">
+      <c r="AB4" s="119" t="s">
         <v>487</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="85">
+      <c r="A5" s="116">
         <v>3</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="118" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="119" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="119" t="s">
         <v>483</v>
       </c>
-      <c r="E5" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="45">
+      <c r="E5" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="119">
         <v>262824</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="G5" s="119" t="s">
         <v>486</v>
       </c>
-      <c r="H5" s="45">
+      <c r="H5" s="119">
         <v>350</v>
       </c>
-      <c r="I5" s="47">
+      <c r="I5" s="120">
         <v>0.63900000000000001</v>
       </c>
-      <c r="J5" s="47">
+      <c r="J5" s="120">
         <v>1.9019999999999999</v>
       </c>
-      <c r="K5" s="45" t="s">
+      <c r="K5" s="119" t="s">
         <v>485</v>
       </c>
-      <c r="L5" s="47">
+      <c r="L5" s="120">
         <v>425.38200000000001</v>
       </c>
-      <c r="M5" s="48">
+      <c r="M5" s="121">
         <v>332.8</v>
       </c>
-      <c r="N5" s="49">
+      <c r="N5" s="122">
         <v>4.6199999999999998E-2</v>
       </c>
-      <c r="O5" s="50">
+      <c r="O5" s="123">
         <v>2.77</v>
       </c>
-      <c r="P5" s="45">
+      <c r="P5" s="119">
         <v>134</v>
       </c>
-      <c r="Q5" s="45">
+      <c r="Q5" s="119">
         <v>2</v>
       </c>
-      <c r="R5" s="45">
+      <c r="R5" s="119">
         <v>1300</v>
       </c>
-      <c r="S5" s="47">
+      <c r="S5" s="120">
         <v>1.278</v>
       </c>
-      <c r="T5" s="45">
+      <c r="T5" s="119">
         <v>22</v>
       </c>
-      <c r="U5" s="49">
+      <c r="U5" s="122">
         <v>1.6899999999999998E-2</v>
       </c>
-      <c r="V5" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="45" t="s">
+      <c r="V5" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="119" t="s">
         <v>38</v>
       </c>
-      <c r="AB5" s="45" t="s">
+      <c r="AB5" s="119" t="s">
         <v>484</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="85">
+      <c r="A6" s="116">
         <v>4</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="118" t="s">
         <v>460</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="61">
+      <c r="D6" s="124">
         <v>46297</v>
       </c>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45">
+      <c r="E6" s="119"/>
+      <c r="F6" s="119">
         <v>262829</v>
       </c>
-      <c r="G6" s="45">
+      <c r="G6" s="119">
         <v>81</v>
       </c>
-      <c r="H6" s="45">
+      <c r="H6" s="119">
         <v>2000</v>
       </c>
-      <c r="I6" s="47">
+      <c r="I6" s="120">
         <v>0.54</v>
       </c>
-      <c r="J6" s="47">
+      <c r="J6" s="120">
         <v>1.61</v>
       </c>
-      <c r="K6" s="45" t="s">
+      <c r="K6" s="119" t="s">
         <v>497</v>
       </c>
-      <c r="L6" s="47">
+      <c r="L6" s="120">
         <v>1738.8</v>
       </c>
-      <c r="M6" s="48">
+      <c r="M6" s="121">
         <v>1610</v>
       </c>
-      <c r="N6" s="49">
+      <c r="N6" s="122">
         <v>0.22359999999999999</v>
       </c>
-      <c r="O6" s="50">
+      <c r="O6" s="123">
         <v>13.42</v>
       </c>
-      <c r="P6" s="45">
+      <c r="P6" s="119">
         <v>617.29999999999995</v>
       </c>
-      <c r="Q6" s="45">
+      <c r="Q6" s="119">
         <v>2</v>
       </c>
-      <c r="R6" s="45">
+      <c r="R6" s="119">
         <v>1100</v>
       </c>
-      <c r="S6" s="47">
+      <c r="S6" s="120">
         <v>1.08</v>
       </c>
-      <c r="T6" s="45">
+      <c r="T6" s="119">
         <v>20</v>
       </c>
-      <c r="U6" s="49">
+      <c r="U6" s="122">
         <v>1.8200000000000001E-2</v>
       </c>
-      <c r="V6" s="45" t="s">
+      <c r="V6" s="119" t="s">
         <v>29</v>
       </c>
-      <c r="W6" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="45" t="s">
+      <c r="W6" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="119" t="s">
         <v>29</v>
       </c>
-      <c r="Y6" s="45"/>
-      <c r="Z6" s="45"/>
-      <c r="AA6" s="45">
+      <c r="Y6" s="119"/>
+      <c r="Z6" s="119"/>
+      <c r="AA6" s="119">
         <v>3</v>
       </c>
-      <c r="AB6" s="45" t="s">
+      <c r="AB6" s="119" t="s">
         <v>498</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="85">
+      <c r="A7" s="116">
         <v>5</v>
       </c>
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="118" t="s">
         <v>126</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="119" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="119" t="s">
         <v>483</v>
       </c>
-      <c r="E7" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="45">
+      <c r="E7" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="119">
         <v>262825</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="119" t="s">
         <v>482</v>
       </c>
-      <c r="H7" s="45">
+      <c r="H7" s="119">
         <v>1175</v>
       </c>
-      <c r="I7" s="47">
+      <c r="I7" s="120">
         <v>0.49199999999999999</v>
       </c>
-      <c r="J7" s="47">
+      <c r="J7" s="120">
         <v>0.87</v>
       </c>
-      <c r="K7" s="45" t="s">
+      <c r="K7" s="119" t="s">
         <v>481</v>
       </c>
-      <c r="L7" s="47">
+      <c r="L7" s="120">
         <v>502.947</v>
       </c>
-      <c r="M7" s="48">
+      <c r="M7" s="121">
         <v>511.1</v>
       </c>
-      <c r="N7" s="49">
+      <c r="N7" s="122">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="O7" s="50">
+      <c r="O7" s="123">
         <v>4.26</v>
       </c>
-      <c r="P7" s="45">
+      <c r="P7" s="119">
         <v>158.4</v>
       </c>
-      <c r="Q7" s="45">
+      <c r="Q7" s="119">
         <v>2</v>
       </c>
-      <c r="R7" s="45">
+      <c r="R7" s="119">
         <v>1050</v>
       </c>
-      <c r="S7" s="47">
+      <c r="S7" s="120">
         <v>0.98399999999999999</v>
       </c>
-      <c r="T7" s="45">
+      <c r="T7" s="119">
         <v>66</v>
       </c>
-      <c r="U7" s="49">
+      <c r="U7" s="122">
         <v>6.2899999999999998E-2</v>
       </c>
-      <c r="V7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="45" t="s">
+      <c r="V7" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="119" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="119" t="s">
         <v>38</v>
       </c>
-      <c r="AB7" s="45" t="s">
+      <c r="AB7" s="119" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="52">
+      <c r="A8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="125">
         <v>1825</v>
       </c>
-      <c r="I8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="N8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="O8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="52">
+      <c r="I8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="125">
         <v>390.3</v>
       </c>
-      <c r="Q8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="R8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="T8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="V8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="W8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="X8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB8" s="52" t="s">
+      <c r="Q8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="125" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3009,7 +3078,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="1.79" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="90" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="78" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 10:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADAC36BF-4518-4A63-8056-618153600ACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60EB9E73-9385-4E0F-9ADD-195716CC1BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1246" sheetId="176" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4790" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4868" uniqueCount="527">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1587,6 +1587,57 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - ABAPEL COMERCIO DE EMBALAGENS LTDA  —  OF: 001246</t>
+  </si>
+  <si>
+    <t>1514x2251</t>
+  </si>
+  <si>
+    <t>412x670x412</t>
+  </si>
+  <si>
+    <t>1790</t>
+  </si>
+  <si>
+    <t>1336x1264</t>
+  </si>
+  <si>
+    <t>313x58x574x58x313</t>
+  </si>
+  <si>
+    <t>1797</t>
+  </si>
+  <si>
+    <t>620x2387</t>
+  </si>
+  <si>
+    <t>203x194x203</t>
+  </si>
+  <si>
+    <t>1788</t>
+  </si>
+  <si>
+    <t>1130x2323</t>
+  </si>
+  <si>
+    <t>278x554x278</t>
+  </si>
+  <si>
+    <t>1786</t>
+  </si>
+  <si>
+    <t>1013x1901</t>
+  </si>
+  <si>
+    <t>97x799x97</t>
+  </si>
+  <si>
+    <t>1793</t>
+  </si>
+  <si>
+    <t>1020x3420</t>
+  </si>
+  <si>
+    <t>1787</t>
   </si>
 </sst>
 </file>
@@ -1823,7 +1874,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2203,6 +2254,24 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -23821,7 +23890,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF841B48-E833-4DBA-8A4F-DEEF6290C316}">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="33" customWidth="1"/>
@@ -24026,863 +24095,1381 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="41">
+    <row r="3" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="45">
         <v>1</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E3" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="41">
+      <c r="E3" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="45">
         <v>262736</v>
       </c>
-      <c r="G3" s="41" t="s">
+      <c r="G3" s="45" t="s">
         <v>389</v>
       </c>
-      <c r="H3" s="41">
+      <c r="H3" s="45">
         <v>150</v>
       </c>
-      <c r="I3" s="42">
+      <c r="I3" s="47">
         <v>1.498</v>
       </c>
-      <c r="J3" s="42">
+      <c r="J3" s="47">
         <v>1.6830000000000001</v>
       </c>
-      <c r="K3" s="41" t="s">
+      <c r="K3" s="45" t="s">
         <v>395</v>
       </c>
-      <c r="L3" s="38">
+      <c r="L3" s="47">
         <v>378.17</v>
       </c>
-      <c r="M3" s="40">
+      <c r="M3" s="48">
         <v>252.5</v>
       </c>
-      <c r="N3" s="37">
+      <c r="N3" s="49">
         <v>7.0099999999999996E-2</v>
       </c>
-      <c r="O3" s="39">
+      <c r="O3" s="50">
         <v>4.21</v>
       </c>
-      <c r="P3" s="36">
+      <c r="P3" s="45">
         <v>203.5</v>
       </c>
-      <c r="Q3" s="36">
+      <c r="Q3" s="45">
         <v>1</v>
       </c>
-      <c r="R3" s="36">
+      <c r="R3" s="45">
         <v>1550</v>
       </c>
-      <c r="S3" s="38">
+      <c r="S3" s="47">
         <v>1.498</v>
       </c>
-      <c r="T3" s="36">
+      <c r="T3" s="45">
         <v>52</v>
       </c>
-      <c r="U3" s="37">
+      <c r="U3" s="49">
         <v>3.3500000000000002E-2</v>
       </c>
-      <c r="V3" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="36" t="s">
+      <c r="V3" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="36" t="s">
+      <c r="X3" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AB3" s="36" t="s">
+      <c r="AB3" s="45" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="41">
+    <row r="4" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="45">
         <v>2</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E4" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="41">
+      <c r="E4" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="45">
         <v>262735</v>
       </c>
-      <c r="G4" s="41" t="s">
+      <c r="G4" s="45" t="s">
         <v>389</v>
       </c>
-      <c r="H4" s="41">
+      <c r="H4" s="45">
         <v>150</v>
       </c>
-      <c r="I4" s="42">
+      <c r="I4" s="47">
         <v>1.488</v>
       </c>
-      <c r="J4" s="42">
+      <c r="J4" s="47">
         <v>2.0830000000000002</v>
       </c>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="45" t="s">
         <v>393</v>
       </c>
-      <c r="L4" s="38">
+      <c r="L4" s="47">
         <v>464.92599999999999</v>
       </c>
-      <c r="M4" s="40">
+      <c r="M4" s="48">
         <v>312.5</v>
       </c>
-      <c r="N4" s="37">
+      <c r="N4" s="49">
         <v>8.6800000000000002E-2</v>
       </c>
-      <c r="O4" s="39">
+      <c r="O4" s="50">
         <v>5.21</v>
       </c>
-      <c r="P4" s="36">
+      <c r="P4" s="45">
         <v>250.1</v>
       </c>
-      <c r="Q4" s="36">
+      <c r="Q4" s="45">
         <v>1</v>
       </c>
-      <c r="R4" s="36">
+      <c r="R4" s="45">
         <v>1550</v>
       </c>
-      <c r="S4" s="38">
+      <c r="S4" s="47">
         <v>1.488</v>
       </c>
-      <c r="T4" s="36">
+      <c r="T4" s="45">
         <v>62</v>
       </c>
-      <c r="U4" s="37">
+      <c r="U4" s="49">
         <v>0.04</v>
       </c>
-      <c r="V4" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="36" t="s">
+      <c r="V4" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="36" t="s">
+      <c r="X4" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AB4" s="36" t="s">
+      <c r="AB4" s="45" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="41">
+    <row r="5" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="45">
         <v>3</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="140" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="135" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="135" t="s">
+        <v>483</v>
+      </c>
+      <c r="E5" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="135">
+        <v>262837</v>
+      </c>
+      <c r="G5" s="135" t="s">
+        <v>512</v>
+      </c>
+      <c r="H5" s="135">
+        <v>140</v>
+      </c>
+      <c r="I5" s="137">
+        <v>1.494</v>
+      </c>
+      <c r="J5" s="137">
+        <v>2.2309999999999999</v>
+      </c>
+      <c r="K5" s="135" t="s">
+        <v>511</v>
+      </c>
+      <c r="L5" s="137">
+        <v>466.63600000000002</v>
+      </c>
+      <c r="M5" s="139">
+        <v>312.3</v>
+      </c>
+      <c r="N5" s="136">
+        <v>8.6800000000000002E-2</v>
+      </c>
+      <c r="O5" s="138">
+        <v>5.21</v>
+      </c>
+      <c r="P5" s="135">
+        <v>265</v>
+      </c>
+      <c r="Q5" s="135">
+        <v>1</v>
+      </c>
+      <c r="R5" s="135">
+        <v>1550</v>
+      </c>
+      <c r="S5" s="137">
+        <v>1.494</v>
+      </c>
+      <c r="T5" s="135">
+        <v>56</v>
+      </c>
+      <c r="U5" s="136">
+        <v>3.61E-2</v>
+      </c>
+      <c r="V5" s="135" t="s">
+        <v>34</v>
+      </c>
+      <c r="W5" s="135" t="s">
+        <v>39</v>
+      </c>
+      <c r="X5" s="135" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y5" s="135" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z5" s="135" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA5" s="135" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB5" s="135" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="45">
+        <v>4</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D6" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E5" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="41">
+      <c r="E6" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="45">
         <v>262733</v>
       </c>
-      <c r="G5" s="41" t="s">
+      <c r="G6" s="45" t="s">
         <v>389</v>
       </c>
-      <c r="H5" s="41">
+      <c r="H6" s="45">
         <v>150</v>
       </c>
-      <c r="I5" s="42">
+      <c r="I6" s="47">
         <v>1.478</v>
       </c>
-      <c r="J5" s="42">
+      <c r="J6" s="47">
         <v>2.0030000000000001</v>
       </c>
-      <c r="K5" s="41" t="s">
+      <c r="K6" s="45" t="s">
         <v>391</v>
       </c>
-      <c r="L5" s="38">
+      <c r="L6" s="47">
         <v>444.065</v>
       </c>
-      <c r="M5" s="40">
+      <c r="M6" s="48">
         <v>300.5</v>
       </c>
-      <c r="N5" s="37">
+      <c r="N6" s="49">
         <v>8.3500000000000005E-2</v>
       </c>
-      <c r="O5" s="39">
+      <c r="O6" s="50">
         <v>5.01</v>
       </c>
-      <c r="P5" s="36">
+      <c r="P6" s="45">
         <v>238.9</v>
       </c>
-      <c r="Q5" s="36">
+      <c r="Q6" s="45">
         <v>1</v>
       </c>
-      <c r="R5" s="36">
+      <c r="R6" s="45">
         <v>1500</v>
       </c>
-      <c r="S5" s="38">
+      <c r="S6" s="47">
         <v>1.478</v>
       </c>
-      <c r="T5" s="36">
+      <c r="T6" s="45">
         <v>22</v>
       </c>
-      <c r="U5" s="37">
+      <c r="U6" s="49">
         <v>1.47E-2</v>
       </c>
-      <c r="V5" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="36" t="s">
+      <c r="V6" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="36" t="s">
+      <c r="X6" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AB5" s="36" t="s">
+      <c r="AB6" s="45" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="41">
-        <v>4</v>
-      </c>
-      <c r="B6" s="43" t="s">
+    <row r="7" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="45">
+        <v>5</v>
+      </c>
+      <c r="B7" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C7" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D7" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E6" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="41">
+      <c r="E7" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="45">
         <v>262734</v>
       </c>
-      <c r="G6" s="41" t="s">
+      <c r="G7" s="45" t="s">
         <v>389</v>
       </c>
-      <c r="H6" s="41">
+      <c r="H7" s="45">
         <v>150</v>
       </c>
-      <c r="I6" s="42">
+      <c r="I7" s="47">
         <v>1.3380000000000001</v>
       </c>
-      <c r="J6" s="42">
+      <c r="J7" s="47">
         <v>2.0830000000000002</v>
       </c>
-      <c r="K6" s="41" t="s">
+      <c r="K7" s="45" t="s">
         <v>388</v>
       </c>
-      <c r="L6" s="38">
+      <c r="L7" s="47">
         <v>418.05799999999999</v>
       </c>
-      <c r="M6" s="40">
+      <c r="M7" s="48">
         <v>312.5</v>
       </c>
-      <c r="N6" s="37">
+      <c r="N7" s="49">
         <v>8.6800000000000002E-2</v>
       </c>
-      <c r="O6" s="39">
+      <c r="O7" s="50">
         <v>5.21</v>
       </c>
-      <c r="P6" s="36">
+      <c r="P7" s="45">
         <v>224.9</v>
       </c>
-      <c r="Q6" s="36">
+      <c r="Q7" s="45">
         <v>1</v>
       </c>
-      <c r="R6" s="36">
+      <c r="R7" s="45">
         <v>1400</v>
       </c>
-      <c r="S6" s="38">
+      <c r="S7" s="47">
         <v>1.3380000000000001</v>
       </c>
-      <c r="T6" s="36">
+      <c r="T7" s="45">
         <v>62</v>
       </c>
-      <c r="U6" s="37">
+      <c r="U7" s="49">
         <v>4.4299999999999999E-2</v>
       </c>
-      <c r="V6" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="36" t="s">
+      <c r="V7" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="36" t="s">
+      <c r="X7" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AB6" s="36" t="s">
+      <c r="AB7" s="45" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="41">
-        <v>5</v>
-      </c>
-      <c r="B7" s="43" t="s">
+    <row r="8" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="45">
+        <v>6</v>
+      </c>
+      <c r="B8" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C8" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D8" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E7" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="41">
+      <c r="E8" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="45">
         <v>262731</v>
       </c>
-      <c r="G7" s="41" t="s">
+      <c r="G8" s="45" t="s">
         <v>386</v>
       </c>
-      <c r="H7" s="41">
+      <c r="H8" s="45">
         <v>1250</v>
       </c>
-      <c r="I7" s="42">
+      <c r="I8" s="47">
         <v>0.75</v>
       </c>
-      <c r="J7" s="42">
+      <c r="J8" s="47">
         <v>0.75</v>
       </c>
-      <c r="K7" s="41" t="s">
+      <c r="K8" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="L7" s="38">
+      <c r="L8" s="47">
         <v>703.125</v>
       </c>
-      <c r="M7" s="40">
+      <c r="M8" s="48">
         <v>468.8</v>
       </c>
-      <c r="N7" s="37">
+      <c r="N8" s="49">
         <v>6.5100000000000005E-2</v>
       </c>
-      <c r="O7" s="39">
+      <c r="O8" s="50">
         <v>3.91</v>
       </c>
-      <c r="P7" s="36">
+      <c r="P8" s="45">
         <v>309.39999999999998</v>
       </c>
-      <c r="Q7" s="36">
+      <c r="Q8" s="45">
         <v>2</v>
       </c>
-      <c r="R7" s="36">
+      <c r="R8" s="45">
         <v>1550</v>
       </c>
-      <c r="S7" s="38">
+      <c r="S8" s="47">
         <v>1.5</v>
       </c>
-      <c r="T7" s="36">
+      <c r="T8" s="45">
         <v>50</v>
       </c>
-      <c r="U7" s="37">
+      <c r="U8" s="49">
         <v>3.2300000000000002E-2</v>
       </c>
-      <c r="V7" s="36" t="s">
+      <c r="V8" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="W7" s="36" t="s">
+      <c r="W8" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="X7" s="36" t="s">
+      <c r="X8" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="Y7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="36" t="s">
+      <c r="Y8" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="36" t="s">
+      <c r="AB8" s="45" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="41">
-        <v>6</v>
-      </c>
-      <c r="B8" s="43" t="s">
+    <row r="9" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="45">
+        <v>7</v>
+      </c>
+      <c r="B9" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C9" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D9" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E8" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="41">
+      <c r="E9" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="45">
         <v>262732</v>
       </c>
-      <c r="G8" s="41" t="s">
+      <c r="G9" s="45" t="s">
         <v>386</v>
       </c>
-      <c r="H8" s="41">
+      <c r="H9" s="45">
         <v>1500</v>
       </c>
-      <c r="I8" s="42">
+      <c r="I9" s="47">
         <v>0.75</v>
       </c>
-      <c r="J8" s="42">
+      <c r="J9" s="47">
         <v>0.75</v>
       </c>
-      <c r="K8" s="41" t="s">
+      <c r="K9" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="L8" s="38">
+      <c r="L9" s="47">
         <v>843.75</v>
       </c>
-      <c r="M8" s="40">
+      <c r="M9" s="48">
         <v>562.5</v>
       </c>
-      <c r="N8" s="37">
+      <c r="N9" s="49">
         <v>7.8100000000000003E-2</v>
       </c>
-      <c r="O8" s="39">
+      <c r="O9" s="50">
         <v>4.6900000000000004</v>
       </c>
-      <c r="P8" s="36">
+      <c r="P9" s="45">
         <v>371.3</v>
       </c>
-      <c r="Q8" s="36">
+      <c r="Q9" s="45">
         <v>2</v>
       </c>
-      <c r="R8" s="36">
+      <c r="R9" s="45">
         <v>1550</v>
       </c>
-      <c r="S8" s="38">
+      <c r="S9" s="47">
         <v>1.5</v>
       </c>
-      <c r="T8" s="36">
+      <c r="T9" s="45">
         <v>50</v>
       </c>
-      <c r="U8" s="37">
+      <c r="U9" s="49">
         <v>3.2300000000000002E-2</v>
       </c>
-      <c r="V8" s="36" t="s">
+      <c r="V9" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="W8" s="36" t="s">
+      <c r="W9" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="X8" s="36" t="s">
+      <c r="X9" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="Y8" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="36" t="s">
+      <c r="Y9" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="AB8" s="36" t="s">
+      <c r="AB9" s="45" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A9" s="41">
-        <v>7</v>
-      </c>
-      <c r="B9" s="43" t="s">
+    <row r="10" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="45">
+        <v>8</v>
+      </c>
+      <c r="B10" s="140" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C10" s="135" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D10" s="135" t="s">
+        <v>483</v>
+      </c>
+      <c r="E10" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="135">
+        <v>262839</v>
+      </c>
+      <c r="G10" s="135" t="s">
+        <v>515</v>
+      </c>
+      <c r="H10" s="135">
+        <v>150</v>
+      </c>
+      <c r="I10" s="137">
+        <v>1.3160000000000001</v>
+      </c>
+      <c r="J10" s="137">
+        <v>1.244</v>
+      </c>
+      <c r="K10" s="135" t="s">
+        <v>514</v>
+      </c>
+      <c r="L10" s="137">
+        <v>245.566</v>
+      </c>
+      <c r="M10" s="139">
+        <v>186.6</v>
+      </c>
+      <c r="N10" s="136">
+        <v>5.1799999999999999E-2</v>
+      </c>
+      <c r="O10" s="138">
+        <v>3.11</v>
+      </c>
+      <c r="P10" s="135">
+        <v>77.400000000000006</v>
+      </c>
+      <c r="Q10" s="135">
+        <v>1</v>
+      </c>
+      <c r="R10" s="135">
+        <v>1350</v>
+      </c>
+      <c r="S10" s="137">
+        <v>1.3160000000000001</v>
+      </c>
+      <c r="T10" s="135">
+        <v>34</v>
+      </c>
+      <c r="U10" s="136">
+        <v>2.52E-2</v>
+      </c>
+      <c r="V10" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="135" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB10" s="135" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="45">
+        <v>9</v>
+      </c>
+      <c r="B11" s="140" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="135" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="135" t="s">
+        <v>483</v>
+      </c>
+      <c r="E11" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="135">
+        <v>262835</v>
+      </c>
+      <c r="G11" s="135" t="s">
+        <v>518</v>
+      </c>
+      <c r="H11" s="135">
+        <v>500</v>
+      </c>
+      <c r="I11" s="137">
+        <v>0.6</v>
+      </c>
+      <c r="J11" s="137">
+        <v>2.367</v>
+      </c>
+      <c r="K11" s="135" t="s">
+        <v>517</v>
+      </c>
+      <c r="L11" s="137">
+        <v>710.1</v>
+      </c>
+      <c r="M11" s="139">
+        <v>591.79999999999995</v>
+      </c>
+      <c r="N11" s="136">
+        <v>8.2199999999999995E-2</v>
+      </c>
+      <c r="O11" s="138">
+        <v>4.93</v>
+      </c>
+      <c r="P11" s="135">
+        <v>223.7</v>
+      </c>
+      <c r="Q11" s="135">
+        <v>2</v>
+      </c>
+      <c r="R11" s="135">
+        <v>1250</v>
+      </c>
+      <c r="S11" s="137">
+        <v>1.2</v>
+      </c>
+      <c r="T11" s="135">
+        <v>50</v>
+      </c>
+      <c r="U11" s="136">
+        <v>0.04</v>
+      </c>
+      <c r="V11" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="135" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB11" s="135" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="45">
+        <v>10</v>
+      </c>
+      <c r="B12" s="140" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="135" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="135" t="s">
+        <v>483</v>
+      </c>
+      <c r="E12" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="135">
+        <v>262834</v>
+      </c>
+      <c r="G12" s="135" t="s">
+        <v>521</v>
+      </c>
+      <c r="H12" s="135">
+        <v>200</v>
+      </c>
+      <c r="I12" s="137">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="J12" s="137">
+        <v>2.3029999999999999</v>
+      </c>
+      <c r="K12" s="135" t="s">
+        <v>520</v>
+      </c>
+      <c r="L12" s="137">
+        <v>511.26600000000002</v>
+      </c>
+      <c r="M12" s="139">
+        <v>460.6</v>
+      </c>
+      <c r="N12" s="136">
+        <v>0.12790000000000001</v>
+      </c>
+      <c r="O12" s="138">
+        <v>7.68</v>
+      </c>
+      <c r="P12" s="135">
+        <v>161</v>
+      </c>
+      <c r="Q12" s="135">
+        <v>1</v>
+      </c>
+      <c r="R12" s="135">
+        <v>1150</v>
+      </c>
+      <c r="S12" s="137">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="T12" s="135">
+        <v>40</v>
+      </c>
+      <c r="U12" s="136">
+        <v>3.4799999999999998E-2</v>
+      </c>
+      <c r="V12" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="135" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB12" s="135" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="45">
+        <v>11</v>
+      </c>
+      <c r="B13" s="140" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="135" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="135" t="s">
+        <v>483</v>
+      </c>
+      <c r="E13" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="135">
+        <v>262838</v>
+      </c>
+      <c r="G13" s="135" t="s">
+        <v>524</v>
+      </c>
+      <c r="H13" s="135">
+        <v>1200</v>
+      </c>
+      <c r="I13" s="137">
+        <v>0.99299999999999999</v>
+      </c>
+      <c r="J13" s="137">
+        <v>0.627</v>
+      </c>
+      <c r="K13" s="135" t="s">
+        <v>523</v>
+      </c>
+      <c r="L13" s="137">
+        <v>747.13300000000004</v>
+      </c>
+      <c r="M13" s="139">
+        <v>752.4</v>
+      </c>
+      <c r="N13" s="136">
+        <v>0.20899999999999999</v>
+      </c>
+      <c r="O13" s="138">
+        <v>12.54</v>
+      </c>
+      <c r="P13" s="135">
+        <v>235.3</v>
+      </c>
+      <c r="Q13" s="135">
+        <v>1</v>
+      </c>
+      <c r="R13" s="135">
+        <v>1050</v>
+      </c>
+      <c r="S13" s="137">
+        <v>0.99299999999999999</v>
+      </c>
+      <c r="T13" s="135">
+        <v>57</v>
+      </c>
+      <c r="U13" s="136">
+        <v>5.4300000000000001E-2</v>
+      </c>
+      <c r="V13" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="135" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB13" s="135" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="45">
+        <v>12</v>
+      </c>
+      <c r="B14" s="140" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="135" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="135" t="s">
+        <v>483</v>
+      </c>
+      <c r="E14" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="135">
+        <v>262836</v>
+      </c>
+      <c r="G14" s="135" t="s">
+        <v>526</v>
+      </c>
+      <c r="H14" s="135">
+        <v>800</v>
+      </c>
+      <c r="I14" s="137">
+        <v>1</v>
+      </c>
+      <c r="J14" s="137">
+        <v>3.4</v>
+      </c>
+      <c r="K14" s="135" t="s">
+        <v>33</v>
+      </c>
+      <c r="L14" s="137">
+        <v>2720</v>
+      </c>
+      <c r="M14" s="139">
+        <v>2720</v>
+      </c>
+      <c r="N14" s="136">
+        <v>0.75560000000000005</v>
+      </c>
+      <c r="O14" s="138">
+        <v>45.33</v>
+      </c>
+      <c r="P14" s="135">
+        <v>856.8</v>
+      </c>
+      <c r="Q14" s="135">
+        <v>1</v>
+      </c>
+      <c r="R14" s="135">
+        <v>1050</v>
+      </c>
+      <c r="S14" s="137">
+        <v>1</v>
+      </c>
+      <c r="T14" s="135">
+        <v>50</v>
+      </c>
+      <c r="U14" s="136">
+        <v>4.7600000000000003E-2</v>
+      </c>
+      <c r="V14" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="135" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB14" s="135" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="45">
+        <v>13</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E9" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="41">
+      <c r="E15" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="45">
         <v>262737</v>
       </c>
-      <c r="G9" s="41" t="s">
+      <c r="G15" s="45" t="s">
         <v>379</v>
       </c>
-      <c r="H9" s="41">
+      <c r="H15" s="45">
         <v>600</v>
       </c>
-      <c r="I9" s="42">
+      <c r="I15" s="47">
         <v>0.47</v>
       </c>
-      <c r="J9" s="42">
+      <c r="J15" s="47">
         <v>1.7869999999999999</v>
       </c>
-      <c r="K9" s="41" t="s">
+      <c r="K15" s="45" t="s">
         <v>384</v>
       </c>
-      <c r="L9" s="38">
+      <c r="L15" s="47">
         <v>503.93400000000003</v>
       </c>
-      <c r="M9" s="40">
+      <c r="M15" s="48">
         <v>536.1</v>
       </c>
-      <c r="N9" s="37">
+      <c r="N15" s="49">
         <v>7.4499999999999997E-2</v>
       </c>
-      <c r="O9" s="39">
+      <c r="O15" s="50">
         <v>4.47</v>
       </c>
-      <c r="P9" s="36">
+      <c r="P15" s="45">
         <v>158.69999999999999</v>
       </c>
-      <c r="Q9" s="36">
+      <c r="Q15" s="45">
         <v>2</v>
       </c>
-      <c r="R9" s="36">
+      <c r="R15" s="45">
         <v>1000</v>
       </c>
-      <c r="S9" s="38">
+      <c r="S15" s="47">
         <v>0.94</v>
       </c>
-      <c r="T9" s="36">
+      <c r="T15" s="45">
         <v>60</v>
       </c>
-      <c r="U9" s="37">
+      <c r="U15" s="49">
         <v>0.06</v>
       </c>
-      <c r="V9" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="36" t="s">
+      <c r="V15" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AB9" s="36" t="s">
+      <c r="AB15" s="45" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A10" s="41">
-        <v>8</v>
-      </c>
-      <c r="B10" s="43" t="s">
+    <row r="16" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="45">
+        <v>14</v>
+      </c>
+      <c r="B16" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C16" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D16" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E10" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="41">
+      <c r="E16" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="45">
         <v>262739</v>
       </c>
-      <c r="G10" s="41" t="s">
+      <c r="G16" s="45" t="s">
         <v>379</v>
       </c>
-      <c r="H10" s="41">
+      <c r="H16" s="45">
         <v>300</v>
       </c>
-      <c r="I10" s="42">
+      <c r="I16" s="47">
         <v>0.86</v>
       </c>
-      <c r="J10" s="42">
+      <c r="J16" s="47">
         <v>1.8029999999999999</v>
       </c>
-      <c r="K10" s="41" t="s">
+      <c r="K16" s="45" t="s">
         <v>382</v>
       </c>
-      <c r="L10" s="38">
+      <c r="L16" s="47">
         <v>465.17399999999998</v>
       </c>
-      <c r="M10" s="40">
+      <c r="M16" s="48">
         <v>540.9</v>
       </c>
-      <c r="N10" s="37">
+      <c r="N16" s="49">
         <v>0.1502</v>
       </c>
-      <c r="O10" s="39">
+      <c r="O16" s="50">
         <v>9.01</v>
       </c>
-      <c r="P10" s="36">
+      <c r="P16" s="45">
         <v>146.5</v>
       </c>
-      <c r="Q10" s="36">
+      <c r="Q16" s="45">
         <v>1</v>
       </c>
-      <c r="R10" s="36">
+      <c r="R16" s="45">
         <v>900</v>
       </c>
-      <c r="S10" s="38">
+      <c r="S16" s="47">
         <v>0.86</v>
       </c>
-      <c r="T10" s="36">
+      <c r="T16" s="45">
         <v>40</v>
       </c>
-      <c r="U10" s="37">
+      <c r="U16" s="49">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="V10" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="36" t="s">
+      <c r="V16" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y16" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z16" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA16" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AB10" s="36" t="s">
+      <c r="AB16" s="45" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" s="41">
-        <v>9</v>
-      </c>
-      <c r="B11" s="43" t="s">
+    <row r="17" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="45">
+        <v>15</v>
+      </c>
+      <c r="B17" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C11" s="41" t="s">
+      <c r="C17" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D17" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="E11" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="41">
+      <c r="E17" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="45">
         <v>262738</v>
       </c>
-      <c r="G11" s="41" t="s">
+      <c r="G17" s="45" t="s">
         <v>379</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H17" s="45">
         <v>600</v>
       </c>
-      <c r="I11" s="42">
+      <c r="I17" s="47">
         <v>0.39</v>
       </c>
-      <c r="J11" s="42">
+      <c r="J17" s="47">
         <v>1.7829999999999999</v>
       </c>
-      <c r="K11" s="41" t="s">
+      <c r="K17" s="45" t="s">
         <v>378</v>
       </c>
-      <c r="L11" s="38">
+      <c r="L17" s="47">
         <v>417.22199999999998</v>
       </c>
-      <c r="M11" s="40">
+      <c r="M17" s="48">
         <v>534.9</v>
       </c>
-      <c r="N11" s="37">
+      <c r="N17" s="49">
         <v>7.4300000000000005E-2</v>
       </c>
-      <c r="O11" s="39">
+      <c r="O17" s="50">
         <v>4.46</v>
       </c>
-      <c r="P11" s="36">
+      <c r="P17" s="45">
         <v>131.4</v>
       </c>
-      <c r="Q11" s="36">
+      <c r="Q17" s="45">
         <v>2</v>
       </c>
-      <c r="R11" s="36">
+      <c r="R17" s="45">
         <v>800</v>
       </c>
-      <c r="S11" s="38">
+      <c r="S17" s="47">
         <v>0.78</v>
       </c>
-      <c r="T11" s="36">
+      <c r="T17" s="45">
         <v>20</v>
       </c>
-      <c r="U11" s="37">
+      <c r="U17" s="49">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="V11" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="36" t="s">
+      <c r="V17" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W17" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="X17" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y17" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AB11" s="36" t="s">
+      <c r="AB17" s="45" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="35">
-        <v>4850</v>
-      </c>
-      <c r="I12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="34">
-        <v>2034.7</v>
-      </c>
-      <c r="Q12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="34" t="s">
+    <row r="18" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="H18" s="52">
+        <f>SUM(H3:H17)</f>
+        <v>7840</v>
+      </c>
+      <c r="I18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="K18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="L18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="M18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="O18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="P18" s="52">
+        <f>SUM(P3:P17)</f>
+        <v>3853.9</v>
+      </c>
+      <c r="Q18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="R18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="S18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="T18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="U18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="V18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="W18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="X18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB18" s="52" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 11:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6B7BC6-A1B1-4636-B5B3-31D297B256C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697F74AC-DFA1-4F14-9FDE-B99CC077E4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1249" sheetId="178" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="HARMONY EMBALAGENS 1231 P" sheetId="168" r:id="rId10"/>
     <sheet name="RM Embalagens P" sheetId="166" r:id="rId11"/>
     <sheet name="PCBOX EMBALAGENS LTDA 1222 P" sheetId="164" r:id="rId12"/>
-    <sheet name="FORBOX 1220" sheetId="163" r:id="rId13"/>
+    <sheet name="FORBOX 1220 P" sheetId="163" r:id="rId13"/>
     <sheet name="HARMONY EMBALAGENS 1217 P" sheetId="162" r:id="rId14"/>
     <sheet name="Z4A EMBALAGENS LTDA 1216" sheetId="161" r:id="rId15"/>
     <sheet name="ABAPEL 1213" sheetId="159" r:id="rId16"/>
@@ -9178,7 +9178,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD2CB328-92D9-4132-AB19-3AEA902CFC6F}">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="33" customWidth="1"/>
@@ -9209,88 +9209,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="101" t="s">
         <v>278</v>
       </c>
-      <c r="B1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="102" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="102" t="s">
+      <c r="B1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="101" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="101" t="s">
         <v>27</v>
       </c>
     </row>
@@ -9380,7 +9380,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="41">
         <v>1</v>
       </c>
@@ -9466,7 +9466,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="41">
         <v>2</v>
       </c>
@@ -9552,7 +9552,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="41">
         <v>3</v>
       </c>
@@ -9638,7 +9638,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="41">
         <v>4</v>
       </c>
@@ -9722,7 +9722,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="35" t="s">
         <v>27</v>
       </c>
@@ -9808,11 +9808,13 @@
         <v>27</v>
       </c>
     </row>
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 11:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697F74AC-DFA1-4F14-9FDE-B99CC077E4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AF219F-4326-4B4A-891D-89F187082164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1249" sheetId="178" r:id="rId1"/>
@@ -1999,7 +1999,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="151">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2427,6 +2427,24 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2659,7 +2677,7 @@
     <col min="4" max="4" width="11.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8.33203125" style="33" customWidth="1"/>
     <col min="6" max="6" width="7.33203125" style="33" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="33" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" style="33" customWidth="1"/>
     <col min="8" max="8" width="7.33203125" style="33" customWidth="1"/>
     <col min="9" max="9" width="7.21875" style="33" customWidth="1"/>
     <col min="10" max="10" width="7.33203125" style="33" customWidth="1"/>
@@ -3199,89 +3217,89 @@
         <v>559</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="45">
+    <row r="7" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="89">
         <v>5</v>
       </c>
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="89" t="s">
         <v>380</v>
       </c>
-      <c r="E7" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="45">
+      <c r="E7" s="89" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="89">
         <v>262859</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="89" t="s">
         <v>547</v>
       </c>
-      <c r="H7" s="45">
+      <c r="H7" s="89">
         <v>600</v>
       </c>
-      <c r="I7" s="47">
+      <c r="I7" s="152">
         <v>1.236</v>
       </c>
-      <c r="J7" s="47">
+      <c r="J7" s="152">
         <v>2.5910000000000002</v>
       </c>
-      <c r="K7" s="45" t="s">
+      <c r="K7" s="89" t="s">
         <v>104</v>
       </c>
-      <c r="L7" s="47">
+      <c r="L7" s="152">
         <v>1921.4860000000001</v>
       </c>
-      <c r="M7" s="48">
+      <c r="M7" s="153">
         <v>1554.6</v>
       </c>
-      <c r="N7" s="49">
+      <c r="N7" s="154">
         <v>0.43180000000000002</v>
       </c>
-      <c r="O7" s="50">
+      <c r="O7" s="155">
         <v>25.91</v>
       </c>
-      <c r="P7" s="45">
+      <c r="P7" s="89">
         <v>1214.4000000000001</v>
       </c>
-      <c r="Q7" s="45">
+      <c r="Q7" s="89">
         <v>1</v>
       </c>
-      <c r="R7" s="45">
+      <c r="R7" s="89">
         <v>1300</v>
       </c>
-      <c r="S7" s="47">
+      <c r="S7" s="152">
         <v>1.236</v>
       </c>
-      <c r="T7" s="45">
+      <c r="T7" s="89">
         <v>64</v>
       </c>
-      <c r="U7" s="49">
+      <c r="U7" s="154">
         <v>4.9200000000000001E-2</v>
       </c>
-      <c r="V7" s="45" t="s">
+      <c r="V7" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="W7" s="45" t="s">
+      <c r="W7" s="89" t="s">
         <v>39</v>
       </c>
-      <c r="X7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="45" t="s">
+      <c r="X7" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="AA7" s="45" t="s">
+      <c r="AA7" s="89" t="s">
         <v>31</v>
       </c>
-      <c r="AB7" s="45" t="s">
+      <c r="AB7" s="89" t="s">
         <v>103</v>
       </c>
     </row>
@@ -3457,261 +3475,261 @@
         <v>555</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="45">
+    <row r="10" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="89">
         <v>8</v>
       </c>
-      <c r="B10" s="46" t="s">
+      <c r="B10" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="45" t="s">
+      <c r="C10" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="D10" s="89" t="s">
         <v>380</v>
       </c>
-      <c r="E10" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="45">
+      <c r="E10" s="89" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="89">
         <v>262858</v>
       </c>
-      <c r="G10" s="45" t="s">
+      <c r="G10" s="89" t="s">
         <v>547</v>
       </c>
-      <c r="H10" s="45">
+      <c r="H10" s="89">
         <v>1200</v>
       </c>
-      <c r="I10" s="47">
+      <c r="I10" s="152">
         <v>1.196</v>
       </c>
-      <c r="J10" s="47">
+      <c r="J10" s="152">
         <v>1.6910000000000001</v>
       </c>
-      <c r="K10" s="45" t="s">
+      <c r="K10" s="89" t="s">
         <v>101</v>
       </c>
-      <c r="L10" s="47">
+      <c r="L10" s="152">
         <v>2426.9229999999998</v>
       </c>
-      <c r="M10" s="48">
+      <c r="M10" s="153">
         <v>2029.2</v>
       </c>
-      <c r="N10" s="49">
+      <c r="N10" s="154">
         <v>0.56369999999999998</v>
       </c>
-      <c r="O10" s="50">
+      <c r="O10" s="155">
         <v>33.82</v>
       </c>
-      <c r="P10" s="45">
+      <c r="P10" s="89">
         <v>1533.8</v>
       </c>
-      <c r="Q10" s="45">
+      <c r="Q10" s="89">
         <v>1</v>
       </c>
-      <c r="R10" s="45">
+      <c r="R10" s="89">
         <v>1250</v>
       </c>
-      <c r="S10" s="47">
+      <c r="S10" s="152">
         <v>1.196</v>
       </c>
-      <c r="T10" s="45">
+      <c r="T10" s="89">
         <v>54</v>
       </c>
-      <c r="U10" s="49">
+      <c r="U10" s="154">
         <v>4.3200000000000002E-2</v>
       </c>
-      <c r="V10" s="45" t="s">
+      <c r="V10" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="W10" s="45" t="s">
+      <c r="W10" s="89" t="s">
         <v>39</v>
       </c>
-      <c r="X10" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z10" s="45" t="s">
+      <c r="X10" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z10" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="AA10" s="45" t="s">
+      <c r="AA10" s="89" t="s">
         <v>54</v>
       </c>
-      <c r="AB10" s="45" t="s">
+      <c r="AB10" s="89" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="45">
+    <row r="11" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="89">
         <v>9</v>
       </c>
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="C11" s="45" t="s">
+      <c r="C11" s="89" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="89" t="s">
         <v>380</v>
       </c>
-      <c r="E11" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="45">
+      <c r="E11" s="89" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="89">
         <v>262857</v>
       </c>
-      <c r="G11" s="45" t="s">
+      <c r="G11" s="89" t="s">
         <v>547</v>
       </c>
-      <c r="H11" s="45">
+      <c r="H11" s="89">
         <v>1700</v>
       </c>
-      <c r="I11" s="47">
+      <c r="I11" s="152">
         <v>1.2050000000000001</v>
       </c>
-      <c r="J11" s="47">
+      <c r="J11" s="152">
         <v>2.5110000000000001</v>
       </c>
-      <c r="K11" s="45" t="s">
+      <c r="K11" s="89" t="s">
         <v>554</v>
       </c>
-      <c r="L11" s="47">
+      <c r="L11" s="152">
         <v>5143.7839999999997</v>
       </c>
-      <c r="M11" s="48">
+      <c r="M11" s="153">
         <v>4268.7</v>
       </c>
-      <c r="N11" s="49">
+      <c r="N11" s="154">
         <v>1.1857</v>
       </c>
-      <c r="O11" s="50">
+      <c r="O11" s="155">
         <v>71.14</v>
       </c>
-      <c r="P11" s="45">
+      <c r="P11" s="89">
         <v>2921.7</v>
       </c>
-      <c r="Q11" s="45">
+      <c r="Q11" s="89">
         <v>1</v>
       </c>
-      <c r="R11" s="45">
+      <c r="R11" s="89">
         <v>1250</v>
       </c>
-      <c r="S11" s="47">
+      <c r="S11" s="152">
         <v>1.2050000000000001</v>
       </c>
-      <c r="T11" s="45">
+      <c r="T11" s="89">
         <v>45</v>
       </c>
-      <c r="U11" s="49">
+      <c r="U11" s="154">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="V11" s="45" t="s">
+      <c r="V11" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="W11" s="45" t="s">
+      <c r="W11" s="89" t="s">
         <v>39</v>
       </c>
-      <c r="X11" s="45" t="s">
+      <c r="X11" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="Y11" s="45" t="s">
+      <c r="Y11" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="Z11" s="45" t="s">
+      <c r="Z11" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="AA11" s="45" t="s">
+      <c r="AA11" s="89" t="s">
         <v>63</v>
       </c>
-      <c r="AB11" s="45" t="s">
+      <c r="AB11" s="89" t="s">
         <v>553</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="45">
+    <row r="12" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="89">
         <v>10</v>
       </c>
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="45" t="s">
+      <c r="C12" s="89" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="45" t="s">
+      <c r="D12" s="89" t="s">
         <v>380</v>
       </c>
-      <c r="E12" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="45">
+      <c r="E12" s="89" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="89">
         <v>262856</v>
       </c>
-      <c r="G12" s="45" t="s">
+      <c r="G12" s="89" t="s">
         <v>547</v>
       </c>
-      <c r="H12" s="45">
+      <c r="H12" s="89">
         <v>1400</v>
       </c>
-      <c r="I12" s="47">
+      <c r="I12" s="152">
         <v>1.2050000000000001</v>
       </c>
-      <c r="J12" s="47">
+      <c r="J12" s="152">
         <v>2.5910000000000002</v>
       </c>
-      <c r="K12" s="45" t="s">
+      <c r="K12" s="89" t="s">
         <v>50</v>
       </c>
-      <c r="L12" s="47">
+      <c r="L12" s="152">
         <v>4371.0169999999998</v>
       </c>
-      <c r="M12" s="48">
+      <c r="M12" s="153">
         <v>3627.4</v>
       </c>
-      <c r="N12" s="49">
+      <c r="N12" s="154">
         <v>1.0076000000000001</v>
       </c>
-      <c r="O12" s="50">
+      <c r="O12" s="155">
         <v>60.46</v>
       </c>
-      <c r="P12" s="45">
+      <c r="P12" s="89">
         <v>2482.6999999999998</v>
       </c>
-      <c r="Q12" s="45">
+      <c r="Q12" s="89">
         <v>1</v>
       </c>
-      <c r="R12" s="45">
+      <c r="R12" s="89">
         <v>1250</v>
       </c>
-      <c r="S12" s="47">
+      <c r="S12" s="152">
         <v>1.2050000000000001</v>
       </c>
-      <c r="T12" s="45">
+      <c r="T12" s="89">
         <v>45</v>
       </c>
-      <c r="U12" s="49">
+      <c r="U12" s="154">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="V12" s="45" t="s">
+      <c r="V12" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="W12" s="45" t="s">
+      <c r="W12" s="89" t="s">
         <v>39</v>
       </c>
-      <c r="X12" s="45" t="s">
+      <c r="X12" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="Y12" s="45" t="s">
+      <c r="Y12" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="Z12" s="45" t="s">
+      <c r="Z12" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="AA12" s="45" t="s">
+      <c r="AA12" s="89" t="s">
         <v>52</v>
       </c>
-      <c r="AB12" s="45" t="s">
+      <c r="AB12" s="89" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3887,89 +3905,89 @@
         <v>548</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="45">
+    <row r="15" spans="1:28" s="156" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="89">
         <v>13</v>
       </c>
-      <c r="B15" s="46" t="s">
+      <c r="B15" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="45" t="s">
+      <c r="C15" s="89" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="45" t="s">
+      <c r="D15" s="89" t="s">
         <v>380</v>
       </c>
-      <c r="E15" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="45">
+      <c r="E15" s="89" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="89">
         <v>262860</v>
       </c>
-      <c r="G15" s="45" t="s">
+      <c r="G15" s="89" t="s">
         <v>547</v>
       </c>
-      <c r="H15" s="45">
+      <c r="H15" s="89">
         <v>1300</v>
       </c>
-      <c r="I15" s="47">
+      <c r="I15" s="152">
         <v>0.97599999999999998</v>
       </c>
-      <c r="J15" s="47">
+      <c r="J15" s="152">
         <v>2.331</v>
       </c>
-      <c r="K15" s="45" t="s">
+      <c r="K15" s="89" t="s">
         <v>546</v>
       </c>
-      <c r="L15" s="47">
+      <c r="L15" s="152">
         <v>2957.5729999999999</v>
       </c>
-      <c r="M15" s="48">
+      <c r="M15" s="153">
         <v>3030.3</v>
       </c>
-      <c r="N15" s="49">
+      <c r="N15" s="154">
         <v>0.8417</v>
       </c>
-      <c r="O15" s="50">
+      <c r="O15" s="155">
         <v>50.5</v>
       </c>
-      <c r="P15" s="45">
+      <c r="P15" s="89">
         <v>1591.2</v>
       </c>
-      <c r="Q15" s="45">
+      <c r="Q15" s="89">
         <v>1</v>
       </c>
-      <c r="R15" s="45">
+      <c r="R15" s="89">
         <v>1000</v>
       </c>
-      <c r="S15" s="47">
+      <c r="S15" s="152">
         <v>0.97599999999999998</v>
       </c>
-      <c r="T15" s="45">
+      <c r="T15" s="89">
         <v>24</v>
       </c>
-      <c r="U15" s="49">
+      <c r="U15" s="154">
         <v>2.4E-2</v>
       </c>
-      <c r="V15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="45" t="s">
+      <c r="V15" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="X15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA15" s="45" t="s">
+      <c r="X15" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z15" s="89" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA15" s="89" t="s">
         <v>54</v>
       </c>
-      <c r="AB15" s="45" t="s">
+      <c r="AB15" s="89" t="s">
         <v>545</v>
       </c>
     </row>
@@ -4666,6 +4684,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9178,6 +9197,9 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD2CB328-92D9-4132-AB19-3AEA902CFC6F}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -9813,8 +9835,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.17" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="97" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 14:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AF219F-4326-4B4A-891D-89F187082164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E570DF-96F3-4137-81ED-B155F1CDF9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1249" sheetId="178" r:id="rId1"/>
@@ -1934,7 +1934,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1965,6 +1965,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF66"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1999,7 +2005,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2445,6 +2451,28 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="7" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="7" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="7" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="3" applyFill="1"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -24678,7 +24706,7 @@
     <col min="7" max="7" width="5.109375" style="33" customWidth="1"/>
     <col min="8" max="8" width="8" style="33" customWidth="1"/>
     <col min="9" max="9" width="10.77734375" style="33" customWidth="1"/>
-    <col min="10" max="10" width="7.109375" style="33" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="33" customWidth="1"/>
     <col min="11" max="11" width="21" style="33" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="33" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="33" hidden="1" customWidth="1"/>
@@ -24897,7 +24925,7 @@
       <c r="I3" s="116">
         <v>0.39400000000000002</v>
       </c>
-      <c r="J3" s="116">
+      <c r="J3" s="164">
         <v>1.07</v>
       </c>
       <c r="K3" s="116" t="s">
@@ -25381,7 +25409,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="1.79" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="78" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="77" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -27873,89 +27901,89 @@
         <v>476</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="106">
+    <row r="8" spans="1:28" s="163" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="157">
         <v>6</v>
       </c>
-      <c r="B8" s="107" t="s">
+      <c r="B8" s="158" t="s">
         <v>463</v>
       </c>
-      <c r="C8" s="106" t="s">
+      <c r="C8" s="157" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="106" t="s">
+      <c r="D8" s="157" t="s">
         <v>404</v>
       </c>
-      <c r="E8" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="106">
+      <c r="E8" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="157">
         <v>262794</v>
       </c>
-      <c r="G8" s="106" t="s">
+      <c r="G8" s="157" t="s">
         <v>462</v>
       </c>
-      <c r="H8" s="106">
+      <c r="H8" s="157">
         <v>5000</v>
       </c>
-      <c r="I8" s="108">
+      <c r="I8" s="159">
         <v>0.46</v>
       </c>
-      <c r="J8" s="108">
+      <c r="J8" s="159">
         <v>0.92</v>
       </c>
-      <c r="K8" s="106" t="s">
+      <c r="K8" s="157" t="s">
         <v>33</v>
       </c>
-      <c r="L8" s="108">
+      <c r="L8" s="159">
         <v>2116</v>
       </c>
-      <c r="M8" s="109">
+      <c r="M8" s="160">
         <v>1533.3</v>
       </c>
-      <c r="N8" s="110">
+      <c r="N8" s="161">
         <v>0.14199999999999999</v>
       </c>
-      <c r="O8" s="111">
+      <c r="O8" s="162">
         <v>8.52</v>
       </c>
-      <c r="P8" s="106">
+      <c r="P8" s="157">
         <v>666.5</v>
       </c>
-      <c r="Q8" s="106">
+      <c r="Q8" s="157">
         <v>3</v>
       </c>
-      <c r="R8" s="106">
+      <c r="R8" s="157">
         <v>1400</v>
       </c>
-      <c r="S8" s="108">
+      <c r="S8" s="159">
         <v>1.38</v>
       </c>
-      <c r="T8" s="106">
+      <c r="T8" s="157">
         <v>20</v>
       </c>
-      <c r="U8" s="110">
+      <c r="U8" s="161">
         <v>1.43E-2</v>
       </c>
-      <c r="V8" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="106" t="s">
+      <c r="V8" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="157" t="s">
         <v>31</v>
       </c>
-      <c r="AB8" s="106" t="s">
+      <c r="AB8" s="157" t="s">
         <v>475</v>
       </c>
     </row>
@@ -28131,89 +28159,89 @@
         <v>474</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="106">
+    <row r="11" spans="1:28" s="163" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="157">
         <v>9</v>
       </c>
-      <c r="B11" s="107" t="s">
+      <c r="B11" s="158" t="s">
         <v>463</v>
       </c>
-      <c r="C11" s="106" t="s">
+      <c r="C11" s="157" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="106" t="s">
+      <c r="D11" s="157" t="s">
         <v>404</v>
       </c>
-      <c r="E11" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="106">
+      <c r="E11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="157">
         <v>262795</v>
       </c>
-      <c r="G11" s="106" t="s">
+      <c r="G11" s="157" t="s">
         <v>462</v>
       </c>
-      <c r="H11" s="106">
+      <c r="H11" s="157">
         <v>1000</v>
       </c>
-      <c r="I11" s="108">
+      <c r="I11" s="159">
         <v>0.66</v>
       </c>
-      <c r="J11" s="108">
+      <c r="J11" s="159">
         <v>0.82</v>
       </c>
-      <c r="K11" s="106" t="s">
+      <c r="K11" s="157" t="s">
         <v>33</v>
       </c>
-      <c r="L11" s="108">
+      <c r="L11" s="159">
         <v>541.20000000000005</v>
       </c>
-      <c r="M11" s="109">
+      <c r="M11" s="160">
         <v>410</v>
       </c>
-      <c r="N11" s="110">
+      <c r="N11" s="161">
         <v>5.6899999999999999E-2</v>
       </c>
-      <c r="O11" s="111">
+      <c r="O11" s="162">
         <v>3.42</v>
       </c>
-      <c r="P11" s="106">
+      <c r="P11" s="157">
         <v>170.5</v>
       </c>
-      <c r="Q11" s="106">
+      <c r="Q11" s="157">
         <v>2</v>
       </c>
-      <c r="R11" s="106">
+      <c r="R11" s="157">
         <v>1350</v>
       </c>
-      <c r="S11" s="108">
+      <c r="S11" s="159">
         <v>1.32</v>
       </c>
-      <c r="T11" s="106">
+      <c r="T11" s="157">
         <v>30</v>
       </c>
-      <c r="U11" s="110">
+      <c r="U11" s="161">
         <v>2.2200000000000001E-2</v>
       </c>
-      <c r="V11" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="106" t="s">
+      <c r="V11" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="157" t="s">
         <v>38</v>
       </c>
-      <c r="AB11" s="106" t="s">
+      <c r="AB11" s="157" t="s">
         <v>473</v>
       </c>
     </row>
@@ -28475,89 +28503,89 @@
         <v>469</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="106">
+    <row r="15" spans="1:28" s="163" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="157">
         <v>13</v>
       </c>
-      <c r="B15" s="107" t="s">
+      <c r="B15" s="158" t="s">
         <v>463</v>
       </c>
-      <c r="C15" s="106" t="s">
+      <c r="C15" s="157" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="106" t="s">
+      <c r="D15" s="157" t="s">
         <v>404</v>
       </c>
-      <c r="E15" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="106">
+      <c r="E15" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="157">
         <v>262797</v>
       </c>
-      <c r="G15" s="106" t="s">
+      <c r="G15" s="157" t="s">
         <v>462</v>
       </c>
-      <c r="H15" s="106">
+      <c r="H15" s="157">
         <v>500</v>
       </c>
-      <c r="I15" s="108">
+      <c r="I15" s="159">
         <v>0.59</v>
       </c>
-      <c r="J15" s="108">
+      <c r="J15" s="159">
         <v>0.88</v>
       </c>
-      <c r="K15" s="106" t="s">
+      <c r="K15" s="157" t="s">
         <v>33</v>
       </c>
-      <c r="L15" s="108">
+      <c r="L15" s="159">
         <v>259.60000000000002</v>
       </c>
-      <c r="M15" s="109">
+      <c r="M15" s="160">
         <v>220</v>
       </c>
-      <c r="N15" s="110">
+      <c r="N15" s="161">
         <v>3.0599999999999999E-2</v>
       </c>
-      <c r="O15" s="111">
+      <c r="O15" s="162">
         <v>1.83</v>
       </c>
-      <c r="P15" s="106">
+      <c r="P15" s="157">
         <v>81.8</v>
       </c>
-      <c r="Q15" s="106">
+      <c r="Q15" s="157">
         <v>2</v>
       </c>
-      <c r="R15" s="106">
+      <c r="R15" s="157">
         <v>1200</v>
       </c>
-      <c r="S15" s="108">
+      <c r="S15" s="159">
         <v>1.18</v>
       </c>
-      <c r="T15" s="106">
+      <c r="T15" s="157">
         <v>20</v>
       </c>
-      <c r="U15" s="110">
+      <c r="U15" s="161">
         <v>1.67E-2</v>
       </c>
-      <c r="V15" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="X15" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="106" t="s">
+      <c r="V15" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="157" t="s">
         <v>38</v>
       </c>
-      <c r="AB15" s="106" t="s">
+      <c r="AB15" s="157" t="s">
         <v>468</v>
       </c>
     </row>
@@ -28647,89 +28675,89 @@
         <v>464</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="106">
+    <row r="17" spans="1:28" s="163" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="157">
         <v>15</v>
       </c>
-      <c r="B17" s="107" t="s">
+      <c r="B17" s="158" t="s">
         <v>463</v>
       </c>
-      <c r="C17" s="106" t="s">
+      <c r="C17" s="157" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="106" t="s">
+      <c r="D17" s="157" t="s">
         <v>404</v>
       </c>
-      <c r="E17" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="106">
+      <c r="E17" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="157">
         <v>262796</v>
       </c>
-      <c r="G17" s="106" t="s">
+      <c r="G17" s="157" t="s">
         <v>462</v>
       </c>
-      <c r="H17" s="106">
+      <c r="H17" s="157">
         <v>1000</v>
       </c>
-      <c r="I17" s="108">
+      <c r="I17" s="159">
         <v>0.56000000000000005</v>
       </c>
-      <c r="J17" s="108">
+      <c r="J17" s="159">
         <v>0.62</v>
       </c>
-      <c r="K17" s="106" t="s">
+      <c r="K17" s="157" t="s">
         <v>33</v>
       </c>
-      <c r="L17" s="108">
+      <c r="L17" s="159">
         <v>347.2</v>
       </c>
-      <c r="M17" s="109">
+      <c r="M17" s="160">
         <v>310</v>
       </c>
-      <c r="N17" s="110">
+      <c r="N17" s="161">
         <v>4.3099999999999999E-2</v>
       </c>
-      <c r="O17" s="111">
+      <c r="O17" s="162">
         <v>2.58</v>
       </c>
-      <c r="P17" s="106">
+      <c r="P17" s="157">
         <v>109.4</v>
       </c>
-      <c r="Q17" s="106">
+      <c r="Q17" s="157">
         <v>2</v>
       </c>
-      <c r="R17" s="106">
+      <c r="R17" s="157">
         <v>1150</v>
       </c>
-      <c r="S17" s="108">
+      <c r="S17" s="159">
         <v>1.1200000000000001</v>
       </c>
-      <c r="T17" s="106">
+      <c r="T17" s="157">
         <v>30</v>
       </c>
-      <c r="U17" s="110">
+      <c r="U17" s="161">
         <v>2.6100000000000002E-2</v>
       </c>
-      <c r="V17" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="W17" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="X17" s="106" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y17" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z17" s="106" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA17" s="106" t="s">
+      <c r="V17" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="W17" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="X17" s="157" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y17" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="157" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="157" t="s">
         <v>38</v>
       </c>
-      <c r="AB17" s="106" t="s">
+      <c r="AB17" s="157" t="s">
         <v>461</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 15:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA82C317-D1FB-4751-B47F-CB128B17E11F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1E8BF1-8EFA-4FBB-A9AB-E4287FA0B5B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2730,7 +2730,7 @@
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8" style="1" customWidth="1"/>
     <col min="6" max="6" width="7.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" style="1" customWidth="1"/>
     <col min="8" max="8" width="6.21875" style="1" customWidth="1"/>
     <col min="9" max="9" width="6.6640625" style="1" customWidth="1"/>
     <col min="10" max="10" width="7.21875" style="1" customWidth="1"/>
@@ -2934,7 +2934,7 @@
         <v>570</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>333</v>
@@ -3276,7 +3276,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="85" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="85" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/10/2026 15:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1E8BF1-8EFA-4FBB-A9AB-E4287FA0B5B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278E5CB9-B83F-495E-95CE-CBA8B8CFCBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR EMBALAGENS 1250" sheetId="179" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5426" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5433" uniqueCount="575">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -31531,7 +31531,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF841B48-E833-4DBA-8A4F-DEEF6290C316}">
-  <dimension ref="A1:AB18"/>
+  <dimension ref="A1:AB19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="33" customWidth="1"/>
@@ -32338,90 +32338,84 @@
         <v>385</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="45">
         <v>8</v>
       </c>
-      <c r="B10" s="150" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" s="145" t="s">
+      <c r="B10" s="46" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="145" t="s">
-        <v>483</v>
-      </c>
-      <c r="E10" s="145" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="145">
-        <v>262839</v>
-      </c>
-      <c r="G10" s="145" t="s">
-        <v>515</v>
-      </c>
-      <c r="H10" s="145">
-        <v>150</v>
-      </c>
-      <c r="I10" s="147">
-        <v>1.3160000000000001</v>
-      </c>
-      <c r="J10" s="147">
-        <v>1.244</v>
-      </c>
-      <c r="K10" s="145" t="s">
-        <v>514</v>
-      </c>
-      <c r="L10" s="147">
-        <v>245.566</v>
-      </c>
-      <c r="M10" s="149">
-        <v>186.6</v>
-      </c>
-      <c r="N10" s="146">
-        <v>5.1799999999999999E-2</v>
-      </c>
-      <c r="O10" s="148">
-        <v>3.11</v>
-      </c>
-      <c r="P10" s="145">
-        <v>77.400000000000006</v>
-      </c>
-      <c r="Q10" s="145">
-        <v>1</v>
-      </c>
-      <c r="R10" s="145">
-        <v>1350</v>
-      </c>
-      <c r="S10" s="147">
-        <v>1.3160000000000001</v>
-      </c>
-      <c r="T10" s="145">
-        <v>34</v>
-      </c>
-      <c r="U10" s="146">
-        <v>2.52E-2</v>
-      </c>
-      <c r="V10" s="145" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="145" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="145" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="145" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="145" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="145" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB10" s="145" t="s">
-        <v>513</v>
+      <c r="D10" s="61">
+        <v>46297</v>
+      </c>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45">
+        <v>262864</v>
+      </c>
+      <c r="G10" s="45">
+        <v>1798</v>
+      </c>
+      <c r="H10" s="45">
+        <v>2000</v>
+      </c>
+      <c r="I10" s="47">
+        <v>1.3</v>
+      </c>
+      <c r="J10" s="47">
+        <v>1.6</v>
+      </c>
+      <c r="K10" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="L10" s="47">
+        <v>4160</v>
+      </c>
+      <c r="M10" s="48">
+        <v>1066.7</v>
+      </c>
+      <c r="N10" s="49">
+        <v>9.8799999999999999E-2</v>
+      </c>
+      <c r="O10" s="50">
+        <v>5.93</v>
+      </c>
+      <c r="P10" s="45">
+        <v>1310.4000000000001</v>
+      </c>
+      <c r="Q10" s="45">
+        <v>3</v>
+      </c>
+      <c r="R10" s="45">
+        <v>1550</v>
+      </c>
+      <c r="S10" s="47">
+        <v>3.9</v>
+      </c>
+      <c r="T10" s="45">
+        <v>-2350</v>
+      </c>
+      <c r="U10" s="49">
+        <v>-1.5161</v>
+      </c>
+      <c r="V10" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="45"/>
+      <c r="Z10" s="45"/>
+      <c r="AA10" s="45">
+        <v>2</v>
+      </c>
+      <c r="AB10" s="45" t="s">
+        <v>572</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -32441,52 +32435,52 @@
         <v>27</v>
       </c>
       <c r="F11" s="145">
-        <v>262835</v>
+        <v>262839</v>
       </c>
       <c r="G11" s="145" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H11" s="145">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="I11" s="147">
-        <v>0.6</v>
+        <v>1.3160000000000001</v>
       </c>
       <c r="J11" s="147">
-        <v>2.367</v>
+        <v>1.244</v>
       </c>
       <c r="K11" s="145" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="L11" s="147">
-        <v>710.1</v>
+        <v>245.566</v>
       </c>
       <c r="M11" s="149">
-        <v>591.79999999999995</v>
+        <v>186.6</v>
       </c>
       <c r="N11" s="146">
-        <v>8.2199999999999995E-2</v>
+        <v>5.1799999999999999E-2</v>
       </c>
       <c r="O11" s="148">
-        <v>4.93</v>
+        <v>3.11</v>
       </c>
       <c r="P11" s="145">
-        <v>223.7</v>
+        <v>77.400000000000006</v>
       </c>
       <c r="Q11" s="145">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R11" s="145">
-        <v>1250</v>
+        <v>1350</v>
       </c>
       <c r="S11" s="147">
-        <v>1.2</v>
+        <v>1.3160000000000001</v>
       </c>
       <c r="T11" s="145">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="U11" s="146">
-        <v>0.04</v>
+        <v>2.52E-2</v>
       </c>
       <c r="V11" s="145" t="s">
         <v>28</v>
@@ -32504,10 +32498,10 @@
         <v>27</v>
       </c>
       <c r="AA11" s="145" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="AB11" s="145" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -32527,52 +32521,52 @@
         <v>27</v>
       </c>
       <c r="F12" s="145">
-        <v>262834</v>
+        <v>262835</v>
       </c>
       <c r="G12" s="145" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H12" s="145">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I12" s="147">
-        <v>1.1100000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J12" s="147">
-        <v>2.3029999999999999</v>
+        <v>2.367</v>
       </c>
       <c r="K12" s="145" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="L12" s="147">
-        <v>511.26600000000002</v>
+        <v>710.1</v>
       </c>
       <c r="M12" s="149">
-        <v>460.6</v>
+        <v>591.79999999999995</v>
       </c>
       <c r="N12" s="146">
-        <v>0.12790000000000001</v>
+        <v>8.2199999999999995E-2</v>
       </c>
       <c r="O12" s="148">
-        <v>7.68</v>
+        <v>4.93</v>
       </c>
       <c r="P12" s="145">
-        <v>161</v>
+        <v>223.7</v>
       </c>
       <c r="Q12" s="145">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="145">
-        <v>1150</v>
+        <v>1250</v>
       </c>
       <c r="S12" s="147">
-        <v>1.1100000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="T12" s="145">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="U12" s="146">
-        <v>3.4799999999999998E-2</v>
+        <v>0.04</v>
       </c>
       <c r="V12" s="145" t="s">
         <v>28</v>
@@ -32590,10 +32584,10 @@
         <v>27</v>
       </c>
       <c r="AA12" s="145" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="AB12" s="145" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -32613,52 +32607,52 @@
         <v>27</v>
       </c>
       <c r="F13" s="145">
-        <v>262838</v>
+        <v>262834</v>
       </c>
       <c r="G13" s="145" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="H13" s="145">
-        <v>1200</v>
+        <v>200</v>
       </c>
       <c r="I13" s="147">
-        <v>0.99299999999999999</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="J13" s="147">
-        <v>0.627</v>
+        <v>2.3029999999999999</v>
       </c>
       <c r="K13" s="145" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="L13" s="147">
-        <v>747.13300000000004</v>
+        <v>511.26600000000002</v>
       </c>
       <c r="M13" s="149">
-        <v>752.4</v>
+        <v>460.6</v>
       </c>
       <c r="N13" s="146">
-        <v>0.20899999999999999</v>
+        <v>0.12790000000000001</v>
       </c>
       <c r="O13" s="148">
-        <v>12.54</v>
+        <v>7.68</v>
       </c>
       <c r="P13" s="145">
-        <v>235.3</v>
+        <v>161</v>
       </c>
       <c r="Q13" s="145">
         <v>1</v>
       </c>
       <c r="R13" s="145">
-        <v>1050</v>
+        <v>1150</v>
       </c>
       <c r="S13" s="147">
-        <v>0.99299999999999999</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="T13" s="145">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="U13" s="146">
-        <v>5.4300000000000001E-2</v>
+        <v>3.4799999999999998E-2</v>
       </c>
       <c r="V13" s="145" t="s">
         <v>28</v>
@@ -32679,7 +32673,7 @@
         <v>38</v>
       </c>
       <c r="AB13" s="145" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -32699,37 +32693,37 @@
         <v>27</v>
       </c>
       <c r="F14" s="145">
-        <v>262836</v>
+        <v>262838</v>
       </c>
       <c r="G14" s="145" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="H14" s="145">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="I14" s="147">
-        <v>1</v>
+        <v>0.99299999999999999</v>
       </c>
       <c r="J14" s="147">
-        <v>3.4</v>
+        <v>0.627</v>
       </c>
       <c r="K14" s="145" t="s">
-        <v>33</v>
+        <v>523</v>
       </c>
       <c r="L14" s="147">
-        <v>2720</v>
+        <v>747.13300000000004</v>
       </c>
       <c r="M14" s="149">
-        <v>2720</v>
+        <v>752.4</v>
       </c>
       <c r="N14" s="146">
-        <v>0.75560000000000005</v>
+        <v>0.20899999999999999</v>
       </c>
       <c r="O14" s="148">
-        <v>45.33</v>
+        <v>12.54</v>
       </c>
       <c r="P14" s="145">
-        <v>856.8</v>
+        <v>235.3</v>
       </c>
       <c r="Q14" s="145">
         <v>1</v>
@@ -32738,13 +32732,13 @@
         <v>1050</v>
       </c>
       <c r="S14" s="147">
-        <v>1</v>
+        <v>0.99299999999999999</v>
       </c>
       <c r="T14" s="145">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="U14" s="146">
-        <v>4.7600000000000003E-2</v>
+        <v>5.4300000000000001E-2</v>
       </c>
       <c r="V14" s="145" t="s">
         <v>28</v>
@@ -32762,96 +32756,96 @@
         <v>27</v>
       </c>
       <c r="AA14" s="145" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="AB14" s="145" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="45">
         <v>13</v>
       </c>
-      <c r="B15" s="46" t="s">
+      <c r="B15" s="150" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="45" t="s">
+      <c r="C15" s="145" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="45" t="s">
-        <v>380</v>
-      </c>
-      <c r="E15" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="45">
-        <v>262737</v>
-      </c>
-      <c r="G15" s="45" t="s">
-        <v>379</v>
-      </c>
-      <c r="H15" s="45">
-        <v>600</v>
-      </c>
-      <c r="I15" s="47">
-        <v>0.47</v>
-      </c>
-      <c r="J15" s="47">
-        <v>1.7869999999999999</v>
-      </c>
-      <c r="K15" s="45" t="s">
-        <v>384</v>
-      </c>
-      <c r="L15" s="47">
-        <v>503.93400000000003</v>
-      </c>
-      <c r="M15" s="48">
-        <v>536.1</v>
-      </c>
-      <c r="N15" s="49">
-        <v>7.4499999999999997E-2</v>
-      </c>
-      <c r="O15" s="50">
-        <v>4.47</v>
-      </c>
-      <c r="P15" s="45">
-        <v>158.69999999999999</v>
-      </c>
-      <c r="Q15" s="45">
-        <v>2</v>
-      </c>
-      <c r="R15" s="45">
-        <v>1000</v>
-      </c>
-      <c r="S15" s="47">
-        <v>0.94</v>
-      </c>
-      <c r="T15" s="45">
-        <v>60</v>
-      </c>
-      <c r="U15" s="49">
-        <v>0.06</v>
-      </c>
-      <c r="V15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="X15" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB15" s="45" t="s">
-        <v>383</v>
+      <c r="D15" s="145" t="s">
+        <v>483</v>
+      </c>
+      <c r="E15" s="145" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="145">
+        <v>262836</v>
+      </c>
+      <c r="G15" s="145" t="s">
+        <v>526</v>
+      </c>
+      <c r="H15" s="145">
+        <v>800</v>
+      </c>
+      <c r="I15" s="147">
+        <v>1</v>
+      </c>
+      <c r="J15" s="147">
+        <v>3.4</v>
+      </c>
+      <c r="K15" s="145" t="s">
+        <v>33</v>
+      </c>
+      <c r="L15" s="147">
+        <v>2720</v>
+      </c>
+      <c r="M15" s="149">
+        <v>2720</v>
+      </c>
+      <c r="N15" s="146">
+        <v>0.75560000000000005</v>
+      </c>
+      <c r="O15" s="148">
+        <v>45.33</v>
+      </c>
+      <c r="P15" s="145">
+        <v>856.8</v>
+      </c>
+      <c r="Q15" s="145">
+        <v>1</v>
+      </c>
+      <c r="R15" s="145">
+        <v>1050</v>
+      </c>
+      <c r="S15" s="147">
+        <v>1</v>
+      </c>
+      <c r="T15" s="145">
+        <v>50</v>
+      </c>
+      <c r="U15" s="146">
+        <v>4.7600000000000003E-2</v>
+      </c>
+      <c r="V15" s="145" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="145" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="145" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="145" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="145" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="145" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB15" s="145" t="s">
+        <v>525</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -32871,52 +32865,52 @@
         <v>27</v>
       </c>
       <c r="F16" s="45">
-        <v>262739</v>
+        <v>262737</v>
       </c>
       <c r="G16" s="45" t="s">
         <v>379</v>
       </c>
       <c r="H16" s="45">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="I16" s="47">
-        <v>0.86</v>
+        <v>0.47</v>
       </c>
       <c r="J16" s="47">
-        <v>1.8029999999999999</v>
+        <v>1.7869999999999999</v>
       </c>
       <c r="K16" s="45" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="L16" s="47">
-        <v>465.17399999999998</v>
+        <v>503.93400000000003</v>
       </c>
       <c r="M16" s="48">
-        <v>540.9</v>
+        <v>536.1</v>
       </c>
       <c r="N16" s="49">
-        <v>0.1502</v>
+        <v>7.4499999999999997E-2</v>
       </c>
       <c r="O16" s="50">
-        <v>9.01</v>
+        <v>4.47</v>
       </c>
       <c r="P16" s="45">
-        <v>146.5</v>
+        <v>158.69999999999999</v>
       </c>
       <c r="Q16" s="45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R16" s="45">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="S16" s="47">
-        <v>0.86</v>
+        <v>0.94</v>
       </c>
       <c r="T16" s="45">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="U16" s="49">
-        <v>4.4400000000000002E-2</v>
+        <v>0.06</v>
       </c>
       <c r="V16" s="45" t="s">
         <v>28</v>
@@ -32937,7 +32931,7 @@
         <v>38</v>
       </c>
       <c r="AB16" s="45" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -32957,52 +32951,52 @@
         <v>27</v>
       </c>
       <c r="F17" s="45">
-        <v>262738</v>
+        <v>262739</v>
       </c>
       <c r="G17" s="45" t="s">
         <v>379</v>
       </c>
       <c r="H17" s="45">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="I17" s="47">
-        <v>0.39</v>
+        <v>0.86</v>
       </c>
       <c r="J17" s="47">
-        <v>1.7829999999999999</v>
+        <v>1.8029999999999999</v>
       </c>
       <c r="K17" s="45" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="L17" s="47">
-        <v>417.22199999999998</v>
+        <v>465.17399999999998</v>
       </c>
       <c r="M17" s="48">
-        <v>534.9</v>
+        <v>540.9</v>
       </c>
       <c r="N17" s="49">
-        <v>7.4300000000000005E-2</v>
+        <v>0.1502</v>
       </c>
       <c r="O17" s="50">
-        <v>4.46</v>
+        <v>9.01</v>
       </c>
       <c r="P17" s="45">
-        <v>131.4</v>
+        <v>146.5</v>
       </c>
       <c r="Q17" s="45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R17" s="45">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="S17" s="47">
-        <v>0.78</v>
+        <v>0.86</v>
       </c>
       <c r="T17" s="45">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="U17" s="49">
-        <v>2.5000000000000001E-2</v>
+        <v>4.4400000000000002E-2</v>
       </c>
       <c r="V17" s="45" t="s">
         <v>28</v>
@@ -33023,94 +33017,180 @@
         <v>38</v>
       </c>
       <c r="AB17" s="45" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="45">
+        <v>16</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="45" t="s">
+        <v>380</v>
+      </c>
+      <c r="E18" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="45">
+        <v>262738</v>
+      </c>
+      <c r="G18" s="45" t="s">
+        <v>379</v>
+      </c>
+      <c r="H18" s="45">
+        <v>600</v>
+      </c>
+      <c r="I18" s="47">
+        <v>0.39</v>
+      </c>
+      <c r="J18" s="47">
+        <v>1.7829999999999999</v>
+      </c>
+      <c r="K18" s="45" t="s">
+        <v>378</v>
+      </c>
+      <c r="L18" s="47">
+        <v>417.22199999999998</v>
+      </c>
+      <c r="M18" s="48">
+        <v>534.9</v>
+      </c>
+      <c r="N18" s="49">
+        <v>7.4300000000000005E-2</v>
+      </c>
+      <c r="O18" s="50">
+        <v>4.46</v>
+      </c>
+      <c r="P18" s="45">
+        <v>131.4</v>
+      </c>
+      <c r="Q18" s="45">
+        <v>2</v>
+      </c>
+      <c r="R18" s="45">
+        <v>800</v>
+      </c>
+      <c r="S18" s="47">
+        <v>0.78</v>
+      </c>
+      <c r="T18" s="45">
+        <v>20</v>
+      </c>
+      <c r="U18" s="49">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="V18" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="W18" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="X18" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y18" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="45" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB18" s="45" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="D18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="H18" s="52">
-        <f>SUM(H3:H17)</f>
-        <v>7840</v>
-      </c>
-      <c r="I18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="J18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="K18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="L18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="M18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="N18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="O18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="P18" s="52">
-        <f>SUM(P3:P17)</f>
-        <v>3853.9</v>
-      </c>
-      <c r="Q18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="R18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="S18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="T18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="U18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="V18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="W18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="X18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA18" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB18" s="52" t="s">
+    <row r="19" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" s="52">
+        <f>SUM(H3:H18)</f>
+        <v>9840</v>
+      </c>
+      <c r="I19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="K19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="L19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="M19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="O19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="P19" s="52">
+        <f>SUM(P3:P18)</f>
+        <v>5164.2999999999993</v>
+      </c>
+      <c r="Q19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="R19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="S19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="T19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="U19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="V19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="W19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="X19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB19" s="52" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (05/10/2026 09:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CEE783B-4EEC-4F75-91F3-210808B74177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9959169-1EA4-4549-BD6C-B0E71EF567EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR EMBALAGENS 1250" sheetId="179" r:id="rId1"/>
-    <sheet name="HARMONY EMBALAGENS 1249" sheetId="178" r:id="rId2"/>
+    <sheet name="HARMONY EMBALAGENS 1249 P" sheetId="178" r:id="rId2"/>
     <sheet name="FAVINCO 1248 AMOSTRA" sheetId="177" r:id="rId3"/>
     <sheet name="ABAPEL 1246" sheetId="176" r:id="rId4"/>
     <sheet name="FAVINCO 1243 P" sheetId="175" r:id="rId5"/>
@@ -14307,7 +14307,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A982AD08-A19C-4AB3-8139-90400A7A453C}">
-  <dimension ref="A1:AB23"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="33" customWidth="1"/>
@@ -14341,88 +14344,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="158" t="s">
+      <c r="A1" s="162" t="s">
         <v>567</v>
       </c>
-      <c r="B1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="158" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="158" t="s">
+      <c r="B1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="162" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="162" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14512,7 +14515,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="45">
         <v>1</v>
       </c>
@@ -14598,7 +14601,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="45">
         <v>2</v>
       </c>
@@ -14684,7 +14687,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="45">
         <v>3</v>
       </c>
@@ -14770,7 +14773,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="45">
         <v>4</v>
       </c>
@@ -14856,7 +14859,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="148" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="89">
         <v>5</v>
       </c>
@@ -14942,7 +14945,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="45">
         <v>6</v>
       </c>
@@ -15028,7 +15031,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="45">
         <v>7</v>
       </c>
@@ -15114,7 +15117,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="148" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="89">
         <v>8</v>
       </c>
@@ -15200,7 +15203,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="148" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="89">
         <v>9</v>
       </c>
@@ -15286,7 +15289,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="148" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89">
         <v>10</v>
       </c>
@@ -15372,7 +15375,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="45">
         <v>11</v>
       </c>
@@ -15458,7 +15461,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="45">
         <v>12</v>
       </c>
@@ -15544,7 +15547,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="148" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="89">
         <v>13</v>
       </c>
@@ -15630,7 +15633,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="45">
         <v>14</v>
       </c>
@@ -15716,7 +15719,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="45">
         <v>15</v>
       </c>
@@ -15802,7 +15805,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="45">
         <v>16</v>
       </c>
@@ -15888,7 +15891,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="45">
         <v>17</v>
       </c>
@@ -15974,7 +15977,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="20" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="45">
         <v>18</v>
       </c>
@@ -16060,7 +16063,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="21" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="45">
         <v>19</v>
       </c>
@@ -16146,7 +16149,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="22" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="45">
         <v>20</v>
       </c>
@@ -16232,7 +16235,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="23" spans="1:28" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="52" t="s">
         <v>27</v>
       </c>
@@ -16318,12 +16321,14 @@
         <v>27</v>
       </c>
     </row>
+    <row r="24" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="81" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -31531,6 +31536,9 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF841B48-E833-4DBA-8A4F-DEEF6290C316}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -31650,7 +31658,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="44" t="s">
         <v>0</v>
       </c>
@@ -33199,6 +33207,6 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup scale="93" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (05/10/2026 10:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075DB83B-CF0F-428F-BF1E-D1E56B133A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF46A25-667E-44F0-86FC-066BF26619DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2737,28 +2737,32 @@
   <dimension ref="A1:AB5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.77734375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="4.44140625" style="1" customWidth="1"/>
+    <col min="8" max="9" width="6.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.21875" style="1" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="8.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="13.77734375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="11.77734375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="6.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.21875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.6640625" style="1" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="26" width="11.77734375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="10.77734375" style="1" customWidth="1"/>
-    <col min="28" max="28" width="16.77734375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="8.33203125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.44140625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.21875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="10.109375" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.6640625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10.5546875" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
@@ -2848,7 +2852,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (05/10/2026 11:13)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A316E6-FD51-4C96-8D53-D0B97F039A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD9D4E2-0FA0-4065-A337-D60D25DE509C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RR STELLA 1253" sheetId="181" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5649" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5648" uniqueCount="587">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -15426,8 +15426,8 @@
       <c r="F4" s="126">
         <v>262866</v>
       </c>
-      <c r="G4" s="126" t="s">
-        <v>576</v>
+      <c r="G4" s="126">
+        <v>83</v>
       </c>
       <c r="H4" s="126">
         <v>1000</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (05/10/2026 15:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099EA770-8F96-4CD7-8CF7-41073B9A3D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6960A02B-4981-4184-95C0-6E74ECC4E621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="10" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE EMBALAGENS LTDA 1254" sheetId="182" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (05/10/2026 15:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6960A02B-4981-4184-95C0-6E74ECC4E621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFDBC572-9731-4EAA-A8C3-C6AD5DAE4334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="10" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-10830" windowWidth="38620" windowHeight="21100" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE EMBALAGENS LTDA 1254" sheetId="182" r:id="rId1"/>
@@ -1193,9 +1193,6 @@
     <t>1298x1810</t>
   </si>
   <si>
-    <t>PROGRAMAÇÃO ONDULADEIRA - RM Embalagens ( Daiane Marques Canossa ME )  —  OF: 001232</t>
-  </si>
-  <si>
     <t>1190x1803</t>
   </si>
   <si>
@@ -1854,6 +1851,9 @@
   </si>
   <si>
     <t>780x2198</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - RM Embalagens   —  OF: 001232</t>
   </si>
 </sst>
 </file>
@@ -2096,7 +2096,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2544,6 +2544,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2801,7 +2802,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="152" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B1" s="152" t="s">
         <v>27</v>
@@ -2982,7 +2983,7 @@
         <v>35</v>
       </c>
       <c r="D3" s="126" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="E3" s="126" t="s">
         <v>27</v>
@@ -2991,7 +2992,7 @@
         <v>262870</v>
       </c>
       <c r="G3" s="126" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="H3" s="126">
         <v>200</v>
@@ -3054,7 +3055,7 @@
         <v>38</v>
       </c>
       <c r="AB3" s="121" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -3191,7 +3192,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="154" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B1" s="154" t="s">
         <v>27</v>
@@ -3452,13 +3453,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="101" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C4" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D4" s="100" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E4" s="100" t="s">
         <v>27</v>
@@ -3467,7 +3468,7 @@
         <v>262800</v>
       </c>
       <c r="G4" s="100" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="H4" s="100">
         <v>1000</v>
@@ -3530,7 +3531,7 @@
         <v>38</v>
       </c>
       <c r="AB4" s="100" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="106" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3624,7 +3625,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="101" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C6" s="100" t="s">
         <v>35</v>
@@ -3637,7 +3638,7 @@
         <v>262827</v>
       </c>
       <c r="G6" s="100" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="H6" s="100">
         <v>1000</v>
@@ -3696,7 +3697,7 @@
         <v>1</v>
       </c>
       <c r="AB6" s="100" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="106" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3704,13 +3705,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="101" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C7" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D7" s="100" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E7" s="100" t="s">
         <v>27</v>
@@ -3719,7 +3720,7 @@
         <v>262802</v>
       </c>
       <c r="G7" s="100" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H7" s="100">
         <v>2000</v>
@@ -3782,7 +3783,7 @@
         <v>38</v>
       </c>
       <c r="AB7" s="100" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3790,13 +3791,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="143" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C8" s="142" t="s">
         <v>35</v>
       </c>
       <c r="D8" s="142" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E8" s="142" t="s">
         <v>27</v>
@@ -3805,7 +3806,7 @@
         <v>262794</v>
       </c>
       <c r="G8" s="142" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="H8" s="142">
         <v>5000</v>
@@ -3868,7 +3869,7 @@
         <v>31</v>
       </c>
       <c r="AB8" s="142" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="106" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3876,13 +3877,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="101" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C9" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D9" s="100" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E9" s="100" t="s">
         <v>27</v>
@@ -3891,7 +3892,7 @@
         <v>262804</v>
       </c>
       <c r="G9" s="100" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H9" s="100">
         <v>2000</v>
@@ -3962,13 +3963,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="101" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C10" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D10" s="100" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E10" s="100" t="s">
         <v>27</v>
@@ -3977,7 +3978,7 @@
         <v>262799</v>
       </c>
       <c r="G10" s="100" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="H10" s="100">
         <v>1000</v>
@@ -4040,7 +4041,7 @@
         <v>38</v>
       </c>
       <c r="AB10" s="100" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4048,13 +4049,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="143" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C11" s="142" t="s">
         <v>35</v>
       </c>
       <c r="D11" s="142" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E11" s="142" t="s">
         <v>27</v>
@@ -4063,7 +4064,7 @@
         <v>262795</v>
       </c>
       <c r="G11" s="142" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="H11" s="142">
         <v>1000</v>
@@ -4126,7 +4127,7 @@
         <v>38</v>
       </c>
       <c r="AB11" s="142" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="106" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4220,13 +4221,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="101" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C13" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D13" s="100" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E13" s="100" t="s">
         <v>27</v>
@@ -4235,7 +4236,7 @@
         <v>262798</v>
       </c>
       <c r="G13" s="100" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="H13" s="100">
         <v>300</v>
@@ -4298,7 +4299,7 @@
         <v>38</v>
       </c>
       <c r="AB13" s="100" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="106" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4306,13 +4307,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="101" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C14" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D14" s="100" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E14" s="100" t="s">
         <v>27</v>
@@ -4321,7 +4322,7 @@
         <v>262803</v>
       </c>
       <c r="G14" s="100" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H14" s="100">
         <v>2000</v>
@@ -4384,7 +4385,7 @@
         <v>32</v>
       </c>
       <c r="AB14" s="100" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4392,13 +4393,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="143" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C15" s="142" t="s">
         <v>35</v>
       </c>
       <c r="D15" s="142" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E15" s="142" t="s">
         <v>27</v>
@@ -4407,7 +4408,7 @@
         <v>262797</v>
       </c>
       <c r="G15" s="142" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="H15" s="142">
         <v>500</v>
@@ -4470,7 +4471,7 @@
         <v>38</v>
       </c>
       <c r="AB15" s="142" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="106" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4478,13 +4479,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="101" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C16" s="100" t="s">
         <v>35</v>
       </c>
       <c r="D16" s="100" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E16" s="100" t="s">
         <v>27</v>
@@ -4493,7 +4494,7 @@
         <v>262801</v>
       </c>
       <c r="G16" s="100" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H16" s="100">
         <v>1000</v>
@@ -4556,7 +4557,7 @@
         <v>32</v>
       </c>
       <c r="AB16" s="100" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="148" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4564,13 +4565,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="143" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C17" s="142" t="s">
         <v>35</v>
       </c>
       <c r="D17" s="142" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E17" s="142" t="s">
         <v>27</v>
@@ -4579,7 +4580,7 @@
         <v>262796</v>
       </c>
       <c r="G17" s="142" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="H17" s="142">
         <v>1000</v>
@@ -4642,7 +4643,7 @@
         <v>38</v>
       </c>
       <c r="AB17" s="142" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="18" spans="1:28" s="106" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4822,7 +4823,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="101" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C20" s="100" t="s">
         <v>35</v>
@@ -4835,7 +4836,7 @@
         <v>262826</v>
       </c>
       <c r="G20" s="100" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H20" s="100">
         <v>1000</v>
@@ -4894,7 +4895,7 @@
         <v>1</v>
       </c>
       <c r="AB20" s="100" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.3">
@@ -5063,7 +5064,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="155" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B1" s="155" t="s">
         <v>27</v>
@@ -5244,7 +5245,7 @@
         <v>144</v>
       </c>
       <c r="D3" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E3" s="53" t="s">
         <v>27</v>
@@ -5253,7 +5254,7 @@
         <v>262787</v>
       </c>
       <c r="G3" s="53" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="H3" s="53">
         <v>650</v>
@@ -5265,7 +5266,7 @@
         <v>1.5620000000000001</v>
       </c>
       <c r="K3" s="53" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="L3" s="55">
         <v>519.83399999999995</v>
@@ -5316,7 +5317,7 @@
         <v>38</v>
       </c>
       <c r="AB3" s="53" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="59" customFormat="1" x14ac:dyDescent="0.3">
@@ -5330,7 +5331,7 @@
         <v>35</v>
       </c>
       <c r="D4" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E4" s="53" t="s">
         <v>27</v>
@@ -5339,7 +5340,7 @@
         <v>262785</v>
       </c>
       <c r="G4" s="53" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="H4" s="53">
         <v>1000</v>
@@ -5416,7 +5417,7 @@
         <v>35</v>
       </c>
       <c r="D5" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E5" s="53" t="s">
         <v>27</v>
@@ -5425,7 +5426,7 @@
         <v>262784</v>
       </c>
       <c r="G5" s="53" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="H5" s="53">
         <v>1000</v>
@@ -5502,7 +5503,7 @@
         <v>144</v>
       </c>
       <c r="D6" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E6" s="53" t="s">
         <v>27</v>
@@ -5511,7 +5512,7 @@
         <v>262786</v>
       </c>
       <c r="G6" s="53" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="H6" s="53">
         <v>1000</v>
@@ -5523,7 +5524,7 @@
         <v>1.3879999999999999</v>
       </c>
       <c r="K6" s="53" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="L6" s="55">
         <v>581.572</v>
@@ -5574,7 +5575,7 @@
         <v>32</v>
       </c>
       <c r="AB6" s="53" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="59" customFormat="1" x14ac:dyDescent="0.3">
@@ -5588,7 +5589,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E7" s="53" t="s">
         <v>27</v>
@@ -5597,7 +5598,7 @@
         <v>262783</v>
       </c>
       <c r="G7" s="53" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="H7" s="53">
         <v>1000</v>
@@ -5660,7 +5661,7 @@
         <v>38</v>
       </c>
       <c r="AB7" s="53" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="59" customFormat="1" x14ac:dyDescent="0.3">
@@ -5668,7 +5669,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="54" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C8" s="53" t="s">
         <v>35</v>
@@ -5754,7 +5755,7 @@
         <v>35</v>
       </c>
       <c r="D9" s="53" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E9" s="53" t="s">
         <v>27</v>
@@ -5763,7 +5764,7 @@
         <v>262782</v>
       </c>
       <c r="G9" s="53" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="H9" s="53">
         <v>1000</v>
@@ -5965,7 +5966,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="155" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B1" s="155" t="s">
         <v>27</v>
@@ -6146,7 +6147,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E3" s="45" t="s">
         <v>27</v>
@@ -6155,7 +6156,7 @@
         <v>262736</v>
       </c>
       <c r="G3" s="45" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H3" s="45">
         <v>150</v>
@@ -6167,7 +6168,7 @@
         <v>1.6830000000000001</v>
       </c>
       <c r="K3" s="45" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L3" s="47">
         <v>378.17</v>
@@ -6218,7 +6219,7 @@
         <v>38</v>
       </c>
       <c r="AB3" s="45" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6232,7 +6233,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E4" s="45" t="s">
         <v>27</v>
@@ -6241,7 +6242,7 @@
         <v>262735</v>
       </c>
       <c r="G4" s="45" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H4" s="45">
         <v>150</v>
@@ -6253,7 +6254,7 @@
         <v>2.0830000000000002</v>
       </c>
       <c r="K4" s="45" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="L4" s="47">
         <v>464.92599999999999</v>
@@ -6304,7 +6305,7 @@
         <v>38</v>
       </c>
       <c r="AB4" s="45" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6318,7 +6319,7 @@
         <v>44</v>
       </c>
       <c r="D5" s="130" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E5" s="130" t="s">
         <v>27</v>
@@ -6327,7 +6328,7 @@
         <v>262837</v>
       </c>
       <c r="G5" s="130" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H5" s="130">
         <v>140</v>
@@ -6339,7 +6340,7 @@
         <v>2.2309999999999999</v>
       </c>
       <c r="K5" s="130" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="L5" s="132">
         <v>466.63600000000002</v>
@@ -6390,7 +6391,7 @@
         <v>38</v>
       </c>
       <c r="AB5" s="130" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6404,7 +6405,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E6" s="45" t="s">
         <v>27</v>
@@ -6413,7 +6414,7 @@
         <v>262733</v>
       </c>
       <c r="G6" s="45" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H6" s="45">
         <v>150</v>
@@ -6425,7 +6426,7 @@
         <v>2.0030000000000001</v>
       </c>
       <c r="K6" s="45" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L6" s="47">
         <v>444.065</v>
@@ -6476,7 +6477,7 @@
         <v>38</v>
       </c>
       <c r="AB6" s="45" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6490,7 +6491,7 @@
         <v>26</v>
       </c>
       <c r="D7" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E7" s="45" t="s">
         <v>27</v>
@@ -6499,7 +6500,7 @@
         <v>262734</v>
       </c>
       <c r="G7" s="45" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H7" s="45">
         <v>150</v>
@@ -6511,7 +6512,7 @@
         <v>2.0830000000000002</v>
       </c>
       <c r="K7" s="45" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="L7" s="47">
         <v>418.05799999999999</v>
@@ -6562,7 +6563,7 @@
         <v>38</v>
       </c>
       <c r="AB7" s="45" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6576,7 +6577,7 @@
         <v>45</v>
       </c>
       <c r="D8" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E8" s="45" t="s">
         <v>27</v>
@@ -6585,7 +6586,7 @@
         <v>262731</v>
       </c>
       <c r="G8" s="45" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H8" s="45">
         <v>1250</v>
@@ -6648,7 +6649,7 @@
         <v>32</v>
       </c>
       <c r="AB8" s="45" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6662,7 +6663,7 @@
         <v>45</v>
       </c>
       <c r="D9" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E9" s="45" t="s">
         <v>27</v>
@@ -6671,7 +6672,7 @@
         <v>262732</v>
       </c>
       <c r="G9" s="45" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H9" s="45">
         <v>1500</v>
@@ -6734,7 +6735,7 @@
         <v>30</v>
       </c>
       <c r="AB9" s="45" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6814,7 +6815,7 @@
         <v>2</v>
       </c>
       <c r="AB10" s="45" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6828,7 +6829,7 @@
         <v>35</v>
       </c>
       <c r="D11" s="130" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E11" s="130" t="s">
         <v>27</v>
@@ -6837,7 +6838,7 @@
         <v>262839</v>
       </c>
       <c r="G11" s="130" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="H11" s="130">
         <v>150</v>
@@ -6849,7 +6850,7 @@
         <v>1.244</v>
       </c>
       <c r="K11" s="130" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="L11" s="132">
         <v>245.566</v>
@@ -6900,7 +6901,7 @@
         <v>38</v>
       </c>
       <c r="AB11" s="130" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6914,7 +6915,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="130" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E12" s="130" t="s">
         <v>27</v>
@@ -6923,7 +6924,7 @@
         <v>262835</v>
       </c>
       <c r="G12" s="130" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="H12" s="130">
         <v>500</v>
@@ -6935,7 +6936,7 @@
         <v>2.367</v>
       </c>
       <c r="K12" s="130" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="L12" s="132">
         <v>710.1</v>
@@ -6986,7 +6987,7 @@
         <v>32</v>
       </c>
       <c r="AB12" s="130" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7000,7 +7001,7 @@
         <v>35</v>
       </c>
       <c r="D13" s="130" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E13" s="130" t="s">
         <v>27</v>
@@ -7009,7 +7010,7 @@
         <v>262834</v>
       </c>
       <c r="G13" s="130" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H13" s="130">
         <v>200</v>
@@ -7021,7 +7022,7 @@
         <v>2.3029999999999999</v>
       </c>
       <c r="K13" s="130" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L13" s="132">
         <v>511.26600000000002</v>
@@ -7072,7 +7073,7 @@
         <v>38</v>
       </c>
       <c r="AB13" s="130" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7086,7 +7087,7 @@
         <v>35</v>
       </c>
       <c r="D14" s="130" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E14" s="130" t="s">
         <v>27</v>
@@ -7095,7 +7096,7 @@
         <v>262838</v>
       </c>
       <c r="G14" s="130" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H14" s="130">
         <v>1200</v>
@@ -7107,7 +7108,7 @@
         <v>0.627</v>
       </c>
       <c r="K14" s="130" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="L14" s="132">
         <v>747.13300000000004</v>
@@ -7158,7 +7159,7 @@
         <v>38</v>
       </c>
       <c r="AB14" s="130" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="98" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7172,7 +7173,7 @@
         <v>35</v>
       </c>
       <c r="D15" s="130" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E15" s="130" t="s">
         <v>27</v>
@@ -7181,7 +7182,7 @@
         <v>262836</v>
       </c>
       <c r="G15" s="130" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H15" s="130">
         <v>800</v>
@@ -7244,7 +7245,7 @@
         <v>32</v>
       </c>
       <c r="AB15" s="130" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7258,7 +7259,7 @@
         <v>35</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E16" s="45" t="s">
         <v>27</v>
@@ -7267,7 +7268,7 @@
         <v>262737</v>
       </c>
       <c r="G16" s="45" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H16" s="45">
         <v>600</v>
@@ -7279,7 +7280,7 @@
         <v>1.7869999999999999</v>
       </c>
       <c r="K16" s="45" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="L16" s="47">
         <v>503.93400000000003</v>
@@ -7330,7 +7331,7 @@
         <v>38</v>
       </c>
       <c r="AB16" s="45" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7344,7 +7345,7 @@
         <v>35</v>
       </c>
       <c r="D17" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E17" s="45" t="s">
         <v>27</v>
@@ -7353,7 +7354,7 @@
         <v>262739</v>
       </c>
       <c r="G17" s="45" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H17" s="45">
         <v>300</v>
@@ -7365,7 +7366,7 @@
         <v>1.8029999999999999</v>
       </c>
       <c r="K17" s="45" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="L17" s="47">
         <v>465.17399999999998</v>
@@ -7416,7 +7417,7 @@
         <v>38</v>
       </c>
       <c r="AB17" s="45" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="18" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7430,7 +7431,7 @@
         <v>35</v>
       </c>
       <c r="D18" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E18" s="45" t="s">
         <v>27</v>
@@ -7439,7 +7440,7 @@
         <v>262738</v>
       </c>
       <c r="G18" s="45" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H18" s="45">
         <v>600</v>
@@ -7451,7 +7452,7 @@
         <v>1.7829999999999999</v>
       </c>
       <c r="K18" s="45" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="L18" s="47">
         <v>417.22199999999998</v>
@@ -7502,7 +7503,7 @@
         <v>38</v>
       </c>
       <c r="AB18" s="45" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="19" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7637,8 +7638,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="151" t="s">
-        <v>376</v>
+      <c r="A1" s="159" t="s">
+        <v>596</v>
       </c>
       <c r="B1" s="151" t="s">
         <v>27</v>
@@ -15327,7 +15328,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="152" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B1" s="152" t="s">
         <v>27</v>
@@ -15502,13 +15503,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="128" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="C3" s="126" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D3" s="126" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E3" s="126" t="s">
         <v>27</v>
@@ -15517,7 +15518,7 @@
         <v>262868</v>
       </c>
       <c r="G3" s="126" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="H3" s="126">
         <v>2000</v>
@@ -15580,7 +15581,7 @@
         <v>32</v>
       </c>
       <c r="AB3" s="121" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -15588,13 +15589,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="128" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="C4" s="126" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D4" s="126" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E4" s="126" t="s">
         <v>27</v>
@@ -15603,7 +15604,7 @@
         <v>262867</v>
       </c>
       <c r="G4" s="126" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="H4" s="126">
         <v>7000</v>
@@ -15666,7 +15667,7 @@
         <v>40</v>
       </c>
       <c r="AB4" s="121" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -15984,7 +15985,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="91" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E3" s="91" t="s">
         <v>27</v>
@@ -15993,7 +15994,7 @@
         <v>262778</v>
       </c>
       <c r="G3" s="91" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="H3" s="91">
         <v>430</v>
@@ -16005,7 +16006,7 @@
         <v>1.64</v>
       </c>
       <c r="K3" s="91" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="L3" s="93">
         <v>530.30999999999995</v>
@@ -16056,7 +16057,7 @@
         <v>30</v>
       </c>
       <c r="AB3" s="91" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="90" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16070,7 +16071,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="91" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E4" s="91" t="s">
         <v>27</v>
@@ -16079,7 +16080,7 @@
         <v>262777</v>
       </c>
       <c r="G4" s="91" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H4" s="91">
         <v>450</v>
@@ -16091,7 +16092,7 @@
         <v>2.11</v>
       </c>
       <c r="K4" s="91" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="L4" s="93">
         <v>695.98299999999995</v>
@@ -16142,7 +16143,7 @@
         <v>30</v>
       </c>
       <c r="AB4" s="91" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="90" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16156,7 +16157,7 @@
         <v>26</v>
       </c>
       <c r="D5" s="91" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E5" s="91" t="s">
         <v>27</v>
@@ -16165,7 +16166,7 @@
         <v>262774</v>
       </c>
       <c r="G5" s="91" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H5" s="91">
         <v>550</v>
@@ -16177,7 +16178,7 @@
         <v>1.4990000000000001</v>
       </c>
       <c r="K5" s="91" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L5" s="93">
         <v>582.88599999999997</v>
@@ -16228,7 +16229,7 @@
         <v>30</v>
       </c>
       <c r="AB5" s="91" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="90" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16242,7 +16243,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="91" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E6" s="91" t="s">
         <v>27</v>
@@ -16251,7 +16252,7 @@
         <v>262775</v>
       </c>
       <c r="G6" s="91" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H6" s="91">
         <v>385</v>
@@ -16263,7 +16264,7 @@
         <v>2.0990000000000002</v>
       </c>
       <c r="K6" s="91" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="L6" s="93">
         <v>576.18600000000004</v>
@@ -16314,7 +16315,7 @@
         <v>32</v>
       </c>
       <c r="AB6" s="91" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="90" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16400,7 +16401,7 @@
         <v>30</v>
       </c>
       <c r="AB7" s="91" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="90" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16586,7 +16587,7 @@
         <v>26</v>
       </c>
       <c r="D10" s="91" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E10" s="91" t="s">
         <v>27</v>
@@ -16595,7 +16596,7 @@
         <v>262776</v>
       </c>
       <c r="G10" s="91" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H10" s="91">
         <v>285</v>
@@ -16658,7 +16659,7 @@
         <v>32</v>
       </c>
       <c r="AB10" s="91" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="90" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16672,7 +16673,7 @@
         <v>26</v>
       </c>
       <c r="D11" s="91" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E11" s="91" t="s">
         <v>27</v>
@@ -16681,7 +16682,7 @@
         <v>262779</v>
       </c>
       <c r="G11" s="91" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="H11" s="91">
         <v>450</v>
@@ -16744,7 +16745,7 @@
         <v>30</v>
       </c>
       <c r="AB11" s="91" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="90" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -16758,7 +16759,7 @@
         <v>59</v>
       </c>
       <c r="D12" s="91" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E12" s="91" t="s">
         <v>27</v>
@@ -16767,7 +16768,7 @@
         <v>262772</v>
       </c>
       <c r="G12" s="91" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="H12" s="91">
         <v>9500</v>
@@ -16844,7 +16845,7 @@
         <v>59</v>
       </c>
       <c r="D13" s="91" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E13" s="91" t="s">
         <v>27</v>
@@ -16853,7 +16854,7 @@
         <v>262773</v>
       </c>
       <c r="G13" s="91" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="H13" s="91">
         <v>930</v>
@@ -27306,7 +27307,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="152" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B1" s="152" t="s">
         <v>27</v>
@@ -27487,7 +27488,7 @@
         <v>35</v>
       </c>
       <c r="D3" s="126" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E3" s="126" t="s">
         <v>27</v>
@@ -27496,7 +27497,7 @@
         <v>262865</v>
       </c>
       <c r="G3" s="126" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="H3" s="126">
         <v>1400</v>
@@ -27508,7 +27509,7 @@
         <v>0.83</v>
       </c>
       <c r="K3" s="126" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="L3" s="123">
         <v>517.09</v>
@@ -27559,7 +27560,7 @@
         <v>38</v>
       </c>
       <c r="AB3" s="121" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -27573,7 +27574,7 @@
         <v>35</v>
       </c>
       <c r="D4" s="126" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E4" s="126" t="s">
         <v>27</v>
@@ -27645,7 +27646,7 @@
         <v>38</v>
       </c>
       <c r="AB4" s="121" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -28430,7 +28431,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="150" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B1" s="150" t="s">
         <v>27</v>
@@ -28605,7 +28606,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>55</v>
@@ -28620,7 +28621,7 @@
         <v>262863</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="H3" s="5">
         <v>2000</v>
@@ -28683,7 +28684,7 @@
         <v>32</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -28691,13 +28692,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>27</v>
@@ -28706,7 +28707,7 @@
         <v>262861</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="H4" s="5">
         <v>2550</v>
@@ -28769,7 +28770,7 @@
         <v>30</v>
       </c>
       <c r="AB4" s="5" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -28777,13 +28778,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>27</v>
@@ -28792,7 +28793,7 @@
         <v>262862</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="H5" s="5">
         <v>500</v>
@@ -28855,7 +28856,7 @@
         <v>38</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -28994,7 +28995,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="155" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B1" s="155" t="s">
         <v>27</v>
@@ -29175,7 +29176,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E3" s="45" t="s">
         <v>27</v>
@@ -29184,7 +29185,7 @@
         <v>262848</v>
       </c>
       <c r="G3" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H3" s="45">
         <v>300</v>
@@ -29196,7 +29197,7 @@
         <v>1.7789999999999999</v>
       </c>
       <c r="K3" s="45" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L3" s="47">
         <v>263.64800000000002</v>
@@ -29247,7 +29248,7 @@
         <v>38</v>
       </c>
       <c r="AB3" s="45" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -29261,7 +29262,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E4" s="45" t="s">
         <v>27</v>
@@ -29270,7 +29271,7 @@
         <v>262853</v>
       </c>
       <c r="G4" s="45" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H4" s="45">
         <v>1000</v>
@@ -29282,7 +29283,7 @@
         <v>1.7190000000000001</v>
       </c>
       <c r="K4" s="45" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L4" s="47">
         <v>1287.5309999999999</v>
@@ -29333,7 +29334,7 @@
         <v>40</v>
       </c>
       <c r="AB4" s="45" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -29347,7 +29348,7 @@
         <v>26</v>
       </c>
       <c r="D5" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E5" s="45" t="s">
         <v>27</v>
@@ -29356,7 +29357,7 @@
         <v>262844</v>
       </c>
       <c r="G5" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H5" s="45">
         <v>400</v>
@@ -29368,7 +29369,7 @@
         <v>1.7190000000000001</v>
       </c>
       <c r="K5" s="45" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="L5" s="47">
         <v>511.57400000000001</v>
@@ -29419,7 +29420,7 @@
         <v>30</v>
       </c>
       <c r="AB5" s="45" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -29433,7 +29434,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E6" s="45" t="s">
         <v>27</v>
@@ -29442,7 +29443,7 @@
         <v>262854</v>
       </c>
       <c r="G6" s="45" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H6" s="45">
         <v>400</v>
@@ -29454,7 +29455,7 @@
         <v>1.0589999999999999</v>
       </c>
       <c r="K6" s="45" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="L6" s="47">
         <v>143.6</v>
@@ -29505,7 +29506,7 @@
         <v>38</v>
       </c>
       <c r="AB6" s="45" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="141" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -29519,7 +29520,7 @@
         <v>57</v>
       </c>
       <c r="D7" s="89" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E7" s="89" t="s">
         <v>27</v>
@@ -29528,7 +29529,7 @@
         <v>262859</v>
       </c>
       <c r="G7" s="89" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H7" s="89">
         <v>600</v>
@@ -29605,7 +29606,7 @@
         <v>26</v>
       </c>
       <c r="D8" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E8" s="45" t="s">
         <v>27</v>
@@ -29614,7 +29615,7 @@
         <v>262855</v>
       </c>
       <c r="G8" s="45" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H8" s="45">
         <v>200</v>
@@ -29626,7 +29627,7 @@
         <v>1.2589999999999999</v>
       </c>
       <c r="K8" s="45" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="L8" s="47">
         <v>154.60499999999999</v>
@@ -29677,7 +29678,7 @@
         <v>32</v>
       </c>
       <c r="AB8" s="45" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -29691,7 +29692,7 @@
         <v>26</v>
       </c>
       <c r="D9" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E9" s="45" t="s">
         <v>27</v>
@@ -29700,7 +29701,7 @@
         <v>262843</v>
       </c>
       <c r="G9" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H9" s="45">
         <v>500</v>
@@ -29712,7 +29713,7 @@
         <v>1.629</v>
       </c>
       <c r="K9" s="45" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="L9" s="47">
         <v>488.7</v>
@@ -29763,7 +29764,7 @@
         <v>30</v>
       </c>
       <c r="AB9" s="45" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="141" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -29777,7 +29778,7 @@
         <v>57</v>
       </c>
       <c r="D10" s="89" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E10" s="89" t="s">
         <v>27</v>
@@ -29786,7 +29787,7 @@
         <v>262858</v>
       </c>
       <c r="G10" s="89" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H10" s="89">
         <v>1200</v>
@@ -29863,7 +29864,7 @@
         <v>44</v>
       </c>
       <c r="D11" s="89" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E11" s="89" t="s">
         <v>27</v>
@@ -29872,7 +29873,7 @@
         <v>262857</v>
       </c>
       <c r="G11" s="89" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H11" s="89">
         <v>1700</v>
@@ -29884,7 +29885,7 @@
         <v>2.5110000000000001</v>
       </c>
       <c r="K11" s="89" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="L11" s="137">
         <v>5143.7839999999997</v>
@@ -29935,7 +29936,7 @@
         <v>63</v>
       </c>
       <c r="AB11" s="89" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="141" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -29949,7 +29950,7 @@
         <v>44</v>
       </c>
       <c r="D12" s="89" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E12" s="89" t="s">
         <v>27</v>
@@ -29958,7 +29959,7 @@
         <v>262856</v>
       </c>
       <c r="G12" s="89" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H12" s="89">
         <v>1400</v>
@@ -30035,7 +30036,7 @@
         <v>26</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E13" s="45" t="s">
         <v>27</v>
@@ -30044,7 +30045,7 @@
         <v>262851</v>
       </c>
       <c r="G13" s="45" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H13" s="45">
         <v>15000</v>
@@ -30056,7 +30057,7 @@
         <v>0.95899999999999996</v>
       </c>
       <c r="K13" s="45" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L13" s="47">
         <v>4229.1899999999996</v>
@@ -30104,10 +30105,10 @@
         <v>28</v>
       </c>
       <c r="AA13" s="45" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="AB13" s="45" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30121,7 +30122,7 @@
         <v>26</v>
       </c>
       <c r="D14" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E14" s="45" t="s">
         <v>27</v>
@@ -30130,7 +30131,7 @@
         <v>262841</v>
       </c>
       <c r="G14" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H14" s="45">
         <v>300</v>
@@ -30142,7 +30143,7 @@
         <v>2.024</v>
       </c>
       <c r="K14" s="45" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="L14" s="47">
         <v>626.02300000000002</v>
@@ -30193,7 +30194,7 @@
         <v>32</v>
       </c>
       <c r="AB14" s="45" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="141" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30207,7 +30208,7 @@
         <v>26</v>
       </c>
       <c r="D15" s="89" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E15" s="89" t="s">
         <v>27</v>
@@ -30216,7 +30217,7 @@
         <v>262860</v>
       </c>
       <c r="G15" s="89" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H15" s="89">
         <v>1300</v>
@@ -30228,7 +30229,7 @@
         <v>2.331</v>
       </c>
       <c r="K15" s="89" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="L15" s="137">
         <v>2957.5729999999999</v>
@@ -30279,7 +30280,7 @@
         <v>54</v>
       </c>
       <c r="AB15" s="89" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30293,7 +30294,7 @@
         <v>44</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E16" s="45" t="s">
         <v>27</v>
@@ -30302,7 +30303,7 @@
         <v>262845</v>
       </c>
       <c r="G16" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H16" s="45">
         <v>200</v>
@@ -30314,7 +30315,7 @@
         <v>2.069</v>
       </c>
       <c r="K16" s="45" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="L16" s="47">
         <v>349.24700000000001</v>
@@ -30365,7 +30366,7 @@
         <v>32</v>
       </c>
       <c r="AB16" s="45" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30379,7 +30380,7 @@
         <v>35</v>
       </c>
       <c r="D17" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E17" s="45" t="s">
         <v>27</v>
@@ -30388,7 +30389,7 @@
         <v>262842</v>
       </c>
       <c r="G17" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H17" s="45">
         <v>1500</v>
@@ -30400,7 +30401,7 @@
         <v>1.0129999999999999</v>
       </c>
       <c r="K17" s="45" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="L17" s="47">
         <v>572.851</v>
@@ -30451,7 +30452,7 @@
         <v>38</v>
       </c>
       <c r="AB17" s="45" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="18" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30465,7 +30466,7 @@
         <v>35</v>
       </c>
       <c r="D18" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E18" s="45" t="s">
         <v>27</v>
@@ -30474,7 +30475,7 @@
         <v>262846</v>
       </c>
       <c r="G18" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H18" s="45">
         <v>550</v>
@@ -30486,7 +30487,7 @@
         <v>1.409</v>
       </c>
       <c r="K18" s="45" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="L18" s="47">
         <v>382.82499999999999</v>
@@ -30537,7 +30538,7 @@
         <v>38</v>
       </c>
       <c r="AB18" s="45" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="19" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30551,7 +30552,7 @@
         <v>35</v>
       </c>
       <c r="D19" s="45" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E19" s="45" t="s">
         <v>27</v>
@@ -30560,7 +30561,7 @@
         <v>262847</v>
       </c>
       <c r="G19" s="45" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H19" s="45">
         <v>350</v>
@@ -30572,7 +30573,7 @@
         <v>1.929</v>
       </c>
       <c r="K19" s="45" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L19" s="47">
         <v>506.363</v>
@@ -30623,7 +30624,7 @@
         <v>38</v>
       </c>
       <c r="AB19" s="45" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="20" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30637,7 +30638,7 @@
         <v>35</v>
       </c>
       <c r="D20" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E20" s="45" t="s">
         <v>27</v>
@@ -30646,7 +30647,7 @@
         <v>262852</v>
       </c>
       <c r="G20" s="45" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H20" s="45">
         <v>1500</v>
@@ -30658,7 +30659,7 @@
         <v>0.95299999999999996</v>
       </c>
       <c r="K20" s="45" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L20" s="47">
         <v>517.47900000000004</v>
@@ -30709,7 +30710,7 @@
         <v>38</v>
       </c>
       <c r="AB20" s="45" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="21" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30723,7 +30724,7 @@
         <v>35</v>
       </c>
       <c r="D21" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E21" s="45" t="s">
         <v>27</v>
@@ -30732,7 +30733,7 @@
         <v>262849</v>
       </c>
       <c r="G21" s="45" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H21" s="45">
         <v>3000</v>
@@ -30744,7 +30745,7 @@
         <v>0.90900000000000003</v>
       </c>
       <c r="K21" s="45" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="L21" s="47">
         <v>1210.788</v>
@@ -30795,7 +30796,7 @@
         <v>32</v>
       </c>
       <c r="AB21" s="45" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="22" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -30809,7 +30810,7 @@
         <v>35</v>
       </c>
       <c r="D22" s="45" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E22" s="45" t="s">
         <v>27</v>
@@ -30818,7 +30819,7 @@
         <v>262850</v>
       </c>
       <c r="G22" s="45" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H22" s="45">
         <v>400</v>
@@ -30881,7 +30882,7 @@
         <v>38</v>
       </c>
       <c r="AB22" s="45" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="23" spans="1:28" s="51" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -31021,7 +31022,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="150" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B1" s="150" t="s">
         <v>27</v>
@@ -31202,7 +31203,7 @@
         <v>44</v>
       </c>
       <c r="D3" s="126" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="E3" s="126" t="s">
         <v>27</v>
@@ -31211,7 +31212,7 @@
         <v>262840</v>
       </c>
       <c r="G3" s="126" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="H3" s="126">
         <v>6</v>
@@ -31274,7 +31275,7 @@
         <v>38</v>
       </c>
       <c r="AB3" s="121" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -31413,7 +31414,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="150" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B1" s="150" t="s">
         <v>27</v>
@@ -31594,7 +31595,7 @@
         <v>26</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>27</v>
@@ -31603,7 +31604,7 @@
         <v>262830</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="H3" s="5">
         <v>1100</v>
@@ -31615,7 +31616,7 @@
         <v>2.68</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L3" s="7">
         <v>1524.116</v>
@@ -31666,7 +31667,7 @@
         <v>40</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -31680,7 +31681,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>27</v>
@@ -31689,7 +31690,7 @@
         <v>262832</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="H4" s="5">
         <v>660</v>
@@ -31701,7 +31702,7 @@
         <v>2.1</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L4" s="7">
         <v>1264.0319999999999</v>
@@ -31752,7 +31753,7 @@
         <v>31</v>
       </c>
       <c r="AB4" s="5" t="s">
- 